<commit_message>
LLenando las descripciones y tablas del muestreo de datos
</commit_message>
<xml_diff>
--- a/Muestreo de datos.xlsx
+++ b/Muestreo de datos.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\leand\Desktop\DOO\DOO\Extra clase\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jesus\OneDrive\Escritorio\leo\Doo\Barberia proyecto\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2CCD1F91-2196-458D-9B07-860EEE4AAA01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D5778858-64E9-47C9-A2D8-63B1F0A5B398}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="5" xr2:uid="{09A6C7D7-663F-4C06-9D71-8A4E97495CF9}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{09A6C7D7-663F-4C06-9D71-8A4E97495CF9}"/>
   </bookViews>
   <sheets>
     <sheet name="Modelo de Dominio" sheetId="1" r:id="rId1"/>
@@ -52,7 +52,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="137" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="177" uniqueCount="111">
   <si>
     <t>Nombre</t>
   </si>
@@ -162,118 +162,229 @@
     <t>fecha</t>
   </si>
   <si>
+    <t>Representa los dias y horas en que algo está disponible para operar, un rango de hora de inicio y hora de fin, asociado a un día de la semana. Se usa en dos contextos distintos dentro del sistema en Barberia, representa cuando abre y cierra el negocio en general, en Agenda representa en que dias y horas trabaja un barbero específico, siempre dentro de los limites que ya definió la Barbería.</t>
+  </si>
+  <si>
+    <t>barberoId</t>
+  </si>
+  <si>
+    <t>servicioId</t>
+  </si>
+  <si>
+    <t>idAgenda</t>
+  </si>
+  <si>
+    <t>clienteId</t>
+  </si>
+  <si>
+    <t>agendaId</t>
+  </si>
+  <si>
+    <t>hora_inicio</t>
+  </si>
+  <si>
+    <t>estado</t>
+  </si>
+  <si>
+    <t>citaId</t>
+  </si>
+  <si>
+    <t>monto</t>
+  </si>
+  <si>
+    <t>pagada</t>
+  </si>
+  <si>
+    <t>precioAlMomento</t>
+  </si>
+  <si>
+    <t>duracionAlMomento</t>
+  </si>
+  <si>
+    <t>id</t>
+  </si>
+  <si>
+    <t>&lt;&lt;&lt;&lt; Ir al modulo de dominio</t>
+  </si>
+  <si>
+    <t>&lt;&lt;&lt;&lt; Ir a objetos de dominio</t>
+  </si>
+  <si>
+    <t>aquí</t>
+  </si>
+  <si>
+    <t>Reprsenta el numero de celular de la persona que le va aescribir al barbero por WhatsApp para pedirle una cita</t>
+  </si>
+  <si>
+    <t>Combinación única 1</t>
+  </si>
+  <si>
+    <t>Juan Gómez</t>
+  </si>
+  <si>
+    <t>Simon Ramirez Perez</t>
+  </si>
+  <si>
+    <t>Representa el nombre completo (pude ser un apellido o dos pedendiendo lo que el barbero necesite) de la persona, que va a estar llendo a la barberia para las citas</t>
+  </si>
+  <si>
+    <t>Simon Ochoa Ramirez</t>
+  </si>
+  <si>
+    <t>Alexis Gallego</t>
+  </si>
+  <si>
+    <t>Combinacion única que indica que no puede existir más de un departamento dentro del mismo pais</t>
+  </si>
+  <si>
+    <t>toleranciaTardanza</t>
+  </si>
+  <si>
+    <t>Representa la cantidad de minutos que el cliente puede llegarle tarde un cliente a la cita establecida con el barbero, despues de eso el barbero lo podrá multar</t>
+  </si>
+  <si>
+    <t>Representa la maxima de multas que pueda tener un cliente sin pagar, a partir de esta cantidad se le hace un veto al cliente</t>
+  </si>
+  <si>
+    <t>barberia</t>
+  </si>
+  <si>
+    <t>Representa el nombre del servicio que va estar en la barberia, que el barbero ofrece y en las citas que esta</t>
+  </si>
+  <si>
+    <t>duracion</t>
+  </si>
+  <si>
+    <t>Representa lo que va durar en minutos el servicio</t>
+  </si>
+  <si>
+    <t>Representa cuanto va a valer el servicio en pesos colombianos</t>
+  </si>
+  <si>
+    <t>Representa la cantidad de dinero que el cliente debe de pagar en pesos colombianos, por superar la toleranciaTardanza</t>
+  </si>
+  <si>
+    <t>Revisar la logica de Regla, Multa y Barberia</t>
+  </si>
+  <si>
+    <t>Se tenia planeado que fuera el precio de los servicios</t>
+  </si>
+  <si>
+    <t>Motilada</t>
+  </si>
+  <si>
+    <t>Ir a objetos de dominio &gt;&gt;&gt;&gt;</t>
+  </si>
+  <si>
+    <t>barbero</t>
+  </si>
+  <si>
+    <t>servicio</t>
+  </si>
+  <si>
+    <t>correo</t>
+  </si>
+  <si>
+    <t>vigente</t>
+  </si>
+  <si>
+    <t>cliente</t>
+  </si>
+  <si>
+    <t>Corregir</t>
+  </si>
+  <si>
+    <t>Corregir Barberia o barbero</t>
+  </si>
+  <si>
+    <t>combinacion unica 1</t>
+  </si>
+  <si>
+    <t>Combinacion única que indica que no puede existir más de un servicio con el mismo nombre</t>
+  </si>
+  <si>
+    <t>Corte de barba</t>
+  </si>
+  <si>
+    <t>Perfilada de barba</t>
+  </si>
+  <si>
+    <t>Arreglo completo de barba con toalla caliente</t>
+  </si>
+  <si>
+    <t>Representa el nombre del barbero que trabaja en barbería</t>
+  </si>
+  <si>
+    <t>Representa el numero de celular del barbero</t>
+  </si>
+  <si>
+    <t>Representa si el barbero sigue o no trabajando en la barberia</t>
+  </si>
+  <si>
+    <t>si</t>
+  </si>
+  <si>
+    <t>no</t>
+  </si>
+  <si>
+    <t>apellidos</t>
+  </si>
+  <si>
+    <t>Representa los dos apellidos del barbero que trabaja en la barbería</t>
+  </si>
+  <si>
+    <t>Combinacion única que indica que no puede existir más de un barbero con el mismo numero de celular</t>
+  </si>
+  <si>
+    <t>Juan Fernando</t>
+  </si>
+  <si>
+    <t>Juan David</t>
+  </si>
+  <si>
+    <t>Carlos</t>
+  </si>
+  <si>
+    <t>Andres</t>
+  </si>
+  <si>
+    <t>García Lopez</t>
+  </si>
+  <si>
+    <t>Ortiz Sanchez</t>
+  </si>
+  <si>
+    <t>Arbeladez Montoya</t>
+  </si>
+  <si>
+    <t>Ramirez Patiño</t>
+  </si>
+  <si>
+    <t>juanfer234535@gmail.com</t>
+  </si>
+  <si>
+    <t>Representa el correo electronico del barbero</t>
+  </si>
+  <si>
+    <t>juandaviddd2525@gmail.com</t>
+  </si>
+  <si>
+    <t>carlosbeladez@gmail.com</t>
+  </si>
+  <si>
+    <t>andresramirezpatino123@gmail.com</t>
+  </si>
+  <si>
     <t>activo</t>
   </si>
   <si>
-    <t>Representa los dias y horas en que algo está disponible para operar, un rango de hora de inicio y hora de fin, asociado a un día de la semana. Se usa en dos contextos distintos dentro del sistema en Barberia, representa cuando abre y cierra el negocio en general, en Agenda representa en que dias y horas trabaja un barbero específico, siempre dentro de los limites que ya definió la Barbería.</t>
-  </si>
-  <si>
-    <t>barberoId</t>
-  </si>
-  <si>
-    <t>servicioId</t>
-  </si>
-  <si>
-    <t>idAgenda</t>
-  </si>
-  <si>
-    <t>clienteId</t>
-  </si>
-  <si>
-    <t>agendaId</t>
-  </si>
-  <si>
-    <t>hora_inicio</t>
-  </si>
-  <si>
-    <t>estado</t>
-  </si>
-  <si>
-    <t>citaId</t>
-  </si>
-  <si>
-    <t>monto</t>
-  </si>
-  <si>
-    <t>pagada</t>
-  </si>
-  <si>
-    <t>precioAlMomento</t>
-  </si>
-  <si>
-    <t>duracionAlMomento</t>
-  </si>
-  <si>
-    <t>id</t>
-  </si>
-  <si>
-    <t>&lt;&lt;&lt;&lt; Ir al modulo de dominio</t>
-  </si>
-  <si>
-    <t>&lt;&lt;&lt;&lt; Ir a objetos de dominio</t>
-  </si>
-  <si>
-    <t>aquí</t>
-  </si>
-  <si>
-    <t>Reprsenta el numero de celular de la persona que le va aescribir al barbero por WhatsApp para pedirle una cita</t>
-  </si>
-  <si>
-    <t>Combinación única 1</t>
-  </si>
-  <si>
-    <t>Juan Gómez</t>
-  </si>
-  <si>
-    <t>Simon Ramirez Perez</t>
-  </si>
-  <si>
-    <t>Representa el nombre completo (pude ser un apellido o dos pedendiendo lo que el barbero necesite) de la persona, que va a estar llendo a la barberia para las citas</t>
-  </si>
-  <si>
-    <t>Simon Ochoa Ramirez</t>
-  </si>
-  <si>
-    <t>Alexis Gallego</t>
-  </si>
-  <si>
-    <t>Combinacion única que indica que no puede existir más de un departamento dentro del mismo pais</t>
-  </si>
-  <si>
-    <t>toleranciaTardanza</t>
-  </si>
-  <si>
-    <t>Representa la cantidad de minutos que el cliente puede llegarle tarde un cliente a la cita establecida con el barbero, despues de eso el barbero lo podrá multar</t>
-  </si>
-  <si>
-    <t>Representa la maxima de multas que pueda tener un cliente sin pagar, a partir de esta cantidad se le hace un veto al cliente</t>
-  </si>
-  <si>
-    <t>barberia</t>
-  </si>
-  <si>
-    <t>Representa el nombre del servicio que va estar en la barberia, que el barbero ofrece y en las citas que esta</t>
-  </si>
-  <si>
-    <t>duracion</t>
-  </si>
-  <si>
-    <t>Representa lo que va durar en minutos el servicio</t>
-  </si>
-  <si>
-    <t>Representa cuanto va a valer el servicio en pesos colombianos</t>
-  </si>
-  <si>
-    <t>Representa la cantidad de dinero que el cliente debe de pagar en pesos colombianos, por superar la toleranciaTardanza</t>
-  </si>
-  <si>
-    <t>Revisar la logica de Regla, Multa y Barberia</t>
-  </si>
-  <si>
-    <t>Se tenia planeado que fuera el precio de los servicios</t>
-  </si>
-  <si>
-    <t>Motilada</t>
+    <t>Combinacion única 1</t>
+  </si>
+  <si>
+    <t>Representa el numero de celular del cliente al que se veto, es decir al que no se le podra agendar más citas</t>
+  </si>
+  <si>
+    <t>Representa la fecha en el que se veto al cliente, por acomular y no pagar las multas</t>
   </si>
 </sst>
 </file>
@@ -281,9 +392,9 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="166" formatCode="&quot;$&quot;\ #,##0"/>
+    <numFmt numFmtId="164" formatCode="&quot;$&quot;\ #,##0"/>
   </numFmts>
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -327,8 +438,17 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="10">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -343,12 +463,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="2" tint="-0.249977111117893"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="9"/>
         <bgColor indexed="64"/>
       </patternFill>
@@ -356,6 +470,36 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="7" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="2" tint="-9.9978637043366805E-2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-0.14999847407452621"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.59999389629810485"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -388,7 +532,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="46">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -421,39 +565,79 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -483,8 +667,8 @@
       <xdr:rowOff>57149</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>17</xdr:col>
-      <xdr:colOff>475710</xdr:colOff>
+      <xdr:col>16</xdr:col>
+      <xdr:colOff>244801</xdr:colOff>
       <xdr:row>27</xdr:row>
       <xdr:rowOff>85724</xdr:rowOff>
     </xdr:to>
@@ -857,9 +1041,15 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D2495362-94CF-4E08-8433-6F4780C6375E}">
   <dimension ref="A1:AD50"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="26.28515625" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:30" x14ac:dyDescent="0.25">
+      <c r="A1" s="6" t="s">
+        <v>73</v>
+      </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
@@ -890,7 +1080,7 @@
       <c r="AC1" s="1"/>
       <c r="AD1" s="1"/>
     </row>
-    <row r="2" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A2" s="1"/>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
@@ -922,7 +1112,7 @@
       <c r="AC2" s="1"/>
       <c r="AD2" s="1"/>
     </row>
-    <row r="3" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
       <c r="B3" s="1"/>
       <c r="C3" s="1"/>
@@ -954,7 +1144,7 @@
       <c r="AC3" s="1"/>
       <c r="AD3" s="1"/>
     </row>
-    <row r="4" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A4" s="1"/>
       <c r="B4" s="1"/>
       <c r="C4" s="1"/>
@@ -986,7 +1176,7 @@
       <c r="AC4" s="1"/>
       <c r="AD4" s="1"/>
     </row>
-    <row r="5" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A5" s="1"/>
       <c r="B5" s="1"/>
       <c r="C5" s="1"/>
@@ -1018,7 +1208,7 @@
       <c r="AC5" s="1"/>
       <c r="AD5" s="1"/>
     </row>
-    <row r="6" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A6" s="1"/>
       <c r="B6" s="1"/>
       <c r="D6" s="1"/>
@@ -1049,7 +1239,7 @@
       <c r="AC6" s="1"/>
       <c r="AD6" s="1"/>
     </row>
-    <row r="7" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A7" s="1"/>
       <c r="B7" s="1"/>
       <c r="C7" s="1"/>
@@ -1081,7 +1271,7 @@
       <c r="AC7" s="1"/>
       <c r="AD7" s="1"/>
     </row>
-    <row r="8" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A8" s="1"/>
       <c r="B8" s="1"/>
       <c r="C8" s="1"/>
@@ -1113,7 +1303,7 @@
       <c r="AC8" s="1"/>
       <c r="AD8" s="1"/>
     </row>
-    <row r="9" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A9" s="1"/>
       <c r="B9" s="1"/>
       <c r="C9" s="1"/>
@@ -1145,7 +1335,7 @@
       <c r="AC9" s="1"/>
       <c r="AD9" s="1"/>
     </row>
-    <row r="10" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A10" s="1"/>
       <c r="B10" s="1"/>
       <c r="C10" s="1"/>
@@ -1177,7 +1367,7 @@
       <c r="AC10" s="1"/>
       <c r="AD10" s="1"/>
     </row>
-    <row r="11" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A11" s="1"/>
       <c r="B11" s="1"/>
       <c r="C11" s="1"/>
@@ -1209,7 +1399,7 @@
       <c r="AC11" s="1"/>
       <c r="AD11" s="1"/>
     </row>
-    <row r="12" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A12" s="1"/>
       <c r="B12" s="1"/>
       <c r="C12" s="1"/>
@@ -1241,7 +1431,7 @@
       <c r="AC12" s="1"/>
       <c r="AD12" s="1"/>
     </row>
-    <row r="13" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A13" s="1"/>
       <c r="B13" s="1"/>
       <c r="C13" s="1"/>
@@ -1273,7 +1463,7 @@
       <c r="AC13" s="1"/>
       <c r="AD13" s="1"/>
     </row>
-    <row r="14" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A14" s="1"/>
       <c r="B14" s="1"/>
       <c r="C14" s="1"/>
@@ -1305,7 +1495,7 @@
       <c r="AC14" s="1"/>
       <c r="AD14" s="1"/>
     </row>
-    <row r="15" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A15" s="1"/>
       <c r="B15" s="1"/>
       <c r="C15" s="1"/>
@@ -1337,7 +1527,7 @@
       <c r="AC15" s="1"/>
       <c r="AD15" s="1"/>
     </row>
-    <row r="16" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A16" s="1"/>
       <c r="B16" s="1"/>
       <c r="C16" s="1"/>
@@ -1369,7 +1559,7 @@
       <c r="AC16" s="1"/>
       <c r="AD16" s="1"/>
     </row>
-    <row r="17" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A17" s="1"/>
       <c r="B17" s="1"/>
       <c r="C17" s="1"/>
@@ -1401,7 +1591,7 @@
       <c r="AC17" s="1"/>
       <c r="AD17" s="1"/>
     </row>
-    <row r="18" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A18" s="1"/>
       <c r="B18" s="1"/>
       <c r="C18" s="1"/>
@@ -1433,7 +1623,7 @@
       <c r="AC18" s="1"/>
       <c r="AD18" s="1"/>
     </row>
-    <row r="19" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A19" s="1"/>
       <c r="B19" s="1"/>
       <c r="C19" s="1"/>
@@ -1465,7 +1655,7 @@
       <c r="AC19" s="1"/>
       <c r="AD19" s="1"/>
     </row>
-    <row r="20" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A20" s="1"/>
       <c r="B20" s="1"/>
       <c r="C20" s="1"/>
@@ -1497,7 +1687,7 @@
       <c r="AC20" s="1"/>
       <c r="AD20" s="1"/>
     </row>
-    <row r="21" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A21" s="1"/>
       <c r="B21" s="1"/>
       <c r="C21" s="1"/>
@@ -1529,7 +1719,7 @@
       <c r="AC21" s="1"/>
       <c r="AD21" s="1"/>
     </row>
-    <row r="22" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A22" s="1"/>
       <c r="B22" s="1"/>
       <c r="C22" s="1"/>
@@ -1561,7 +1751,7 @@
       <c r="AC22" s="1"/>
       <c r="AD22" s="1"/>
     </row>
-    <row r="23" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A23" s="1"/>
       <c r="B23" s="1"/>
       <c r="C23" s="1"/>
@@ -1593,7 +1783,7 @@
       <c r="AC23" s="1"/>
       <c r="AD23" s="1"/>
     </row>
-    <row r="24" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A24" s="1"/>
       <c r="B24" s="1"/>
       <c r="C24" s="1"/>
@@ -1625,7 +1815,7 @@
       <c r="AC24" s="1"/>
       <c r="AD24" s="1"/>
     </row>
-    <row r="25" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A25" s="1"/>
       <c r="B25" s="1"/>
       <c r="C25" s="1"/>
@@ -1657,7 +1847,7 @@
       <c r="AC25" s="1"/>
       <c r="AD25" s="1"/>
     </row>
-    <row r="26" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A26" s="1"/>
       <c r="B26" s="1"/>
       <c r="C26" s="1"/>
@@ -1689,7 +1879,7 @@
       <c r="AC26" s="1"/>
       <c r="AD26" s="1"/>
     </row>
-    <row r="27" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A27" s="1"/>
       <c r="B27" s="1"/>
       <c r="C27" s="1"/>
@@ -1721,7 +1911,7 @@
       <c r="AC27" s="1"/>
       <c r="AD27" s="1"/>
     </row>
-    <row r="28" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A28" s="1"/>
       <c r="B28" s="1"/>
       <c r="C28" s="1"/>
@@ -1753,7 +1943,7 @@
       <c r="AC28" s="1"/>
       <c r="AD28" s="1"/>
     </row>
-    <row r="29" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A29" s="1"/>
       <c r="B29" s="1"/>
       <c r="C29" s="1"/>
@@ -1785,7 +1975,7 @@
       <c r="AC29" s="1"/>
       <c r="AD29" s="1"/>
     </row>
-    <row r="30" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A30" s="1"/>
       <c r="B30" s="1"/>
       <c r="C30" s="1"/>
@@ -1817,7 +2007,7 @@
       <c r="AC30" s="1"/>
       <c r="AD30" s="1"/>
     </row>
-    <row r="31" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A31" s="1"/>
       <c r="B31" s="1"/>
       <c r="C31" s="1"/>
@@ -1849,7 +2039,7 @@
       <c r="AC31" s="1"/>
       <c r="AD31" s="1"/>
     </row>
-    <row r="32" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A32" s="1"/>
       <c r="B32" s="1"/>
       <c r="C32" s="1"/>
@@ -1881,7 +2071,7 @@
       <c r="AC32" s="1"/>
       <c r="AD32" s="1"/>
     </row>
-    <row r="33" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A33" s="1"/>
       <c r="B33" s="1"/>
       <c r="C33" s="1"/>
@@ -1913,7 +2103,7 @@
       <c r="AC33" s="1"/>
       <c r="AD33" s="1"/>
     </row>
-    <row r="34" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A34" s="1"/>
       <c r="B34" s="1"/>
       <c r="C34" s="1"/>
@@ -1945,7 +2135,7 @@
       <c r="AC34" s="1"/>
       <c r="AD34" s="1"/>
     </row>
-    <row r="35" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A35" s="1"/>
       <c r="B35" s="1"/>
       <c r="C35" s="1"/>
@@ -1977,7 +2167,7 @@
       <c r="AC35" s="1"/>
       <c r="AD35" s="1"/>
     </row>
-    <row r="36" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A36" s="1"/>
       <c r="B36" s="1"/>
       <c r="C36" s="1"/>
@@ -2009,7 +2199,7 @@
       <c r="AC36" s="1"/>
       <c r="AD36" s="1"/>
     </row>
-    <row r="37" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A37" s="1"/>
       <c r="B37" s="1"/>
       <c r="C37" s="1"/>
@@ -2041,7 +2231,7 @@
       <c r="AC37" s="1"/>
       <c r="AD37" s="1"/>
     </row>
-    <row r="38" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A38" s="1"/>
       <c r="B38" s="1"/>
       <c r="C38" s="1"/>
@@ -2073,7 +2263,7 @@
       <c r="AC38" s="1"/>
       <c r="AD38" s="1"/>
     </row>
-    <row r="39" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A39" s="1"/>
       <c r="B39" s="1"/>
       <c r="C39" s="1"/>
@@ -2105,7 +2295,7 @@
       <c r="AC39" s="1"/>
       <c r="AD39" s="1"/>
     </row>
-    <row r="40" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A40" s="1"/>
       <c r="B40" s="1"/>
       <c r="C40" s="1"/>
@@ -2137,7 +2327,7 @@
       <c r="AC40" s="1"/>
       <c r="AD40" s="1"/>
     </row>
-    <row r="41" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A41" s="1"/>
       <c r="B41" s="1"/>
       <c r="C41" s="1"/>
@@ -2169,7 +2359,7 @@
       <c r="AC41" s="1"/>
       <c r="AD41" s="1"/>
     </row>
-    <row r="42" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A42" s="1"/>
       <c r="B42" s="1"/>
       <c r="C42" s="1"/>
@@ -2201,7 +2391,7 @@
       <c r="AC42" s="1"/>
       <c r="AD42" s="1"/>
     </row>
-    <row r="43" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A43" s="1"/>
       <c r="B43" s="1"/>
       <c r="C43" s="1"/>
@@ -2233,7 +2423,7 @@
       <c r="AC43" s="1"/>
       <c r="AD43" s="1"/>
     </row>
-    <row r="44" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A44" s="1"/>
       <c r="B44" s="1"/>
       <c r="C44" s="1"/>
@@ -2265,7 +2455,7 @@
       <c r="AC44" s="1"/>
       <c r="AD44" s="1"/>
     </row>
-    <row r="45" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A45" s="1"/>
       <c r="B45" s="1"/>
       <c r="C45" s="1"/>
@@ -2297,7 +2487,7 @@
       <c r="AC45" s="1"/>
       <c r="AD45" s="1"/>
     </row>
-    <row r="46" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A46" s="1"/>
       <c r="B46" s="1"/>
       <c r="C46" s="1"/>
@@ -2329,7 +2519,7 @@
       <c r="AC46" s="1"/>
       <c r="AD46" s="1"/>
     </row>
-    <row r="47" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A47" s="1"/>
       <c r="B47" s="1"/>
       <c r="C47" s="1"/>
@@ -2361,7 +2551,7 @@
       <c r="AC47" s="1"/>
       <c r="AD47" s="1"/>
     </row>
-    <row r="48" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A48" s="1"/>
       <c r="B48" s="1"/>
       <c r="C48" s="1"/>
@@ -2393,7 +2583,7 @@
       <c r="AC48" s="1"/>
       <c r="AD48" s="1"/>
     </row>
-    <row r="49" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A49" s="1"/>
       <c r="B49" s="1"/>
       <c r="C49" s="1"/>
@@ -2425,7 +2615,7 @@
       <c r="AC49" s="1"/>
       <c r="AD49" s="1"/>
     </row>
-    <row r="50" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A50" s="1"/>
       <c r="B50" s="1"/>
       <c r="C50" s="1"/>
@@ -2458,6 +2648,9 @@
       <c r="AD50" s="1"/>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A1" location="'Objetos de Dominio'!A1" display="&lt;&lt;&lt;&lt; Ir a objetos de dominio" xr:uid="{1E6C5FA1-E9A9-4758-8F5D-35278D15B010}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
   <drawing r:id="rId2"/>
@@ -2467,32 +2660,35 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2921A3C4-B96A-49A7-8353-9FD37D2F2B74}">
   <dimension ref="A1:C3"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="23.88671875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="23.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="23.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="23.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="B1" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="B1" s="6" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" ht="30" x14ac:dyDescent="0.3">
-      <c r="A2" s="7" t="s">
+    </row>
+    <row r="2" spans="1:3" ht="28.5" x14ac:dyDescent="0.25">
+      <c r="A2" s="25" t="s">
         <v>28</v>
       </c>
       <c r="B2" s="6"/>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" s="3" t="s">
+        <v>49</v>
+      </c>
       <c r="B3" s="3" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
   </sheetData>
@@ -2506,29 +2702,34 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C1DFEC6B-639A-456B-87BA-BB123C224403}">
-  <dimension ref="A1:B3"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:D9"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="23.88671875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="23.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="23.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="23.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="B1" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="B1" s="6" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" ht="30" x14ac:dyDescent="0.3">
-      <c r="A2" s="7" t="s">
+    </row>
+    <row r="2" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
+      <c r="A2" s="25" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>50</v>
+        <v>49</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D9" t="s">
+        <v>80</v>
       </c>
     </row>
   </sheetData>
@@ -2543,44 +2744,44 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1429879F-6697-4F1F-AF5D-52C4860B7B3E}">
   <dimension ref="A1:F3"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="23.88671875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="23.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="23.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="23.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="B1" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="B1" s="6" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" ht="30" x14ac:dyDescent="0.3">
-      <c r="A2" s="7" t="s">
+    </row>
+    <row r="2" spans="1:6" ht="28.5" x14ac:dyDescent="0.25">
+      <c r="A2" s="25" t="s">
         <v>28</v>
       </c>
       <c r="B2" s="6"/>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B3" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="C3" s="3" t="s">
         <v>41</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>42</v>
       </c>
       <c r="D3" s="3" t="s">
         <v>35</v>
       </c>
       <c r="E3" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="F3" s="3" t="s">
         <v>43</v>
-      </c>
-      <c r="F3" s="3" t="s">
-        <v>44</v>
       </c>
     </row>
   </sheetData>
@@ -2595,41 +2796,41 @@
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{766573FB-AAA2-4254-B83C-7C7505540365}">
   <dimension ref="A1:E3"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="23.88671875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="23.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="23.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="23.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="B1" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="B1" s="6" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" ht="30" x14ac:dyDescent="0.3">
+    </row>
+    <row r="2" spans="1:5" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A2" s="7" t="s">
         <v>28</v>
       </c>
       <c r="B2" s="6"/>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C3" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D3" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="E3" s="3" t="s">
         <v>46</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>47</v>
       </c>
     </row>
   </sheetData>
@@ -2644,43 +2845,43 @@
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F470C5A4-8D15-43DA-95FC-91C9614E5EEA}">
   <dimension ref="A1:E3"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="23.88671875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="23.33203125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="17.109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="19.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="23.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="23.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="17.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="19.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="B1" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="B1" s="6" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" ht="30" x14ac:dyDescent="0.3">
+    </row>
+    <row r="2" spans="1:5" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A2" s="7" t="s">
         <v>28</v>
       </c>
       <c r="B2" s="6"/>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D3" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="E3" s="3" t="s">
         <v>48</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>49</v>
       </c>
     </row>
   </sheetData>
@@ -2694,211 +2895,217 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7A5AA025-A9A3-4E3E-A766-44885AA770B6}">
-  <dimension ref="A1:D13"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:D14"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="16.33203125" customWidth="1"/>
-    <col min="2" max="2" width="54.5546875" customWidth="1"/>
-    <col min="3" max="3" width="12.44140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="7.6640625" customWidth="1"/>
+    <col min="1" max="1" width="27" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="54.5703125" customWidth="1"/>
+    <col min="3" max="3" width="12.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="7.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A1" s="8" t="s">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1" s="6" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="8" t="s">
+      <c r="B2" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="8" t="s">
+      <c r="C2" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="8" t="s">
+      <c r="D2" s="8" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A2" s="9" t="s">
+    <row r="3" spans="1:4" ht="60" x14ac:dyDescent="0.25">
+      <c r="A3" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="10" t="s">
+      <c r="B3" s="10" t="s">
         <v>15</v>
-      </c>
-      <c r="C2" s="9">
-        <v>1</v>
-      </c>
-      <c r="D2" s="11" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A3" s="9" t="s">
-        <v>11</v>
-      </c>
-      <c r="B3" s="10" t="s">
-        <v>16</v>
       </c>
       <c r="C3" s="9">
         <v>1</v>
       </c>
       <c r="D3" s="11" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="60" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="B4" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="C4" s="9">
+        <v>1</v>
+      </c>
+      <c r="D4" s="11" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="75" x14ac:dyDescent="0.25">
+      <c r="A5" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="B4" s="10" t="s">
+      <c r="B5" s="10" t="s">
         <v>22</v>
-      </c>
-      <c r="C4" s="9">
-        <v>2</v>
-      </c>
-      <c r="D4" s="11" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A5" s="9" t="s">
-        <v>6</v>
-      </c>
-      <c r="B5" s="10" t="s">
-        <v>17</v>
       </c>
       <c r="C5" s="9">
         <v>2</v>
       </c>
       <c r="D5" s="11" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="75" x14ac:dyDescent="0.25">
       <c r="A6" s="9" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B6" s="10" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C6" s="9">
         <v>2</v>
       </c>
       <c r="D6" s="11" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" ht="45" x14ac:dyDescent="0.25">
       <c r="A7" s="9" t="s">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="B7" s="10" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="C7" s="9">
         <v>2</v>
       </c>
       <c r="D7" s="11" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" ht="60" x14ac:dyDescent="0.25">
       <c r="A8" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="B8" s="10" t="s">
+        <v>20</v>
+      </c>
+      <c r="C8" s="9">
+        <v>2</v>
+      </c>
+      <c r="D8" s="11" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" ht="45" x14ac:dyDescent="0.25">
+      <c r="A9" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="B8" s="10" t="s">
+      <c r="B9" s="10" t="s">
         <v>19</v>
-      </c>
-      <c r="C8" s="9">
-        <v>3</v>
-      </c>
-      <c r="D8" s="11" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A9" s="9" t="s">
-        <v>9</v>
-      </c>
-      <c r="B9" s="10" t="s">
-        <v>21</v>
       </c>
       <c r="C9" s="9">
         <v>3</v>
       </c>
       <c r="D9" s="11" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" ht="100.8" x14ac:dyDescent="0.3">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" ht="75" x14ac:dyDescent="0.25">
       <c r="A10" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="B10" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="C10" s="9">
+        <v>3</v>
+      </c>
+      <c r="D10" s="11" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" ht="120" x14ac:dyDescent="0.25">
+      <c r="A11" s="9" t="s">
         <v>29</v>
       </c>
-      <c r="B10" s="10" t="s">
-        <v>37</v>
-      </c>
-      <c r="C10" s="9">
-        <v>4</v>
-      </c>
-      <c r="D10" s="11" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" ht="129.6" x14ac:dyDescent="0.3">
-      <c r="A11" s="9" t="s">
-        <v>10</v>
-      </c>
       <c r="B11" s="10" t="s">
-        <v>23</v>
+        <v>36</v>
       </c>
       <c r="C11" s="9">
         <v>4</v>
       </c>
       <c r="D11" s="11" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" ht="150" x14ac:dyDescent="0.25">
       <c r="A12" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="B12" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="C12" s="9">
+        <v>4</v>
+      </c>
+      <c r="D12" s="11" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" ht="60" x14ac:dyDescent="0.25">
+      <c r="A13" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="B12" s="10" t="s">
+      <c r="B13" s="10" t="s">
         <v>24</v>
-      </c>
-      <c r="C12" s="9">
-        <v>5</v>
-      </c>
-      <c r="D12" s="11" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A13" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="B13" s="10" t="s">
-        <v>25</v>
       </c>
       <c r="C13" s="9">
         <v>5</v>
       </c>
       <c r="D13" s="11" t="s">
-        <v>53</v>
+        <v>52</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" ht="75" x14ac:dyDescent="0.25">
+      <c r="A14" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="B14" s="10" t="s">
+        <v>25</v>
+      </c>
+      <c r="C14" s="9">
+        <v>5</v>
+      </c>
+      <c r="D14" s="11" t="s">
+        <v>52</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="D2" location="Barberia_D!A1" display="aquí" xr:uid="{4DD4FFDC-FEC3-4024-8B2A-15ECCC25F1B4}"/>
-    <hyperlink ref="D3" location="Cliente_D!A1" display="aquí" xr:uid="{36147D48-0B43-4DA0-AD5A-85C9F3A80142}"/>
-    <hyperlink ref="D4" location="Regla_D!A1" display="aquí" xr:uid="{CE75E08E-3AEF-4772-B979-C6C2C9E47B76}"/>
-    <hyperlink ref="D5" location="Servicio_D!A1" display="aquí" xr:uid="{FA9DCCF5-D4AD-44C7-B850-A147A771879F}"/>
-    <hyperlink ref="D6" location="Barbero_D!A1" display="aquí" xr:uid="{D986BDF3-3679-4C1D-B75C-941AB0C17E00}"/>
-    <hyperlink ref="D7" location="Veto_D!A1" display="aquí" xr:uid="{50EEB4A4-A05B-458F-A616-2C079D7BA2A1}"/>
-    <hyperlink ref="D8" location="BarberoServicio_D!A1" display="aquí" xr:uid="{AC14820F-CB56-4CB4-B9D5-B9DDBC302113}"/>
-    <hyperlink ref="D9" location="Agenda_D!A1" display="aquí" xr:uid="{F2DC45FC-06BF-43EC-8765-3A2CBBBD79CD}"/>
-    <hyperlink ref="D10" location="HorarioSemanal_D!A1" display="aquí" xr:uid="{2BEC7AC9-1950-45BF-A932-EE8AB8B8E00C}"/>
-    <hyperlink ref="D11" location="Cita_D!A1" display="aquí" xr:uid="{3BDFED20-FFB7-4345-9356-B30AC1240BDC}"/>
-    <hyperlink ref="D12" location="Multa_D!A1" display="aquí" xr:uid="{5D100657-ADBE-4AA9-A971-9C9D942C9DAD}"/>
-    <hyperlink ref="D13" location="CitaServicio_D!A1" display="aquí" xr:uid="{F49154C9-A497-4677-B686-F9CF5B536DEC}"/>
+    <hyperlink ref="D3" location="Barberia_D!A1" display="aquí" xr:uid="{4DD4FFDC-FEC3-4024-8B2A-15ECCC25F1B4}"/>
+    <hyperlink ref="D4" location="Cliente_D!A1" display="aquí" xr:uid="{36147D48-0B43-4DA0-AD5A-85C9F3A80142}"/>
+    <hyperlink ref="D5" location="Regla_D!A1" display="aquí" xr:uid="{CE75E08E-3AEF-4772-B979-C6C2C9E47B76}"/>
+    <hyperlink ref="D6" location="Servicio_D!A1" display="aquí" xr:uid="{FA9DCCF5-D4AD-44C7-B850-A147A771879F}"/>
+    <hyperlink ref="D7" location="Barbero_D!A1" display="aquí" xr:uid="{D986BDF3-3679-4C1D-B75C-941AB0C17E00}"/>
+    <hyperlink ref="D8" location="Veto_D!A1" display="aquí" xr:uid="{50EEB4A4-A05B-458F-A616-2C079D7BA2A1}"/>
+    <hyperlink ref="D9" location="BarberoServicio_D!A1" display="aquí" xr:uid="{AC14820F-CB56-4CB4-B9D5-B9DDBC302113}"/>
+    <hyperlink ref="D10" location="Agenda_D!A1" display="aquí" xr:uid="{F2DC45FC-06BF-43EC-8765-3A2CBBBD79CD}"/>
+    <hyperlink ref="D11" location="HorarioSemanal_D!A1" display="aquí" xr:uid="{2BEC7AC9-1950-45BF-A932-EE8AB8B8E00C}"/>
+    <hyperlink ref="D12" location="Cita_D!A1" display="aquí" xr:uid="{3BDFED20-FFB7-4345-9356-B30AC1240BDC}"/>
+    <hyperlink ref="D13" location="Multa_D!A1" display="aquí" xr:uid="{5D100657-ADBE-4AA9-A971-9C9D942C9DAD}"/>
+    <hyperlink ref="D14" location="CitaServicio_D!A1" display="aquí" xr:uid="{F49154C9-A497-4677-B686-F9CF5B536DEC}"/>
+    <hyperlink ref="A1" location="'Modelo de Dominio'!A1" display="&lt;&lt;&lt;&lt; Ir al modulo de dominio" xr:uid="{A3D1E053-3C90-4C85-85FB-01CE6B92A5EE}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2906,30 +3113,30 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AAA22F8C-1648-4644-8301-765EB2B8C50B}">
-  <dimension ref="A1:C4"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:E8"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="33.88671875" customWidth="1"/>
-    <col min="2" max="2" width="23.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="33.85546875" customWidth="1"/>
+    <col min="2" max="2" width="26" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="B1" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="B1" s="6" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" ht="20.399999999999999" x14ac:dyDescent="0.3">
+    </row>
+    <row r="2" spans="1:5" ht="19.5" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A3" s="3" t="s">
-        <v>50</v>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3" s="21" t="s">
+        <v>49</v>
       </c>
       <c r="B3" s="3" t="s">
         <v>26</v>
@@ -2938,7 +3145,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>1</v>
       </c>
@@ -2947,6 +3154,11 @@
       </c>
       <c r="C4" s="4">
         <v>0.79166666666666663</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E8" t="s">
+        <v>79</v>
       </c>
     </row>
   </sheetData>
@@ -2961,41 +3173,41 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{28259140-2713-4A98-8730-76D57DC1D653}">
   <dimension ref="A1:D7"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="23.88671875" style="12" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="23.33203125" style="12" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="19.33203125" style="12" customWidth="1"/>
-    <col min="4" max="4" width="18.44140625" style="12" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="26.85546875" style="12" customWidth="1"/>
+    <col min="2" max="2" width="26.28515625" style="12" customWidth="1"/>
+    <col min="3" max="3" width="19.28515625" style="12" customWidth="1"/>
+    <col min="4" max="4" width="20.28515625" style="12" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="13" t="s">
+        <v>50</v>
+      </c>
+      <c r="B1" s="13" t="s">
         <v>51</v>
-      </c>
-      <c r="B1" s="13" t="s">
-        <v>52</v>
       </c>
       <c r="C1" s="14"/>
       <c r="D1" s="14"/>
     </row>
-    <row r="2" spans="1:4" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="A2" s="16" t="s">
+    <row r="2" spans="1:4" ht="37.5" x14ac:dyDescent="0.25">
+      <c r="A2" s="22" t="s">
         <v>28</v>
       </c>
-      <c r="B2" s="16" t="s">
-        <v>58</v>
-      </c>
-      <c r="C2" s="17" t="s">
-        <v>54</v>
-      </c>
-      <c r="D2" s="18" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A3" s="19" t="s">
-        <v>50</v>
+      <c r="B2" s="22" t="s">
+        <v>57</v>
+      </c>
+      <c r="C2" s="23" t="s">
+        <v>53</v>
+      </c>
+      <c r="D2" s="24" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" s="16" t="s">
+        <v>49</v>
       </c>
       <c r="B3" s="15" t="s">
         <v>30</v>
@@ -3003,16 +3215,16 @@
       <c r="C3" s="15" t="s">
         <v>31</v>
       </c>
-      <c r="D3" s="20" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D3" s="17" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="14">
         <v>1</v>
       </c>
       <c r="B4" s="14" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C4" s="14">
         <v>3234528921</v>
@@ -3022,12 +3234,12 @@
         <v>3234528921</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="14">
         <v>2</v>
       </c>
       <c r="B5" s="14" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C5" s="14">
         <v>3161657782</v>
@@ -3037,12 +3249,12 @@
         <v>3161657782</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="14">
         <v>3</v>
       </c>
       <c r="B6" s="14" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C6" s="14">
         <v>3119884321</v>
@@ -3052,12 +3264,12 @@
         <v>3119884321</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="14">
         <v>4</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C7" s="14">
         <v>3245267189</v>
@@ -3079,42 +3291,42 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B0E77388-6266-4A55-B7A3-4FCD2B643D29}">
   <dimension ref="A1:F5"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="23.88671875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="23.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="19.88671875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="18.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="23.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="23.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="18.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="B1" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="B1" s="6" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="A2" s="7" t="s">
+    </row>
+    <row r="2" spans="1:6" ht="46.5" x14ac:dyDescent="0.25">
+      <c r="A2" s="25" t="s">
         <v>28</v>
       </c>
-      <c r="B2" s="5" t="s">
+      <c r="B2" s="26" t="s">
+        <v>62</v>
+      </c>
+      <c r="C2" s="26" t="s">
+        <v>69</v>
+      </c>
+      <c r="D2" s="26" t="s">
         <v>63</v>
       </c>
-      <c r="C2" s="5" t="s">
-        <v>70</v>
-      </c>
-      <c r="D2" s="5" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A3" s="3" t="s">
-        <v>50</v>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" s="21" t="s">
+        <v>49</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C3" s="3" t="s">
         <v>32</v>
@@ -3122,30 +3334,30 @@
       <c r="D3" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="E3" s="3" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E3" s="28" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>1</v>
       </c>
       <c r="B4">
         <v>10</v>
       </c>
-      <c r="C4" s="21">
+      <c r="C4" s="18">
         <v>10000</v>
       </c>
-      <c r="D4" s="21">
+      <c r="D4" s="18">
         <v>20000</v>
       </c>
     </row>
-    <row r="5" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:6" ht="45" x14ac:dyDescent="0.25">
       <c r="D5" s="2" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="F5" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
   </sheetData>
@@ -3159,120 +3371,162 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C97B567D-D27E-4BE3-B1E4-8CA267790151}">
-  <dimension ref="A1:D12"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:E12"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="23.88671875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="23.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="16.33203125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="17.33203125" customWidth="1"/>
+    <col min="1" max="1" width="28.140625" customWidth="1"/>
+    <col min="2" max="2" width="26.5703125" customWidth="1"/>
+    <col min="3" max="3" width="16.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="17.28515625" customWidth="1"/>
+    <col min="5" max="5" width="26.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A1" s="22" t="s">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1" s="19" t="s">
+        <v>50</v>
+      </c>
+      <c r="B1" s="19" t="s">
         <v>51</v>
       </c>
-      <c r="B1" s="22" t="s">
-        <v>52</v>
-      </c>
-      <c r="C1" s="23"/>
-      <c r="D1" s="23"/>
-    </row>
-    <row r="2" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A2" s="24" t="s">
+      <c r="C1" s="20"/>
+      <c r="D1" s="20"/>
+      <c r="E1" s="12"/>
+    </row>
+    <row r="2" spans="1:5" ht="28.5" x14ac:dyDescent="0.25">
+      <c r="A2" s="29" t="s">
         <v>28</v>
       </c>
-      <c r="B2" s="24" t="s">
+      <c r="B2" s="29" t="s">
+        <v>65</v>
+      </c>
+      <c r="C2" s="30" t="s">
+        <v>67</v>
+      </c>
+      <c r="D2" s="30" t="s">
+        <v>68</v>
+      </c>
+      <c r="E2" s="23" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3" s="31" t="s">
+        <v>49</v>
+      </c>
+      <c r="B3" s="32" t="s">
+        <v>30</v>
+      </c>
+      <c r="C3" s="32" t="s">
         <v>66</v>
       </c>
-      <c r="C2" s="25" t="s">
-        <v>68</v>
-      </c>
-      <c r="D2" s="25" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A3" s="26" t="s">
-        <v>50</v>
-      </c>
-      <c r="B3" s="26" t="s">
+      <c r="D3" s="32" t="s">
+        <v>34</v>
+      </c>
+      <c r="E3" s="17" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4" s="33">
+        <v>1</v>
+      </c>
+      <c r="B4" s="33" t="s">
+        <v>72</v>
+      </c>
+      <c r="C4" s="33">
+        <v>45</v>
+      </c>
+      <c r="D4" s="34">
+        <v>22000</v>
+      </c>
+      <c r="E4" s="14" t="str">
+        <f>B4</f>
+        <v>Motilada</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5" s="33">
+        <v>2</v>
+      </c>
+      <c r="B5" s="33" t="s">
+        <v>83</v>
+      </c>
+      <c r="C5" s="33">
+        <v>10</v>
+      </c>
+      <c r="D5" s="34">
+        <v>12000</v>
+      </c>
+      <c r="E5" s="14" t="str">
+        <f t="shared" ref="E5:E7" si="0">B5</f>
+        <v>Corte de barba</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6" s="33">
+        <v>3</v>
+      </c>
+      <c r="B6" s="33" t="s">
+        <v>84</v>
+      </c>
+      <c r="C6" s="33">
+        <v>15</v>
+      </c>
+      <c r="D6" s="34">
+        <v>15000</v>
+      </c>
+      <c r="E6" s="14" t="str">
+        <f t="shared" si="0"/>
+        <v>Perfilada de barba</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A7" s="33">
+        <v>4</v>
+      </c>
+      <c r="B7" s="35" t="s">
+        <v>85</v>
+      </c>
+      <c r="C7" s="33">
         <v>30</v>
       </c>
-      <c r="C3" s="26" t="s">
-        <v>67</v>
-      </c>
-      <c r="D3" s="26" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A4" s="23">
-        <v>1</v>
-      </c>
-      <c r="B4" s="23" t="s">
-        <v>73</v>
-      </c>
-      <c r="C4" s="23">
-        <v>45</v>
-      </c>
-      <c r="D4" s="27">
-        <v>22000</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A5" s="23">
-        <v>2</v>
-      </c>
-      <c r="B5" s="23"/>
-      <c r="C5" s="23"/>
-      <c r="D5" s="23"/>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A6" s="23">
-        <v>3</v>
-      </c>
-      <c r="B6" s="23"/>
-      <c r="C6" s="23"/>
-      <c r="D6" s="23"/>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A7" s="23">
-        <v>4</v>
-      </c>
-      <c r="B7" s="23"/>
-      <c r="C7" s="23"/>
-      <c r="D7" s="23"/>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A8" s="23"/>
-      <c r="B8" s="23"/>
-      <c r="C8" s="23"/>
-      <c r="D8" s="23"/>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A9" s="23"/>
-      <c r="B9" s="23"/>
-      <c r="C9" s="23"/>
-      <c r="D9" s="23"/>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A10" s="23"/>
-      <c r="B10" s="23"/>
-      <c r="C10" s="23"/>
-      <c r="D10" s="23"/>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A11" s="23"/>
-      <c r="B11" s="23"/>
-      <c r="C11" s="23"/>
-      <c r="D11" s="23"/>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A12" s="23"/>
-      <c r="B12" s="23"/>
-      <c r="C12" s="23"/>
-      <c r="D12" s="23"/>
+      <c r="D7" s="34">
+        <v>35000</v>
+      </c>
+      <c r="E7" s="36" t="str">
+        <f t="shared" si="0"/>
+        <v>Arreglo completo de barba con toalla caliente</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A8" s="20"/>
+      <c r="B8" s="20"/>
+      <c r="C8" s="20"/>
+      <c r="D8" s="20"/>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A9" s="20"/>
+      <c r="B9" s="20"/>
+      <c r="C9" s="20"/>
+      <c r="D9" s="20"/>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A10" s="20"/>
+      <c r="B10" s="20"/>
+      <c r="C10" s="20"/>
+      <c r="D10" s="20"/>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A11" s="20"/>
+      <c r="B11" s="20"/>
+      <c r="C11" s="20"/>
+      <c r="D11" s="20"/>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A12" s="20"/>
+      <c r="B12" s="20"/>
+      <c r="C12" s="20"/>
+      <c r="D12" s="20"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -3285,42 +3539,176 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2DAE59AB-4103-4731-9C3C-4C276F8A29F8}">
-  <dimension ref="A1:C3"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:G7"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="23.88671875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="23.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="27" bestFit="1" customWidth="1"/>
+    <col min="2" max="3" width="26.7109375" customWidth="1"/>
+    <col min="4" max="4" width="16.28515625" customWidth="1"/>
+    <col min="5" max="5" width="40.7109375" customWidth="1"/>
+    <col min="6" max="6" width="18.85546875" customWidth="1"/>
+    <col min="7" max="7" width="25.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="B1" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="B1" s="6" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" ht="30" x14ac:dyDescent="0.3">
-      <c r="A2" s="7" t="s">
+      <c r="C1" s="6"/>
+    </row>
+    <row r="2" spans="1:7" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="38" t="s">
         <v>28</v>
       </c>
-      <c r="B2" s="6"/>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A3" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="B3" s="3" t="s">
+      <c r="B2" s="38" t="s">
+        <v>86</v>
+      </c>
+      <c r="C2" s="38" t="s">
+        <v>92</v>
+      </c>
+      <c r="D2" s="39" t="s">
+        <v>87</v>
+      </c>
+      <c r="E2" s="39" t="s">
+        <v>103</v>
+      </c>
+      <c r="F2" s="39" t="s">
+        <v>88</v>
+      </c>
+      <c r="G2" s="40" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="B3" s="15" t="s">
         <v>30</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="C3" s="15" t="s">
+        <v>91</v>
+      </c>
+      <c r="D3" s="15" t="s">
         <v>31</v>
+      </c>
+      <c r="E3" s="15" t="s">
+        <v>76</v>
+      </c>
+      <c r="F3" s="15" t="s">
+        <v>77</v>
+      </c>
+      <c r="G3" s="41" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" s="14">
+        <v>1</v>
+      </c>
+      <c r="B4" s="14" t="s">
+        <v>94</v>
+      </c>
+      <c r="C4" s="14" t="s">
+        <v>98</v>
+      </c>
+      <c r="D4" s="14">
+        <v>3245627890</v>
+      </c>
+      <c r="E4" s="13" t="s">
+        <v>102</v>
+      </c>
+      <c r="F4" s="14" t="s">
+        <v>89</v>
+      </c>
+      <c r="G4" s="14">
+        <f>D4</f>
+        <v>3245627890</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" s="14">
+        <v>2</v>
+      </c>
+      <c r="B5" s="14" t="s">
+        <v>95</v>
+      </c>
+      <c r="C5" s="14" t="s">
+        <v>99</v>
+      </c>
+      <c r="D5" s="14">
+        <v>3124518923</v>
+      </c>
+      <c r="E5" s="13" t="s">
+        <v>104</v>
+      </c>
+      <c r="F5" s="14" t="s">
+        <v>90</v>
+      </c>
+      <c r="G5" s="14">
+        <f t="shared" ref="G5:G7" si="0">D5</f>
+        <v>3124518923</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" s="14">
+        <v>3</v>
+      </c>
+      <c r="B6" s="14" t="s">
+        <v>96</v>
+      </c>
+      <c r="C6" s="14" t="s">
+        <v>100</v>
+      </c>
+      <c r="D6" s="14">
+        <v>3214533321</v>
+      </c>
+      <c r="E6" s="13" t="s">
+        <v>105</v>
+      </c>
+      <c r="F6" s="14" t="s">
+        <v>89</v>
+      </c>
+      <c r="G6" s="14">
+        <f t="shared" si="0"/>
+        <v>3214533321</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" s="14">
+        <v>4</v>
+      </c>
+      <c r="B7" s="14" t="s">
+        <v>97</v>
+      </c>
+      <c r="C7" s="14" t="s">
+        <v>101</v>
+      </c>
+      <c r="D7" s="14">
+        <v>3161769863</v>
+      </c>
+      <c r="E7" s="13" t="s">
+        <v>106</v>
+      </c>
+      <c r="F7" s="14" t="s">
+        <v>89</v>
+      </c>
+      <c r="G7" s="14">
+        <f t="shared" si="0"/>
+        <v>3161769863</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="A1" location="'Modelo de Dominio'!A1" display="&lt;&lt;&lt;&lt; Ir al modulo de dominio" xr:uid="{E687A9B1-2F94-41F4-9C64-B065CF803569}"/>
     <hyperlink ref="B1" location="'Objetos de Dominio'!A1" display="&lt;&lt;&lt;&lt; Ir a objetos de dominio" xr:uid="{B11349A8-A5E5-4188-AE93-A5D086816413}"/>
+    <hyperlink ref="E4" r:id="rId1" xr:uid="{60EA2572-583B-4C21-A5A4-79AC0F810621}"/>
+    <hyperlink ref="E5" r:id="rId2" xr:uid="{6DE7DFDC-37F8-4F9E-9AEF-2A9B5D465DE8}"/>
+    <hyperlink ref="E6" r:id="rId3" xr:uid="{4550EE1F-4989-43BD-948F-5BD527B9D531}"/>
+    <hyperlink ref="E7" r:id="rId4" xr:uid="{72EF9758-1786-4FA4-86ED-08E3A4E7C6AD}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -3328,45 +3716,74 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C828B98D-AAA9-4184-8373-FE2E421AAE23}">
-  <dimension ref="A1:D3"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:E4"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="23.88671875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="23.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="23.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28.85546875" customWidth="1"/>
+    <col min="3" max="3" width="29" customWidth="1"/>
+    <col min="5" max="5" width="19.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="B1" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="B1" s="6" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" ht="30" x14ac:dyDescent="0.3">
-      <c r="A2" s="7" t="s">
+    </row>
+    <row r="2" spans="1:5" ht="28.5" x14ac:dyDescent="0.25">
+      <c r="A2" s="25" t="s">
         <v>28</v>
       </c>
-      <c r="B2" s="6"/>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A3" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>41</v>
+      <c r="B2" s="25" t="s">
+        <v>109</v>
+      </c>
+      <c r="C2" s="45" t="s">
+        <v>110</v>
+      </c>
+      <c r="D2" s="42"/>
+      <c r="E2" s="42"/>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3" s="21" t="s">
+        <v>49</v>
+      </c>
+      <c r="B3" s="43" t="s">
+        <v>78</v>
       </c>
       <c r="C3" s="3" t="s">
         <v>35</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>36</v>
+        <v>107</v>
+      </c>
+      <c r="E3" s="37" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>1</v>
+      </c>
+      <c r="B4" s="6">
+        <f>Cliente_D!C4</f>
+        <v>3234528921</v>
+      </c>
+      <c r="C4" s="44">
+        <v>45789</v>
+      </c>
+      <c r="D4" t="s">
+        <v>90</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="A1" location="'Modelo de Dominio'!A1" display="&lt;&lt;&lt;&lt; Ir al modulo de dominio" xr:uid="{F755F618-0A40-4479-913F-8F6060E94F5B}"/>
     <hyperlink ref="B1" location="'Objetos de Dominio'!A1" display="&lt;&lt;&lt;&lt; Ir a objetos de dominio" xr:uid="{C5748D80-5E29-4CD8-BA51-198180E61202}"/>
+    <hyperlink ref="B3" location="Cliente_D!A1" display="cliente" xr:uid="{F7C47FD3-2FEB-4E40-8CE8-9FEC66E905E0}"/>
+    <hyperlink ref="B4" location="Cliente_D!A4" display="Cliente_D!A4" xr:uid="{7F6CACFC-57C0-447E-811A-802403EBA0AC}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -3375,35 +3792,35 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A24A074A-5C83-448D-978C-7C1005CE378E}">
   <dimension ref="A1:C3"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="23.88671875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="23.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="23.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="23.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="B1" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="B1" s="6" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" ht="30" x14ac:dyDescent="0.3">
-      <c r="A2" s="7" t="s">
+    </row>
+    <row r="2" spans="1:3" ht="28.5" x14ac:dyDescent="0.25">
+      <c r="A2" s="25" t="s">
         <v>28</v>
       </c>
       <c r="B2" s="6"/>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A3" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>39</v>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" s="21" t="s">
+        <v>49</v>
+      </c>
+      <c r="B3" s="27" t="s">
+        <v>74</v>
+      </c>
+      <c r="C3" s="27" t="s">
+        <v>75</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Se corrigió el modelo de domonio y se llenó las tablas
</commit_message>
<xml_diff>
--- a/Muestreo de datos.xlsx
+++ b/Muestreo de datos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jesus\OneDrive\Escritorio\leo\Doo\Barberia proyecto\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D5778858-64E9-47C9-A2D8-63B1F0A5B398}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{115416B5-1CE8-47C2-B36F-135C986E3E2F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{09A6C7D7-663F-4C06-9D71-8A4E97495CF9}"/>
   </bookViews>
@@ -18,15 +18,16 @@
     <sheet name="Barberia_D" sheetId="5" r:id="rId3"/>
     <sheet name="Cliente_D" sheetId="6" r:id="rId4"/>
     <sheet name="Regla_D" sheetId="7" r:id="rId5"/>
-    <sheet name="Servicio_D" sheetId="8" r:id="rId6"/>
-    <sheet name="Barbero_D" sheetId="9" r:id="rId7"/>
-    <sheet name="Veto_D" sheetId="10" r:id="rId8"/>
-    <sheet name="BarberoServicio_D" sheetId="11" r:id="rId9"/>
-    <sheet name="Agenda_D" sheetId="12" r:id="rId10"/>
-    <sheet name="HorarioSemanal_D" sheetId="15" r:id="rId11"/>
-    <sheet name="Cita_D" sheetId="13" r:id="rId12"/>
-    <sheet name="Multa_D" sheetId="16" r:id="rId13"/>
-    <sheet name="CitaServicio_D" sheetId="17" r:id="rId14"/>
+    <sheet name="HorarioBarberia_D" sheetId="18" r:id="rId6"/>
+    <sheet name="Servicio_D" sheetId="8" r:id="rId7"/>
+    <sheet name="Barbero_D" sheetId="9" r:id="rId8"/>
+    <sheet name="Veto_D" sheetId="10" r:id="rId9"/>
+    <sheet name="BarberoServicio_D" sheetId="11" r:id="rId10"/>
+    <sheet name="Agenda_D" sheetId="12" r:id="rId11"/>
+    <sheet name="HorarioBarbero_D" sheetId="20" r:id="rId12"/>
+    <sheet name="Cita_D" sheetId="13" r:id="rId13"/>
+    <sheet name="Multa_D" sheetId="16" r:id="rId14"/>
+    <sheet name="CitaServicio_D" sheetId="17" r:id="rId15"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -52,7 +53,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="177" uniqueCount="111">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="246" uniqueCount="151">
   <si>
     <t>Nombre</t>
   </si>
@@ -102,9 +103,6 @@
     <t>Representa el negocio donde trabajan los barberos, agrupa el catalogo de servicios que ofrece y las reglas de tolerancia, multas y veto que aplican para todos sus clientes</t>
   </si>
   <si>
-    <t>Representa a la persona que solicita citas en la barbería, el se las pide a un barbero por WhatsApp. Esta entidad solo es para que en el sistema tenga un historial de las citas que ha pedido, de multas y de vetos</t>
-  </si>
-  <si>
     <t>Representa un tipo de servicio que ofrece la barbería, por ejemplo, motilada, afeitada de barba, perfilar barba, con su duración y su precio. Este precio es el que se usa para calcular la multa cuando un cliente no se presenta a una cita</t>
   </si>
   <si>
@@ -132,18 +130,9 @@
     <t>Representa cada servicio incluido dentro de una cita puntual, guardando el precio y la duración que tenía ese servicio en el momento exacto en que se agendó, para que cambios futuros en el catálogo no alteren citas ya registradas</t>
   </si>
   <si>
-    <t>horarioApertura</t>
-  </si>
-  <si>
-    <t>horarioCierre</t>
-  </si>
-  <si>
     <t>Representa un identificador que hará unico cada objeto de dominio de este tipo, no se puede repetir</t>
   </si>
   <si>
-    <t>HorarioSemanal</t>
-  </si>
-  <si>
     <t>nombre</t>
   </si>
   <si>
@@ -153,42 +142,15 @@
     <t>montoMultaTardanza</t>
   </si>
   <si>
-    <t>numeroMultasVeto</t>
-  </si>
-  <si>
     <t>precio</t>
   </si>
   <si>
     <t>fecha</t>
   </si>
   <si>
-    <t>Representa los dias y horas en que algo está disponible para operar, un rango de hora de inicio y hora de fin, asociado a un día de la semana. Se usa en dos contextos distintos dentro del sistema en Barberia, representa cuando abre y cierra el negocio en general, en Agenda representa en que dias y horas trabaja un barbero específico, siempre dentro de los limites que ya definió la Barbería.</t>
-  </si>
-  <si>
-    <t>barberoId</t>
-  </si>
-  <si>
-    <t>servicioId</t>
-  </si>
-  <si>
-    <t>idAgenda</t>
-  </si>
-  <si>
-    <t>clienteId</t>
-  </si>
-  <si>
-    <t>agendaId</t>
-  </si>
-  <si>
-    <t>hora_inicio</t>
-  </si>
-  <si>
     <t>estado</t>
   </si>
   <si>
-    <t>citaId</t>
-  </si>
-  <si>
     <t>monto</t>
   </si>
   <si>
@@ -216,9 +178,6 @@
     <t>Reprsenta el numero de celular de la persona que le va aescribir al barbero por WhatsApp para pedirle una cita</t>
   </si>
   <si>
-    <t>Combinación única 1</t>
-  </si>
-  <si>
     <t>Juan Gómez</t>
   </si>
   <si>
@@ -264,12 +223,6 @@
     <t>Representa la cantidad de dinero que el cliente debe de pagar en pesos colombianos, por superar la toleranciaTardanza</t>
   </si>
   <si>
-    <t>Revisar la logica de Regla, Multa y Barberia</t>
-  </si>
-  <si>
-    <t>Se tenia planeado que fuera el precio de los servicios</t>
-  </si>
-  <si>
     <t>Motilada</t>
   </si>
   <si>
@@ -291,15 +244,6 @@
     <t>cliente</t>
   </si>
   <si>
-    <t>Corregir</t>
-  </si>
-  <si>
-    <t>Corregir Barberia o barbero</t>
-  </si>
-  <si>
-    <t>combinacion unica 1</t>
-  </si>
-  <si>
     <t>Combinacion única que indica que no puede existir más de un servicio con el mismo nombre</t>
   </si>
   <si>
@@ -378,13 +322,192 @@
     <t>activo</t>
   </si>
   <si>
-    <t>Combinacion única 1</t>
-  </si>
-  <si>
     <t>Representa el numero de celular del cliente al que se veto, es decir al que no se le podra agendar más citas</t>
   </si>
   <si>
-    <t>Representa la fecha en el que se veto al cliente, por acomular y no pagar las multas</t>
+    <t>Representa si el veto está vigente o no. Es el dato que indica si el cliente se le quito la sancion del veto o no</t>
+  </si>
+  <si>
+    <t>Combinacion única que indica que no puede existir más de un veto con el mismo cliente y la misma fecha</t>
+  </si>
+  <si>
+    <t>Representa la fecha en el que se veto al cliente, por acomular y no pagar las multas, el numero para que se de el veto lo define la regla de la barbería</t>
+  </si>
+  <si>
+    <t>numeroCelularCliente</t>
+  </si>
+  <si>
+    <t>agenda</t>
+  </si>
+  <si>
+    <t>Representa el nombre y apellidos del barbero</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Representa el nombre del servicio de la barberia </t>
+  </si>
+  <si>
+    <t>horaInicio</t>
+  </si>
+  <si>
+    <t>Representa el nombre completo del cliente que va a estar en la cita, para que luego el barbero se acuerde a quien tiene que atender</t>
+  </si>
+  <si>
+    <t>agendada</t>
+  </si>
+  <si>
+    <t>Representa el nombre de como se llama la barberia en donde trabajan los barberos</t>
+  </si>
+  <si>
+    <t>Barbería Oriental</t>
+  </si>
+  <si>
+    <t>numeroMultasMaxima</t>
+  </si>
+  <si>
+    <t>Representa el nombre de la barberia que va a estar asociado la regla</t>
+  </si>
+  <si>
+    <t>Combinación única</t>
+  </si>
+  <si>
+    <t xml:space="preserve">combinacion única </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Combinación única </t>
+  </si>
+  <si>
+    <t>Combinacion única</t>
+  </si>
+  <si>
+    <t>HorarioBarberia</t>
+  </si>
+  <si>
+    <t>HorarioBarbero</t>
+  </si>
+  <si>
+    <t>Representa a la persona que solicita citas en la barbería, el se las pide a un barbero por WhatsApp. Cada uno solo es para que en el sistema tenga un historial de las citas que ha pedido, de multas y de vetos</t>
+  </si>
+  <si>
+    <t>Representa cada dia de la semana, hora en el que entra, hora a la que sale, para que la agenda del barbero sepa que dias trabaja el</t>
+  </si>
+  <si>
+    <t>Representa cada día de la semana en los que la barberia abre, la hora a la que abre y cierra la barberia</t>
+  </si>
+  <si>
+    <t>Representa el nombre de la barberia que va pertencer los horarios de la barberia</t>
+  </si>
+  <si>
+    <t>dia</t>
+  </si>
+  <si>
+    <t>horaApertura</t>
+  </si>
+  <si>
+    <t>horaCierre</t>
+  </si>
+  <si>
+    <t>Lunes</t>
+  </si>
+  <si>
+    <t>Martes</t>
+  </si>
+  <si>
+    <t>Miércoles</t>
+  </si>
+  <si>
+    <t>Jueves</t>
+  </si>
+  <si>
+    <t>Viernes</t>
+  </si>
+  <si>
+    <t>Sábado</t>
+  </si>
+  <si>
+    <t>Referencia a que barbero es el dueño de esta agenda, es el dato que conecta el calendario con la persona que lo usa para organizar su tiempo y sus citas</t>
+  </si>
+  <si>
+    <t>Combinación única que indica que un barbero no puede tener más de una agenda, cada barbero organiza todo su tiempo en un único lugar</t>
+  </si>
+  <si>
+    <t>horaFin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+Hace referencia a la agenda (y por lo tanto al barbero) a la que pertenece este horario, permite saber de quién es cada bloque de disponibilidad</t>
+  </si>
+  <si>
+    <t>Representa el día de la semana en que aplica este horario, es necesario porque un barbero puede trabajar unos días sí y otros no</t>
+  </si>
+  <si>
+    <t>Representa la hora en la que el barbero empieza a estar disponible ese dia</t>
+  </si>
+  <si>
+    <t>Representa la hora en la que el barbero deja de estar disponible ese día, junto con horaInicio, es lo que la aplicación usa para saber si hay campo para agendar una cita nueva</t>
+  </si>
+  <si>
+    <t>Combinación única que indica que una misma agenda no puede tener dos horarios distintos para el mismo día</t>
+  </si>
+  <si>
+    <t>Representa en qué momento del proceso está la cita: agendada (se creó y espera a que el cliente), atendida (la cita se cumpli sin ningún inconveniente), incumplida (el cliente violó una de las reglas) o cancelada (el cliente avisó con anticipación que ya no la quiere)</t>
+  </si>
+  <si>
+    <t>Hace referencia a en la agenda de qué barbero quedó registrada esta cita, es lo que permite validar que no se cruce con otra cita del mismo barbero</t>
+  </si>
+  <si>
+    <t>Representa la fecha en el que se va a realizar la cita</t>
+  </si>
+  <si>
+    <t>Representa la hora en la que empieza la cita, junto con la duración de los servicios pedidos, permite calcular hasta qué hora queda ocupado el barbero con el cliente</t>
+  </si>
+  <si>
+    <t>31/09/2026</t>
+  </si>
+  <si>
+    <t>atendida</t>
+  </si>
+  <si>
+    <t>incumplida</t>
+  </si>
+  <si>
+    <t>cancelada</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+Combinación única que indica que una cita no puede existir dentro de una agenda con la misma fecha y hora de inicio</t>
+  </si>
+  <si>
+    <t>cita</t>
+  </si>
+  <si>
+    <t>Hace referencia a que cliente se le esta cobrando la multa, es el dato que se usa para sumar cuántas multas sin pagar tiene una persona y decidir si debe ser vetada, dependiendo de como se definio en regla</t>
+  </si>
+  <si>
+    <t>Hace referencia a la cita puntual que el cliente incumplió (llegando tarde fuera de la tolerancia o no presentándose), de esa cita es de donde sale el valor de monto si fue el caso de no presentase</t>
+  </si>
+  <si>
+    <t>Representa cuanto dinero en pesos colombianos debe pagar el cliente, según la política definida en Regla, puede ser el monto fijo por tardanza o la suma del precio de los servicios que tenía esa cita</t>
+  </si>
+  <si>
+    <t>Representa si el cliente ya pagó o no esta multa, es el dato que se revisa para decidir si un cliente llega al número de multas sin pagar que activa el veto</t>
+  </si>
+  <si>
+    <t>Combinación única que indica que una misma cita no puede generar más de una multa</t>
+  </si>
+  <si>
+    <t>Hace referencia a la cita puntual en la que se pidió este servicio</t>
+  </si>
+  <si>
+    <t>Hace referencia a cual servicio del catalogo fue el que se pidió en esa cita</t>
+  </si>
+  <si>
+    <t>Representa cuanto valía el servicio en el momento exacto en que se agendó la cita, se guarda aparte del precio del catalogo por si el precio de ese servicio cambia después, las citas ya registradas no se vean afectadas</t>
+  </si>
+  <si>
+    <t>Representa cuanto duraba el servicio en el momento en que se agendó, junto con la hora de inicio de la cita permite calcular hasta que hora queda ocupado el barbero</t>
+  </si>
+  <si>
+    <t>Combinación única que indica que un mismo servicio no puede repetirse dos veces dentro de la misma cita</t>
   </si>
 </sst>
 </file>
@@ -394,7 +517,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="&quot;$&quot;\ #,##0"/>
   </numFmts>
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -443,6 +566,12 @@
       <u/>
       <sz val="11"/>
       <color theme="10"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -532,7 +661,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="46">
+  <cellXfs count="56">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -540,13 +669,7 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="18" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
@@ -594,7 +717,6 @@
     <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
@@ -620,7 +742,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="4" fillId="8" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
@@ -633,11 +754,51 @@
     <xf numFmtId="0" fontId="1" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="18" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="18" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="18" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -662,22 +823,22 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>57149</xdr:rowOff>
+      <xdr:colOff>202045</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>192423</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>16</xdr:col>
-      <xdr:colOff>244801</xdr:colOff>
-      <xdr:row>27</xdr:row>
-      <xdr:rowOff>85724</xdr:rowOff>
+      <xdr:col>18</xdr:col>
+      <xdr:colOff>329247</xdr:colOff>
+      <xdr:row>31</xdr:row>
+      <xdr:rowOff>163560</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="4" name="Imagen 3">
+        <xdr:cNvPr id="2" name="Imagen 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{CE24C749-19DF-5C13-B186-1AD4A1B1B53D}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{ABE419C4-ED6D-F2DD-03E4-99972CEE0EE1}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -700,8 +861,8 @@
       </xdr:blipFill>
       <xdr:spPr bwMode="auto">
         <a:xfrm>
-          <a:off x="0" y="247649"/>
-          <a:ext cx="13429710" cy="4981575"/>
+          <a:off x="202045" y="577271"/>
+          <a:ext cx="14799550" cy="5551441"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1047,8 +1208,8 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:30" x14ac:dyDescent="0.25">
-      <c r="A1" s="6" t="s">
-        <v>73</v>
+      <c r="A1" s="5" t="s">
+        <v>57</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -1145,7 +1306,6 @@
       <c r="AD3" s="1"/>
     </row>
     <row r="4" spans="1:30" x14ac:dyDescent="0.25">
-      <c r="A4" s="1"/>
       <c r="B4" s="1"/>
       <c r="C4" s="1"/>
       <c r="D4" s="1"/>
@@ -2658,37 +2818,217 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2921A3C4-B96A-49A7-8353-9FD37D2F2B74}">
-  <dimension ref="A1:C3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A24A074A-5C83-448D-978C-7C1005CE378E}">
+  <dimension ref="A1:D7"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="23.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="23.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="29.140625" customWidth="1"/>
+    <col min="2" max="2" width="30" customWidth="1"/>
+    <col min="3" max="3" width="41.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="63.28515625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="20" t="s">
+        <v>25</v>
+      </c>
+      <c r="B2" s="42" t="s">
+        <v>95</v>
+      </c>
+      <c r="C2" s="39" t="s">
+        <v>96</v>
+      </c>
+      <c r="D2" s="43"/>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" s="14" t="s">
+        <v>36</v>
+      </c>
+      <c r="B3" s="44" t="s">
+        <v>58</v>
+      </c>
+      <c r="C3" s="44" t="s">
+        <v>59</v>
+      </c>
+      <c r="D3" s="45" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" s="12">
+        <v>1</v>
+      </c>
+      <c r="B4" s="12" t="str">
+        <f>_xlfn.CONCAT(Barbero_D!B4,"-",Barbero_D!C4)</f>
+        <v>Juan Fernando-García Lopez</v>
+      </c>
+      <c r="C4" s="12" t="str">
+        <f>Servicio_D!B4</f>
+        <v>Motilada</v>
+      </c>
+      <c r="D4" s="12" t="str">
+        <f>_xlfn.CONCAT(B4,"-",C4)</f>
+        <v>Juan Fernando-García Lopez-Motilada</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5" s="12">
+        <v>2</v>
+      </c>
+      <c r="B5" s="12" t="str">
+        <f>_xlfn.CONCAT(Barbero_D!B5,"-",Barbero_D!C5)</f>
+        <v>Juan David-Ortiz Sanchez</v>
+      </c>
+      <c r="C5" s="12" t="str">
+        <f>Servicio_D!B5</f>
+        <v>Corte de barba</v>
+      </c>
+      <c r="D5" s="12" t="str">
+        <f t="shared" ref="D5:D7" si="0">_xlfn.CONCAT(B5,"-",C5)</f>
+        <v>Juan David-Ortiz Sanchez-Corte de barba</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6" s="12">
+        <v>3</v>
+      </c>
+      <c r="B6" s="12" t="str">
+        <f>_xlfn.CONCAT(Barbero_D!B6,"-",Barbero_D!C6)</f>
+        <v>Carlos-Arbeladez Montoya</v>
+      </c>
+      <c r="C6" s="12" t="str">
+        <f>Servicio_D!B6</f>
+        <v>Perfilada de barba</v>
+      </c>
+      <c r="D6" s="12" t="str">
+        <f t="shared" si="0"/>
+        <v>Carlos-Arbeladez Montoya-Perfilada de barba</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7" s="12">
+        <v>4</v>
+      </c>
+      <c r="B7" s="12" t="str">
+        <f>_xlfn.CONCAT(Barbero_D!B7,"-",Barbero_D!C7)</f>
+        <v>Andres-Ramirez Patiño</v>
+      </c>
+      <c r="C7" s="12" t="str">
+        <f>Servicio_D!B7</f>
+        <v>Arreglo completo de barba con toalla caliente</v>
+      </c>
+      <c r="D7" s="12" t="str">
+        <f t="shared" si="0"/>
+        <v>Andres-Ramirez Patiño-Arreglo completo de barba con toalla caliente</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A1" location="'Modelo de Dominio'!A1" display="&lt;&lt;&lt;&lt; Ir al modulo de dominio" xr:uid="{FFA03467-D9E8-4922-8DD1-EB697146AC1B}"/>
+    <hyperlink ref="B1" location="'Objetos de Dominio'!A1" display="&lt;&lt;&lt;&lt; Ir a objetos de dominio" xr:uid="{971E0EFC-60C0-48A1-B837-6AAF98E7514B}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2921A3C4-B96A-49A7-8353-9FD37D2F2B74}">
+  <dimension ref="A1:C7"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="30" customWidth="1"/>
+    <col min="2" max="2" width="42.28515625" customWidth="1"/>
+    <col min="3" max="3" width="37.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" s="6" t="s">
-        <v>50</v>
-      </c>
-      <c r="B1" s="6" t="s">
-        <v>51</v>
+      <c r="A1" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="2" spans="1:3" ht="28.5" x14ac:dyDescent="0.25">
-      <c r="A2" s="25" t="s">
-        <v>28</v>
-      </c>
-      <c r="B2" s="6"/>
+      <c r="A2" s="20" t="s">
+        <v>25</v>
+      </c>
+      <c r="B2" s="20" t="s">
+        <v>123</v>
+      </c>
+      <c r="C2" s="21" t="s">
+        <v>124</v>
+      </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>37</v>
+      <c r="A3" s="14" t="s">
+        <v>36</v>
+      </c>
+      <c r="B3" s="44" t="s">
+        <v>58</v>
+      </c>
+      <c r="C3" s="37" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" s="12">
+        <v>1</v>
+      </c>
+      <c r="B4" s="12" t="str">
+        <f>_xlfn.CONCAT(Barbero_D!B4," ",Barbero_D!C4)</f>
+        <v>Juan Fernando García Lopez</v>
+      </c>
+      <c r="C4" s="12" t="str">
+        <f>B4</f>
+        <v>Juan Fernando García Lopez</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" s="12">
+        <v>2</v>
+      </c>
+      <c r="B5" s="12" t="str">
+        <f>_xlfn.CONCAT(Barbero_D!B5," ",Barbero_D!C5)</f>
+        <v>Juan David Ortiz Sanchez</v>
+      </c>
+      <c r="C5" s="12" t="str">
+        <f t="shared" ref="C5:C7" si="0">B5</f>
+        <v>Juan David Ortiz Sanchez</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" s="12">
+        <v>3</v>
+      </c>
+      <c r="B6" s="12" t="str">
+        <f>_xlfn.CONCAT(Barbero_D!B6," ",Barbero_D!C6)</f>
+        <v>Carlos Arbeladez Montoya</v>
+      </c>
+      <c r="C6" s="12" t="str">
+        <f t="shared" si="0"/>
+        <v>Carlos Arbeladez Montoya</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" s="12">
+        <v>4</v>
+      </c>
+      <c r="B7" s="12" t="str">
+        <f>_xlfn.CONCAT(Barbero_D!B7," ",Barbero_D!C7)</f>
+        <v>Andres Ramirez Patiño</v>
+      </c>
+      <c r="C7" s="12" t="str">
+        <f t="shared" si="0"/>
+        <v>Andres Ramirez Patiño</v>
       </c>
     </row>
   </sheetData>
@@ -2700,89 +3040,344 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C1DFEC6B-639A-456B-87BA-BB123C224403}">
-  <dimension ref="A1:D9"/>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5CFE76D0-FBB4-4C81-85CC-F644057A8847}">
+  <dimension ref="A1:F7"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="23.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="23.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="27" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="37.140625" customWidth="1"/>
+    <col min="3" max="3" width="28" customWidth="1"/>
+    <col min="4" max="4" width="18.7109375" customWidth="1"/>
+    <col min="5" max="5" width="31.7109375" customWidth="1"/>
+    <col min="6" max="6" width="37.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1" s="6" t="s">
-        <v>50</v>
-      </c>
-      <c r="B1" s="6" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
-      <c r="A2" s="25" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" s="3" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D9" t="s">
-        <v>80</v>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" ht="40.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="21" t="s">
+        <v>25</v>
+      </c>
+      <c r="B2" s="21" t="s">
+        <v>126</v>
+      </c>
+      <c r="C2" s="21" t="s">
+        <v>127</v>
+      </c>
+      <c r="D2" s="21" t="s">
+        <v>128</v>
+      </c>
+      <c r="E2" s="21" t="s">
+        <v>129</v>
+      </c>
+      <c r="F2" s="21" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" s="14" t="s">
+        <v>36</v>
+      </c>
+      <c r="B3" s="44" t="s">
+        <v>94</v>
+      </c>
+      <c r="C3" s="50" t="s">
+        <v>114</v>
+      </c>
+      <c r="D3" s="13" t="s">
+        <v>97</v>
+      </c>
+      <c r="E3" s="13" t="s">
+        <v>125</v>
+      </c>
+      <c r="F3" s="37" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" s="12">
+        <v>1</v>
+      </c>
+      <c r="B4" s="48" t="str">
+        <f>Agenda_D!C4</f>
+        <v>Juan Fernando García Lopez</v>
+      </c>
+      <c r="C4" s="48" t="s">
+        <v>117</v>
+      </c>
+      <c r="D4" s="48">
+        <v>0.41666666666666669</v>
+      </c>
+      <c r="E4" s="48">
+        <v>0.66666666666666663</v>
+      </c>
+      <c r="F4" s="12" t="str">
+        <f>_xlfn.CONCAT(B4,"-",C4,"-",TEXT(D4,"hh;mm"),"-",TEXT(E4,"hh;mm"))</f>
+        <v>Juan Fernando García Lopez-Lunes-10-16</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" s="12">
+        <v>2</v>
+      </c>
+      <c r="B5" s="48" t="str">
+        <f>Agenda_D!C5</f>
+        <v>Juan David Ortiz Sanchez</v>
+      </c>
+      <c r="C5" s="12" t="s">
+        <v>118</v>
+      </c>
+      <c r="D5" s="48">
+        <v>0.375</v>
+      </c>
+      <c r="E5" s="48">
+        <v>0.625</v>
+      </c>
+      <c r="F5" s="12" t="str">
+        <f t="shared" ref="F5:F7" si="0">_xlfn.CONCAT(B5,"-",C5,"-",TEXT(D5,"hh;mm"),"-",TEXT(E5,"hh;mm"))</f>
+        <v>Juan David Ortiz Sanchez-Martes-09-15</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" s="12">
+        <v>3</v>
+      </c>
+      <c r="B6" s="48" t="str">
+        <f>Agenda_D!C6</f>
+        <v>Carlos Arbeladez Montoya</v>
+      </c>
+      <c r="C6" s="12" t="s">
+        <v>120</v>
+      </c>
+      <c r="D6" s="48">
+        <v>0.54166666666666663</v>
+      </c>
+      <c r="E6" s="48">
+        <v>0.79166666666666663</v>
+      </c>
+      <c r="F6" s="12" t="str">
+        <f t="shared" si="0"/>
+        <v>Carlos Arbeladez Montoya-Jueves-13-19</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" s="12">
+        <v>4</v>
+      </c>
+      <c r="B7" s="48" t="str">
+        <f>Agenda_D!C7</f>
+        <v>Andres Ramirez Patiño</v>
+      </c>
+      <c r="C7" s="12" t="s">
+        <v>122</v>
+      </c>
+      <c r="D7" s="48">
+        <v>0.33333333333333331</v>
+      </c>
+      <c r="E7" s="48">
+        <v>0.58333333333333337</v>
+      </c>
+      <c r="F7" s="12" t="str">
+        <f t="shared" si="0"/>
+        <v>Andres Ramirez Patiño-Sábado-08-14</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="A1" location="'Modelo de Dominio'!A1" display="&lt;&lt;&lt;&lt; Ir al modulo de dominio" xr:uid="{F874FBF9-ADBF-4432-A887-3E2F20C26347}"/>
-    <hyperlink ref="B1" location="'Objetos de Dominio'!A1" display="&lt;&lt;&lt;&lt; Ir a objetos de dominio" xr:uid="{77CB29A5-4A2F-4570-859B-63ABC144D952}"/>
+    <hyperlink ref="A1" location="'Modelo de Dominio'!A1" display="&lt;&lt;&lt;&lt; Ir al modulo de dominio" xr:uid="{98F427D6-B9F6-42D5-A84C-3F68DE3A5B6E}"/>
+    <hyperlink ref="B1" location="'Objetos de Dominio'!A1" display="&lt;&lt;&lt;&lt; Ir a objetos de dominio" xr:uid="{9EA36EAB-A0B6-4F6C-A61D-44A86E61BF9F}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1429879F-6697-4F1F-AF5D-52C4860B7B3E}">
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:G15"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="23.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="23.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="28" customWidth="1"/>
+    <col min="2" max="2" width="26.5703125" customWidth="1"/>
+    <col min="3" max="3" width="30.42578125" customWidth="1"/>
+    <col min="4" max="4" width="17.85546875" customWidth="1"/>
+    <col min="5" max="5" width="36.5703125" customWidth="1"/>
+    <col min="6" max="6" width="52.85546875" customWidth="1"/>
+    <col min="7" max="7" width="39.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A1" s="6" t="s">
-        <v>50</v>
-      </c>
-      <c r="B1" s="6" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" ht="28.5" x14ac:dyDescent="0.25">
-      <c r="A2" s="25" t="s">
-        <v>28</v>
-      </c>
-      <c r="B2" s="6"/>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>41</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="F3" s="3" t="s">
-        <v>43</v>
-      </c>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A1" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="20" t="s">
+        <v>25</v>
+      </c>
+      <c r="B2" s="20" t="s">
+        <v>98</v>
+      </c>
+      <c r="C2" s="39" t="s">
+        <v>132</v>
+      </c>
+      <c r="D2" s="39" t="s">
+        <v>133</v>
+      </c>
+      <c r="E2" s="39" t="s">
+        <v>134</v>
+      </c>
+      <c r="F2" s="39" t="s">
+        <v>131</v>
+      </c>
+      <c r="G2" s="39" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" s="14" t="s">
+        <v>36</v>
+      </c>
+      <c r="B3" s="44" t="s">
+        <v>62</v>
+      </c>
+      <c r="C3" s="44" t="s">
+        <v>94</v>
+      </c>
+      <c r="D3" s="13" t="s">
+        <v>30</v>
+      </c>
+      <c r="E3" s="13" t="s">
+        <v>97</v>
+      </c>
+      <c r="F3" s="13" t="s">
+        <v>31</v>
+      </c>
+      <c r="G3" s="37" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" s="12">
+        <v>1</v>
+      </c>
+      <c r="B4" s="12" t="str">
+        <f>Cliente_D!B4</f>
+        <v>Juan Gómez</v>
+      </c>
+      <c r="C4" s="12" t="str">
+        <f>Agenda_D!C4</f>
+        <v>Juan Fernando García Lopez</v>
+      </c>
+      <c r="D4" s="41" t="s">
+        <v>135</v>
+      </c>
+      <c r="E4" s="48">
+        <v>0.41666666666666669</v>
+      </c>
+      <c r="F4" s="12" t="s">
+        <v>99</v>
+      </c>
+      <c r="G4" s="12" t="str">
+        <f>_xlfn.CONCAT(C4,"-",TEXT(D4,"dd/mm/yyyy"),"-",TEXT(E4,"hh;mm"))</f>
+        <v>Juan Fernando García Lopez-31/09/2026-10</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" s="12">
+        <v>2</v>
+      </c>
+      <c r="B5" s="12" t="str">
+        <f>Cliente_D!B5</f>
+        <v>Simon Ramirez Perez</v>
+      </c>
+      <c r="C5" s="12" t="str">
+        <f>Agenda_D!C5</f>
+        <v>Juan David Ortiz Sanchez</v>
+      </c>
+      <c r="D5" s="41">
+        <v>45983</v>
+      </c>
+      <c r="E5" s="48">
+        <v>0.45833333333333298</v>
+      </c>
+      <c r="F5" s="12" t="s">
+        <v>136</v>
+      </c>
+      <c r="G5" s="12" t="str">
+        <f t="shared" ref="G5:G7" si="0">_xlfn.CONCAT(C5,"-",TEXT(D5,"dd/mm/yyyy"),"-",TEXT(E5,"hh;mm"))</f>
+        <v>Juan David Ortiz Sanchez-22/11/2025-11</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" s="12">
+        <v>3</v>
+      </c>
+      <c r="B6" s="12" t="str">
+        <f>Cliente_D!B6</f>
+        <v>Simon Ochoa Ramirez</v>
+      </c>
+      <c r="C6" s="12" t="str">
+        <f>Agenda_D!C6</f>
+        <v>Carlos Arbeladez Montoya</v>
+      </c>
+      <c r="D6" s="41">
+        <v>45514</v>
+      </c>
+      <c r="E6" s="48">
+        <v>0.58333333333333337</v>
+      </c>
+      <c r="F6" s="12" t="s">
+        <v>137</v>
+      </c>
+      <c r="G6" s="12" t="str">
+        <f t="shared" si="0"/>
+        <v>Carlos Arbeladez Montoya-10/08/2024-14</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" s="12">
+        <v>4</v>
+      </c>
+      <c r="B7" s="12" t="str">
+        <f>Cliente_D!B7</f>
+        <v>Alexis Gallego</v>
+      </c>
+      <c r="C7" s="12" t="str">
+        <f>Agenda_D!C7</f>
+        <v>Andres Ramirez Patiño</v>
+      </c>
+      <c r="D7" s="41">
+        <v>46289</v>
+      </c>
+      <c r="E7" s="48">
+        <v>0.54166666666666696</v>
+      </c>
+      <c r="F7" s="12" t="s">
+        <v>138</v>
+      </c>
+      <c r="G7" s="12" t="str">
+        <f t="shared" si="0"/>
+        <v>Andres Ramirez Patiño-24/09/2026-13</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="D13" s="54"/>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="D14" s="54"/>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="D15" s="54"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -2793,44 +3388,157 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{766573FB-AAA2-4254-B83C-7C7505540365}">
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="23.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="23.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="26.7109375" customWidth="1"/>
+    <col min="2" max="2" width="38.5703125" customWidth="1"/>
+    <col min="3" max="3" width="39.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="39.7109375" customWidth="1"/>
+    <col min="5" max="5" width="29.85546875" customWidth="1"/>
+    <col min="6" max="6" width="39.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1" s="6" t="s">
-        <v>50</v>
-      </c>
-      <c r="B1" s="6" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" ht="28.5" x14ac:dyDescent="0.25">
-      <c r="A2" s="7" t="s">
-        <v>28</v>
-      </c>
-      <c r="B2" s="6"/>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>45</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>46</v>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="20" t="s">
+        <v>25</v>
+      </c>
+      <c r="B2" s="20" t="s">
+        <v>141</v>
+      </c>
+      <c r="C2" s="39" t="s">
+        <v>142</v>
+      </c>
+      <c r="D2" s="39" t="s">
+        <v>143</v>
+      </c>
+      <c r="E2" s="39" t="s">
+        <v>144</v>
+      </c>
+      <c r="F2" s="39" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" s="14" t="s">
+        <v>36</v>
+      </c>
+      <c r="B3" s="44" t="s">
+        <v>62</v>
+      </c>
+      <c r="C3" s="44" t="s">
+        <v>140</v>
+      </c>
+      <c r="D3" s="13" t="s">
+        <v>32</v>
+      </c>
+      <c r="E3" s="13" t="s">
+        <v>33</v>
+      </c>
+      <c r="F3" s="37" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" s="12">
+        <v>1</v>
+      </c>
+      <c r="B4" s="12" t="str">
+        <f>Cliente_D!B4</f>
+        <v>Juan Gómez</v>
+      </c>
+      <c r="C4" s="12" t="str">
+        <f>Cita_D!G4</f>
+        <v>Juan Fernando García Lopez-31/09/2026-10</v>
+      </c>
+      <c r="D4" s="12">
+        <v>22000</v>
+      </c>
+      <c r="E4" s="12" t="s">
+        <v>71</v>
+      </c>
+      <c r="F4" s="12" t="str">
+        <f>C4</f>
+        <v>Juan Fernando García Lopez-31/09/2026-10</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" s="12">
+        <v>2</v>
+      </c>
+      <c r="B5" s="12" t="str">
+        <f>Cliente_D!B5</f>
+        <v>Simon Ramirez Perez</v>
+      </c>
+      <c r="C5" s="12" t="str">
+        <f>Cita_D!G5</f>
+        <v>Juan David Ortiz Sanchez-22/11/2025-11</v>
+      </c>
+      <c r="D5" s="12">
+        <v>37000</v>
+      </c>
+      <c r="E5" s="12" t="s">
+        <v>70</v>
+      </c>
+      <c r="F5" s="12" t="str">
+        <f t="shared" ref="F5:F7" si="0">C5</f>
+        <v>Juan David Ortiz Sanchez-22/11/2025-11</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" s="12">
+        <v>3</v>
+      </c>
+      <c r="B6" s="12" t="str">
+        <f>Cliente_D!B6</f>
+        <v>Simon Ochoa Ramirez</v>
+      </c>
+      <c r="C6" s="12" t="str">
+        <f>Cita_D!G6</f>
+        <v>Carlos Arbeladez Montoya-10/08/2024-14</v>
+      </c>
+      <c r="D6" s="12">
+        <v>10000</v>
+      </c>
+      <c r="E6" s="12" t="s">
+        <v>71</v>
+      </c>
+      <c r="F6" s="12" t="str">
+        <f t="shared" si="0"/>
+        <v>Carlos Arbeladez Montoya-10/08/2024-14</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" s="12">
+        <v>4</v>
+      </c>
+      <c r="B7" s="12" t="str">
+        <f>Cliente_D!B7</f>
+        <v>Alexis Gallego</v>
+      </c>
+      <c r="C7" s="12" t="str">
+        <f>Cita_D!G7</f>
+        <v>Andres Ramirez Patiño-24/09/2026-13</v>
+      </c>
+      <c r="D7" s="12">
+        <v>10000</v>
+      </c>
+      <c r="E7" s="12" t="s">
+        <v>70</v>
+      </c>
+      <c r="F7" s="12" t="str">
+        <f t="shared" si="0"/>
+        <v>Andres Ramirez Patiño-24/09/2026-13</v>
       </c>
     </row>
   </sheetData>
@@ -2842,46 +3550,157 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F470C5A4-8D15-43DA-95FC-91C9614E5EEA}">
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="23.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="23.28515625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="17.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="19.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="26.42578125" customWidth="1"/>
+    <col min="2" max="2" width="39.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="21.85546875" customWidth="1"/>
+    <col min="4" max="4" width="41.85546875" customWidth="1"/>
+    <col min="5" max="5" width="32.140625" customWidth="1"/>
+    <col min="6" max="6" width="54.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1" s="6" t="s">
-        <v>50</v>
-      </c>
-      <c r="B1" s="6" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" ht="28.5" x14ac:dyDescent="0.25">
-      <c r="A2" s="7" t="s">
-        <v>28</v>
-      </c>
-      <c r="B2" s="6"/>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="C3" s="3" t="s">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="B1" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="D3" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>48</v>
+    </row>
+    <row r="2" spans="1:6" ht="33" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="20" t="s">
+        <v>25</v>
+      </c>
+      <c r="B2" s="20" t="s">
+        <v>146</v>
+      </c>
+      <c r="C2" s="39" t="s">
+        <v>147</v>
+      </c>
+      <c r="D2" s="39" t="s">
+        <v>148</v>
+      </c>
+      <c r="E2" s="39" t="s">
+        <v>149</v>
+      </c>
+      <c r="F2" s="39" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" s="55" t="s">
+        <v>36</v>
+      </c>
+      <c r="B3" s="44" t="s">
+        <v>140</v>
+      </c>
+      <c r="C3" s="44" t="s">
+        <v>59</v>
+      </c>
+      <c r="D3" s="13" t="s">
+        <v>34</v>
+      </c>
+      <c r="E3" s="13" t="s">
+        <v>35</v>
+      </c>
+      <c r="F3" s="37" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" s="12">
+        <v>1</v>
+      </c>
+      <c r="B4" s="12" t="str">
+        <f>Cita_D!G4</f>
+        <v>Juan Fernando García Lopez-31/09/2026-10</v>
+      </c>
+      <c r="C4" s="12" t="str">
+        <f>Servicio_D!E4</f>
+        <v>Motilada</v>
+      </c>
+      <c r="D4" s="12">
+        <v>22000</v>
+      </c>
+      <c r="E4" s="12">
+        <v>45</v>
+      </c>
+      <c r="F4" s="12" t="str">
+        <f>_xlfn.CONCAT(B4,"-",C4)</f>
+        <v>Juan Fernando García Lopez-31/09/2026-10-Motilada</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" s="12">
+        <v>2</v>
+      </c>
+      <c r="B5" s="12" t="str">
+        <f>Cita_D!G5</f>
+        <v>Juan David Ortiz Sanchez-22/11/2025-11</v>
+      </c>
+      <c r="C5" s="12" t="str">
+        <f>Servicio_D!E4</f>
+        <v>Motilada</v>
+      </c>
+      <c r="D5" s="12">
+        <v>22000</v>
+      </c>
+      <c r="E5" s="12">
+        <v>45</v>
+      </c>
+      <c r="F5" s="12" t="str">
+        <f t="shared" ref="F5:F7" si="0">_xlfn.CONCAT(B5,"-",C5)</f>
+        <v>Juan David Ortiz Sanchez-22/11/2025-11-Motilada</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" s="12">
+        <v>3</v>
+      </c>
+      <c r="B6" s="12" t="str">
+        <f>Cita_D!G6</f>
+        <v>Carlos Arbeladez Montoya-10/08/2024-14</v>
+      </c>
+      <c r="C6" s="12" t="str">
+        <f>Servicio_D!E6</f>
+        <v>Perfilada de barba</v>
+      </c>
+      <c r="D6" s="12">
+        <v>15000</v>
+      </c>
+      <c r="E6" s="12">
+        <v>15</v>
+      </c>
+      <c r="F6" s="12" t="str">
+        <f t="shared" si="0"/>
+        <v>Carlos Arbeladez Montoya-10/08/2024-14-Perfilada de barba</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" ht="45" x14ac:dyDescent="0.25">
+      <c r="A7" s="12">
+        <v>4</v>
+      </c>
+      <c r="B7" s="12" t="str">
+        <f>Cita_D!G7</f>
+        <v>Andres Ramirez Patiño-24/09/2026-13</v>
+      </c>
+      <c r="C7" s="33" t="str">
+        <f>Servicio_D!E7</f>
+        <v>Arreglo completo de barba con toalla caliente</v>
+      </c>
+      <c r="D7" s="12">
+        <v>35000</v>
+      </c>
+      <c r="E7" s="12">
+        <v>30</v>
+      </c>
+      <c r="F7" s="33" t="str">
+        <f t="shared" si="0"/>
+        <v>Andres Ramirez Patiño-24/09/2026-13-Arreglo completo de barba con toalla caliente</v>
       </c>
     </row>
   </sheetData>
@@ -2895,200 +3714,214 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7A5AA025-A9A3-4E3E-A766-44885AA770B6}">
-  <dimension ref="A1:D14"/>
+  <dimension ref="A1:D15"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="27" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="54.5703125" customWidth="1"/>
-    <col min="3" max="3" width="12.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.42578125" customWidth="1"/>
     <col min="4" max="4" width="7.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1" s="6" t="s">
-        <v>50</v>
+      <c r="A1" s="5" t="s">
+        <v>37</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" s="8" t="s">
+      <c r="A2" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="8" t="s">
+      <c r="B2" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="8" t="s">
+      <c r="C2" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="8" t="s">
+      <c r="D2" s="6" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="60" x14ac:dyDescent="0.25">
-      <c r="A3" s="9" t="s">
+      <c r="A3" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="10" t="s">
+      <c r="B3" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="C3" s="9">
+      <c r="C3" s="7">
         <v>1</v>
       </c>
-      <c r="D3" s="11" t="s">
-        <v>52</v>
+      <c r="D3" s="9" t="s">
+        <v>39</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="60" x14ac:dyDescent="0.25">
-      <c r="A4" s="9" t="s">
+      <c r="A4" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="B4" s="10" t="s">
+      <c r="B4" s="8" t="s">
+        <v>110</v>
+      </c>
+      <c r="C4" s="7">
+        <v>1</v>
+      </c>
+      <c r="D4" s="9" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="75" x14ac:dyDescent="0.25">
+      <c r="A5" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="B5" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="C5" s="7">
+        <v>2</v>
+      </c>
+      <c r="D5" s="9" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="A6" s="7" t="s">
+        <v>108</v>
+      </c>
+      <c r="B6" s="8" t="s">
+        <v>112</v>
+      </c>
+      <c r="C6" s="7">
+        <v>2</v>
+      </c>
+      <c r="D6" s="9" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" ht="75" x14ac:dyDescent="0.25">
+      <c r="A7" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="B7" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="C4" s="9">
-        <v>1</v>
-      </c>
-      <c r="D4" s="11" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" ht="75" x14ac:dyDescent="0.25">
-      <c r="A5" s="9" t="s">
+      <c r="C7" s="7">
+        <v>2</v>
+      </c>
+      <c r="D7" s="9" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" ht="45" x14ac:dyDescent="0.25">
+      <c r="A8" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="B8" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="C8" s="7">
+        <v>2</v>
+      </c>
+      <c r="D8" s="9" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" ht="60" x14ac:dyDescent="0.25">
+      <c r="A9" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="B9" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="C9" s="7">
+        <v>2</v>
+      </c>
+      <c r="D9" s="9" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" ht="45" x14ac:dyDescent="0.25">
+      <c r="A10" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="B10" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="C10" s="7">
+        <v>3</v>
+      </c>
+      <c r="D10" s="9" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" ht="75" x14ac:dyDescent="0.25">
+      <c r="A11" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="B11" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="C11" s="7">
+        <v>3</v>
+      </c>
+      <c r="D11" s="9" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" ht="45" x14ac:dyDescent="0.25">
+      <c r="A12" s="7" t="s">
+        <v>109</v>
+      </c>
+      <c r="B12" s="8" t="s">
+        <v>111</v>
+      </c>
+      <c r="C12" s="7">
+        <v>4</v>
+      </c>
+      <c r="D12" s="9" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" ht="150" x14ac:dyDescent="0.25">
+      <c r="A13" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="B13" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="C13" s="7">
+        <v>4</v>
+      </c>
+      <c r="D13" s="9" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" ht="60" x14ac:dyDescent="0.25">
+      <c r="A14" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="B14" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="C14" s="7">
         <v>5</v>
       </c>
-      <c r="B5" s="10" t="s">
-        <v>22</v>
-      </c>
-      <c r="C5" s="9">
-        <v>2</v>
-      </c>
-      <c r="D5" s="11" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" ht="75" x14ac:dyDescent="0.25">
-      <c r="A6" s="9" t="s">
-        <v>6</v>
-      </c>
-      <c r="B6" s="10" t="s">
-        <v>17</v>
-      </c>
-      <c r="C6" s="9">
-        <v>2</v>
-      </c>
-      <c r="D6" s="11" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" ht="45" x14ac:dyDescent="0.25">
-      <c r="A7" s="9" t="s">
-        <v>7</v>
-      </c>
-      <c r="B7" s="10" t="s">
-        <v>18</v>
-      </c>
-      <c r="C7" s="9">
-        <v>2</v>
-      </c>
-      <c r="D7" s="11" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" ht="60" x14ac:dyDescent="0.25">
-      <c r="A8" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="B8" s="10" t="s">
-        <v>20</v>
-      </c>
-      <c r="C8" s="9">
-        <v>2</v>
-      </c>
-      <c r="D8" s="11" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" ht="45" x14ac:dyDescent="0.25">
-      <c r="A9" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="B9" s="10" t="s">
-        <v>19</v>
-      </c>
-      <c r="C9" s="9">
-        <v>3</v>
-      </c>
-      <c r="D9" s="11" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" ht="75" x14ac:dyDescent="0.25">
-      <c r="A10" s="9" t="s">
-        <v>9</v>
-      </c>
-      <c r="B10" s="10" t="s">
-        <v>21</v>
-      </c>
-      <c r="C10" s="9">
-        <v>3</v>
-      </c>
-      <c r="D10" s="11" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" ht="120" x14ac:dyDescent="0.25">
-      <c r="A11" s="9" t="s">
-        <v>29</v>
-      </c>
-      <c r="B11" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="C11" s="9">
-        <v>4</v>
-      </c>
-      <c r="D11" s="11" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" ht="150" x14ac:dyDescent="0.25">
-      <c r="A12" s="9" t="s">
-        <v>10</v>
-      </c>
-      <c r="B12" s="10" t="s">
-        <v>23</v>
-      </c>
-      <c r="C12" s="9">
-        <v>4</v>
-      </c>
-      <c r="D12" s="11" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" ht="60" x14ac:dyDescent="0.25">
-      <c r="A13" s="9" t="s">
-        <v>12</v>
-      </c>
-      <c r="B13" s="10" t="s">
+      <c r="D14" s="9" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" ht="75" x14ac:dyDescent="0.25">
+      <c r="A15" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="B15" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="C13" s="9">
+      <c r="C15" s="7">
         <v>5</v>
       </c>
-      <c r="D13" s="11" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" ht="75" x14ac:dyDescent="0.25">
-      <c r="A14" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="B14" s="10" t="s">
-        <v>25</v>
-      </c>
-      <c r="C14" s="9">
-        <v>5</v>
-      </c>
-      <c r="D14" s="11" t="s">
-        <v>52</v>
+      <c r="D15" s="9" t="s">
+        <v>39</v>
       </c>
     </row>
   </sheetData>
@@ -3096,16 +3929,17 @@
     <hyperlink ref="D3" location="Barberia_D!A1" display="aquí" xr:uid="{4DD4FFDC-FEC3-4024-8B2A-15ECCC25F1B4}"/>
     <hyperlink ref="D4" location="Cliente_D!A1" display="aquí" xr:uid="{36147D48-0B43-4DA0-AD5A-85C9F3A80142}"/>
     <hyperlink ref="D5" location="Regla_D!A1" display="aquí" xr:uid="{CE75E08E-3AEF-4772-B979-C6C2C9E47B76}"/>
-    <hyperlink ref="D6" location="Servicio_D!A1" display="aquí" xr:uid="{FA9DCCF5-D4AD-44C7-B850-A147A771879F}"/>
-    <hyperlink ref="D7" location="Barbero_D!A1" display="aquí" xr:uid="{D986BDF3-3679-4C1D-B75C-941AB0C17E00}"/>
-    <hyperlink ref="D8" location="Veto_D!A1" display="aquí" xr:uid="{50EEB4A4-A05B-458F-A616-2C079D7BA2A1}"/>
-    <hyperlink ref="D9" location="BarberoServicio_D!A1" display="aquí" xr:uid="{AC14820F-CB56-4CB4-B9D5-B9DDBC302113}"/>
-    <hyperlink ref="D10" location="Agenda_D!A1" display="aquí" xr:uid="{F2DC45FC-06BF-43EC-8765-3A2CBBBD79CD}"/>
-    <hyperlink ref="D11" location="HorarioSemanal_D!A1" display="aquí" xr:uid="{2BEC7AC9-1950-45BF-A932-EE8AB8B8E00C}"/>
-    <hyperlink ref="D12" location="Cita_D!A1" display="aquí" xr:uid="{3BDFED20-FFB7-4345-9356-B30AC1240BDC}"/>
-    <hyperlink ref="D13" location="Multa_D!A1" display="aquí" xr:uid="{5D100657-ADBE-4AA9-A971-9C9D942C9DAD}"/>
-    <hyperlink ref="D14" location="CitaServicio_D!A1" display="aquí" xr:uid="{F49154C9-A497-4677-B686-F9CF5B536DEC}"/>
+    <hyperlink ref="D7" location="Servicio_D!A1" display="aquí" xr:uid="{FA9DCCF5-D4AD-44C7-B850-A147A771879F}"/>
+    <hyperlink ref="D8" location="Barbero_D!A1" display="aquí" xr:uid="{D986BDF3-3679-4C1D-B75C-941AB0C17E00}"/>
+    <hyperlink ref="D9" location="Veto_D!A1" display="aquí" xr:uid="{50EEB4A4-A05B-458F-A616-2C079D7BA2A1}"/>
+    <hyperlink ref="D10" location="BarberoServicio_D!A1" display="aquí" xr:uid="{AC14820F-CB56-4CB4-B9D5-B9DDBC302113}"/>
+    <hyperlink ref="D11" location="Agenda_D!A1" display="aquí" xr:uid="{F2DC45FC-06BF-43EC-8765-3A2CBBBD79CD}"/>
+    <hyperlink ref="D13" location="Cita_D!A1" display="aquí" xr:uid="{3BDFED20-FFB7-4345-9356-B30AC1240BDC}"/>
+    <hyperlink ref="D14" location="Multa_D!A1" display="aquí" xr:uid="{5D100657-ADBE-4AA9-A971-9C9D942C9DAD}"/>
+    <hyperlink ref="D15" location="CitaServicio_D!A1" display="aquí" xr:uid="{F49154C9-A497-4677-B686-F9CF5B536DEC}"/>
     <hyperlink ref="A1" location="'Modelo de Dominio'!A1" display="&lt;&lt;&lt;&lt; Ir al modulo de dominio" xr:uid="{A3D1E053-3C90-4C85-85FB-01CE6B92A5EE}"/>
+    <hyperlink ref="D6" location="HorarioBarberia_D!A1" display="aquí" xr:uid="{CE45E0DE-1B75-4BE0-8664-81F7834039D9}"/>
+    <hyperlink ref="D12" location="HorarioBarbero_D!A1" display="aquí" xr:uid="{3B048927-BA4F-418A-BCDC-3E65406B8FD1}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -3113,53 +3947,48 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AAA22F8C-1648-4644-8301-765EB2B8C50B}">
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:C4"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="33.85546875" customWidth="1"/>
-    <col min="2" max="2" width="26" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="29.140625" customWidth="1"/>
+    <col min="3" max="3" width="21" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1" s="6" t="s">
-        <v>50</v>
-      </c>
-      <c r="B1" s="6" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" ht="19.5" x14ac:dyDescent="0.25">
-      <c r="A2" s="5" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" s="21" t="s">
-        <v>49</v>
-      </c>
-      <c r="B3" s="3" t="s">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="21" t="s">
+        <v>25</v>
+      </c>
+      <c r="B2" s="21" t="s">
+        <v>100</v>
+      </c>
+      <c r="C2" s="47"/>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" s="14" t="s">
+        <v>36</v>
+      </c>
+      <c r="B3" s="13" t="s">
         <v>26</v>
       </c>
-      <c r="C3" s="3" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4">
+      <c r="C3" s="46"/>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" s="12">
         <v>1</v>
       </c>
-      <c r="B4" s="4">
-        <v>0.375</v>
-      </c>
-      <c r="C4" s="4">
-        <v>0.79166666666666663</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="E8" t="s">
-        <v>79</v>
-      </c>
+      <c r="B4" s="48" t="s">
+        <v>101</v>
+      </c>
+      <c r="C4" s="4"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -3175,106 +4004,106 @@
   <dimension ref="A1:D7"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="26.85546875" style="12" customWidth="1"/>
-    <col min="2" max="2" width="26.28515625" style="12" customWidth="1"/>
-    <col min="3" max="3" width="19.28515625" style="12" customWidth="1"/>
-    <col min="4" max="4" width="20.28515625" style="12" customWidth="1"/>
+    <col min="1" max="1" width="26.85546875" style="10" customWidth="1"/>
+    <col min="2" max="2" width="26.28515625" style="10" customWidth="1"/>
+    <col min="3" max="3" width="19.28515625" style="10" customWidth="1"/>
+    <col min="4" max="4" width="20.28515625" style="10" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1" s="13" t="s">
-        <v>50</v>
-      </c>
-      <c r="B1" s="13" t="s">
-        <v>51</v>
-      </c>
-      <c r="C1" s="14"/>
-      <c r="D1" s="14"/>
+      <c r="A1" s="11" t="s">
+        <v>37</v>
+      </c>
+      <c r="B1" s="11" t="s">
+        <v>38</v>
+      </c>
+      <c r="C1" s="12"/>
+      <c r="D1" s="12"/>
     </row>
     <row r="2" spans="1:4" ht="37.5" x14ac:dyDescent="0.25">
-      <c r="A2" s="22" t="s">
-        <v>28</v>
-      </c>
-      <c r="B2" s="22" t="s">
-        <v>57</v>
-      </c>
-      <c r="C2" s="23" t="s">
-        <v>53</v>
-      </c>
-      <c r="D2" s="24" t="s">
-        <v>60</v>
+      <c r="A2" s="20" t="s">
+        <v>25</v>
+      </c>
+      <c r="B2" s="20" t="s">
+        <v>43</v>
+      </c>
+      <c r="C2" s="21" t="s">
+        <v>40</v>
+      </c>
+      <c r="D2" s="22" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" s="16" t="s">
-        <v>49</v>
-      </c>
-      <c r="B3" s="15" t="s">
-        <v>30</v>
-      </c>
-      <c r="C3" s="15" t="s">
-        <v>31</v>
-      </c>
-      <c r="D3" s="17" t="s">
-        <v>54</v>
+      <c r="A3" s="14" t="s">
+        <v>36</v>
+      </c>
+      <c r="B3" s="13" t="s">
+        <v>26</v>
+      </c>
+      <c r="C3" s="13" t="s">
+        <v>27</v>
+      </c>
+      <c r="D3" s="15" t="s">
+        <v>104</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4" s="14">
+      <c r="A4" s="12">
         <v>1</v>
       </c>
-      <c r="B4" s="14" t="s">
-        <v>55</v>
-      </c>
-      <c r="C4" s="14">
+      <c r="B4" s="12" t="s">
+        <v>41</v>
+      </c>
+      <c r="C4" s="12">
         <v>3234528921</v>
       </c>
-      <c r="D4" s="14">
+      <c r="D4" s="12">
         <f>C4</f>
         <v>3234528921</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A5" s="14">
+      <c r="A5" s="12">
         <v>2</v>
       </c>
-      <c r="B5" s="14" t="s">
-        <v>56</v>
-      </c>
-      <c r="C5" s="14">
+      <c r="B5" s="12" t="s">
+        <v>42</v>
+      </c>
+      <c r="C5" s="12">
         <v>3161657782</v>
       </c>
-      <c r="D5" s="14">
+      <c r="D5" s="12">
         <f t="shared" ref="D5:D7" si="0">C5</f>
         <v>3161657782</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A6" s="14">
+      <c r="A6" s="12">
         <v>3</v>
       </c>
-      <c r="B6" s="14" t="s">
-        <v>58</v>
-      </c>
-      <c r="C6" s="14">
+      <c r="B6" s="12" t="s">
+        <v>44</v>
+      </c>
+      <c r="C6" s="12">
         <v>3119884321</v>
       </c>
-      <c r="D6" s="14">
+      <c r="D6" s="12">
         <f t="shared" si="0"/>
         <v>3119884321</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A7" s="14">
+      <c r="A7" s="12">
         <v>4</v>
       </c>
-      <c r="B7" s="14" t="s">
-        <v>59</v>
-      </c>
-      <c r="C7" s="14">
+      <c r="B7" s="12" t="s">
+        <v>45</v>
+      </c>
+      <c r="C7" s="12">
         <v>3245267189</v>
       </c>
-      <c r="D7" s="14">
+      <c r="D7" s="12">
         <f t="shared" si="0"/>
         <v>3245267189</v>
       </c>
@@ -3293,50 +4122,57 @@
   <dimension ref="A1:F5"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="23.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="23.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="26.85546875" customWidth="1"/>
+    <col min="2" max="2" width="27.28515625" customWidth="1"/>
     <col min="3" max="3" width="19.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="18.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="16.28515625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="18.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A1" s="6" t="s">
+      <c r="A1" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" ht="46.5" x14ac:dyDescent="0.25">
+      <c r="A2" s="23" t="s">
+        <v>25</v>
+      </c>
+      <c r="B2" s="24" t="s">
+        <v>48</v>
+      </c>
+      <c r="C2" s="24" t="s">
+        <v>55</v>
+      </c>
+      <c r="D2" s="24" t="s">
+        <v>49</v>
+      </c>
+      <c r="E2" s="24" t="s">
+        <v>103</v>
+      </c>
+      <c r="F2" s="47"/>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" s="19" t="s">
+        <v>36</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>102</v>
+      </c>
+      <c r="E3" s="25" t="s">
         <v>50</v>
       </c>
-      <c r="B1" s="6" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" ht="46.5" x14ac:dyDescent="0.25">
-      <c r="A2" s="25" t="s">
-        <v>28</v>
-      </c>
-      <c r="B2" s="26" t="s">
-        <v>62</v>
-      </c>
-      <c r="C2" s="26" t="s">
-        <v>69</v>
-      </c>
-      <c r="D2" s="26" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" s="21" t="s">
-        <v>49</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>61</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="E3" s="28" t="s">
-        <v>64</v>
-      </c>
+      <c r="F3" s="49"/>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4">
@@ -3345,20 +4181,23 @@
       <c r="B4">
         <v>10</v>
       </c>
-      <c r="C4" s="18">
+      <c r="C4" s="16">
         <v>10000</v>
       </c>
-      <c r="D4" s="18">
-        <v>20000</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" ht="45" x14ac:dyDescent="0.25">
-      <c r="D5" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="F5" t="s">
-        <v>70</v>
-      </c>
+      <c r="D4">
+        <v>3</v>
+      </c>
+      <c r="E4" s="4" t="str">
+        <f>Barberia_D!B4</f>
+        <v>Barbería Oriental</v>
+      </c>
+      <c r="F4" t="str">
+        <f>_xlfn.CONCAT(D9)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="D5" s="2"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -3370,6 +4209,204 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2190E1EC-B79B-40C0-AC5B-0E2726DDD399}">
+  <dimension ref="A1:F10"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="27" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="26" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13" customWidth="1"/>
+    <col min="6" max="6" width="34.85546875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="21" t="s">
+        <v>25</v>
+      </c>
+      <c r="B2" s="21" t="s">
+        <v>113</v>
+      </c>
+      <c r="C2" s="43"/>
+      <c r="D2" s="43"/>
+      <c r="E2" s="43"/>
+      <c r="F2" s="43"/>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" s="14" t="s">
+        <v>36</v>
+      </c>
+      <c r="B3" s="44" t="s">
+        <v>50</v>
+      </c>
+      <c r="C3" s="50" t="s">
+        <v>114</v>
+      </c>
+      <c r="D3" s="13" t="s">
+        <v>115</v>
+      </c>
+      <c r="E3" s="13" t="s">
+        <v>116</v>
+      </c>
+      <c r="F3" s="45" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" s="12">
+        <v>1</v>
+      </c>
+      <c r="B4" s="48" t="str">
+        <f>Barberia_D!B4</f>
+        <v>Barbería Oriental</v>
+      </c>
+      <c r="C4" s="48" t="s">
+        <v>117</v>
+      </c>
+      <c r="D4" s="48">
+        <v>0.375</v>
+      </c>
+      <c r="E4" s="48">
+        <v>0.79166666666666663</v>
+      </c>
+      <c r="F4" s="12" t="str">
+        <f>_xlfn.CONCAT(B4,"-",C4,"-",TEXT(D4,"hh:mm"),"-",TEXT(E4,"hh:mm"))</f>
+        <v>Barbería Oriental-Lunes-09:00-19:00</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" s="12">
+        <v>2</v>
+      </c>
+      <c r="B5" s="48" t="str">
+        <f>Barberia_D!B4</f>
+        <v>Barbería Oriental</v>
+      </c>
+      <c r="C5" s="12" t="s">
+        <v>118</v>
+      </c>
+      <c r="D5" s="48">
+        <v>0.375</v>
+      </c>
+      <c r="E5" s="48">
+        <v>0.79166666666666663</v>
+      </c>
+      <c r="F5" s="12" t="str">
+        <f t="shared" ref="F5:F9" si="0">_xlfn.CONCAT(B5,"-",C5,"-",TEXT(D5,"hh:mm"),"-",TEXT(E5,"hh:mm"))</f>
+        <v>Barbería Oriental-Martes-09:00-19:00</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" s="12">
+        <v>3</v>
+      </c>
+      <c r="B6" s="48" t="str">
+        <f>Barberia_D!B4</f>
+        <v>Barbería Oriental</v>
+      </c>
+      <c r="C6" s="48" t="s">
+        <v>119</v>
+      </c>
+      <c r="D6" s="48">
+        <v>0.375</v>
+      </c>
+      <c r="E6" s="48">
+        <v>0.79166666666666696</v>
+      </c>
+      <c r="F6" s="12" t="str">
+        <f t="shared" si="0"/>
+        <v>Barbería Oriental-Miércoles-09:00-19:00</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" s="12">
+        <v>4</v>
+      </c>
+      <c r="B7" s="48" t="str">
+        <f>Barberia_D!B4</f>
+        <v>Barbería Oriental</v>
+      </c>
+      <c r="C7" s="12" t="s">
+        <v>120</v>
+      </c>
+      <c r="D7" s="48">
+        <v>0.375</v>
+      </c>
+      <c r="E7" s="48">
+        <v>0.79166666666666696</v>
+      </c>
+      <c r="F7" s="12" t="str">
+        <f t="shared" si="0"/>
+        <v>Barbería Oriental-Jueves-09:00-19:00</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" s="12">
+        <v>5</v>
+      </c>
+      <c r="B8" s="48" t="str">
+        <f>Barberia_D!B4</f>
+        <v>Barbería Oriental</v>
+      </c>
+      <c r="C8" s="48" t="s">
+        <v>121</v>
+      </c>
+      <c r="D8" s="48">
+        <v>0.375</v>
+      </c>
+      <c r="E8" s="48">
+        <v>0.79166666666666696</v>
+      </c>
+      <c r="F8" s="12" t="str">
+        <f t="shared" si="0"/>
+        <v>Barbería Oriental-Viernes-09:00-19:00</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" s="12">
+        <v>6</v>
+      </c>
+      <c r="B9" s="48" t="str">
+        <f>Barberia_D!B4</f>
+        <v>Barbería Oriental</v>
+      </c>
+      <c r="C9" s="12" t="s">
+        <v>122</v>
+      </c>
+      <c r="D9" s="53">
+        <v>0.33333333333333331</v>
+      </c>
+      <c r="E9" s="48">
+        <v>0.875</v>
+      </c>
+      <c r="F9" s="12" t="str">
+        <f t="shared" si="0"/>
+        <v>Barbería Oriental-Sábado-08:00-21:00</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" s="51"/>
+      <c r="B10" s="52"/>
+      <c r="C10" s="52"/>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="7" type="noConversion"/>
+  <hyperlinks>
+    <hyperlink ref="A1" location="'Modelo de Dominio'!A1" display="&lt;&lt;&lt;&lt; Ir al modulo de dominio" xr:uid="{8FE767F6-22F1-4F43-85BA-468D80B0CB91}"/>
+    <hyperlink ref="B1" location="'Objetos de Dominio'!A1" display="&lt;&lt;&lt;&lt; Ir a objetos de dominio" xr:uid="{FCE2B5DC-7C40-48F2-89BF-3ECFD15A2C41}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C97B567D-D27E-4BE3-B1E4-8CA267790151}">
   <dimension ref="A1:E12"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -3382,151 +4419,151 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1" s="19" t="s">
-        <v>50</v>
-      </c>
-      <c r="B1" s="19" t="s">
+      <c r="A1" s="17" t="s">
+        <v>37</v>
+      </c>
+      <c r="B1" s="17" t="s">
+        <v>38</v>
+      </c>
+      <c r="C1" s="18"/>
+      <c r="D1" s="18"/>
+      <c r="E1" s="10"/>
+    </row>
+    <row r="2" spans="1:5" ht="28.5" x14ac:dyDescent="0.25">
+      <c r="A2" s="26" t="s">
+        <v>25</v>
+      </c>
+      <c r="B2" s="26" t="s">
         <v>51</v>
       </c>
-      <c r="C1" s="20"/>
-      <c r="D1" s="20"/>
-      <c r="E1" s="12"/>
-    </row>
-    <row r="2" spans="1:5" ht="28.5" x14ac:dyDescent="0.25">
-      <c r="A2" s="29" t="s">
-        <v>28</v>
-      </c>
-      <c r="B2" s="29" t="s">
-        <v>65</v>
-      </c>
-      <c r="C2" s="30" t="s">
-        <v>67</v>
-      </c>
-      <c r="D2" s="30" t="s">
-        <v>68</v>
-      </c>
-      <c r="E2" s="23" t="s">
-        <v>82</v>
+      <c r="C2" s="27" t="s">
+        <v>53</v>
+      </c>
+      <c r="D2" s="27" t="s">
+        <v>54</v>
+      </c>
+      <c r="E2" s="21" t="s">
+        <v>63</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" s="31" t="s">
-        <v>49</v>
-      </c>
-      <c r="B3" s="32" t="s">
-        <v>30</v>
-      </c>
-      <c r="C3" s="32" t="s">
-        <v>66</v>
-      </c>
-      <c r="D3" s="32" t="s">
-        <v>34</v>
-      </c>
-      <c r="E3" s="17" t="s">
-        <v>81</v>
+      <c r="A3" s="28" t="s">
+        <v>36</v>
+      </c>
+      <c r="B3" s="29" t="s">
+        <v>26</v>
+      </c>
+      <c r="C3" s="29" t="s">
+        <v>52</v>
+      </c>
+      <c r="D3" s="29" t="s">
+        <v>29</v>
+      </c>
+      <c r="E3" s="15" t="s">
+        <v>105</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" s="33">
+      <c r="A4" s="30">
         <v>1</v>
       </c>
-      <c r="B4" s="33" t="s">
-        <v>72</v>
-      </c>
-      <c r="C4" s="33">
+      <c r="B4" s="30" t="s">
+        <v>56</v>
+      </c>
+      <c r="C4" s="30">
         <v>45</v>
       </c>
-      <c r="D4" s="34">
+      <c r="D4" s="31">
         <v>22000</v>
       </c>
-      <c r="E4" s="14" t="str">
+      <c r="E4" s="12" t="str">
         <f>B4</f>
         <v>Motilada</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5" s="33">
+      <c r="A5" s="30">
         <v>2</v>
       </c>
-      <c r="B5" s="33" t="s">
-        <v>83</v>
-      </c>
-      <c r="C5" s="33">
+      <c r="B5" s="30" t="s">
+        <v>64</v>
+      </c>
+      <c r="C5" s="30">
         <v>10</v>
       </c>
-      <c r="D5" s="34">
+      <c r="D5" s="31">
         <v>12000</v>
       </c>
-      <c r="E5" s="14" t="str">
+      <c r="E5" s="12" t="str">
         <f t="shared" ref="E5:E7" si="0">B5</f>
         <v>Corte de barba</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" s="33">
+      <c r="A6" s="30">
         <v>3</v>
       </c>
-      <c r="B6" s="33" t="s">
-        <v>84</v>
-      </c>
-      <c r="C6" s="33">
+      <c r="B6" s="30" t="s">
+        <v>65</v>
+      </c>
+      <c r="C6" s="30">
         <v>15</v>
       </c>
-      <c r="D6" s="34">
+      <c r="D6" s="31">
         <v>15000</v>
       </c>
-      <c r="E6" s="14" t="str">
+      <c r="E6" s="12" t="str">
         <f t="shared" si="0"/>
         <v>Perfilada de barba</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="30" x14ac:dyDescent="0.25">
-      <c r="A7" s="33">
+      <c r="A7" s="30">
         <v>4</v>
       </c>
-      <c r="B7" s="35" t="s">
-        <v>85</v>
-      </c>
-      <c r="C7" s="33">
+      <c r="B7" s="32" t="s">
+        <v>66</v>
+      </c>
+      <c r="C7" s="30">
         <v>30</v>
       </c>
-      <c r="D7" s="34">
+      <c r="D7" s="31">
         <v>35000</v>
       </c>
-      <c r="E7" s="36" t="str">
+      <c r="E7" s="33" t="str">
         <f t="shared" si="0"/>
         <v>Arreglo completo de barba con toalla caliente</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A8" s="20"/>
-      <c r="B8" s="20"/>
-      <c r="C8" s="20"/>
-      <c r="D8" s="20"/>
+      <c r="A8" s="18"/>
+      <c r="B8" s="18"/>
+      <c r="C8" s="18"/>
+      <c r="D8" s="18"/>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A9" s="20"/>
-      <c r="B9" s="20"/>
-      <c r="C9" s="20"/>
-      <c r="D9" s="20"/>
+      <c r="A9" s="18"/>
+      <c r="B9" s="18"/>
+      <c r="C9" s="18"/>
+      <c r="D9" s="18"/>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A10" s="20"/>
-      <c r="B10" s="20"/>
-      <c r="C10" s="20"/>
-      <c r="D10" s="20"/>
+      <c r="A10" s="18"/>
+      <c r="B10" s="18"/>
+      <c r="C10" s="18"/>
+      <c r="D10" s="18"/>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A11" s="20"/>
-      <c r="B11" s="20"/>
-      <c r="C11" s="20"/>
-      <c r="D11" s="20"/>
+      <c r="A11" s="18"/>
+      <c r="B11" s="18"/>
+      <c r="C11" s="18"/>
+      <c r="D11" s="18"/>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A12" s="20"/>
-      <c r="B12" s="20"/>
-      <c r="C12" s="20"/>
-      <c r="D12" s="20"/>
+      <c r="A12" s="18"/>
+      <c r="B12" s="18"/>
+      <c r="C12" s="18"/>
+      <c r="D12" s="18"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -3537,7 +4574,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2DAE59AB-4103-4731-9C3C-4C276F8A29F8}">
   <dimension ref="A1:G7"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -3547,156 +4584,156 @@
     <col min="4" max="4" width="16.28515625" customWidth="1"/>
     <col min="5" max="5" width="40.7109375" customWidth="1"/>
     <col min="6" max="6" width="18.85546875" customWidth="1"/>
-    <col min="7" max="7" width="25.140625" customWidth="1"/>
+    <col min="7" max="7" width="37.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A1" s="6" t="s">
-        <v>50</v>
-      </c>
-      <c r="B1" s="6" t="s">
-        <v>51</v>
-      </c>
-      <c r="C1" s="6"/>
+      <c r="A1" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="C1" s="5"/>
     </row>
     <row r="2" spans="1:7" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="38" t="s">
-        <v>28</v>
-      </c>
-      <c r="B2" s="38" t="s">
-        <v>86</v>
-      </c>
-      <c r="C2" s="38" t="s">
-        <v>92</v>
-      </c>
-      <c r="D2" s="39" t="s">
-        <v>87</v>
-      </c>
-      <c r="E2" s="39" t="s">
-        <v>103</v>
-      </c>
-      <c r="F2" s="39" t="s">
-        <v>88</v>
-      </c>
-      <c r="G2" s="40" t="s">
-        <v>93</v>
+      <c r="A2" s="34" t="s">
+        <v>25</v>
+      </c>
+      <c r="B2" s="34" t="s">
+        <v>67</v>
+      </c>
+      <c r="C2" s="34" t="s">
+        <v>73</v>
+      </c>
+      <c r="D2" s="35" t="s">
+        <v>68</v>
+      </c>
+      <c r="E2" s="35" t="s">
+        <v>84</v>
+      </c>
+      <c r="F2" s="35" t="s">
+        <v>69</v>
+      </c>
+      <c r="G2" s="36" t="s">
+        <v>74</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A3" s="16" t="s">
-        <v>49</v>
-      </c>
-      <c r="B3" s="15" t="s">
-        <v>30</v>
-      </c>
-      <c r="C3" s="15" t="s">
-        <v>91</v>
-      </c>
-      <c r="D3" s="15" t="s">
-        <v>31</v>
-      </c>
-      <c r="E3" s="15" t="s">
-        <v>76</v>
-      </c>
-      <c r="F3" s="15" t="s">
-        <v>77</v>
-      </c>
-      <c r="G3" s="41" t="s">
-        <v>54</v>
+      <c r="A3" s="14" t="s">
+        <v>36</v>
+      </c>
+      <c r="B3" s="13" t="s">
+        <v>26</v>
+      </c>
+      <c r="C3" s="13" t="s">
+        <v>72</v>
+      </c>
+      <c r="D3" s="13" t="s">
+        <v>27</v>
+      </c>
+      <c r="E3" s="13" t="s">
+        <v>60</v>
+      </c>
+      <c r="F3" s="13" t="s">
+        <v>61</v>
+      </c>
+      <c r="G3" s="37" t="s">
+        <v>106</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A4" s="14">
+      <c r="A4" s="12">
         <v>1</v>
       </c>
-      <c r="B4" s="14" t="s">
-        <v>94</v>
-      </c>
-      <c r="C4" s="14" t="s">
-        <v>98</v>
-      </c>
-      <c r="D4" s="14">
+      <c r="B4" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C4" s="12" t="s">
+        <v>79</v>
+      </c>
+      <c r="D4" s="12">
         <v>3245627890</v>
       </c>
-      <c r="E4" s="13" t="s">
-        <v>102</v>
-      </c>
-      <c r="F4" s="14" t="s">
-        <v>89</v>
-      </c>
-      <c r="G4" s="14">
+      <c r="E4" s="11" t="s">
+        <v>83</v>
+      </c>
+      <c r="F4" s="12" t="s">
+        <v>70</v>
+      </c>
+      <c r="G4" s="12">
         <f>D4</f>
         <v>3245627890</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A5" s="14">
+      <c r="A5" s="12">
         <v>2</v>
       </c>
-      <c r="B5" s="14" t="s">
-        <v>95</v>
-      </c>
-      <c r="C5" s="14" t="s">
-        <v>99</v>
-      </c>
-      <c r="D5" s="14">
+      <c r="B5" s="12" t="s">
+        <v>76</v>
+      </c>
+      <c r="C5" s="12" t="s">
+        <v>80</v>
+      </c>
+      <c r="D5" s="12">
         <v>3124518923</v>
       </c>
-      <c r="E5" s="13" t="s">
-        <v>104</v>
-      </c>
-      <c r="F5" s="14" t="s">
-        <v>90</v>
-      </c>
-      <c r="G5" s="14">
+      <c r="E5" s="11" t="s">
+        <v>85</v>
+      </c>
+      <c r="F5" s="12" t="s">
+        <v>71</v>
+      </c>
+      <c r="G5" s="12">
         <f t="shared" ref="G5:G7" si="0">D5</f>
         <v>3124518923</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A6" s="14">
+      <c r="A6" s="12">
         <v>3</v>
       </c>
-      <c r="B6" s="14" t="s">
-        <v>96</v>
-      </c>
-      <c r="C6" s="14" t="s">
-        <v>100</v>
-      </c>
-      <c r="D6" s="14">
+      <c r="B6" s="12" t="s">
+        <v>77</v>
+      </c>
+      <c r="C6" s="12" t="s">
+        <v>81</v>
+      </c>
+      <c r="D6" s="12">
         <v>3214533321</v>
       </c>
-      <c r="E6" s="13" t="s">
-        <v>105</v>
-      </c>
-      <c r="F6" s="14" t="s">
-        <v>89</v>
-      </c>
-      <c r="G6" s="14">
+      <c r="E6" s="11" t="s">
+        <v>86</v>
+      </c>
+      <c r="F6" s="12" t="s">
+        <v>70</v>
+      </c>
+      <c r="G6" s="12">
         <f t="shared" si="0"/>
         <v>3214533321</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A7" s="14">
+      <c r="A7" s="12">
         <v>4</v>
       </c>
-      <c r="B7" s="14" t="s">
-        <v>97</v>
-      </c>
-      <c r="C7" s="14" t="s">
-        <v>101</v>
-      </c>
-      <c r="D7" s="14">
+      <c r="B7" s="12" t="s">
+        <v>78</v>
+      </c>
+      <c r="C7" s="12" t="s">
+        <v>82</v>
+      </c>
+      <c r="D7" s="12">
         <v>3161769863</v>
       </c>
-      <c r="E7" s="13" t="s">
-        <v>106</v>
-      </c>
-      <c r="F7" s="14" t="s">
-        <v>89</v>
-      </c>
-      <c r="G7" s="14">
+      <c r="E7" s="11" t="s">
+        <v>87</v>
+      </c>
+      <c r="F7" s="12" t="s">
+        <v>70</v>
+      </c>
+      <c r="G7" s="12">
         <f t="shared" si="0"/>
         <v>3161769863</v>
       </c>
@@ -3714,69 +4751,138 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C828B98D-AAA9-4184-8373-FE2E421AAE23}">
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="23.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="27" customWidth="1"/>
     <col min="2" max="2" width="28.85546875" customWidth="1"/>
-    <col min="3" max="3" width="29" customWidth="1"/>
-    <col min="5" max="5" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="41" customWidth="1"/>
+    <col min="4" max="5" width="26.85546875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1" s="6" t="s">
-        <v>50</v>
-      </c>
-      <c r="B1" s="6" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" ht="28.5" x14ac:dyDescent="0.25">
-      <c r="A2" s="25" t="s">
-        <v>28</v>
-      </c>
-      <c r="B2" s="25" t="s">
-        <v>109</v>
-      </c>
-      <c r="C2" s="45" t="s">
-        <v>110</v>
-      </c>
-      <c r="D2" s="42"/>
-      <c r="E2" s="42"/>
+      <c r="A1" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="20" t="s">
+        <v>25</v>
+      </c>
+      <c r="B2" s="20" t="s">
+        <v>89</v>
+      </c>
+      <c r="C2" s="39" t="s">
+        <v>92</v>
+      </c>
+      <c r="D2" s="39" t="s">
+        <v>90</v>
+      </c>
+      <c r="E2" s="39" t="s">
+        <v>91</v>
+      </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" s="21" t="s">
-        <v>49</v>
-      </c>
-      <c r="B3" s="43" t="s">
-        <v>78</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="D3" s="3" t="s">
+      <c r="A3" s="14" t="s">
+        <v>36</v>
+      </c>
+      <c r="B3" s="40" t="s">
+        <v>93</v>
+      </c>
+      <c r="C3" s="13" t="s">
+        <v>30</v>
+      </c>
+      <c r="D3" s="13" t="s">
+        <v>88</v>
+      </c>
+      <c r="E3" s="37" t="s">
         <v>107</v>
       </c>
-      <c r="E3" s="37" t="s">
-        <v>108</v>
-      </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4">
+      <c r="A4" s="12">
         <v>1</v>
       </c>
-      <c r="B4" s="6">
+      <c r="B4" s="11">
         <f>Cliente_D!C4</f>
         <v>3234528921</v>
       </c>
-      <c r="C4" s="44">
-        <v>45789</v>
-      </c>
-      <c r="D4" t="s">
-        <v>90</v>
-      </c>
+      <c r="C4" s="41">
+        <v>45255</v>
+      </c>
+      <c r="D4" s="12" t="s">
+        <v>71</v>
+      </c>
+      <c r="E4" s="12" t="str">
+        <f>_xlfn.CONCAT(B4,"-",TEXT(C4,"dd/mm/yyyy"))</f>
+        <v>3234528921-25/11/2023</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5" s="12">
+        <v>2</v>
+      </c>
+      <c r="B5" s="11">
+        <f>Cliente_D!C5</f>
+        <v>3161657782</v>
+      </c>
+      <c r="C5" s="41">
+        <v>45372</v>
+      </c>
+      <c r="D5" s="12" t="s">
+        <v>71</v>
+      </c>
+      <c r="E5" s="12" t="str">
+        <f t="shared" ref="E5:E7" si="0">_xlfn.CONCAT(B5,"-",TEXT(C5,"dd/mm/yyyy"))</f>
+        <v>3161657782-21/03/2024</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6" s="12">
+        <v>3</v>
+      </c>
+      <c r="B6" s="11">
+        <f>Cliente_D!C6</f>
+        <v>3119884321</v>
+      </c>
+      <c r="C6" s="41">
+        <v>45556</v>
+      </c>
+      <c r="D6" s="12" t="s">
+        <v>70</v>
+      </c>
+      <c r="E6" s="12" t="str">
+        <f t="shared" si="0"/>
+        <v>3119884321-21/09/2024</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7" s="12">
+        <v>4</v>
+      </c>
+      <c r="B7" s="11">
+        <f>Cliente_D!C7</f>
+        <v>3245267189</v>
+      </c>
+      <c r="C7" s="41">
+        <v>46002</v>
+      </c>
+      <c r="D7" s="12" t="s">
+        <v>70</v>
+      </c>
+      <c r="E7" s="12" t="str">
+        <f t="shared" si="0"/>
+        <v>3245267189-11/12/2025</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="C8" s="38"/>
+      <c r="D8" s="38"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -3784,49 +4890,9 @@
     <hyperlink ref="B1" location="'Objetos de Dominio'!A1" display="&lt;&lt;&lt;&lt; Ir a objetos de dominio" xr:uid="{C5748D80-5E29-4CD8-BA51-198180E61202}"/>
     <hyperlink ref="B3" location="Cliente_D!A1" display="cliente" xr:uid="{F7C47FD3-2FEB-4E40-8CE8-9FEC66E905E0}"/>
     <hyperlink ref="B4" location="Cliente_D!A4" display="Cliente_D!A4" xr:uid="{7F6CACFC-57C0-447E-811A-802403EBA0AC}"/>
-  </hyperlinks>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A24A074A-5C83-448D-978C-7C1005CE378E}">
-  <dimension ref="A1:C3"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="23.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="23.28515625" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" s="6" t="s">
-        <v>50</v>
-      </c>
-      <c r="B1" s="6" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" ht="28.5" x14ac:dyDescent="0.25">
-      <c r="A2" s="25" t="s">
-        <v>28</v>
-      </c>
-      <c r="B2" s="6"/>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" s="21" t="s">
-        <v>49</v>
-      </c>
-      <c r="B3" s="27" t="s">
-        <v>74</v>
-      </c>
-      <c r="C3" s="27" t="s">
-        <v>75</v>
-      </c>
-    </row>
-  </sheetData>
-  <hyperlinks>
-    <hyperlink ref="A1" location="'Modelo de Dominio'!A1" display="&lt;&lt;&lt;&lt; Ir al modulo de dominio" xr:uid="{FFA03467-D9E8-4922-8DD1-EB697146AC1B}"/>
-    <hyperlink ref="B1" location="'Objetos de Dominio'!A1" display="&lt;&lt;&lt;&lt; Ir a objetos de dominio" xr:uid="{971E0EFC-60C0-48A1-B837-6AAF98E7514B}"/>
+    <hyperlink ref="B5" location="Cliente_D!A5" display="Cliente_D!A5" xr:uid="{EE87A799-0DAD-412E-8BF4-24089411596B}"/>
+    <hyperlink ref="B6" location="Cliente_D!A6" display="Cliente_D!A6" xr:uid="{D95F6EBA-51E7-42CB-9EFD-6676C5924513}"/>
+    <hyperlink ref="B7" location="Cliente_D!A7" display="Cliente_D!A7" xr:uid="{9BA1680E-A8A5-4CE9-866D-EC3B5A4F5B91}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Añadiendole atributos a objetos de dominio y corregí una linea torcida en el modelo anemico
</commit_message>
<xml_diff>
--- a/Muestreo de datos.xlsx
+++ b/Muestreo de datos.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\leand\Desktop\DOO\DOO\Barberia\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{12A4D0AF-3649-471C-8937-4D4C6C781C8A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{81BFAD6D-9C90-4CE7-B6FE-4D8B9CAEDEAD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="8" activeTab="14" xr2:uid="{09A6C7D7-663F-4C06-9D71-8A4E97495CF9}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{09A6C7D7-663F-4C06-9D71-8A4E97495CF9}"/>
   </bookViews>
   <sheets>
     <sheet name="Modelo de Dominio" sheetId="1" r:id="rId1"/>
@@ -53,7 +53,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="293" uniqueCount="191">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="297" uniqueCount="191">
   <si>
     <t>Nombre</t>
   </si>
@@ -401,9 +401,6 @@
     <t>Combinación única que indica que una misma agenda no puede tener dos horarios distintos para el mismo día</t>
   </si>
   <si>
-    <t>Hace referencia a en la agenda de qué barbero quedó registrada esta cita, es lo que permite validar que no se cruce con otra cita del mismo barbero</t>
-  </si>
-  <si>
     <t>atendida</t>
   </si>
   <si>
@@ -591,12 +588,6 @@
   </si>
   <si>
     <t>Representa si el barbero sigue o no trabajando en la barberia, es un dato calculado cuando el barbero tiene en su agenda un horario de trabajo si es vigente y si no tiene horario de trabajo dice no es vigente</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Creo que falta por poner un atributo de referencia barberia, para saber que trabaja en esa barberia </t>
-  </si>
-  <si>
-    <t>Creo que falta poner la referencia del nombre de la barberia</t>
   </si>
   <si>
     <t>fechaHora</t>
@@ -609,25 +600,34 @@
 Combinación única que indica que una cita no puede existir dentro de una agenda con la misma fecha y hora de inicio para la cita</t>
   </si>
   <si>
-    <t>Representa en qué momento del proceso está la cita: agendada (se creó y espera a que el cliente llegue), atendida (la cita se cumplió sin ningún inconveniente), retraso (el cliente llegó, pero pasada la tolerancia de tiempo) ,incumplida (el cliente nunca llegó) o cancelada (el cliente avisó con anticipación que ya no la quiere)</t>
-  </si>
-  <si>
     <t>retraso</t>
   </si>
   <si>
     <t xml:space="preserve">Representa cuanto dinero en pesos colombianos debe pagar el cliente la multa, si es por retraso se el monto es el que dice en regla y si es por incumplida el monto es del o los servicios que pidio </t>
   </si>
   <si>
-    <t>Parece que multa depende de citaservicio</t>
-  </si>
-  <si>
-    <t>Parece que veto depende de multa</t>
-  </si>
-  <si>
     <t>Combinacion única que indica que no puede existir más de un cliente con un mismo nombre, apellidos, prefijo de celular y número de celular</t>
   </si>
   <si>
     <t>Representa la hora prevista a la que finaliza una cita, es un dato calculado a partir de la hora en que empieza la cita y la duración del servicio, sumándole la duración del servicio a la hora de inicio</t>
+  </si>
+  <si>
+    <t>Representa el nombre de la barbería que pertenece el servicio</t>
+  </si>
+  <si>
+    <t>Representa la barbería en la que trabaja el barbero</t>
+  </si>
+  <si>
+    <t>Hace referencia a en la agenda de que barbero quedó registrada esta cita, es lo que permite validar que no se cruce con otra cita del mismo barbero</t>
+  </si>
+  <si>
+    <t>Representa en que momento del proceso está la cita: agendada (se creó y espera a que el cliente llegue), atendida (la cita se cumplió sin ningún inconveniente), retraso (el cliente llegó, pero pasada la tolerancia de tiempo) ,incumplida (el cliente nunca llegó) o cancelada (el cliente avisó con anticipación que ya no la quiere)</t>
+  </si>
+  <si>
+    <t>tipo</t>
+  </si>
+  <si>
+    <t>Representa el tipo de multa con el que se va sancionar, si es retraso o incumplida. Este es un dato obtenido del estado de cita</t>
   </si>
 </sst>
 </file>
@@ -788,7 +788,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="59">
+  <cellXfs count="63">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -940,6 +940,18 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="18" fontId="3" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -2989,7 +3001,7 @@
         <v>81</v>
       </c>
       <c r="D2" s="47" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
@@ -3015,7 +3027,7 @@
         <v>Juan Fernando García Lopez</v>
       </c>
       <c r="C4" s="11" t="str">
-        <f>Servicio_D!B4</f>
+        <f>Servicio_D!C4</f>
         <v>Motilada</v>
       </c>
       <c r="D4" s="12" t="str">
@@ -3032,7 +3044,7 @@
         <v>Juan David Ortiz Sanchez</v>
       </c>
       <c r="C5" s="11" t="str">
-        <f>Servicio_D!B5</f>
+        <f>Servicio_D!C5</f>
         <v>Corte de barba</v>
       </c>
       <c r="D5" s="12" t="str">
@@ -3049,7 +3061,7 @@
         <v>Carlos Arbeladez</v>
       </c>
       <c r="C6" s="11" t="str">
-        <f>Servicio_D!B6</f>
+        <f>Servicio_D!C6</f>
         <v>Perfilada de barba</v>
       </c>
       <c r="D6" s="12" t="str">
@@ -3066,7 +3078,7 @@
         <v>Andres Ramirez Patiño</v>
       </c>
       <c r="C7" s="11" t="str">
-        <f>Servicio_D!B7</f>
+        <f>Servicio_D!C7</f>
         <v>Arreglo completo de barba con toalla caliente</v>
       </c>
       <c r="D7" s="12" t="str">
@@ -3117,7 +3129,7 @@
         <v>25</v>
       </c>
       <c r="B2" s="18" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="C2" s="19" t="s">
         <v>108</v>
@@ -3396,19 +3408,19 @@
         <v>83</v>
       </c>
       <c r="C2" s="34" t="s">
-        <v>115</v>
+        <v>187</v>
       </c>
       <c r="D2" s="34" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
       <c r="E2" s="34" t="s">
-        <v>190</v>
+        <v>184</v>
       </c>
       <c r="F2" s="34" t="s">
-        <v>184</v>
+        <v>188</v>
       </c>
       <c r="G2" s="34" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -3422,7 +3434,7 @@
         <v>79</v>
       </c>
       <c r="D3" s="13" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
       <c r="E3" s="49" t="s">
         <v>109</v>
@@ -3479,7 +3491,7 @@
         <v>0.48958333333333331</v>
       </c>
       <c r="F5" s="12" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="G5" s="12" t="str">
         <f t="shared" ref="G5:G8" si="0">_xlfn.CONCAT(C5,"-",TEXT(D5,"dd/mm/yyyy/hh:mm"))</f>
@@ -3505,7 +3517,7 @@
         <v>0.59375</v>
       </c>
       <c r="F6" s="12" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
       <c r="G6" s="12" t="str">
         <f t="shared" si="0"/>
@@ -3531,7 +3543,7 @@
         <v>0.5625</v>
       </c>
       <c r="F7" s="12" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="G7" s="12" t="str">
         <f t="shared" si="0"/>
@@ -3557,7 +3569,7 @@
         <v>0.75694444444444442</v>
       </c>
       <c r="F8" s="12" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="G8" s="12" t="str">
         <f t="shared" si="0"/>
@@ -3605,18 +3617,18 @@
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{766573FB-AAA2-4254-B83C-7C7505540365}">
-  <dimension ref="A1:F9"/>
+  <dimension ref="A1:G7"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="26.6640625" customWidth="1"/>
     <col min="2" max="2" width="38.5546875" customWidth="1"/>
     <col min="3" max="3" width="39.33203125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="39.6640625" customWidth="1"/>
-    <col min="5" max="5" width="29.88671875" customWidth="1"/>
-    <col min="6" max="6" width="39.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="39.6640625" customWidth="1"/>
+    <col min="6" max="6" width="34.21875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="39.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" s="5" t="s">
         <v>37</v>
       </c>
@@ -3624,27 +3636,30 @@
         <v>38</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="31.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" ht="31.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="18" t="s">
         <v>25</v>
       </c>
       <c r="B2" s="18" t="s">
+        <v>119</v>
+      </c>
+      <c r="C2" s="34" t="s">
         <v>120</v>
       </c>
-      <c r="C2" s="34" t="s">
+      <c r="D2" s="34" t="s">
+        <v>182</v>
+      </c>
+      <c r="E2" s="34" t="s">
+        <v>190</v>
+      </c>
+      <c r="F2" s="34" t="s">
         <v>121</v>
       </c>
-      <c r="D2" s="34" t="s">
-        <v>186</v>
-      </c>
-      <c r="E2" s="34" t="s">
+      <c r="G2" s="34" t="s">
         <v>122</v>
       </c>
-      <c r="F2" s="34" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" s="14" t="s">
         <v>36</v>
       </c>
@@ -3652,19 +3667,22 @@
         <v>55</v>
       </c>
       <c r="C3" s="35" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="D3" s="38" t="s">
         <v>32</v>
       </c>
-      <c r="E3" s="49" t="s">
+      <c r="E3" s="62" t="s">
+        <v>189</v>
+      </c>
+      <c r="F3" s="49" t="s">
         <v>33</v>
       </c>
-      <c r="F3" s="32" t="s">
+      <c r="G3" s="32" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" s="12">
         <v>1</v>
       </c>
@@ -3681,14 +3699,17 @@
         <v>10000</v>
       </c>
       <c r="E4" s="12" t="s">
+        <v>181</v>
+      </c>
+      <c r="F4" s="12" t="s">
         <v>61</v>
       </c>
-      <c r="F4" s="12" t="str">
+      <c r="G4" s="12" t="str">
         <f>C4</f>
         <v>Carlos Arbeladez-10/08/2024/14:00</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" s="12">
         <v>2</v>
       </c>
@@ -3705,33 +3726,33 @@
         <v>35000</v>
       </c>
       <c r="E5" s="12" t="s">
+        <v>116</v>
+      </c>
+      <c r="F5" s="12" t="s">
         <v>62</v>
       </c>
-      <c r="F5" s="12" t="str">
+      <c r="G5" s="12" t="str">
         <f>C5</f>
         <v>Andres Ramirez Patiño-24/09/2026/13:00</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" s="10"/>
       <c r="B6" s="10"/>
       <c r="C6" s="10"/>
       <c r="D6" s="10"/>
       <c r="E6" s="10"/>
       <c r="F6" s="10"/>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G6" s="10"/>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" s="10"/>
       <c r="B7" s="10"/>
       <c r="C7" s="10"/>
       <c r="D7" s="10"/>
       <c r="E7" s="10"/>
       <c r="F7" s="10"/>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="D9" t="s">
-        <v>187</v>
-      </c>
+      <c r="G7" s="10"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -3774,19 +3795,19 @@
         <v>25</v>
       </c>
       <c r="B2" s="18" t="s">
+        <v>123</v>
+      </c>
+      <c r="C2" s="34" t="s">
         <v>124</v>
       </c>
-      <c r="C2" s="34" t="s">
+      <c r="D2" s="34" t="s">
         <v>125</v>
       </c>
-      <c r="D2" s="34" t="s">
+      <c r="E2" s="34" t="s">
         <v>126</v>
       </c>
-      <c r="E2" s="34" t="s">
+      <c r="F2" s="34" t="s">
         <v>127</v>
-      </c>
-      <c r="F2" s="34" t="s">
-        <v>128</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
@@ -3794,9 +3815,9 @@
         <v>36</v>
       </c>
       <c r="B3" s="35" t="s">
-        <v>119</v>
-      </c>
-      <c r="C3" s="38" t="s">
+        <v>118</v>
+      </c>
+      <c r="C3" s="35" t="s">
         <v>52</v>
       </c>
       <c r="D3" s="13" t="s">
@@ -3817,8 +3838,8 @@
         <f>Cita_D!G4</f>
         <v>Juan Fernando García Lopez-30/09/2026/10:00</v>
       </c>
-      <c r="C4" s="12" t="str">
-        <f>Servicio_D!E4</f>
+      <c r="C4" s="11" t="str">
+        <f>Servicio_D!F4</f>
         <v>Motilada</v>
       </c>
       <c r="D4" s="12">
@@ -3840,8 +3861,8 @@
         <f>Cita_D!G5</f>
         <v>Juan David Ortiz Sanchez-22/11/2025/11:00</v>
       </c>
-      <c r="C5" s="12" t="str">
-        <f>Servicio_D!E4</f>
+      <c r="C5" s="11" t="str">
+        <f>Servicio_D!F4</f>
         <v>Motilada</v>
       </c>
       <c r="D5" s="12">
@@ -3863,8 +3884,8 @@
         <f>Cita_D!G6</f>
         <v>Carlos Arbeladez-10/08/2024/14:00</v>
       </c>
-      <c r="C6" s="12" t="str">
-        <f>Servicio_D!E6</f>
+      <c r="C6" s="11" t="str">
+        <f>Servicio_D!F6</f>
         <v>Perfilada de barba</v>
       </c>
       <c r="D6" s="12">
@@ -3886,8 +3907,8 @@
         <f>Cita_D!G7</f>
         <v>Andres Ramirez Patiño-24/09/2026/13:00</v>
       </c>
-      <c r="C7" s="28" t="str">
-        <f>Servicio_D!E7</f>
+      <c r="C7" s="59" t="str">
+        <f>Servicio_D!F7</f>
         <v>Arreglo completo de barba con toalla caliente</v>
       </c>
       <c r="D7" s="12">
@@ -3909,7 +3930,7 @@
         <f>Cita_D!G8</f>
         <v>Carlos Arbeladez-06/08/2026/18:00</v>
       </c>
-      <c r="C8" s="12" t="s">
+      <c r="C8" s="11" t="s">
         <v>57</v>
       </c>
       <c r="D8" s="12">
@@ -3934,6 +3955,12 @@
     <hyperlink ref="B6" location="Cita_D!A6" display="Cita_D!A6" xr:uid="{7C3F9E66-FC63-4CC5-A67C-8604702403F0}"/>
     <hyperlink ref="B7" location="Cita_D!A7" display="Cita_D!A7" xr:uid="{B03F3CEB-2FAE-4C17-B421-BB7244341FF9}"/>
     <hyperlink ref="B8" location="Cita_D!A8" display="Cita_D!A8" xr:uid="{FA20FBDC-E2C6-44CF-B98E-C85818BE6D1B}"/>
+    <hyperlink ref="C3" location="Servicio_D!A1" display="servicio" xr:uid="{46A59B94-B463-41EF-A1B6-2B1BD97218B9}"/>
+    <hyperlink ref="C4" location="Servicio_D!A4" display="Servicio_D!A4" xr:uid="{E5D47101-7002-491C-A64F-9E08C0E5E166}"/>
+    <hyperlink ref="C5" location="Servicio_D!A4" display="Servicio_D!A4" xr:uid="{EC363894-A006-45A1-A451-8A105D143020}"/>
+    <hyperlink ref="C6" location="Servicio_D!A6" display="Servicio_D!A6" xr:uid="{2F70A83F-4454-46E6-A1E5-B359824AA24F}"/>
+    <hyperlink ref="C7" location="Servicio_D!A7" display="Servicio_D!A7" xr:uid="{36945D0D-E1EC-4BD2-A67D-287FB73A0E8D}"/>
+    <hyperlink ref="C8" location="Servicio_D!A5" display="Corte de barba" xr:uid="{52D089FF-955D-405E-BFF7-8EABA1516B8E}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -4250,30 +4277,30 @@
       <c r="G1" s="12"/>
       <c r="H1" s="12"/>
     </row>
-    <row r="2" spans="1:8" ht="30" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" ht="39.6" x14ac:dyDescent="0.3">
       <c r="A2" s="18" t="s">
         <v>25</v>
       </c>
       <c r="B2" s="18" t="s">
+        <v>154</v>
+      </c>
+      <c r="C2" s="18" t="s">
         <v>155</v>
       </c>
-      <c r="C2" s="18" t="s">
+      <c r="D2" s="18" t="s">
         <v>156</v>
       </c>
-      <c r="D2" s="18" t="s">
+      <c r="E2" s="18" t="s">
         <v>157</v>
       </c>
-      <c r="E2" s="18" t="s">
-        <v>158</v>
-      </c>
       <c r="F2" s="18" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="G2" s="19" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="H2" s="20" t="s">
-        <v>189</v>
+        <v>183</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -4281,19 +4308,19 @@
         <v>36</v>
       </c>
       <c r="B3" s="13" t="s">
+        <v>130</v>
+      </c>
+      <c r="C3" s="13" t="s">
+        <v>132</v>
+      </c>
+      <c r="D3" s="13" t="s">
         <v>131</v>
       </c>
-      <c r="C3" s="13" t="s">
+      <c r="E3" s="13" t="s">
         <v>133</v>
       </c>
-      <c r="D3" s="13" t="s">
-        <v>132</v>
-      </c>
-      <c r="E3" s="13" t="s">
-        <v>134</v>
-      </c>
       <c r="F3" s="13" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="G3" s="13" t="s">
         <v>27</v>
@@ -4307,15 +4334,15 @@
         <v>1</v>
       </c>
       <c r="B4" s="12" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="C4" s="12"/>
       <c r="D4" s="12" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="E4" s="12"/>
       <c r="F4" s="53" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="G4" s="12">
         <v>3234528921</v>
@@ -4330,19 +4357,19 @@
         <v>2</v>
       </c>
       <c r="B5" s="12" t="s">
+        <v>149</v>
+      </c>
+      <c r="C5" s="12" t="s">
         <v>150</v>
       </c>
-      <c r="C5" s="12" t="s">
-        <v>151</v>
-      </c>
       <c r="D5" s="12" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="E5" s="12" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="F5" s="53" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="G5" s="12">
         <v>3161657782</v>
@@ -4357,17 +4384,17 @@
         <v>3</v>
       </c>
       <c r="B6" s="12" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="C6" s="12"/>
       <c r="D6" s="12" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="E6" s="12" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="F6" s="53" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="G6" s="12">
         <v>3119884321</v>
@@ -4382,15 +4409,15 @@
         <v>4</v>
       </c>
       <c r="B7" s="12" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="C7" s="12"/>
       <c r="D7" s="12" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="E7" s="12"/>
       <c r="F7" s="53" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="G7" s="12">
         <v>4127359182</v>
@@ -4533,16 +4560,16 @@
         <v>98</v>
       </c>
       <c r="C2" s="19" t="s">
+        <v>158</v>
+      </c>
+      <c r="D2" s="19" t="s">
         <v>159</v>
       </c>
-      <c r="D2" s="19" t="s">
+      <c r="E2" s="19" t="s">
         <v>160</v>
       </c>
-      <c r="E2" s="19" t="s">
+      <c r="F2" s="19" t="s">
         <v>161</v>
-      </c>
-      <c r="F2" s="19" t="s">
-        <v>162</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
@@ -4721,169 +4748,199 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C97B567D-D27E-4BE3-B1E4-8CA267790151}">
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:F12"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="28.109375" customWidth="1"/>
-    <col min="2" max="2" width="26.5546875" customWidth="1"/>
-    <col min="3" max="3" width="16.33203125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="17.33203125" customWidth="1"/>
-    <col min="5" max="5" width="26.5546875" customWidth="1"/>
+    <col min="1" max="2" width="28.109375" customWidth="1"/>
+    <col min="3" max="3" width="26.5546875" customWidth="1"/>
+    <col min="4" max="4" width="16.33203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="17.33203125" customWidth="1"/>
+    <col min="6" max="6" width="26.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" s="16" t="s">
         <v>37</v>
       </c>
       <c r="B1" s="16" t="s">
         <v>38</v>
       </c>
-      <c r="C1" s="17"/>
       <c r="D1" s="17"/>
-      <c r="E1" s="10"/>
-    </row>
-    <row r="2" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="E1" s="17"/>
+      <c r="F1" s="10"/>
+    </row>
+    <row r="2" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A2" s="21" t="s">
         <v>25</v>
       </c>
       <c r="B2" s="21" t="s">
+        <v>185</v>
+      </c>
+      <c r="C2" s="21" t="s">
         <v>44</v>
       </c>
-      <c r="C2" s="22" t="s">
+      <c r="D2" s="22" t="s">
         <v>46</v>
       </c>
-      <c r="D2" s="22" t="s">
+      <c r="E2" s="22" t="s">
         <v>47</v>
       </c>
-      <c r="E2" s="19" t="s">
+      <c r="F2" s="19" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" s="23" t="s">
         <v>36</v>
       </c>
-      <c r="B3" s="24" t="s">
+      <c r="B3" s="60" t="s">
+        <v>43</v>
+      </c>
+      <c r="C3" s="24" t="s">
         <v>26</v>
       </c>
-      <c r="C3" s="24" t="s">
+      <c r="D3" s="24" t="s">
         <v>45</v>
       </c>
-      <c r="D3" s="24" t="s">
+      <c r="E3" s="24" t="s">
         <v>29</v>
       </c>
-      <c r="E3" s="15" t="s">
+      <c r="F3" s="15" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" s="25">
         <v>1</v>
       </c>
-      <c r="B4" s="25" t="s">
+      <c r="B4" s="61" t="str">
+        <f>Barberia_D!B4</f>
+        <v>Barbería Oriental</v>
+      </c>
+      <c r="C4" s="25" t="s">
         <v>49</v>
       </c>
-      <c r="C4" s="25">
+      <c r="D4" s="25">
         <v>45</v>
       </c>
-      <c r="D4" s="26">
+      <c r="E4" s="26">
         <v>22000</v>
       </c>
-      <c r="E4" s="12" t="str">
-        <f>B4</f>
+      <c r="F4" s="12" t="str">
+        <f>C4</f>
         <v>Motilada</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" s="25">
         <v>2</v>
       </c>
-      <c r="B5" s="25" t="s">
+      <c r="B5" s="61" t="str">
+        <f>Barberia_D!B4</f>
+        <v>Barbería Oriental</v>
+      </c>
+      <c r="C5" s="25" t="s">
         <v>57</v>
       </c>
-      <c r="C5" s="25">
+      <c r="D5" s="25">
         <v>10</v>
       </c>
-      <c r="D5" s="26">
+      <c r="E5" s="26">
         <v>12000</v>
       </c>
-      <c r="E5" s="12" t="str">
-        <f t="shared" ref="E5:E7" si="0">B5</f>
+      <c r="F5" s="12" t="str">
+        <f t="shared" ref="F5:F7" si="0">C5</f>
         <v>Corte de barba</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" s="25">
         <v>3</v>
       </c>
-      <c r="B6" s="25" t="s">
+      <c r="B6" s="61" t="str">
+        <f>Barberia_D!B4</f>
+        <v>Barbería Oriental</v>
+      </c>
+      <c r="C6" s="25" t="s">
         <v>58</v>
       </c>
-      <c r="C6" s="25">
+      <c r="D6" s="25">
         <v>15</v>
       </c>
-      <c r="D6" s="26">
+      <c r="E6" s="26">
         <v>15000</v>
       </c>
-      <c r="E6" s="12" t="str">
+      <c r="F6" s="12" t="str">
         <f t="shared" si="0"/>
         <v>Perfilada de barba</v>
       </c>
     </row>
-    <row r="7" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A7" s="25">
         <v>4</v>
       </c>
-      <c r="B7" s="27" t="s">
+      <c r="B7" s="61" t="str">
+        <f>Barberia_D!B4</f>
+        <v>Barbería Oriental</v>
+      </c>
+      <c r="C7" s="27" t="s">
         <v>59</v>
       </c>
-      <c r="C7" s="25">
+      <c r="D7" s="25">
         <v>30</v>
       </c>
-      <c r="D7" s="26">
+      <c r="E7" s="26">
         <v>35000</v>
       </c>
-      <c r="E7" s="28" t="str">
+      <c r="F7" s="28" t="str">
         <f t="shared" si="0"/>
         <v>Arreglo completo de barba con toalla caliente</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8" s="17"/>
       <c r="B8" s="17"/>
       <c r="C8" s="17"/>
       <c r="D8" s="17"/>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="E8" s="17"/>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A9" s="17"/>
       <c r="B9" s="17"/>
       <c r="C9" s="17"/>
       <c r="D9" s="17"/>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="E9" s="17"/>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A10" s="17"/>
       <c r="B10" s="17"/>
       <c r="C10" s="17"/>
       <c r="D10" s="17"/>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="E10" s="17"/>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A11" s="17"/>
-      <c r="B11" s="17" t="s">
-        <v>180</v>
-      </c>
+      <c r="B11" s="17"/>
       <c r="C11" s="17"/>
       <c r="D11" s="17"/>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="E11" s="17"/>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A12" s="17"/>
       <c r="B12" s="17"/>
       <c r="C12" s="17"/>
       <c r="D12" s="17"/>
+      <c r="E12" s="17"/>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="A1" location="'Modelo de Dominio'!A1" display="&lt;&lt;&lt;&lt; Ir al modulo de dominio" xr:uid="{1232B379-2C8F-4361-B8CE-5CC492F8D207}"/>
     <hyperlink ref="B1" location="'Objetos de Dominio'!A1" display="&lt;&lt;&lt;&lt; Ir a objetos de dominio" xr:uid="{C4612CEA-B79F-4496-B57E-5F6E72A804C7}"/>
+    <hyperlink ref="B3" location="Barberia_D!A1" display="barberia" xr:uid="{49DC9582-0184-41B1-95D7-525F6EE28820}"/>
+    <hyperlink ref="B4" location="Barberia_D!A4" display="Barberia_D!A4" xr:uid="{9C3C8EC0-3D4B-4A80-9FA2-4578065166BB}"/>
+    <hyperlink ref="B5" location="Barberia_D!A4" display="Barberia_D!A4" xr:uid="{1337E6E0-8BBF-46FA-B386-3E8B848525E7}"/>
+    <hyperlink ref="B6" location="Servicio_D!A4" display="Servicio_D!A4" xr:uid="{F14FFAD6-C31D-4D17-A87C-7C4566115E73}"/>
+    <hyperlink ref="B7" location="Barberia_D!A4" display="Barberia_D!A4" xr:uid="{75AD25E9-0697-4BA2-8F6A-B890AAE2A8F8}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -4891,7 +4948,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2DAE59AB-4103-4731-9C3C-4C276F8A29F8}">
-  <dimension ref="A1:K11"/>
+  <dimension ref="A1:L10"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="27" bestFit="1" customWidth="1"/>
@@ -4899,10 +4956,11 @@
     <col min="7" max="7" width="16.33203125" customWidth="1"/>
     <col min="8" max="9" width="40.6640625" customWidth="1"/>
     <col min="10" max="10" width="27.109375" customWidth="1"/>
-    <col min="11" max="11" width="53.109375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="21" customWidth="1"/>
+    <col min="12" max="12" width="53.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A1" s="5" t="s">
         <v>37</v>
       </c>
@@ -4914,59 +4972,62 @@
       <c r="E1" s="5"/>
       <c r="F1" s="5"/>
     </row>
-    <row r="2" spans="1:11" ht="45.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:12" ht="45.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="29" t="s">
         <v>25</v>
       </c>
       <c r="B2" s="29" t="s">
+        <v>141</v>
+      </c>
+      <c r="C2" s="29" t="s">
+        <v>143</v>
+      </c>
+      <c r="D2" s="29" t="s">
         <v>142</v>
       </c>
-      <c r="C2" s="29" t="s">
-        <v>144</v>
-      </c>
-      <c r="D2" s="29" t="s">
-        <v>143</v>
-      </c>
       <c r="E2" s="29" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F2" s="29" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="G2" s="30" t="s">
         <v>60</v>
       </c>
       <c r="H2" s="30" t="s">
+        <v>165</v>
+      </c>
+      <c r="I2" s="30" t="s">
         <v>166</v>
       </c>
-      <c r="I2" s="30" t="s">
-        <v>167</v>
-      </c>
       <c r="J2" s="30" t="s">
-        <v>178</v>
-      </c>
-      <c r="K2" s="31" t="s">
-        <v>171</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
+        <v>177</v>
+      </c>
+      <c r="K2" s="30" t="s">
+        <v>186</v>
+      </c>
+      <c r="L2" s="31" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A3" s="14" t="s">
         <v>36</v>
       </c>
       <c r="B3" s="13" t="s">
+        <v>130</v>
+      </c>
+      <c r="C3" s="13" t="s">
+        <v>132</v>
+      </c>
+      <c r="D3" s="13" t="s">
         <v>131</v>
       </c>
-      <c r="C3" s="13" t="s">
+      <c r="E3" s="13" t="s">
         <v>133</v>
       </c>
-      <c r="D3" s="13" t="s">
-        <v>132</v>
-      </c>
-      <c r="E3" s="13" t="s">
-        <v>134</v>
-      </c>
       <c r="F3" s="13" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="G3" s="13" t="s">
         <v>27</v>
@@ -4975,16 +5036,19 @@
         <v>53</v>
       </c>
       <c r="I3" s="13" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="J3" s="49" t="s">
         <v>54</v>
       </c>
-      <c r="K3" s="32" t="s">
+      <c r="K3" s="35" t="s">
+        <v>43</v>
+      </c>
+      <c r="L3" s="32" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A4" s="12">
         <v>1</v>
       </c>
@@ -4992,16 +5056,16 @@
         <v>63</v>
       </c>
       <c r="C4" s="12" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="D4" s="12" t="s">
         <v>67</v>
       </c>
       <c r="E4" s="12" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="F4" s="53" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="G4" s="12">
         <v>3245627890</v>
@@ -5015,12 +5079,16 @@
       <c r="J4" s="12" t="s">
         <v>61</v>
       </c>
-      <c r="K4" s="12" t="str">
+      <c r="K4" s="55" t="str">
+        <f>Barberia_D!B4</f>
+        <v>Barbería Oriental</v>
+      </c>
+      <c r="L4" s="12" t="str">
         <f>_xlfn.CONCAT(B4,"-",C4,"-",D4,"-",E4,"-",F4,"-",G4)</f>
         <v>Juan Fernando-Fernando-García Lopez-Lopez-+57-3245627890</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A5" s="12">
         <v>2</v>
       </c>
@@ -5028,16 +5096,16 @@
         <v>64</v>
       </c>
       <c r="C5" s="12" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="D5" s="12" t="s">
         <v>68</v>
       </c>
       <c r="E5" s="12" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="F5" s="53" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="G5" s="12">
         <v>3124518923</v>
@@ -5046,17 +5114,21 @@
         <v>71</v>
       </c>
       <c r="I5" s="51" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="J5" s="12" t="s">
         <v>62</v>
       </c>
-      <c r="K5" s="12" t="str">
-        <f t="shared" ref="K5:K7" si="0">_xlfn.CONCAT(B5,"-",C5,"-",D5,"-",E5,"-",F5,"-",G5)</f>
+      <c r="K5" s="55" t="str">
+        <f>Barberia_D!B4</f>
+        <v>Barbería Oriental</v>
+      </c>
+      <c r="L5" s="12" t="str">
+        <f t="shared" ref="L5:L7" si="0">_xlfn.CONCAT(B5,"-",C5,"-",D5,"-",E5,"-",F5,"-",G5)</f>
         <v>Juan David-David-Ortiz Sanchez-Sanchez-+57-3124518923</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A6" s="12">
         <v>3</v>
       </c>
@@ -5065,11 +5137,11 @@
       </c>
       <c r="C6" s="12"/>
       <c r="D6" s="12" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="E6" s="12"/>
       <c r="F6" s="53" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="G6" s="12">
         <v>3214533321</v>
@@ -5078,17 +5150,21 @@
         <v>72</v>
       </c>
       <c r="I6" s="52" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="J6" s="12" t="s">
         <v>61</v>
       </c>
-      <c r="K6" s="12" t="str">
+      <c r="K6" s="55" t="str">
+        <f>Barberia_D!B4</f>
+        <v>Barbería Oriental</v>
+      </c>
+      <c r="L6" s="12" t="str">
         <f t="shared" si="0"/>
         <v>Carlos--Arbeladez--+57-3214533321</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A7" s="12">
         <v>4</v>
       </c>
@@ -5100,10 +5176,10 @@
         <v>69</v>
       </c>
       <c r="E7" s="12" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="F7" s="53" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="G7" s="12">
         <v>9876543210</v>
@@ -5112,24 +5188,23 @@
         <v>73</v>
       </c>
       <c r="I7" s="51" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="J7" s="12" t="s">
         <v>61</v>
       </c>
-      <c r="K7" s="12" t="str">
+      <c r="K7" s="55" t="str">
+        <f>Barberia_D!B4</f>
+        <v>Barbería Oriental</v>
+      </c>
+      <c r="L7" s="12" t="str">
         <f t="shared" si="0"/>
         <v>Andres--Ramirez Patiño-Patiño-+91-9876543210</v>
       </c>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:12" x14ac:dyDescent="0.3">
       <c r="B10" s="10"/>
       <c r="C10" s="10"/>
-    </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="B11" t="s">
-        <v>179</v>
-      </c>
     </row>
   </sheetData>
   <phoneticPr fontId="7" type="noConversion"/>
@@ -5140,6 +5215,9 @@
     <hyperlink ref="H5" r:id="rId2" xr:uid="{6DE7DFDC-37F8-4F9E-9AEF-2A9B5D465DE8}"/>
     <hyperlink ref="H6" r:id="rId3" xr:uid="{4550EE1F-4989-43BD-948F-5BD527B9D531}"/>
     <hyperlink ref="H7" r:id="rId4" xr:uid="{72EF9758-1786-4FA4-86ED-08E3A4E7C6AD}"/>
+    <hyperlink ref="K3" location="Barberia_D!A1" display="barberia" xr:uid="{0A424D71-DFC6-4A9B-AB84-795AF0206DA0}"/>
+    <hyperlink ref="K4" location="Barberia_D!A4" display="Barberia_D!A4" xr:uid="{74759F60-91D9-4AA0-8D34-C14AE4845BDE}"/>
+    <hyperlink ref="K5:K7" location="Barberia_D!A4" display="Barberia_D!A4" xr:uid="{8B3C5650-71BD-4B78-A8B9-12566120F044}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -5176,7 +5254,7 @@
         <v>77</v>
       </c>
       <c r="D2" s="34" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="E2" s="34" t="s">
         <v>76</v>
@@ -5278,11 +5356,6 @@
     <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="C8" s="33"/>
       <c r="D8" s="33"/>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="C10" t="s">
-        <v>188</v>
-      </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.3">
       <c r="C11" s="50"/>

</xml_diff>

<commit_message>
Se añadieron los tipos de datos, valores por defecto, si son o no permitidos; desde Barberia, hasta Barbero. Falta terminar de definir los otros y pensar si los ya definidos están bien.
</commit_message>
<xml_diff>
--- a/Muestreo de datos.xlsx
+++ b/Muestreo de datos.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\leand\Desktop\DOO\DOO\Barberia\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jesus\OneDrive\Escritorio\leo\Doo\Barberia proyecto\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{81BFAD6D-9C90-4CE7-B6FE-4D8B9CAEDEAD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6884477C-7AFB-4EA2-A1F3-CB639B29ADD1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{09A6C7D7-663F-4C06-9D71-8A4E97495CF9}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" firstSheet="1" activeTab="7" xr2:uid="{09A6C7D7-663F-4C06-9D71-8A4E97495CF9}"/>
   </bookViews>
   <sheets>
     <sheet name="Modelo de Dominio" sheetId="1" r:id="rId1"/>
@@ -53,7 +53,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="297" uniqueCount="191">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="306" uniqueCount="194">
   <si>
     <t>Nombre</t>
   </si>
@@ -103,27 +103,12 @@
     <t>Representa el negocio donde trabajan los barberos, agrupa el catalogo de servicios que ofrece y las reglas de tolerancia, multas y veto que aplican para todos sus clientes</t>
   </si>
   <si>
-    <t>Representa un tipo de servicio que ofrece la barbería, por ejemplo, motilada, afeitada de barba, perfilar barba, con su duración y su precio. Este precio es el que se usa para calcular la multa cuando un cliente no se presenta a una cita</t>
-  </si>
-  <si>
     <t>Representa a un trabajador de la barbería que atiende clientes segun los servicios que sabe realizar y que organiza su tiempo a través de su propia agenda</t>
   </si>
   <si>
     <t>Representa que servicios realiza cada barbero, ya que no todos los barberos de la barbería ofrecen los mismos servicios</t>
   </si>
   <si>
-    <t>Representa el historial de estado de bloqueo de un cliente, cuando esta activo, ningun barbero de la barbería puede agendarle nuevas citas. Se activa cuando el cliente llega al número de multas sin pagar definido en Regla</t>
-  </si>
-  <si>
-    <t>Representa el calendario de un barbero, incluye su horario de trabajo, sus bloqueos temporales (permisos, capacitaciones, compromisos que no le permiten trabajar) y las citas que se le van agendando, validando que ninguna se cruce con otra</t>
-  </si>
-  <si>
-    <t>Representa las politicas configurables del negocio, cuantos minutos de tolerancia se permiten antes de aplicar una multa por tardanza, cuanto vale esa multa, y cuantas multas sin pagar se necesitan para que un cliente quede vetado</t>
-  </si>
-  <si>
-    <t>Representa una cita agendada por un cliente con un barbero, incluye la fecha y hora, el o los servicios solicitados, y su estado agendada(indica que se ha creado la cita y esta esperando el cambio de estado depues de la hora prevista de finalizacion), atendida(indica que el barbero atendió correctamente al cliente), incumplida(indica que el cliente violó una de las reglas establecidas) o cancelada(indica que el cliente le pidio al barbero que ya no quiere la cita, por lo que esta cita no va a aparecer en su agenda)</t>
-  </si>
-  <si>
     <t>Representa la sanción económica que se le impone a un cliente por incumplir una cita (llegar tarde fuera de tolerancia o no presentarse), calculada a partir de la cita específica que la originó</t>
   </si>
   <si>
@@ -178,30 +163,12 @@
     <t>toleranciaTardanza</t>
   </si>
   <si>
-    <t>Representa la cantidad de minutos que el cliente puede llegarle tarde un cliente a la cita establecida con el barbero, despues de eso el barbero lo podrá multar</t>
-  </si>
-  <si>
-    <t>Representa la maxima de multas que pueda tener un cliente sin pagar, a partir de esta cantidad se le hace un veto al cliente</t>
-  </si>
-  <si>
     <t>barberia</t>
   </si>
   <si>
-    <t>Representa el nombre del servicio que va estar en la barberia, que el barbero ofrece y en las citas que esta</t>
-  </si>
-  <si>
     <t>duracion</t>
   </si>
   <si>
-    <t>Representa lo que va durar en minutos el servicio</t>
-  </si>
-  <si>
-    <t>Representa cuanto va a valer el servicio en pesos colombianos</t>
-  </si>
-  <si>
-    <t>Representa la cantidad de dinero que el cliente debe de pagar en pesos colombianos, por superar la toleranciaTardanza</t>
-  </si>
-  <si>
     <t>Motilada</t>
   </si>
   <si>
@@ -244,27 +211,12 @@
     <t>no</t>
   </si>
   <si>
-    <t>Juan Fernando</t>
-  </si>
-  <si>
-    <t>Juan David</t>
-  </si>
-  <si>
     <t>Carlos</t>
   </si>
   <si>
     <t>Andres</t>
   </si>
   <si>
-    <t>García Lopez</t>
-  </si>
-  <si>
-    <t>Ortiz Sanchez</t>
-  </si>
-  <si>
-    <t>Ramirez Patiño</t>
-  </si>
-  <si>
     <t>juanfer234535@gmail.com</t>
   </si>
   <si>
@@ -310,9 +262,6 @@
     <t>agendada</t>
   </si>
   <si>
-    <t>Representa el nombre de como se llama la barberia en donde trabajan los barberos</t>
-  </si>
-  <si>
     <t>Barbería Oriental</t>
   </si>
   <si>
@@ -338,15 +287,6 @@
   </si>
   <si>
     <t>HorarioBarbero</t>
-  </si>
-  <si>
-    <t>Representa a la persona que solicita citas en la barbería, el se las pide a un barbero por WhatsApp. Cada uno solo es para que en el sistema tenga un historial de las citas que ha pedido, de multas y de vetos</t>
-  </si>
-  <si>
-    <t>Representa cada dia de la semana, hora en el que entra, hora a la que sale, para que la agenda del barbero sepa que dias trabaja el</t>
-  </si>
-  <si>
-    <t>Representa cada día de la semana en los que la barberia abre, la hora a la que abre y cierra la barberia</t>
   </si>
   <si>
     <t>Representa el nombre de la barberia que va pertencer los horarios de la barberia</t>
@@ -440,9 +380,6 @@
     <t>Combinación única que indica que un mismo servicio no puede repetirse dos veces dentro de la misma cita</t>
   </si>
   <si>
-    <t>Representa el numero de celular de la persona que le va aescribir al barbero por WhatsApp para pedirle una cita</t>
-  </si>
-  <si>
     <t>Combinación única que indica que un mismo barbero no puede aparecer dos veces ofreciendo el mismo servicio</t>
   </si>
   <si>
@@ -476,18 +413,6 @@
     <t>Arbeladez</t>
   </si>
   <si>
-    <t>Representa el segundo apellido del barbero que trabaja en la barbería, su valor por defecto es el vacio y es permitido</t>
-  </si>
-  <si>
-    <t>Representa el primer nombre del barbero que trabaja en barbería, su valor por defecto es el vacio</t>
-  </si>
-  <si>
-    <t>Representa el primer apellido del barbero que trabaja en la barbería, su valor por defecto es el vacio</t>
-  </si>
-  <si>
-    <t>Representa el segundo nombre del barbero que trabaja en barbería, su valor por defecto es el vacio y es permitido</t>
-  </si>
-  <si>
     <t>Gómez</t>
   </si>
   <si>
@@ -518,27 +443,9 @@
     <t>Alexis</t>
   </si>
   <si>
-    <t>Representa el primer nombre de la persona, que va a estar llendo a la barberia para las citas, su valor por defecto es el vacío y no es permitido</t>
-  </si>
-  <si>
-    <t>Representa el segundo nombre de la persona, que va a estar llendo a la barberia para las citas, su valor por defecto es el vacío y es permitido</t>
-  </si>
-  <si>
-    <t>Representa el primer apellido de la persona, que va a estar llendo a la barberia para las citas, su valor por defecto es el vacío y no es permitido</t>
-  </si>
-  <si>
-    <t>Representa el primer apellido de la persona, que va a estar llendo a la barberia para las citas, su valor por defecto es el vacío y es permitido</t>
-  </si>
-  <si>
     <t>Representa el día de la semana en que aplica este horario, es necesario para saber que días abrira la barberia</t>
   </si>
   <si>
-    <t>Representa la hora a la que abre la barbería</t>
-  </si>
-  <si>
-    <t>Representa la hora a la que cierra la barbería</t>
-  </si>
-  <si>
     <t>Combinacion única que indica que no puede existir más de un horario con la misma barberia, dia de la semana, hora de apertura y cierre</t>
   </si>
   <si>
@@ -551,12 +458,6 @@
     <t>contraseña</t>
   </si>
   <si>
-    <t>Representa el correo electronico del barbero, con el que se va a registrar o iniciar seción</t>
-  </si>
-  <si>
-    <t>Representa la contraseña del barbebro, con el que se va a registrar o iniciar sesión</t>
-  </si>
-  <si>
     <t>Carlos.1995</t>
   </si>
   <si>
@@ -566,9 +467,6 @@
     <t>ramirezpatinio23121</t>
   </si>
   <si>
-    <t>Combinacion única que indica que no puede existir más de un barbero con el mismo nombre, apellidos y  número de celular</t>
-  </si>
-  <si>
     <t>prefijo</t>
   </si>
   <si>
@@ -576,12 +474,6 @@
   </si>
   <si>
     <t>+58</t>
-  </si>
-  <si>
-    <t>Representa de que pais es el numero de celular del cliente</t>
-  </si>
-  <si>
-    <t>Representa de que pais es el numero de celular del barbero</t>
   </si>
   <si>
     <t>+91</t>
@@ -628,6 +520,123 @@
   </si>
   <si>
     <t>Representa el tipo de multa con el que se va sancionar, si es retraso o incumplida. Este es un dato obtenido del estado de cita</t>
+  </si>
+  <si>
+    <t>Ortiz</t>
+  </si>
+  <si>
+    <t>García</t>
+  </si>
+  <si>
+    <t>Zambrano</t>
+  </si>
+  <si>
+    <t>+593</t>
+  </si>
+  <si>
+    <t>juancarloszambrano4394@gmail.com</t>
+  </si>
+  <si>
+    <t>Combinacion única que indica que no puede existir más de un barbero con el mismo nombre, apellidos y número de celular</t>
+  </si>
+  <si>
+    <t>Representa a la persona que solicita citas en la barbería, el se las pide a un barbero por WhatsApp. Su valor esta en darle al sistema un historial por persona: que citas ha pedido, que multas tiene y si esta o no vetado, para que cualquier barbero sepa con quien esta tratando antes de agendarle.</t>
+  </si>
+  <si>
+    <t>Representa las políticas de la barbería frente al incumplimiento de los clientes: cuantos minutos de tolerancia se dan antes de considerar tardanza, cuanto vale la multa fija por llegar tarde, y cuantas multas sin pagar activan un veto</t>
+  </si>
+  <si>
+    <t>Representa, día por día, a que hora abre y cierra el negocio. Es el límite dentro del cual tiene que caber el horario de cualquier barbero, nadie puede trabajar antes de que abra ni después de que cierre</t>
+  </si>
+  <si>
+    <t>Representa cada tipo de corte o arreglo que ofrece la barbería, con su duración y su precio. Es el catalogo del que sale tanto lo que un barbero puede ofrecer como lo que termina costando y durando cada cita</t>
+  </si>
+  <si>
+    <t>Representa el historial de bloqueos de un cliente. Cuando esta activo, ningún barbero de la barbería puede agendarle citas nuevas a esa persona. Su valor es proteger a todos los barberos de un mismo cliente problemático, sin que cada uno tenga que enterarse por su cuenta</t>
+  </si>
+  <si>
+    <t>Representa el calendario propio de un barbero. Es donde se organiza su horario de trabajo y las citas que se le van agendando, validando que ninguna se le cruce con otra</t>
+  </si>
+  <si>
+    <t>Representa cada día de la semana, hora en el que entra, hora a la que sale, para que la agenda del barbero sepa que días trabaja el</t>
+  </si>
+  <si>
+    <t>Representa la reserva de un cliente con un barbero para una fecha y hora puntual. De ella sale tanto el cálculo de cuanto queda ocupado el barbero como la funcionalidad de si hay o no una multa (se genera cuando un barbero pone el estado de la cita en retraso o inclumplida), según cómo haya terminado (atendida, con retraso, incumplida o cancelada)</t>
+  </si>
+  <si>
+    <t>Representa el nombre de como se llama la barberia en donde trabajan los barberos. El tipo de dato es alfanumérico, su valor por defecto es el vacio y es permitido</t>
+  </si>
+  <si>
+    <t>Representa el primer nombre de la persona, que va a estar llendo a la barberia para las citas. Su tipo de dato es texto, su valor por defecto es el vacío y no es permitido</t>
+  </si>
+  <si>
+    <t>Representa el segundo nombre de la persona, que va a estar llendo a la barberia para las citas. Su tipo de dato es texto, su valor por defecto es el vacío y es permitido</t>
+  </si>
+  <si>
+    <t>Representa el primer apellido de la persona, que va a estar llendo a la barberia para las citas. Su tipo de dato es texto, su valor por defecto es el vacío y no es permitido</t>
+  </si>
+  <si>
+    <t>Representa el primer apellido de la persona, que va a estar llendo a la barberia para las citas. Su tipo de dato es texto, su valor por defecto es el vacío y es permitido</t>
+  </si>
+  <si>
+    <t>prefijoCelular</t>
+  </si>
+  <si>
+    <t>Representa de que pais es el numero de celular del cliente. Su tipo de dato es alfanumérico, su valor por defecto es +0 (este prefijo no referencia a ningún país) y no es permitido</t>
+  </si>
+  <si>
+    <t>Representa el numero de celular de la persona que le va a escribir al barbero por WhatsApp para pedirle una cita. Su tipo de dato es alfanumérico, su valor por defecto es el 0 y no es permitido</t>
+  </si>
+  <si>
+    <t>Representa la cantidad de minutos que el cliente puede llegarle tarde un cliente a la cita establecida con el barbero, despues de eso el barbero lo podrá multar. Su tipo de dato es numerico, debe de ser mayor o igual a 0, su valor por defecto es el 0 y es permitido</t>
+  </si>
+  <si>
+    <t>Representa la cantidad de dinero que el cliente debe de pagar en pesos colombianos, por superar la toleranciaTardanza. Su tipo de dato es numerico, debe de ser mayor a cero, su valor por defecto es 0 y no es permitido</t>
+  </si>
+  <si>
+    <t>Representa la maxima de multas que pueda tener un cliente sin pagar, a partir de esta cantidad se le hace un veto al cliente. Su tipo de dato es numerico, debe de ser mayor o igual a cero, su valor por defecto es 0 y es permitido</t>
+  </si>
+  <si>
+    <t>Este dato lo tengo pensado como si fuera una lista</t>
+  </si>
+  <si>
+    <t>Representa la hora a la que abre la barbería. Su tipo de dato es hora, su valor por defecto es 00:00 am y es permitido</t>
+  </si>
+  <si>
+    <t>Representa la hora a la que cierra la barbería. Su tipo de dato es hora, su valor por defecto es 00:00 am y es permitido</t>
+  </si>
+  <si>
+    <t>Representa el nombre del servicio que va estar en la barberia, que el barbero ofrece y en las citas que esta. Su tipo de dato es alfanumérico, su valor por defecto es el vacio y no es permitido</t>
+  </si>
+  <si>
+    <t>Representa lo que va durar en minutos el servicio. Su tipo de dato es entero, debe de ser mayor a cero, su valor por defecto es 0 y no es permitido</t>
+  </si>
+  <si>
+    <t>Representa cuanto va a valer el servicio en pesos colombianos. Su tipo de dato es entero, debe de ser mayor a cero, su valor por defecto es 0 y no esta permitido</t>
+  </si>
+  <si>
+    <t>Representa el primer nombre del barbero que trabaja en barbería. Su tipo de dato es texto, su valor por defecto es el vacio y no es permitido</t>
+  </si>
+  <si>
+    <t>Representa el segundo nombre del barbero que trabaja en barbería. Su tipo de dato es texto, su valor por defecto es el vacio y es permitido</t>
+  </si>
+  <si>
+    <t>Representa el primer apellido del barbero que trabaja en la barbería. Su tipo de dato es texto, su valor por defecto es el vacio y no es permitido</t>
+  </si>
+  <si>
+    <t>Representa el segundo apellido del barbero que trabaja en la barbería. Su tipo de dato es texto, su valor por defecto es el vacio y es permitido</t>
+  </si>
+  <si>
+    <t>Realmente se necesita saber el numero del barbero</t>
+  </si>
+  <si>
+    <t>Representa de que pais es el numero de celular del barbero. Su tipo de dato es alfanumérico, su valor por defecto es +0 y no es permitido</t>
+  </si>
+  <si>
+    <t>Representa el correo electronico del barbero, con el que se va a registrar o iniciar seción. Su tipo de dato es alfanumérico, su valor por defecto es el vacio y no es permitido</t>
+  </si>
+  <si>
+    <t>Representa la contraseña del barbebro, con el que se va a registrar o iniciar sesión. Su tipo de dato es alfanumérico, su valor por defecto es el vacio y no esta permitido</t>
   </si>
 </sst>
 </file>
@@ -788,7 +797,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="63">
+  <cellXfs count="62">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -835,12 +844,6 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -952,6 +955,9 @@
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -1356,14 +1362,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D2495362-94CF-4E08-8433-6F4780C6375E}">
   <dimension ref="A1:AD50"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="26.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="26.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
-        <v>50</v>
+        <v>39</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -1395,7 +1401,7 @@
       <c r="AC1" s="1"/>
       <c r="AD1" s="1"/>
     </row>
-    <row r="2" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A2" s="1"/>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
@@ -1427,7 +1433,7 @@
       <c r="AC2" s="1"/>
       <c r="AD2" s="1"/>
     </row>
-    <row r="3" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
       <c r="B3" s="1"/>
       <c r="C3" s="1"/>
@@ -1459,7 +1465,7 @@
       <c r="AC3" s="1"/>
       <c r="AD3" s="1"/>
     </row>
-    <row r="4" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:30" x14ac:dyDescent="0.25">
       <c r="B4" s="1"/>
       <c r="C4" s="1"/>
       <c r="D4" s="1"/>
@@ -1490,7 +1496,7 @@
       <c r="AC4" s="1"/>
       <c r="AD4" s="1"/>
     </row>
-    <row r="5" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A5" s="1"/>
       <c r="B5" s="1"/>
       <c r="C5" s="1"/>
@@ -1522,7 +1528,7 @@
       <c r="AC5" s="1"/>
       <c r="AD5" s="1"/>
     </row>
-    <row r="6" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A6" s="1"/>
       <c r="B6" s="1"/>
       <c r="D6" s="1"/>
@@ -1553,7 +1559,7 @@
       <c r="AC6" s="1"/>
       <c r="AD6" s="1"/>
     </row>
-    <row r="7" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A7" s="1"/>
       <c r="B7" s="1"/>
       <c r="C7" s="1"/>
@@ -1585,7 +1591,7 @@
       <c r="AC7" s="1"/>
       <c r="AD7" s="1"/>
     </row>
-    <row r="8" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A8" s="1"/>
       <c r="B8" s="1"/>
       <c r="C8" s="1"/>
@@ -1617,7 +1623,7 @@
       <c r="AC8" s="1"/>
       <c r="AD8" s="1"/>
     </row>
-    <row r="9" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A9" s="1"/>
       <c r="B9" s="1"/>
       <c r="C9" s="1"/>
@@ -1649,7 +1655,7 @@
       <c r="AC9" s="1"/>
       <c r="AD9" s="1"/>
     </row>
-    <row r="10" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A10" s="1"/>
       <c r="B10" s="1"/>
       <c r="C10" s="1"/>
@@ -1681,7 +1687,7 @@
       <c r="AC10" s="1"/>
       <c r="AD10" s="1"/>
     </row>
-    <row r="11" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A11" s="1"/>
       <c r="B11" s="1"/>
       <c r="C11" s="1"/>
@@ -1713,7 +1719,7 @@
       <c r="AC11" s="1"/>
       <c r="AD11" s="1"/>
     </row>
-    <row r="12" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A12" s="1"/>
       <c r="B12" s="1"/>
       <c r="C12" s="1"/>
@@ -1745,7 +1751,7 @@
       <c r="AC12" s="1"/>
       <c r="AD12" s="1"/>
     </row>
-    <row r="13" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A13" s="1"/>
       <c r="B13" s="1"/>
       <c r="C13" s="1"/>
@@ -1777,7 +1783,7 @@
       <c r="AC13" s="1"/>
       <c r="AD13" s="1"/>
     </row>
-    <row r="14" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A14" s="1"/>
       <c r="B14" s="1"/>
       <c r="C14" s="1"/>
@@ -1809,7 +1815,7 @@
       <c r="AC14" s="1"/>
       <c r="AD14" s="1"/>
     </row>
-    <row r="15" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A15" s="1"/>
       <c r="B15" s="1"/>
       <c r="C15" s="1"/>
@@ -1841,7 +1847,7 @@
       <c r="AC15" s="1"/>
       <c r="AD15" s="1"/>
     </row>
-    <row r="16" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A16" s="1"/>
       <c r="B16" s="1"/>
       <c r="C16" s="1"/>
@@ -1873,7 +1879,7 @@
       <c r="AC16" s="1"/>
       <c r="AD16" s="1"/>
     </row>
-    <row r="17" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A17" s="1"/>
       <c r="B17" s="1"/>
       <c r="C17" s="1"/>
@@ -1905,7 +1911,7 @@
       <c r="AC17" s="1"/>
       <c r="AD17" s="1"/>
     </row>
-    <row r="18" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A18" s="1"/>
       <c r="B18" s="1"/>
       <c r="C18" s="1"/>
@@ -1937,7 +1943,7 @@
       <c r="AC18" s="1"/>
       <c r="AD18" s="1"/>
     </row>
-    <row r="19" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A19" s="1"/>
       <c r="B19" s="1"/>
       <c r="C19" s="1"/>
@@ -1969,7 +1975,7 @@
       <c r="AC19" s="1"/>
       <c r="AD19" s="1"/>
     </row>
-    <row r="20" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A20" s="1"/>
       <c r="B20" s="1"/>
       <c r="C20" s="1"/>
@@ -2001,7 +2007,7 @@
       <c r="AC20" s="1"/>
       <c r="AD20" s="1"/>
     </row>
-    <row r="21" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A21" s="1"/>
       <c r="B21" s="1"/>
       <c r="C21" s="1"/>
@@ -2033,7 +2039,7 @@
       <c r="AC21" s="1"/>
       <c r="AD21" s="1"/>
     </row>
-    <row r="22" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A22" s="1"/>
       <c r="B22" s="1"/>
       <c r="C22" s="1"/>
@@ -2065,7 +2071,7 @@
       <c r="AC22" s="1"/>
       <c r="AD22" s="1"/>
     </row>
-    <row r="23" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A23" s="1"/>
       <c r="B23" s="1"/>
       <c r="C23" s="1"/>
@@ -2097,7 +2103,7 @@
       <c r="AC23" s="1"/>
       <c r="AD23" s="1"/>
     </row>
-    <row r="24" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A24" s="1"/>
       <c r="B24" s="1"/>
       <c r="C24" s="1"/>
@@ -2129,7 +2135,7 @@
       <c r="AC24" s="1"/>
       <c r="AD24" s="1"/>
     </row>
-    <row r="25" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A25" s="1"/>
       <c r="B25" s="1"/>
       <c r="C25" s="1"/>
@@ -2161,7 +2167,7 @@
       <c r="AC25" s="1"/>
       <c r="AD25" s="1"/>
     </row>
-    <row r="26" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A26" s="1"/>
       <c r="B26" s="1"/>
       <c r="C26" s="1"/>
@@ -2193,7 +2199,7 @@
       <c r="AC26" s="1"/>
       <c r="AD26" s="1"/>
     </row>
-    <row r="27" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A27" s="1"/>
       <c r="B27" s="1"/>
       <c r="C27" s="1"/>
@@ -2225,7 +2231,7 @@
       <c r="AC27" s="1"/>
       <c r="AD27" s="1"/>
     </row>
-    <row r="28" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A28" s="1"/>
       <c r="B28" s="1"/>
       <c r="C28" s="1"/>
@@ -2257,7 +2263,7 @@
       <c r="AC28" s="1"/>
       <c r="AD28" s="1"/>
     </row>
-    <row r="29" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A29" s="1"/>
       <c r="B29" s="1"/>
       <c r="C29" s="1"/>
@@ -2289,7 +2295,7 @@
       <c r="AC29" s="1"/>
       <c r="AD29" s="1"/>
     </row>
-    <row r="30" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A30" s="1"/>
       <c r="B30" s="1"/>
       <c r="C30" s="1"/>
@@ -2321,7 +2327,7 @@
       <c r="AC30" s="1"/>
       <c r="AD30" s="1"/>
     </row>
-    <row r="31" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A31" s="1"/>
       <c r="B31" s="1"/>
       <c r="C31" s="1"/>
@@ -2353,7 +2359,7 @@
       <c r="AC31" s="1"/>
       <c r="AD31" s="1"/>
     </row>
-    <row r="32" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A32" s="1"/>
       <c r="B32" s="1"/>
       <c r="C32" s="1"/>
@@ -2385,7 +2391,7 @@
       <c r="AC32" s="1"/>
       <c r="AD32" s="1"/>
     </row>
-    <row r="33" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A33" s="1"/>
       <c r="B33" s="1"/>
       <c r="C33" s="1"/>
@@ -2417,7 +2423,7 @@
       <c r="AC33" s="1"/>
       <c r="AD33" s="1"/>
     </row>
-    <row r="34" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A34" s="1"/>
       <c r="B34" s="1"/>
       <c r="C34" s="1"/>
@@ -2449,7 +2455,7 @@
       <c r="AC34" s="1"/>
       <c r="AD34" s="1"/>
     </row>
-    <row r="35" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A35" s="1"/>
       <c r="B35" s="1"/>
       <c r="C35" s="1"/>
@@ -2481,7 +2487,7 @@
       <c r="AC35" s="1"/>
       <c r="AD35" s="1"/>
     </row>
-    <row r="36" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A36" s="1"/>
       <c r="B36" s="1"/>
       <c r="C36" s="1"/>
@@ -2513,7 +2519,7 @@
       <c r="AC36" s="1"/>
       <c r="AD36" s="1"/>
     </row>
-    <row r="37" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A37" s="1"/>
       <c r="B37" s="1"/>
       <c r="C37" s="1"/>
@@ -2545,7 +2551,7 @@
       <c r="AC37" s="1"/>
       <c r="AD37" s="1"/>
     </row>
-    <row r="38" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A38" s="1"/>
       <c r="B38" s="1"/>
       <c r="C38" s="1"/>
@@ -2577,7 +2583,7 @@
       <c r="AC38" s="1"/>
       <c r="AD38" s="1"/>
     </row>
-    <row r="39" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A39" s="1"/>
       <c r="B39" s="1"/>
       <c r="C39" s="1"/>
@@ -2609,7 +2615,7 @@
       <c r="AC39" s="1"/>
       <c r="AD39" s="1"/>
     </row>
-    <row r="40" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A40" s="1"/>
       <c r="B40" s="1"/>
       <c r="C40" s="1"/>
@@ -2641,7 +2647,7 @@
       <c r="AC40" s="1"/>
       <c r="AD40" s="1"/>
     </row>
-    <row r="41" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A41" s="1"/>
       <c r="B41" s="1"/>
       <c r="C41" s="1"/>
@@ -2673,7 +2679,7 @@
       <c r="AC41" s="1"/>
       <c r="AD41" s="1"/>
     </row>
-    <row r="42" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A42" s="1"/>
       <c r="B42" s="1"/>
       <c r="C42" s="1"/>
@@ -2705,7 +2711,7 @@
       <c r="AC42" s="1"/>
       <c r="AD42" s="1"/>
     </row>
-    <row r="43" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A43" s="1"/>
       <c r="B43" s="1"/>
       <c r="C43" s="1"/>
@@ -2737,7 +2743,7 @@
       <c r="AC43" s="1"/>
       <c r="AD43" s="1"/>
     </row>
-    <row r="44" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A44" s="1"/>
       <c r="B44" s="1"/>
       <c r="C44" s="1"/>
@@ -2769,7 +2775,7 @@
       <c r="AC44" s="1"/>
       <c r="AD44" s="1"/>
     </row>
-    <row r="45" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A45" s="1"/>
       <c r="B45" s="1"/>
       <c r="C45" s="1"/>
@@ -2801,7 +2807,7 @@
       <c r="AC45" s="1"/>
       <c r="AD45" s="1"/>
     </row>
-    <row r="46" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A46" s="1"/>
       <c r="B46" s="1"/>
       <c r="C46" s="1"/>
@@ -2833,7 +2839,7 @@
       <c r="AC46" s="1"/>
       <c r="AD46" s="1"/>
     </row>
-    <row r="47" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A47" s="1"/>
       <c r="B47" s="1"/>
       <c r="C47" s="1"/>
@@ -2865,7 +2871,7 @@
       <c r="AC47" s="1"/>
       <c r="AD47" s="1"/>
     </row>
-    <row r="48" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A48" s="1"/>
       <c r="B48" s="1"/>
       <c r="C48" s="1"/>
@@ -2897,7 +2903,7 @@
       <c r="AC48" s="1"/>
       <c r="AD48" s="1"/>
     </row>
-    <row r="49" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A49" s="1"/>
       <c r="B49" s="1"/>
       <c r="C49" s="1"/>
@@ -2929,7 +2935,7 @@
       <c r="AC49" s="1"/>
       <c r="AD49" s="1"/>
     </row>
-    <row r="50" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A50" s="1"/>
       <c r="B50" s="1"/>
       <c r="C50" s="1"/>
@@ -2974,57 +2980,57 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A24A074A-5C83-448D-978C-7C1005CE378E}">
   <dimension ref="A1:D7"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="29.109375" customWidth="1"/>
+    <col min="1" max="1" width="29.140625" customWidth="1"/>
     <col min="2" max="2" width="30" customWidth="1"/>
-    <col min="3" max="3" width="41.88671875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="61.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="41.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="61.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" ht="36.75" customHeight="1" x14ac:dyDescent="0.3">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="18" t="s">
-        <v>25</v>
-      </c>
-      <c r="B2" s="37" t="s">
-        <v>80</v>
-      </c>
-      <c r="C2" s="34" t="s">
-        <v>81</v>
-      </c>
-      <c r="D2" s="47" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+        <v>20</v>
+      </c>
+      <c r="B2" s="35" t="s">
+        <v>64</v>
+      </c>
+      <c r="C2" s="32" t="s">
+        <v>65</v>
+      </c>
+      <c r="D2" s="45" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="14" t="s">
-        <v>36</v>
-      </c>
-      <c r="B3" s="35" t="s">
-        <v>51</v>
-      </c>
-      <c r="C3" s="35" t="s">
-        <v>52</v>
-      </c>
-      <c r="D3" s="39" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+        <v>31</v>
+      </c>
+      <c r="B3" s="33" t="s">
+        <v>40</v>
+      </c>
+      <c r="C3" s="33" t="s">
+        <v>41</v>
+      </c>
+      <c r="D3" s="37" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="12">
         <v>1</v>
       </c>
       <c r="B4" s="11" t="str">
         <f>_xlfn.CONCAT(Barbero_D!B4," ",Barbero_D!D4)</f>
-        <v>Juan Fernando García Lopez</v>
+        <v>Juan García</v>
       </c>
       <c r="C4" s="11" t="str">
         <f>Servicio_D!C4</f>
@@ -3032,16 +3038,16 @@
       </c>
       <c r="D4" s="12" t="str">
         <f>_xlfn.CONCAT(B4,"-",C4)</f>
-        <v>Juan Fernando García Lopez-Motilada</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+        <v>Juan García-Motilada</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="12">
         <v>2</v>
       </c>
       <c r="B5" s="11" t="str">
         <f>_xlfn.CONCAT(Barbero_D!B5," ",Barbero_D!D5)</f>
-        <v>Juan David Ortiz Sanchez</v>
+        <v>Juan Ortiz</v>
       </c>
       <c r="C5" s="11" t="str">
         <f>Servicio_D!C5</f>
@@ -3049,10 +3055,10 @@
       </c>
       <c r="D5" s="12" t="str">
         <f t="shared" ref="D5:D7" si="0">_xlfn.CONCAT(B5,"-",C5)</f>
-        <v>Juan David Ortiz Sanchez-Corte de barba</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+        <v>Juan Ortiz-Corte de barba</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="12">
         <v>3</v>
       </c>
@@ -3069,13 +3075,13 @@
         <v>Carlos Arbeladez-Perfilada de barba</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="12">
         <v>4</v>
       </c>
       <c r="B7" s="11" t="str">
         <f>_xlfn.CONCAT(Barbero_D!B7," ",Barbero_D!D7)</f>
-        <v>Andres Ramirez Patiño</v>
+        <v>Andres Ramirez</v>
       </c>
       <c r="C7" s="11" t="str">
         <f>Servicio_D!C7</f>
@@ -3083,7 +3089,7 @@
       </c>
       <c r="D7" s="12" t="str">
         <f t="shared" si="0"/>
-        <v>Andres Ramirez Patiño-Arreglo completo de barba con toalla caliente</v>
+        <v>Andres Ramirez-Arreglo completo de barba con toalla caliente</v>
       </c>
     </row>
   </sheetData>
@@ -3109,70 +3115,70 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2921A3C4-B96A-49A7-8353-9FD37D2F2B74}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
-    <col min="2" max="2" width="42.33203125" customWidth="1"/>
-    <col min="3" max="3" width="37.44140625" customWidth="1"/>
+    <col min="2" max="2" width="42.28515625" customWidth="1"/>
+    <col min="3" max="3" width="37.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" ht="30" x14ac:dyDescent="0.3">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A2" s="18" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="B2" s="18" t="s">
-        <v>162</v>
+        <v>131</v>
       </c>
       <c r="C2" s="19" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="14" t="s">
-        <v>36</v>
-      </c>
-      <c r="B3" s="35" t="s">
-        <v>51</v>
-      </c>
-      <c r="C3" s="32" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+        <v>31</v>
+      </c>
+      <c r="B3" s="33" t="s">
+        <v>40</v>
+      </c>
+      <c r="C3" s="30" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="12">
         <v>1</v>
       </c>
       <c r="B4" s="11" t="str">
         <f>_xlfn.CONCAT(Barbero_D!B4," ",Barbero_D!D4)</f>
-        <v>Juan Fernando García Lopez</v>
+        <v>Juan García</v>
       </c>
       <c r="C4" s="12" t="str">
         <f>B4</f>
-        <v>Juan Fernando García Lopez</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+        <v>Juan García</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="12">
         <v>2</v>
       </c>
       <c r="B5" s="11" t="str">
         <f>_xlfn.CONCAT(Barbero_D!B5," ",Barbero_D!D5)</f>
-        <v>Juan David Ortiz Sanchez</v>
+        <v>Juan Ortiz</v>
       </c>
       <c r="C5" s="12" t="str">
         <f t="shared" ref="C5:C7" si="0">B5</f>
-        <v>Juan David Ortiz Sanchez</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+        <v>Juan Ortiz</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="12">
         <v>3</v>
       </c>
@@ -3185,17 +3191,17 @@
         <v>Carlos Arbeladez</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="12">
         <v>4</v>
       </c>
       <c r="B7" s="11" t="str">
         <f>_xlfn.CONCAT(Barbero_D!B7," ",Barbero_D!D7)</f>
-        <v>Andres Ramirez Patiño</v>
+        <v>Andres Ramirez</v>
       </c>
       <c r="C7" s="12" t="str">
         <f t="shared" si="0"/>
-        <v>Andres Ramirez Patiño</v>
+        <v>Andres Ramirez</v>
       </c>
     </row>
   </sheetData>
@@ -3216,123 +3222,123 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5CFE76D0-FBB4-4C81-85CC-F644057A8847}">
   <dimension ref="A1:F7"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="27" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="37.109375" customWidth="1"/>
+    <col min="2" max="2" width="37.140625" customWidth="1"/>
     <col min="3" max="3" width="28" customWidth="1"/>
-    <col min="4" max="4" width="18.6640625" customWidth="1"/>
-    <col min="5" max="5" width="31.6640625" customWidth="1"/>
-    <col min="6" max="6" width="37.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="18.7109375" customWidth="1"/>
+    <col min="5" max="5" width="31.7109375" customWidth="1"/>
+    <col min="6" max="6" width="37.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" ht="40.5" customHeight="1" x14ac:dyDescent="0.3">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" ht="40.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="19" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="B2" s="19" t="s">
-        <v>110</v>
+        <v>90</v>
       </c>
       <c r="C2" s="19" t="s">
-        <v>111</v>
+        <v>91</v>
       </c>
       <c r="D2" s="19" t="s">
-        <v>112</v>
+        <v>92</v>
       </c>
       <c r="E2" s="19" t="s">
-        <v>113</v>
+        <v>93</v>
       </c>
       <c r="F2" s="19" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="14" t="s">
-        <v>36</v>
-      </c>
-      <c r="B3" s="35" t="s">
+        <v>31</v>
+      </c>
+      <c r="B3" s="33" t="s">
+        <v>63</v>
+      </c>
+      <c r="C3" s="40" t="s">
         <v>79</v>
       </c>
-      <c r="C3" s="42" t="s">
-        <v>99</v>
-      </c>
       <c r="D3" s="13" t="s">
-        <v>82</v>
+        <v>66</v>
       </c>
       <c r="E3" s="13" t="s">
-        <v>109</v>
-      </c>
-      <c r="F3" s="32" t="s">
         <v>89</v>
       </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="F3" s="30" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="12">
         <v>1</v>
       </c>
-      <c r="B4" s="55" t="str">
+      <c r="B4" s="53" t="str">
         <f>Agenda_D!C4</f>
-        <v>Juan Fernando García Lopez</v>
-      </c>
-      <c r="C4" s="41" t="s">
-        <v>102</v>
-      </c>
-      <c r="D4" s="41">
+        <v>Juan García</v>
+      </c>
+      <c r="C4" s="39" t="s">
+        <v>82</v>
+      </c>
+      <c r="D4" s="39">
         <v>0.41666666666666669</v>
       </c>
-      <c r="E4" s="41">
+      <c r="E4" s="39">
         <v>0.66666666666666663</v>
       </c>
       <c r="F4" s="12" t="str">
         <f>_xlfn.CONCAT(B4,"-",C4,"-",TEXT(D4,"hh;mm"),"-",TEXT(E4,"hh;mm"))</f>
-        <v>Juan Fernando García Lopez-Lunes-10-16</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+        <v>Juan García-Lunes-10-16</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="12">
         <v>2</v>
       </c>
-      <c r="B5" s="55" t="str">
+      <c r="B5" s="53" t="str">
         <f>Agenda_D!C5</f>
-        <v>Juan David Ortiz Sanchez</v>
+        <v>Juan Ortiz</v>
       </c>
       <c r="C5" s="12" t="s">
-        <v>103</v>
-      </c>
-      <c r="D5" s="41">
+        <v>83</v>
+      </c>
+      <c r="D5" s="39">
         <v>0.375</v>
       </c>
-      <c r="E5" s="41">
+      <c r="E5" s="39">
         <v>0.625</v>
       </c>
       <c r="F5" s="12" t="str">
         <f t="shared" ref="F5:F7" si="0">_xlfn.CONCAT(B5,"-",C5,"-",TEXT(D5,"hh;mm"),"-",TEXT(E5,"hh;mm"))</f>
-        <v>Juan David Ortiz Sanchez-Martes-09-15</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+        <v>Juan Ortiz-Martes-09-15</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="12">
         <v>3</v>
       </c>
-      <c r="B6" s="55" t="str">
+      <c r="B6" s="53" t="str">
         <f>Agenda_D!C6</f>
         <v>Carlos Arbeladez</v>
       </c>
       <c r="C6" s="12" t="s">
-        <v>105</v>
-      </c>
-      <c r="D6" s="41">
+        <v>85</v>
+      </c>
+      <c r="D6" s="39">
         <v>0.54166666666666663</v>
       </c>
-      <c r="E6" s="41">
+      <c r="E6" s="39">
         <v>0.79166666666666663</v>
       </c>
       <c r="F6" s="12" t="str">
@@ -3340,26 +3346,26 @@
         <v>Carlos Arbeladez-Jueves-13-19</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="12">
         <v>4</v>
       </c>
-      <c r="B7" s="55" t="str">
+      <c r="B7" s="53" t="str">
         <f>Agenda_D!C7</f>
-        <v>Andres Ramirez Patiño</v>
+        <v>Andres Ramirez</v>
       </c>
       <c r="C7" s="12" t="s">
-        <v>107</v>
-      </c>
-      <c r="D7" s="41">
+        <v>87</v>
+      </c>
+      <c r="D7" s="39">
         <v>0.33333333333333331</v>
       </c>
-      <c r="E7" s="41">
+      <c r="E7" s="39">
         <v>0.58333333333333337</v>
       </c>
       <c r="F7" s="12" t="str">
         <f t="shared" si="0"/>
-        <v>Andres Ramirez Patiño-Sábado-08-14</v>
+        <v>Andres Ramirez-Sábado-08-14</v>
       </c>
     </row>
   </sheetData>
@@ -3380,73 +3386,73 @@
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1429879F-6697-4F1F-AF5D-52C4860B7B3E}">
   <dimension ref="A1:H15"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="28" customWidth="1"/>
-    <col min="2" max="2" width="26.5546875" customWidth="1"/>
-    <col min="3" max="3" width="30.44140625" customWidth="1"/>
-    <col min="4" max="4" width="27.5546875" customWidth="1"/>
-    <col min="5" max="5" width="36.5546875" customWidth="1"/>
-    <col min="6" max="6" width="60.21875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="39.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="26.5703125" customWidth="1"/>
+    <col min="3" max="3" width="30.42578125" customWidth="1"/>
+    <col min="4" max="4" width="27.5703125" customWidth="1"/>
+    <col min="5" max="5" width="36.5703125" customWidth="1"/>
+    <col min="6" max="6" width="60.28515625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="39.28515625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="22" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" ht="36.75" customHeight="1" x14ac:dyDescent="0.3">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="18" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="B2" s="18" t="s">
-        <v>83</v>
-      </c>
-      <c r="C2" s="34" t="s">
-        <v>187</v>
-      </c>
-      <c r="D2" s="34" t="s">
-        <v>179</v>
-      </c>
-      <c r="E2" s="34" t="s">
-        <v>184</v>
-      </c>
-      <c r="F2" s="34" t="s">
-        <v>188</v>
-      </c>
-      <c r="G2" s="34" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+        <v>67</v>
+      </c>
+      <c r="C2" s="32" t="s">
+        <v>151</v>
+      </c>
+      <c r="D2" s="32" t="s">
+        <v>143</v>
+      </c>
+      <c r="E2" s="32" t="s">
+        <v>148</v>
+      </c>
+      <c r="F2" s="32" t="s">
+        <v>152</v>
+      </c>
+      <c r="G2" s="32" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" s="14" t="s">
-        <v>36</v>
-      </c>
-      <c r="B3" s="35" t="s">
-        <v>55</v>
-      </c>
-      <c r="C3" s="35" t="s">
-        <v>79</v>
+        <v>31</v>
+      </c>
+      <c r="B3" s="33" t="s">
+        <v>44</v>
+      </c>
+      <c r="C3" s="33" t="s">
+        <v>63</v>
       </c>
       <c r="D3" s="13" t="s">
-        <v>178</v>
-      </c>
-      <c r="E3" s="49" t="s">
-        <v>109</v>
+        <v>142</v>
+      </c>
+      <c r="E3" s="47" t="s">
+        <v>89</v>
       </c>
       <c r="F3" s="13" t="s">
-        <v>31</v>
-      </c>
-      <c r="G3" s="32" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+        <v>26</v>
+      </c>
+      <c r="G3" s="30" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" s="12">
         <v>1</v>
       </c>
@@ -3456,23 +3462,23 @@
       </c>
       <c r="C4" s="11" t="str">
         <f>Agenda_D!C4</f>
-        <v>Juan Fernando García Lopez</v>
-      </c>
-      <c r="D4" s="57">
+        <v>Juan García</v>
+      </c>
+      <c r="D4" s="55">
         <v>46295.416666666664</v>
       </c>
-      <c r="E4" s="41">
+      <c r="E4" s="39">
         <v>0.44791666666666669</v>
       </c>
       <c r="F4" s="12" t="s">
-        <v>84</v>
+        <v>68</v>
       </c>
       <c r="G4" s="12" t="str">
         <f>_xlfn.CONCAT(C4,"-",TEXT(D4,"dd/mm/yyyy/hh:mm"))</f>
-        <v>Juan Fernando García Lopez-30/09/2026/10:00</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+        <v>Juan García-30/09/2026/10:00</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" s="12">
         <v>2</v>
       </c>
@@ -3482,23 +3488,23 @@
       </c>
       <c r="C5" s="11" t="str">
         <f>Agenda_D!C5</f>
-        <v>Juan David Ortiz Sanchez</v>
-      </c>
-      <c r="D5" s="57">
+        <v>Juan Ortiz</v>
+      </c>
+      <c r="D5" s="55">
         <v>45983.458333333336</v>
       </c>
-      <c r="E5" s="41">
+      <c r="E5" s="39">
         <v>0.48958333333333331</v>
       </c>
       <c r="F5" s="12" t="s">
-        <v>115</v>
+        <v>95</v>
       </c>
       <c r="G5" s="12" t="str">
         <f t="shared" ref="G5:G8" si="0">_xlfn.CONCAT(C5,"-",TEXT(D5,"dd/mm/yyyy/hh:mm"))</f>
-        <v>Juan David Ortiz Sanchez-22/11/2025/11:00</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+        <v>Juan Ortiz-22/11/2025/11:00</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" s="12">
         <v>3</v>
       </c>
@@ -3510,21 +3516,21 @@
         <f>Agenda_D!C6</f>
         <v>Carlos Arbeladez</v>
       </c>
-      <c r="D6" s="57">
+      <c r="D6" s="55">
         <v>45514.583333333336</v>
       </c>
-      <c r="E6" s="41">
+      <c r="E6" s="39">
         <v>0.59375</v>
       </c>
       <c r="F6" s="12" t="s">
-        <v>181</v>
+        <v>145</v>
       </c>
       <c r="G6" s="12" t="str">
         <f t="shared" si="0"/>
         <v>Carlos Arbeladez-10/08/2024/14:00</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="12">
         <v>4</v>
       </c>
@@ -3534,23 +3540,23 @@
       </c>
       <c r="C7" s="11" t="str">
         <f>Agenda_D!C7</f>
-        <v>Andres Ramirez Patiño</v>
-      </c>
-      <c r="D7" s="57">
+        <v>Andres Ramirez</v>
+      </c>
+      <c r="D7" s="55">
         <v>46289.541666666664</v>
       </c>
-      <c r="E7" s="41">
+      <c r="E7" s="39">
         <v>0.5625</v>
       </c>
       <c r="F7" s="12" t="s">
-        <v>116</v>
+        <v>96</v>
       </c>
       <c r="G7" s="12" t="str">
         <f t="shared" si="0"/>
-        <v>Andres Ramirez Patiño-24/09/2026/13:00</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+        <v>Andres Ramirez-24/09/2026/13:00</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" s="12">
         <v>5</v>
       </c>
@@ -3562,35 +3568,35 @@
         <f>Agenda_D!C6</f>
         <v>Carlos Arbeladez</v>
       </c>
-      <c r="D8" s="57">
+      <c r="D8" s="55">
         <v>46240.75</v>
       </c>
-      <c r="E8" s="41">
+      <c r="E8" s="39">
         <v>0.75694444444444442</v>
       </c>
       <c r="F8" s="12" t="s">
-        <v>117</v>
+        <v>97</v>
       </c>
       <c r="G8" s="12" t="str">
         <f t="shared" si="0"/>
         <v>Carlos Arbeladez-06/08/2026/18:00</v>
       </c>
-      <c r="H8" s="54"/>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="H10" s="56"/>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="D12" s="58"/>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="D13" s="58"/>
-    </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="D14" s="58"/>
-    </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="D15" s="58"/>
+      <c r="H8" s="52"/>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="H10" s="54"/>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="D12" s="56"/>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="D13" s="56"/>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="D14" s="56"/>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="D15" s="56"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -3618,71 +3624,71 @@
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{766573FB-AAA2-4254-B83C-7C7505540365}">
   <dimension ref="A1:G7"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="26.6640625" customWidth="1"/>
-    <col min="2" max="2" width="38.5546875" customWidth="1"/>
-    <col min="3" max="3" width="39.33203125" bestFit="1" customWidth="1"/>
-    <col min="4" max="5" width="39.6640625" customWidth="1"/>
-    <col min="6" max="6" width="34.21875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="39.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="26.7109375" customWidth="1"/>
+    <col min="2" max="2" width="38.5703125" customWidth="1"/>
+    <col min="3" max="3" width="39.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="39.7109375" customWidth="1"/>
+    <col min="6" max="6" width="34.28515625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="39.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" ht="31.5" customHeight="1" x14ac:dyDescent="0.3">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="18" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="B2" s="18" t="s">
-        <v>119</v>
-      </c>
-      <c r="C2" s="34" t="s">
-        <v>120</v>
-      </c>
-      <c r="D2" s="34" t="s">
-        <v>182</v>
-      </c>
-      <c r="E2" s="34" t="s">
-        <v>190</v>
-      </c>
-      <c r="F2" s="34" t="s">
-        <v>121</v>
-      </c>
-      <c r="G2" s="34" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+        <v>99</v>
+      </c>
+      <c r="C2" s="32" t="s">
+        <v>100</v>
+      </c>
+      <c r="D2" s="32" t="s">
+        <v>146</v>
+      </c>
+      <c r="E2" s="32" t="s">
+        <v>154</v>
+      </c>
+      <c r="F2" s="32" t="s">
+        <v>101</v>
+      </c>
+      <c r="G2" s="32" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="14" t="s">
-        <v>36</v>
-      </c>
-      <c r="B3" s="35" t="s">
-        <v>55</v>
-      </c>
-      <c r="C3" s="35" t="s">
-        <v>118</v>
-      </c>
-      <c r="D3" s="38" t="s">
-        <v>32</v>
-      </c>
-      <c r="E3" s="62" t="s">
-        <v>189</v>
-      </c>
-      <c r="F3" s="49" t="s">
-        <v>33</v>
-      </c>
-      <c r="G3" s="32" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+        <v>31</v>
+      </c>
+      <c r="B3" s="33" t="s">
+        <v>44</v>
+      </c>
+      <c r="C3" s="33" t="s">
+        <v>98</v>
+      </c>
+      <c r="D3" s="36" t="s">
+        <v>27</v>
+      </c>
+      <c r="E3" s="60" t="s">
+        <v>153</v>
+      </c>
+      <c r="F3" s="47" t="s">
+        <v>28</v>
+      </c>
+      <c r="G3" s="30" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="12">
         <v>1</v>
       </c>
@@ -3699,17 +3705,17 @@
         <v>10000</v>
       </c>
       <c r="E4" s="12" t="s">
-        <v>181</v>
+        <v>145</v>
       </c>
       <c r="F4" s="12" t="s">
-        <v>61</v>
+        <v>50</v>
       </c>
       <c r="G4" s="12" t="str">
         <f>C4</f>
         <v>Carlos Arbeladez-10/08/2024/14:00</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="12">
         <v>2</v>
       </c>
@@ -3719,24 +3725,24 @@
       </c>
       <c r="C5" s="11" t="str">
         <f>Cita_D!G7</f>
-        <v>Andres Ramirez Patiño-24/09/2026/13:00</v>
+        <v>Andres Ramirez-24/09/2026/13:00</v>
       </c>
       <c r="D5" s="12">
         <f>CitaServicio_D!D7</f>
         <v>35000</v>
       </c>
       <c r="E5" s="12" t="s">
-        <v>116</v>
+        <v>96</v>
       </c>
       <c r="F5" s="12" t="s">
-        <v>62</v>
+        <v>51</v>
       </c>
       <c r="G5" s="12" t="str">
         <f>C5</f>
-        <v>Andres Ramirez Patiño-24/09/2026/13:00</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+        <v>Andres Ramirez-24/09/2026/13:00</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="10"/>
       <c r="B6" s="10"/>
       <c r="C6" s="10"/>
@@ -3745,7 +3751,7 @@
       <c r="F6" s="10"/>
       <c r="G6" s="10"/>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="10"/>
       <c r="B7" s="10"/>
       <c r="C7" s="10"/>
@@ -3772,71 +3778,71 @@
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F470C5A4-8D15-43DA-95FC-91C9614E5EEA}">
   <dimension ref="A1:F8"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="26.44140625" customWidth="1"/>
-    <col min="2" max="2" width="39.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="21.88671875" customWidth="1"/>
-    <col min="4" max="4" width="41.88671875" customWidth="1"/>
-    <col min="5" max="5" width="32.109375" customWidth="1"/>
-    <col min="6" max="6" width="54.88671875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="26.42578125" customWidth="1"/>
+    <col min="2" max="2" width="39.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="21.85546875" customWidth="1"/>
+    <col min="4" max="4" width="41.85546875" customWidth="1"/>
+    <col min="5" max="5" width="32.140625" customWidth="1"/>
+    <col min="6" max="6" width="55.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" ht="33" customHeight="1" x14ac:dyDescent="0.3">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" ht="33" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="18" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="B2" s="18" t="s">
-        <v>123</v>
-      </c>
-      <c r="C2" s="34" t="s">
-        <v>124</v>
-      </c>
-      <c r="D2" s="34" t="s">
-        <v>125</v>
-      </c>
-      <c r="E2" s="34" t="s">
-        <v>126</v>
-      </c>
-      <c r="F2" s="34" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A3" s="45" t="s">
-        <v>36</v>
-      </c>
-      <c r="B3" s="35" t="s">
-        <v>118</v>
-      </c>
-      <c r="C3" s="35" t="s">
-        <v>52</v>
+        <v>103</v>
+      </c>
+      <c r="C2" s="32" t="s">
+        <v>104</v>
+      </c>
+      <c r="D2" s="32" t="s">
+        <v>105</v>
+      </c>
+      <c r="E2" s="32" t="s">
+        <v>106</v>
+      </c>
+      <c r="F2" s="32" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" s="43" t="s">
+        <v>31</v>
+      </c>
+      <c r="B3" s="33" t="s">
+        <v>98</v>
+      </c>
+      <c r="C3" s="33" t="s">
+        <v>41</v>
       </c>
       <c r="D3" s="13" t="s">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="E3" s="13" t="s">
-        <v>35</v>
-      </c>
-      <c r="F3" s="32" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+        <v>30</v>
+      </c>
+      <c r="F3" s="30" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="12">
         <v>1</v>
       </c>
       <c r="B4" s="11" t="str">
         <f>Cita_D!G4</f>
-        <v>Juan Fernando García Lopez-30/09/2026/10:00</v>
+        <v>Juan García-30/09/2026/10:00</v>
       </c>
       <c r="C4" s="11" t="str">
         <f>Servicio_D!F4</f>
@@ -3850,16 +3856,16 @@
       </c>
       <c r="F4" s="12" t="str">
         <f>_xlfn.CONCAT(B4,"-",C4)</f>
-        <v>Juan Fernando García Lopez-30/09/2026/10:00-Motilada</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+        <v>Juan García-30/09/2026/10:00-Motilada</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="12">
         <v>2</v>
       </c>
       <c r="B5" s="11" t="str">
         <f>Cita_D!G5</f>
-        <v>Juan David Ortiz Sanchez-22/11/2025/11:00</v>
+        <v>Juan Ortiz-22/11/2025/11:00</v>
       </c>
       <c r="C5" s="11" t="str">
         <f>Servicio_D!F4</f>
@@ -3873,10 +3879,10 @@
       </c>
       <c r="F5" s="12" t="str">
         <f t="shared" ref="F5:F8" si="0">_xlfn.CONCAT(B5,"-",C5)</f>
-        <v>Juan David Ortiz Sanchez-22/11/2025/11:00-Motilada</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+        <v>Juan Ortiz-22/11/2025/11:00-Motilada</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="12">
         <v>3</v>
       </c>
@@ -3899,15 +3905,15 @@
         <v>Carlos Arbeladez-10/08/2024/14:00-Perfilada de barba</v>
       </c>
     </row>
-    <row r="7" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:6" ht="45" x14ac:dyDescent="0.25">
       <c r="A7" s="12">
         <v>4</v>
       </c>
       <c r="B7" s="11" t="str">
         <f>Cita_D!G7</f>
-        <v>Andres Ramirez Patiño-24/09/2026/13:00</v>
-      </c>
-      <c r="C7" s="59" t="str">
+        <v>Andres Ramirez-24/09/2026/13:00</v>
+      </c>
+      <c r="C7" s="57" t="str">
         <f>Servicio_D!F7</f>
         <v>Arreglo completo de barba con toalla caliente</v>
       </c>
@@ -3917,12 +3923,12 @@
       <c r="E7" s="12">
         <v>30</v>
       </c>
-      <c r="F7" s="28" t="str">
+      <c r="F7" s="26" t="str">
         <f t="shared" si="0"/>
-        <v>Andres Ramirez Patiño-24/09/2026/13:00-Arreglo completo de barba con toalla caliente</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+        <v>Andres Ramirez-24/09/2026/13:00-Arreglo completo de barba con toalla caliente</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="12">
         <v>5</v>
       </c>
@@ -3931,7 +3937,7 @@
         <v>Carlos Arbeladez-06/08/2026/18:00</v>
       </c>
       <c r="C8" s="11" t="s">
-        <v>57</v>
+        <v>46</v>
       </c>
       <c r="D8" s="12">
         <v>12000</v>
@@ -3939,7 +3945,7 @@
       <c r="E8" s="12">
         <v>10</v>
       </c>
-      <c r="F8" s="28" t="str">
+      <c r="F8" s="26" t="str">
         <f t="shared" si="0"/>
         <v>Carlos Arbeladez-06/08/2026/18:00-Corte de barba</v>
       </c>
@@ -3969,20 +3975,20 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7A5AA025-A9A3-4E3E-A766-44885AA770B6}">
   <dimension ref="A1:D15"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="27" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="54.5546875" customWidth="1"/>
-    <col min="3" max="3" width="14.44140625" customWidth="1"/>
-    <col min="4" max="4" width="7.6640625" customWidth="1"/>
+    <col min="2" max="2" width="63.7109375" customWidth="1"/>
+    <col min="3" max="3" width="14.42578125" customWidth="1"/>
+    <col min="4" max="4" width="7.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
         <v>0</v>
       </c>
@@ -3996,7 +4002,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:4" ht="45" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
         <v>4</v>
       </c>
@@ -4007,175 +4013,175 @@
         <v>1</v>
       </c>
       <c r="D3" s="9" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="75" x14ac:dyDescent="0.25">
       <c r="A4" s="7" t="s">
         <v>11</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>95</v>
+        <v>161</v>
       </c>
       <c r="C4" s="7">
         <v>1</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="60" x14ac:dyDescent="0.25">
       <c r="A5" s="7" t="s">
         <v>5</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>21</v>
+        <v>162</v>
       </c>
       <c r="C5" s="7">
         <v>2</v>
       </c>
       <c r="D5" s="9" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="45" x14ac:dyDescent="0.25">
       <c r="A6" s="7" t="s">
-        <v>93</v>
+        <v>76</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>97</v>
+        <v>163</v>
       </c>
       <c r="C6" s="7">
         <v>2</v>
       </c>
       <c r="D6" s="9" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" ht="60" x14ac:dyDescent="0.25">
       <c r="A7" s="7" t="s">
         <v>6</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>16</v>
+        <v>164</v>
       </c>
       <c r="C7" s="7">
         <v>2</v>
       </c>
       <c r="D7" s="9" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" ht="45" x14ac:dyDescent="0.25">
       <c r="A8" s="7" t="s">
         <v>7</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C8" s="7">
         <v>2</v>
       </c>
       <c r="D8" s="9" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" ht="75" x14ac:dyDescent="0.25">
       <c r="A9" s="7" t="s">
         <v>13</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>19</v>
+        <v>165</v>
       </c>
       <c r="C9" s="7">
         <v>2</v>
       </c>
       <c r="D9" s="9" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A10" s="7" t="s">
         <v>8</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C10" s="7">
         <v>3</v>
       </c>
       <c r="D10" s="9" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" ht="45" x14ac:dyDescent="0.25">
       <c r="A11" s="7" t="s">
         <v>9</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>20</v>
+        <v>166</v>
       </c>
       <c r="C11" s="7">
         <v>3</v>
       </c>
       <c r="D11" s="9" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A12" s="7" t="s">
-        <v>94</v>
+        <v>77</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>96</v>
+        <v>167</v>
       </c>
       <c r="C12" s="7">
         <v>4</v>
       </c>
       <c r="D12" s="9" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" ht="129.6" x14ac:dyDescent="0.3">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" ht="90" x14ac:dyDescent="0.25">
       <c r="A13" s="7" t="s">
         <v>10</v>
       </c>
       <c r="B13" s="8" t="s">
-        <v>22</v>
+        <v>168</v>
       </c>
       <c r="C13" s="7">
         <v>4</v>
       </c>
       <c r="D13" s="9" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" ht="45" x14ac:dyDescent="0.25">
       <c r="A14" s="7" t="s">
         <v>12</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="C14" s="7">
         <v>5</v>
       </c>
       <c r="D14" s="9" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" ht="60" x14ac:dyDescent="0.25">
       <c r="A15" s="7" t="s">
         <v>14</v>
       </c>
       <c r="B15" s="8" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="C15" s="7">
         <v>5</v>
       </c>
       <c r="D15" s="9" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
     </row>
   </sheetData>
@@ -4202,44 +4208,44 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AAA22F8C-1648-4644-8301-765EB2B8C50B}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="33.88671875" customWidth="1"/>
-    <col min="2" max="2" width="29.109375" customWidth="1"/>
+    <col min="1" max="1" width="33.85546875" customWidth="1"/>
+    <col min="2" max="2" width="34.7109375" customWidth="1"/>
     <col min="3" max="3" width="21" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="19" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="B2" s="19" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="14" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="B3" s="13" t="s">
-        <v>26</v>
-      </c>
-      <c r="C3" s="40"/>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+        <v>21</v>
+      </c>
+      <c r="C3" s="38"/>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="12">
         <v>1</v>
       </c>
-      <c r="B4" s="41" t="s">
-        <v>86</v>
+      <c r="B4" s="39" t="s">
+        <v>69</v>
       </c>
       <c r="C4" s="4"/>
     </row>
@@ -4255,20 +4261,20 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{28259140-2713-4A98-8730-76D57DC1D653}">
   <dimension ref="A1:H11"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="26.88671875" style="10" customWidth="1"/>
-    <col min="2" max="6" width="26.33203125" style="10" customWidth="1"/>
-    <col min="7" max="7" width="23.109375" style="10" customWidth="1"/>
-    <col min="8" max="8" width="38.5546875" style="10" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="26.85546875" style="10" customWidth="1"/>
+    <col min="2" max="6" width="26.28515625" style="10" customWidth="1"/>
+    <col min="7" max="7" width="23.140625" style="10" customWidth="1"/>
+    <col min="8" max="8" width="38.5703125" style="10" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="11" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="B1" s="11" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="C1" s="11"/>
       <c r="D1" s="11"/>
@@ -4277,72 +4283,72 @@
       <c r="G1" s="12"/>
       <c r="H1" s="12"/>
     </row>
-    <row r="2" spans="1:8" ht="39.6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" ht="55.5" x14ac:dyDescent="0.25">
       <c r="A2" s="18" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="B2" s="18" t="s">
-        <v>154</v>
+        <v>170</v>
       </c>
       <c r="C2" s="18" t="s">
-        <v>155</v>
+        <v>171</v>
       </c>
       <c r="D2" s="18" t="s">
-        <v>156</v>
+        <v>172</v>
       </c>
       <c r="E2" s="18" t="s">
-        <v>157</v>
+        <v>173</v>
       </c>
       <c r="F2" s="18" t="s">
+        <v>175</v>
+      </c>
+      <c r="G2" s="19" t="s">
+        <v>176</v>
+      </c>
+      <c r="H2" s="20" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A3" s="14" t="s">
+        <v>31</v>
+      </c>
+      <c r="B3" s="13" t="s">
+        <v>109</v>
+      </c>
+      <c r="C3" s="13" t="s">
+        <v>111</v>
+      </c>
+      <c r="D3" s="13" t="s">
+        <v>110</v>
+      </c>
+      <c r="E3" s="13" t="s">
+        <v>112</v>
+      </c>
+      <c r="F3" s="13" t="s">
         <v>174</v>
       </c>
-      <c r="G2" s="19" t="s">
-        <v>128</v>
-      </c>
-      <c r="H2" s="20" t="s">
-        <v>183</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A3" s="14" t="s">
-        <v>36</v>
-      </c>
-      <c r="B3" s="13" t="s">
-        <v>130</v>
-      </c>
-      <c r="C3" s="13" t="s">
-        <v>132</v>
-      </c>
-      <c r="D3" s="13" t="s">
-        <v>131</v>
-      </c>
-      <c r="E3" s="13" t="s">
-        <v>133</v>
-      </c>
-      <c r="F3" s="13" t="s">
-        <v>171</v>
-      </c>
       <c r="G3" s="13" t="s">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="H3" s="15" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" s="12">
         <v>1</v>
       </c>
       <c r="B4" s="12" t="s">
-        <v>151</v>
+        <v>126</v>
       </c>
       <c r="C4" s="12"/>
       <c r="D4" s="12" t="s">
-        <v>144</v>
+        <v>119</v>
       </c>
       <c r="E4" s="12"/>
-      <c r="F4" s="53" t="s">
-        <v>172</v>
+      <c r="F4" s="51" t="s">
+        <v>138</v>
       </c>
       <c r="G4" s="12">
         <v>3234528921</v>
@@ -4352,24 +4358,24 @@
         <v>Juan--Gómez--+57-3234528921</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" s="12">
         <v>2</v>
       </c>
       <c r="B5" s="12" t="s">
-        <v>149</v>
+        <v>124</v>
       </c>
       <c r="C5" s="12" t="s">
-        <v>150</v>
+        <v>125</v>
       </c>
       <c r="D5" s="12" t="s">
-        <v>146</v>
+        <v>121</v>
       </c>
       <c r="E5" s="12" t="s">
-        <v>145</v>
-      </c>
-      <c r="F5" s="53" t="s">
-        <v>172</v>
+        <v>120</v>
+      </c>
+      <c r="F5" s="51" t="s">
+        <v>138</v>
       </c>
       <c r="G5" s="12">
         <v>3161657782</v>
@@ -4379,22 +4385,22 @@
         <v>Jose-Miguel-Ramirez-Perez-+57-3161657782</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" s="12">
         <v>3</v>
       </c>
       <c r="B6" s="12" t="s">
-        <v>152</v>
+        <v>127</v>
       </c>
       <c r="C6" s="12"/>
       <c r="D6" s="12" t="s">
-        <v>148</v>
+        <v>123</v>
       </c>
       <c r="E6" s="12" t="s">
-        <v>146</v>
-      </c>
-      <c r="F6" s="53" t="s">
-        <v>172</v>
+        <v>121</v>
+      </c>
+      <c r="F6" s="51" t="s">
+        <v>138</v>
       </c>
       <c r="G6" s="12">
         <v>3119884321</v>
@@ -4404,20 +4410,20 @@
         <v>Simon--Ochoa-Ramirez-+57-3119884321</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="12">
         <v>4</v>
       </c>
       <c r="B7" s="12" t="s">
-        <v>153</v>
+        <v>128</v>
       </c>
       <c r="C7" s="12"/>
       <c r="D7" s="12" t="s">
-        <v>147</v>
+        <v>122</v>
       </c>
       <c r="E7" s="12"/>
-      <c r="F7" s="53" t="s">
-        <v>173</v>
+      <c r="F7" s="51" t="s">
+        <v>139</v>
       </c>
       <c r="G7" s="12">
         <v>4127359182</v>
@@ -4427,7 +4433,7 @@
         <v>Alexis--Gallego--+58-4127359182</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="C11"/>
     </row>
   </sheetData>
@@ -4443,73 +4449,73 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B0E77388-6266-4A55-B7A3-4FCD2B643D29}">
   <dimension ref="A1:F5"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="26.88671875" customWidth="1"/>
-    <col min="2" max="2" width="27.33203125" customWidth="1"/>
-    <col min="3" max="3" width="19.88671875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="16.33203125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="18.44140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="26.85546875" customWidth="1"/>
+    <col min="2" max="2" width="32.5703125" customWidth="1"/>
+    <col min="3" max="3" width="28" customWidth="1"/>
+    <col min="4" max="4" width="26.7109375" customWidth="1"/>
+    <col min="5" max="5" width="16.28515625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="18.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" ht="39.6" x14ac:dyDescent="0.3">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" ht="57" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="18" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="B2" s="19" t="s">
-        <v>41</v>
+        <v>177</v>
       </c>
       <c r="C2" s="19" t="s">
-        <v>48</v>
+        <v>178</v>
       </c>
       <c r="D2" s="19" t="s">
-        <v>42</v>
+        <v>179</v>
       </c>
       <c r="E2" s="19" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="14" t="s">
+        <v>31</v>
+      </c>
+      <c r="B3" s="13" t="s">
+        <v>35</v>
+      </c>
+      <c r="C3" s="13" t="s">
+        <v>23</v>
+      </c>
+      <c r="D3" s="13" t="s">
+        <v>70</v>
+      </c>
+      <c r="E3" s="33" t="s">
         <v>36</v>
       </c>
-      <c r="B3" s="13" t="s">
-        <v>40</v>
-      </c>
-      <c r="C3" s="13" t="s">
-        <v>28</v>
-      </c>
-      <c r="D3" s="13" t="s">
-        <v>87</v>
-      </c>
-      <c r="E3" s="35" t="s">
-        <v>43</v>
-      </c>
       <c r="F3" s="3"/>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="12">
         <v>1</v>
       </c>
       <c r="B4" s="12">
         <v>10</v>
       </c>
-      <c r="C4" s="46">
+      <c r="C4" s="44">
         <v>10000</v>
       </c>
       <c r="D4" s="12">
         <v>3</v>
       </c>
-      <c r="E4" s="55" t="str">
+      <c r="E4" s="53" t="str">
         <f>Barberia_D!B4</f>
         <v>Barbería Oriental</v>
       </c>
@@ -4518,7 +4524,7 @@
         <v/>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="D5" s="2"/>
     </row>
   </sheetData>
@@ -4534,79 +4540,80 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2190E1EC-B79B-40C0-AC5B-0E2726DDD399}">
-  <dimension ref="A1:F10"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:F11"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="27" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="26" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="21.33203125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13" customWidth="1"/>
-    <col min="6" max="6" width="34.88671875" customWidth="1"/>
+    <col min="3" max="3" width="21.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="19.28515625" customWidth="1"/>
+    <col min="5" max="5" width="20.28515625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="34.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" ht="37.5" customHeight="1" x14ac:dyDescent="0.3">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="19" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="B2" s="19" t="s">
-        <v>98</v>
+        <v>78</v>
       </c>
       <c r="C2" s="19" t="s">
-        <v>158</v>
+        <v>129</v>
       </c>
       <c r="D2" s="19" t="s">
-        <v>159</v>
+        <v>181</v>
       </c>
       <c r="E2" s="19" t="s">
-        <v>160</v>
+        <v>182</v>
       </c>
       <c r="F2" s="19" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="14" t="s">
+        <v>31</v>
+      </c>
+      <c r="B3" s="33" t="s">
         <v>36</v>
       </c>
-      <c r="B3" s="35" t="s">
-        <v>43</v>
-      </c>
-      <c r="C3" s="42" t="s">
-        <v>99</v>
-      </c>
-      <c r="D3" s="48" t="s">
-        <v>100</v>
+      <c r="C3" s="40" t="s">
+        <v>79</v>
+      </c>
+      <c r="D3" s="46" t="s">
+        <v>80</v>
       </c>
       <c r="E3" s="13" t="s">
-        <v>101</v>
-      </c>
-      <c r="F3" s="39" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+        <v>81</v>
+      </c>
+      <c r="F3" s="37" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="12">
         <v>1</v>
       </c>
-      <c r="B4" s="55" t="str">
+      <c r="B4" s="53" t="str">
         <f>Barberia_D!B4</f>
         <v>Barbería Oriental</v>
       </c>
-      <c r="C4" s="41" t="s">
-        <v>102</v>
-      </c>
-      <c r="D4" s="41">
+      <c r="C4" s="39" t="s">
+        <v>82</v>
+      </c>
+      <c r="D4" s="39">
         <v>0.375</v>
       </c>
-      <c r="E4" s="41">
+      <c r="E4" s="39">
         <v>0.79166666666666663</v>
       </c>
       <c r="F4" s="12" t="str">
@@ -4614,21 +4621,21 @@
         <v>Barbería Oriental-Lunes-09:00-19:00</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="12">
         <v>2</v>
       </c>
-      <c r="B5" s="55" t="str">
+      <c r="B5" s="53" t="str">
         <f>Barberia_D!B4</f>
         <v>Barbería Oriental</v>
       </c>
       <c r="C5" s="12" t="s">
-        <v>103</v>
-      </c>
-      <c r="D5" s="41">
+        <v>83</v>
+      </c>
+      <c r="D5" s="39">
         <v>0.375</v>
       </c>
-      <c r="E5" s="41">
+      <c r="E5" s="39">
         <v>0.79166666666666663</v>
       </c>
       <c r="F5" s="12" t="str">
@@ -4636,21 +4643,21 @@
         <v>Barbería Oriental-Martes-09:00-19:00</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="12">
         <v>3</v>
       </c>
-      <c r="B6" s="55" t="str">
+      <c r="B6" s="53" t="str">
         <f>Barberia_D!B4</f>
         <v>Barbería Oriental</v>
       </c>
-      <c r="C6" s="41" t="s">
-        <v>104</v>
-      </c>
-      <c r="D6" s="41">
+      <c r="C6" s="39" t="s">
+        <v>84</v>
+      </c>
+      <c r="D6" s="39">
         <v>0.375</v>
       </c>
-      <c r="E6" s="41">
+      <c r="E6" s="39">
         <v>0.79166666666666696</v>
       </c>
       <c r="F6" s="12" t="str">
@@ -4658,21 +4665,21 @@
         <v>Barbería Oriental-Miércoles-09:00-19:00</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="12">
         <v>4</v>
       </c>
-      <c r="B7" s="55" t="str">
+      <c r="B7" s="53" t="str">
         <f>Barberia_D!B4</f>
         <v>Barbería Oriental</v>
       </c>
       <c r="C7" s="12" t="s">
-        <v>105</v>
-      </c>
-      <c r="D7" s="41">
+        <v>85</v>
+      </c>
+      <c r="D7" s="39">
         <v>0.375</v>
       </c>
-      <c r="E7" s="41">
+      <c r="E7" s="39">
         <v>0.79166666666666696</v>
       </c>
       <c r="F7" s="12" t="str">
@@ -4680,21 +4687,21 @@
         <v>Barbería Oriental-Jueves-09:00-19:00</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="12">
         <v>5</v>
       </c>
-      <c r="B8" s="55" t="str">
+      <c r="B8" s="53" t="str">
         <f>Barberia_D!B4</f>
         <v>Barbería Oriental</v>
       </c>
-      <c r="C8" s="41" t="s">
-        <v>106</v>
-      </c>
-      <c r="D8" s="41">
+      <c r="C8" s="39" t="s">
+        <v>86</v>
+      </c>
+      <c r="D8" s="39">
         <v>0.375</v>
       </c>
-      <c r="E8" s="41">
+      <c r="E8" s="39">
         <v>0.79166666666666696</v>
       </c>
       <c r="F8" s="12" t="str">
@@ -4702,21 +4709,21 @@
         <v>Barbería Oriental-Viernes-09:00-19:00</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="12">
         <v>6</v>
       </c>
-      <c r="B9" s="55" t="str">
+      <c r="B9" s="53" t="str">
         <f>Barberia_D!B4</f>
         <v>Barbería Oriental</v>
       </c>
       <c r="C9" s="12" t="s">
-        <v>107</v>
-      </c>
-      <c r="D9" s="44">
+        <v>87</v>
+      </c>
+      <c r="D9" s="42">
         <v>0.33333333333333331</v>
       </c>
-      <c r="E9" s="41">
+      <c r="E9" s="39">
         <v>0.875</v>
       </c>
       <c r="F9" s="12" t="str">
@@ -4724,10 +4731,15 @@
         <v>Barbería Oriental-Sábado-08:00-21:00</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="10"/>
-      <c r="B10" s="43"/>
-      <c r="C10" s="43"/>
+      <c r="B10" s="41"/>
+      <c r="C10" s="41"/>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="C11" s="61" t="s">
+        <v>180</v>
+      </c>
     </row>
   </sheetData>
   <phoneticPr fontId="7" type="noConversion"/>
@@ -4749,81 +4761,81 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C97B567D-D27E-4BE3-B1E4-8CA267790151}">
   <dimension ref="A1:F12"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="2" width="28.109375" customWidth="1"/>
-    <col min="3" max="3" width="26.5546875" customWidth="1"/>
-    <col min="4" max="4" width="16.33203125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="17.33203125" customWidth="1"/>
-    <col min="6" max="6" width="26.5546875" customWidth="1"/>
+    <col min="1" max="2" width="28.140625" customWidth="1"/>
+    <col min="3" max="3" width="26.5703125" customWidth="1"/>
+    <col min="4" max="4" width="24.42578125" customWidth="1"/>
+    <col min="5" max="5" width="25.28515625" customWidth="1"/>
+    <col min="6" max="6" width="26.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="16" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="B1" s="16" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="D1" s="17"/>
       <c r="E1" s="17"/>
       <c r="F1" s="10"/>
     </row>
-    <row r="2" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A2" s="21" t="s">
-        <v>25</v>
-      </c>
-      <c r="B2" s="21" t="s">
+    <row r="2" spans="1:6" ht="45.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="18" t="s">
+        <v>20</v>
+      </c>
+      <c r="B2" s="18" t="s">
+        <v>149</v>
+      </c>
+      <c r="C2" s="18" t="s">
+        <v>183</v>
+      </c>
+      <c r="D2" s="32" t="s">
+        <v>184</v>
+      </c>
+      <c r="E2" s="32" t="s">
         <v>185</v>
       </c>
-      <c r="C2" s="21" t="s">
-        <v>44</v>
-      </c>
-      <c r="D2" s="22" t="s">
-        <v>46</v>
-      </c>
-      <c r="E2" s="22" t="s">
-        <v>47</v>
-      </c>
       <c r="F2" s="19" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A3" s="23" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" s="21" t="s">
+        <v>31</v>
+      </c>
+      <c r="B3" s="58" t="s">
         <v>36</v>
       </c>
-      <c r="B3" s="60" t="s">
-        <v>43</v>
-      </c>
-      <c r="C3" s="24" t="s">
-        <v>26</v>
-      </c>
-      <c r="D3" s="24" t="s">
-        <v>45</v>
-      </c>
-      <c r="E3" s="24" t="s">
-        <v>29</v>
+      <c r="C3" s="22" t="s">
+        <v>21</v>
+      </c>
+      <c r="D3" s="22" t="s">
+        <v>37</v>
+      </c>
+      <c r="E3" s="22" t="s">
+        <v>24</v>
       </c>
       <c r="F3" s="15" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A4" s="25">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" s="23">
         <v>1</v>
       </c>
-      <c r="B4" s="61" t="str">
+      <c r="B4" s="59" t="str">
         <f>Barberia_D!B4</f>
         <v>Barbería Oriental</v>
       </c>
-      <c r="C4" s="25" t="s">
-        <v>49</v>
-      </c>
-      <c r="D4" s="25">
+      <c r="C4" s="23" t="s">
+        <v>38</v>
+      </c>
+      <c r="D4" s="23">
         <v>45</v>
       </c>
-      <c r="E4" s="26">
+      <c r="E4" s="24">
         <v>22000</v>
       </c>
       <c r="F4" s="12" t="str">
@@ -4831,21 +4843,21 @@
         <v>Motilada</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A5" s="25">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" s="23">
         <v>2</v>
       </c>
-      <c r="B5" s="61" t="str">
+      <c r="B5" s="59" t="str">
         <f>Barberia_D!B4</f>
         <v>Barbería Oriental</v>
       </c>
-      <c r="C5" s="25" t="s">
-        <v>57</v>
-      </c>
-      <c r="D5" s="25">
+      <c r="C5" s="23" t="s">
+        <v>46</v>
+      </c>
+      <c r="D5" s="23">
         <v>10</v>
       </c>
-      <c r="E5" s="26">
+      <c r="E5" s="24">
         <v>12000</v>
       </c>
       <c r="F5" s="12" t="str">
@@ -4853,21 +4865,21 @@
         <v>Corte de barba</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A6" s="25">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" s="23">
         <v>3</v>
       </c>
-      <c r="B6" s="61" t="str">
+      <c r="B6" s="59" t="str">
         <f>Barberia_D!B4</f>
         <v>Barbería Oriental</v>
       </c>
-      <c r="C6" s="25" t="s">
-        <v>58</v>
-      </c>
-      <c r="D6" s="25">
+      <c r="C6" s="23" t="s">
+        <v>47</v>
+      </c>
+      <c r="D6" s="23">
         <v>15</v>
       </c>
-      <c r="E6" s="26">
+      <c r="E6" s="24">
         <v>15000</v>
       </c>
       <c r="F6" s="12" t="str">
@@ -4875,57 +4887,57 @@
         <v>Perfilada de barba</v>
       </c>
     </row>
-    <row r="7" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A7" s="25">
+    <row r="7" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A7" s="23">
         <v>4</v>
       </c>
-      <c r="B7" s="61" t="str">
+      <c r="B7" s="59" t="str">
         <f>Barberia_D!B4</f>
         <v>Barbería Oriental</v>
       </c>
-      <c r="C7" s="27" t="s">
-        <v>59</v>
-      </c>
-      <c r="D7" s="25">
+      <c r="C7" s="25" t="s">
+        <v>48</v>
+      </c>
+      <c r="D7" s="23">
         <v>30</v>
       </c>
-      <c r="E7" s="26">
+      <c r="E7" s="24">
         <v>35000</v>
       </c>
-      <c r="F7" s="28" t="str">
+      <c r="F7" s="26" t="str">
         <f t="shared" si="0"/>
         <v>Arreglo completo de barba con toalla caliente</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="17"/>
       <c r="B8" s="17"/>
       <c r="C8" s="17"/>
       <c r="D8" s="17"/>
       <c r="E8" s="17"/>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="17"/>
       <c r="B9" s="17"/>
       <c r="C9" s="17"/>
       <c r="D9" s="17"/>
       <c r="E9" s="17"/>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="17"/>
       <c r="B10" s="17"/>
       <c r="C10" s="17"/>
       <c r="D10" s="17"/>
       <c r="E10" s="17"/>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="17"/>
       <c r="B11" s="17"/>
       <c r="C11" s="17"/>
       <c r="D11" s="17"/>
       <c r="E11" s="17"/>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="17"/>
       <c r="B12" s="17"/>
       <c r="C12" s="17"/>
@@ -4948,214 +4960,214 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2DAE59AB-4103-4731-9C3C-4C276F8A29F8}">
-  <dimension ref="A1:L10"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:L14"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="27" bestFit="1" customWidth="1"/>
-    <col min="2" max="6" width="26.6640625" customWidth="1"/>
-    <col min="7" max="7" width="16.33203125" customWidth="1"/>
-    <col min="8" max="9" width="40.6640625" customWidth="1"/>
-    <col min="10" max="10" width="27.109375" customWidth="1"/>
+    <col min="2" max="6" width="26.7109375" customWidth="1"/>
+    <col min="7" max="7" width="16.28515625" customWidth="1"/>
+    <col min="8" max="9" width="40.7109375" customWidth="1"/>
+    <col min="10" max="10" width="30.28515625" customWidth="1"/>
     <col min="11" max="11" width="21" customWidth="1"/>
-    <col min="12" max="12" width="53.109375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="53.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="C1" s="5"/>
       <c r="D1" s="5"/>
       <c r="E1" s="5"/>
       <c r="F1" s="5"/>
     </row>
-    <row r="2" spans="1:12" ht="45.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="29" t="s">
-        <v>25</v>
-      </c>
-      <c r="B2" s="29" t="s">
+    <row r="2" spans="1:12" ht="45.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="27" t="s">
+        <v>20</v>
+      </c>
+      <c r="B2" s="27" t="s">
+        <v>186</v>
+      </c>
+      <c r="C2" s="27" t="s">
+        <v>187</v>
+      </c>
+      <c r="D2" s="27" t="s">
+        <v>188</v>
+      </c>
+      <c r="E2" s="27" t="s">
+        <v>189</v>
+      </c>
+      <c r="F2" s="27" t="s">
+        <v>191</v>
+      </c>
+      <c r="G2" s="28" t="s">
+        <v>49</v>
+      </c>
+      <c r="H2" s="28" t="s">
+        <v>192</v>
+      </c>
+      <c r="I2" s="28" t="s">
+        <v>193</v>
+      </c>
+      <c r="J2" s="28" t="s">
         <v>141</v>
       </c>
-      <c r="C2" s="29" t="s">
-        <v>143</v>
-      </c>
-      <c r="D2" s="29" t="s">
-        <v>142</v>
-      </c>
-      <c r="E2" s="29" t="s">
-        <v>140</v>
-      </c>
-      <c r="F2" s="29" t="s">
-        <v>175</v>
-      </c>
-      <c r="G2" s="30" t="s">
-        <v>60</v>
-      </c>
-      <c r="H2" s="30" t="s">
-        <v>165</v>
-      </c>
-      <c r="I2" s="30" t="s">
-        <v>166</v>
-      </c>
-      <c r="J2" s="30" t="s">
-        <v>177</v>
-      </c>
-      <c r="K2" s="30" t="s">
-        <v>186</v>
-      </c>
-      <c r="L2" s="31" t="s">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="K2" s="28" t="s">
+        <v>150</v>
+      </c>
+      <c r="L2" s="29" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A3" s="14" t="s">
+        <v>31</v>
+      </c>
+      <c r="B3" s="13" t="s">
+        <v>109</v>
+      </c>
+      <c r="C3" s="13" t="s">
+        <v>111</v>
+      </c>
+      <c r="D3" s="13" t="s">
+        <v>110</v>
+      </c>
+      <c r="E3" s="13" t="s">
+        <v>112</v>
+      </c>
+      <c r="F3" s="13" t="s">
+        <v>137</v>
+      </c>
+      <c r="G3" s="13" t="s">
+        <v>22</v>
+      </c>
+      <c r="H3" s="13" t="s">
+        <v>42</v>
+      </c>
+      <c r="I3" s="13" t="s">
+        <v>133</v>
+      </c>
+      <c r="J3" s="47" t="s">
+        <v>43</v>
+      </c>
+      <c r="K3" s="33" t="s">
         <v>36</v>
       </c>
-      <c r="B3" s="13" t="s">
-        <v>130</v>
-      </c>
-      <c r="C3" s="13" t="s">
-        <v>132</v>
-      </c>
-      <c r="D3" s="13" t="s">
-        <v>131</v>
-      </c>
-      <c r="E3" s="13" t="s">
-        <v>133</v>
-      </c>
-      <c r="F3" s="13" t="s">
-        <v>171</v>
-      </c>
-      <c r="G3" s="13" t="s">
-        <v>27</v>
-      </c>
-      <c r="H3" s="13" t="s">
-        <v>53</v>
-      </c>
-      <c r="I3" s="13" t="s">
-        <v>164</v>
-      </c>
-      <c r="J3" s="49" t="s">
-        <v>54</v>
-      </c>
-      <c r="K3" s="35" t="s">
-        <v>43</v>
-      </c>
-      <c r="L3" s="32" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="L3" s="30" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A4" s="12">
         <v>1</v>
       </c>
       <c r="B4" s="12" t="s">
-        <v>63</v>
+        <v>126</v>
       </c>
       <c r="C4" s="12" t="s">
-        <v>134</v>
+        <v>113</v>
       </c>
       <c r="D4" s="12" t="s">
-        <v>67</v>
+        <v>156</v>
       </c>
       <c r="E4" s="12" t="s">
-        <v>136</v>
-      </c>
-      <c r="F4" s="53" t="s">
-        <v>172</v>
+        <v>115</v>
+      </c>
+      <c r="F4" s="51" t="s">
+        <v>138</v>
       </c>
       <c r="G4" s="12">
         <v>3245627890</v>
       </c>
       <c r="H4" s="11" t="s">
-        <v>70</v>
-      </c>
-      <c r="I4" s="51">
+        <v>54</v>
+      </c>
+      <c r="I4" s="49">
         <v>1264267821</v>
       </c>
       <c r="J4" s="12" t="s">
-        <v>61</v>
-      </c>
-      <c r="K4" s="55" t="str">
+        <v>50</v>
+      </c>
+      <c r="K4" s="53" t="str">
         <f>Barberia_D!B4</f>
         <v>Barbería Oriental</v>
       </c>
       <c r="L4" s="12" t="str">
         <f>_xlfn.CONCAT(B4,"-",C4,"-",D4,"-",E4,"-",F4,"-",G4)</f>
-        <v>Juan Fernando-Fernando-García Lopez-Lopez-+57-3245627890</v>
-      </c>
-    </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
+        <v>Juan-Fernando-García-Lopez-+57-3245627890</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A5" s="12">
         <v>2</v>
       </c>
       <c r="B5" s="12" t="s">
-        <v>64</v>
+        <v>126</v>
       </c>
       <c r="C5" s="12" t="s">
-        <v>135</v>
+        <v>114</v>
       </c>
       <c r="D5" s="12" t="s">
-        <v>68</v>
+        <v>155</v>
       </c>
       <c r="E5" s="12" t="s">
-        <v>137</v>
-      </c>
-      <c r="F5" s="53" t="s">
-        <v>172</v>
+        <v>116</v>
+      </c>
+      <c r="F5" s="51" t="s">
+        <v>138</v>
       </c>
       <c r="G5" s="12">
         <v>3124518923</v>
       </c>
       <c r="H5" s="11" t="s">
-        <v>71</v>
-      </c>
-      <c r="I5" s="51" t="s">
-        <v>168</v>
+        <v>55</v>
+      </c>
+      <c r="I5" s="49" t="s">
+        <v>135</v>
       </c>
       <c r="J5" s="12" t="s">
-        <v>62</v>
-      </c>
-      <c r="K5" s="55" t="str">
+        <v>50</v>
+      </c>
+      <c r="K5" s="53" t="str">
         <f>Barberia_D!B4</f>
         <v>Barbería Oriental</v>
       </c>
       <c r="L5" s="12" t="str">
-        <f t="shared" ref="L5:L7" si="0">_xlfn.CONCAT(B5,"-",C5,"-",D5,"-",E5,"-",F5,"-",G5)</f>
-        <v>Juan David-David-Ortiz Sanchez-Sanchez-+57-3124518923</v>
-      </c>
-    </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.3">
+        <f t="shared" ref="L5:L8" si="0">_xlfn.CONCAT(B5,"-",C5,"-",D5,"-",E5,"-",F5,"-",G5)</f>
+        <v>Juan-David-Ortiz-Sanchez-+57-3124518923</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A6" s="12">
         <v>3</v>
       </c>
       <c r="B6" s="12" t="s">
-        <v>65</v>
+        <v>52</v>
       </c>
       <c r="C6" s="12"/>
       <c r="D6" s="12" t="s">
-        <v>139</v>
+        <v>118</v>
       </c>
       <c r="E6" s="12"/>
-      <c r="F6" s="53" t="s">
-        <v>172</v>
+      <c r="F6" s="51" t="s">
+        <v>138</v>
       </c>
       <c r="G6" s="12">
         <v>3214533321</v>
       </c>
       <c r="H6" s="11" t="s">
-        <v>72</v>
-      </c>
-      <c r="I6" s="52" t="s">
-        <v>167</v>
+        <v>56</v>
+      </c>
+      <c r="I6" s="50" t="s">
+        <v>134</v>
       </c>
       <c r="J6" s="12" t="s">
-        <v>61</v>
-      </c>
-      <c r="K6" s="55" t="str">
+        <v>50</v>
+      </c>
+      <c r="K6" s="53" t="str">
         <f>Barberia_D!B4</f>
         <v>Barbería Oriental</v>
       </c>
@@ -5164,47 +5176,92 @@
         <v>Carlos--Arbeladez--+57-3214533321</v>
       </c>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A7" s="12">
         <v>4</v>
       </c>
       <c r="B7" s="12" t="s">
-        <v>66</v>
+        <v>53</v>
       </c>
       <c r="C7" s="12"/>
       <c r="D7" s="12" t="s">
-        <v>69</v>
+        <v>121</v>
       </c>
       <c r="E7" s="12" t="s">
-        <v>138</v>
-      </c>
-      <c r="F7" s="53" t="s">
-        <v>176</v>
+        <v>117</v>
+      </c>
+      <c r="F7" s="51" t="s">
+        <v>140</v>
       </c>
       <c r="G7" s="12">
         <v>9876543210</v>
       </c>
       <c r="H7" s="11" t="s">
-        <v>73</v>
-      </c>
-      <c r="I7" s="51" t="s">
-        <v>169</v>
+        <v>57</v>
+      </c>
+      <c r="I7" s="49" t="s">
+        <v>136</v>
       </c>
       <c r="J7" s="12" t="s">
-        <v>61</v>
-      </c>
-      <c r="K7" s="55" t="str">
+        <v>50</v>
+      </c>
+      <c r="K7" s="53" t="str">
         <f>Barberia_D!B4</f>
         <v>Barbería Oriental</v>
       </c>
       <c r="L7" s="12" t="str">
         <f t="shared" si="0"/>
-        <v>Andres--Ramirez Patiño-Patiño-+91-9876543210</v>
-      </c>
-    </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.3">
+        <v>Andres--Ramirez-Patiño-+91-9876543210</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A8" s="12">
+        <v>5</v>
+      </c>
+      <c r="B8" s="12" t="s">
+        <v>126</v>
+      </c>
+      <c r="C8" s="12" t="s">
+        <v>52</v>
+      </c>
+      <c r="D8" s="12" t="s">
+        <v>157</v>
+      </c>
+      <c r="E8" s="12" t="s">
+        <v>120</v>
+      </c>
+      <c r="F8" s="51" t="s">
+        <v>158</v>
+      </c>
+      <c r="G8" s="12">
+        <v>998765432</v>
+      </c>
+      <c r="H8" s="11" t="s">
+        <v>159</v>
+      </c>
+      <c r="I8" s="12">
+        <v>312334342</v>
+      </c>
+      <c r="J8" s="12" t="s">
+        <v>51</v>
+      </c>
+      <c r="K8" s="53" t="str">
+        <f>Barberia_D!B4</f>
+        <v>Barbería Oriental</v>
+      </c>
+      <c r="L8" s="12" t="str">
+        <f t="shared" si="0"/>
+        <v>Juan-Carlos-Zambrano-Perez-+593-998765432</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B10" s="10"/>
       <c r="C10" s="10"/>
+    </row>
+    <row r="14" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="F14" t="s">
+        <v>190</v>
+      </c>
     </row>
   </sheetData>
   <phoneticPr fontId="7" type="noConversion"/>
@@ -5218,6 +5275,8 @@
     <hyperlink ref="K3" location="Barberia_D!A1" display="barberia" xr:uid="{0A424D71-DFC6-4A9B-AB84-795AF0206DA0}"/>
     <hyperlink ref="K4" location="Barberia_D!A4" display="Barberia_D!A4" xr:uid="{74759F60-91D9-4AA0-8D34-C14AE4845BDE}"/>
     <hyperlink ref="K5:K7" location="Barberia_D!A4" display="Barberia_D!A4" xr:uid="{8B3C5650-71BD-4B78-A8B9-12566120F044}"/>
+    <hyperlink ref="K8" location="Barberia_D!A4" display="Barberia_D!A4" xr:uid="{B14FD134-98B7-4B6A-849C-ECE5A6600A50}"/>
+    <hyperlink ref="H8" r:id="rId5" xr:uid="{8A2F5CE3-2E3F-41D6-9E52-2EDCD463D69D}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -5226,58 +5285,58 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C828B98D-AAA9-4184-8373-FE2E421AAE23}">
   <dimension ref="A1:E11"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="27" customWidth="1"/>
-    <col min="2" max="2" width="28.88671875" customWidth="1"/>
+    <col min="2" max="2" width="28.85546875" customWidth="1"/>
     <col min="3" max="3" width="41" customWidth="1"/>
-    <col min="4" max="4" width="36.109375" customWidth="1"/>
-    <col min="5" max="5" width="26.88671875" customWidth="1"/>
+    <col min="4" max="4" width="36.140625" customWidth="1"/>
+    <col min="5" max="5" width="26.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" ht="49.8" customHeight="1" x14ac:dyDescent="0.3">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="18" t="s">
+        <v>20</v>
+      </c>
+      <c r="B2" s="18" t="s">
+        <v>59</v>
+      </c>
+      <c r="C2" s="32" t="s">
+        <v>61</v>
+      </c>
+      <c r="D2" s="32" t="s">
+        <v>132</v>
+      </c>
+      <c r="E2" s="32" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3" s="14" t="s">
+        <v>31</v>
+      </c>
+      <c r="B3" s="33" t="s">
+        <v>62</v>
+      </c>
+      <c r="C3" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="B2" s="18" t="s">
+      <c r="D3" s="47" t="s">
+        <v>58</v>
+      </c>
+      <c r="E3" s="30" t="s">
         <v>75</v>
       </c>
-      <c r="C2" s="34" t="s">
-        <v>77</v>
-      </c>
-      <c r="D2" s="34" t="s">
-        <v>163</v>
-      </c>
-      <c r="E2" s="34" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A3" s="14" t="s">
-        <v>36</v>
-      </c>
-      <c r="B3" s="35" t="s">
-        <v>78</v>
-      </c>
-      <c r="C3" s="13" t="s">
-        <v>30</v>
-      </c>
-      <c r="D3" s="49" t="s">
-        <v>74</v>
-      </c>
-      <c r="E3" s="32" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="12">
         <v>1</v>
       </c>
@@ -5285,18 +5344,18 @@
         <f>Cliente_D!G4</f>
         <v>3234528921</v>
       </c>
-      <c r="C4" s="36">
+      <c r="C4" s="34">
         <v>45255</v>
       </c>
       <c r="D4" s="12" t="s">
-        <v>62</v>
+        <v>51</v>
       </c>
       <c r="E4" s="12" t="str">
         <f>_xlfn.CONCAT(B4,"-",TEXT(C4,"dd/mm/yyyy"))</f>
         <v>3234528921-25/11/2023</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="12">
         <v>2</v>
       </c>
@@ -5304,18 +5363,18 @@
         <f>Cliente_D!G5</f>
         <v>3161657782</v>
       </c>
-      <c r="C5" s="36">
+      <c r="C5" s="34">
         <v>45372</v>
       </c>
       <c r="D5" s="12" t="s">
-        <v>62</v>
+        <v>51</v>
       </c>
       <c r="E5" s="12" t="str">
         <f t="shared" ref="E5:E7" si="0">_xlfn.CONCAT(B5,"-",TEXT(C5,"dd/mm/yyyy"))</f>
         <v>3161657782-21/03/2024</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="12">
         <v>3</v>
       </c>
@@ -5323,18 +5382,18 @@
         <f>Cliente_D!G6</f>
         <v>3119884321</v>
       </c>
-      <c r="C6" s="36">
+      <c r="C6" s="34">
         <v>45556</v>
       </c>
       <c r="D6" s="12" t="s">
-        <v>61</v>
+        <v>50</v>
       </c>
       <c r="E6" s="12" t="str">
         <f t="shared" si="0"/>
         <v>3119884321-21/09/2024</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="12">
         <v>4</v>
       </c>
@@ -5342,23 +5401,23 @@
         <f>Cliente_D!G7</f>
         <v>4127359182</v>
       </c>
-      <c r="C7" s="36">
+      <c r="C7" s="34">
         <v>46002</v>
       </c>
       <c r="D7" s="12" t="s">
-        <v>61</v>
+        <v>50</v>
       </c>
       <c r="E7" s="12" t="str">
         <f t="shared" si="0"/>
         <v>4127359182-11/12/2025</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="C8" s="33"/>
-      <c r="D8" s="33"/>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="C11" s="50"/>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="C8" s="31"/>
+      <c r="D8" s="31"/>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="C11" s="48"/>
     </row>
   </sheetData>
   <hyperlinks>

</xml_diff>

<commit_message>
Definiendo los tipos de datos y valores por defecto del muestreo
</commit_message>
<xml_diff>
--- a/Muestreo de datos.xlsx
+++ b/Muestreo de datos.xlsx
@@ -5,29 +5,30 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jesus\OneDrive\Escritorio\leo\Doo\Barberia proyecto\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\leand\Desktop\DOO\DOO\Barberia\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6884477C-7AFB-4EA2-A1F3-CB639B29ADD1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D2C82A5-CE11-488F-916B-C5EEB7B95CE2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" firstSheet="1" activeTab="7" xr2:uid="{09A6C7D7-663F-4C06-9D71-8A4E97495CF9}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{09A6C7D7-663F-4C06-9D71-8A4E97495CF9}"/>
   </bookViews>
   <sheets>
     <sheet name="Modelo de Dominio" sheetId="1" r:id="rId1"/>
     <sheet name="Objetos de Dominio" sheetId="4" r:id="rId2"/>
-    <sheet name="Barberia_D" sheetId="5" r:id="rId3"/>
-    <sheet name="Cliente_D" sheetId="6" r:id="rId4"/>
-    <sheet name="Regla_D" sheetId="7" r:id="rId5"/>
-    <sheet name="HorarioBarberia_D" sheetId="18" r:id="rId6"/>
-    <sheet name="Servicio_D" sheetId="8" r:id="rId7"/>
-    <sheet name="Barbero_D" sheetId="9" r:id="rId8"/>
-    <sheet name="Veto_D" sheetId="10" r:id="rId9"/>
-    <sheet name="BarberoServicio_D" sheetId="11" r:id="rId10"/>
-    <sheet name="Agenda_D" sheetId="12" r:id="rId11"/>
-    <sheet name="HorarioBarbero_D" sheetId="20" r:id="rId12"/>
-    <sheet name="Cita_D" sheetId="13" r:id="rId13"/>
-    <sheet name="Multa_D" sheetId="16" r:id="rId14"/>
-    <sheet name="CitaServicio_D" sheetId="17" r:id="rId15"/>
+    <sheet name="Tipo de datos" sheetId="21" r:id="rId3"/>
+    <sheet name="Barberia_D" sheetId="5" r:id="rId4"/>
+    <sheet name="Cliente_D" sheetId="6" r:id="rId5"/>
+    <sheet name="Regla_D" sheetId="7" r:id="rId6"/>
+    <sheet name="HorarioBarberia_D" sheetId="18" r:id="rId7"/>
+    <sheet name="Servicio_D" sheetId="8" r:id="rId8"/>
+    <sheet name="Barbero_D" sheetId="9" r:id="rId9"/>
+    <sheet name="Veto_D" sheetId="10" r:id="rId10"/>
+    <sheet name="BarberoServicio_D" sheetId="11" r:id="rId11"/>
+    <sheet name="Agenda_D" sheetId="12" r:id="rId12"/>
+    <sheet name="HorarioBarbero_D" sheetId="20" r:id="rId13"/>
+    <sheet name="Cita_D" sheetId="13" r:id="rId14"/>
+    <sheet name="Multa_D" sheetId="16" r:id="rId15"/>
+    <sheet name="CitaServicio_D" sheetId="17" r:id="rId16"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -53,7 +54,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="306" uniqueCount="194">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="333" uniqueCount="220">
   <si>
     <t>Nombre</t>
   </si>
@@ -202,9 +203,6 @@
     <t>Arreglo completo de barba con toalla caliente</t>
   </si>
   <si>
-    <t>Representa el numero de celular del barbero</t>
-  </si>
-  <si>
     <t>si</t>
   </si>
   <si>
@@ -272,9 +270,6 @@
   </si>
   <si>
     <t>Combinación única</t>
-  </si>
-  <si>
-    <t xml:space="preserve">combinacion única </t>
   </si>
   <si>
     <t xml:space="preserve">Combinación única </t>
@@ -329,9 +324,6 @@
 Hace referencia a la agenda (y por lo tanto al barbero) a la que pertenece este horario, permite saber de quién es cada bloque de disponibilidad</t>
   </si>
   <si>
-    <t>Representa el día de la semana en que aplica este horario, es necesario porque un barbero puede trabajar unos días sí y otros no</t>
-  </si>
-  <si>
     <t>Representa la hora en la que el barbero empieza a estar disponible ese dia</t>
   </si>
   <si>
@@ -371,9 +363,6 @@
     <t>Hace referencia a cual servicio del catalogo fue el que se pidió en esa cita</t>
   </si>
   <si>
-    <t>Representa cuanto valía el servicio en el momento exacto en que se agendó la cita, se guarda aparte del precio del catalogo por si el precio de ese servicio cambia después, las citas ya registradas no se vean afectadas</t>
-  </si>
-  <si>
     <t>Representa cuanto duraba el servicio en el momento en que se agendó, junto con la hora de inicio de la cita permite calcular hasta que hora queda ocupado el barbero</t>
   </si>
   <si>
@@ -443,9 +432,6 @@
     <t>Alexis</t>
   </si>
   <si>
-    <t>Representa el día de la semana en que aplica este horario, es necesario para saber que días abrira la barberia</t>
-  </si>
-  <si>
     <t>Combinacion única que indica que no puede existir más de un horario con la misma barberia, dia de la semana, hora de apertura y cierre</t>
   </si>
   <si>
@@ -483,9 +469,6 @@
   </si>
   <si>
     <t>fechaHora</t>
-  </si>
-  <si>
-    <t>Representa la fecha y la hora en el que se va a realizar la cita al cliente</t>
   </si>
   <si>
     <t xml:space="preserve">
@@ -567,54 +550,9 @@
     <t>Representa el nombre de como se llama la barberia en donde trabajan los barberos. El tipo de dato es alfanumérico, su valor por defecto es el vacio y es permitido</t>
   </si>
   <si>
-    <t>Representa el primer nombre de la persona, que va a estar llendo a la barberia para las citas. Su tipo de dato es texto, su valor por defecto es el vacío y no es permitido</t>
-  </si>
-  <si>
-    <t>Representa el segundo nombre de la persona, que va a estar llendo a la barberia para las citas. Su tipo de dato es texto, su valor por defecto es el vacío y es permitido</t>
-  </si>
-  <si>
-    <t>Representa el primer apellido de la persona, que va a estar llendo a la barberia para las citas. Su tipo de dato es texto, su valor por defecto es el vacío y no es permitido</t>
-  </si>
-  <si>
-    <t>Representa el primer apellido de la persona, que va a estar llendo a la barberia para las citas. Su tipo de dato es texto, su valor por defecto es el vacío y es permitido</t>
-  </si>
-  <si>
     <t>prefijoCelular</t>
   </si>
   <si>
-    <t>Representa de que pais es el numero de celular del cliente. Su tipo de dato es alfanumérico, su valor por defecto es +0 (este prefijo no referencia a ningún país) y no es permitido</t>
-  </si>
-  <si>
-    <t>Representa el numero de celular de la persona que le va a escribir al barbero por WhatsApp para pedirle una cita. Su tipo de dato es alfanumérico, su valor por defecto es el 0 y no es permitido</t>
-  </si>
-  <si>
-    <t>Representa la cantidad de minutos que el cliente puede llegarle tarde un cliente a la cita establecida con el barbero, despues de eso el barbero lo podrá multar. Su tipo de dato es numerico, debe de ser mayor o igual a 0, su valor por defecto es el 0 y es permitido</t>
-  </si>
-  <si>
-    <t>Representa la cantidad de dinero que el cliente debe de pagar en pesos colombianos, por superar la toleranciaTardanza. Su tipo de dato es numerico, debe de ser mayor a cero, su valor por defecto es 0 y no es permitido</t>
-  </si>
-  <si>
-    <t>Representa la maxima de multas que pueda tener un cliente sin pagar, a partir de esta cantidad se le hace un veto al cliente. Su tipo de dato es numerico, debe de ser mayor o igual a cero, su valor por defecto es 0 y es permitido</t>
-  </si>
-  <si>
-    <t>Este dato lo tengo pensado como si fuera una lista</t>
-  </si>
-  <si>
-    <t>Representa la hora a la que abre la barbería. Su tipo de dato es hora, su valor por defecto es 00:00 am y es permitido</t>
-  </si>
-  <si>
-    <t>Representa la hora a la que cierra la barbería. Su tipo de dato es hora, su valor por defecto es 00:00 am y es permitido</t>
-  </si>
-  <si>
-    <t>Representa el nombre del servicio que va estar en la barberia, que el barbero ofrece y en las citas que esta. Su tipo de dato es alfanumérico, su valor por defecto es el vacio y no es permitido</t>
-  </si>
-  <si>
-    <t>Representa lo que va durar en minutos el servicio. Su tipo de dato es entero, debe de ser mayor a cero, su valor por defecto es 0 y no es permitido</t>
-  </si>
-  <si>
-    <t>Representa cuanto va a valer el servicio en pesos colombianos. Su tipo de dato es entero, debe de ser mayor a cero, su valor por defecto es 0 y no esta permitido</t>
-  </si>
-  <si>
     <t>Representa el primer nombre del barbero que trabaja en barbería. Su tipo de dato es texto, su valor por defecto es el vacio y no es permitido</t>
   </si>
   <si>
@@ -633,10 +571,151 @@
     <t>Representa de que pais es el numero de celular del barbero. Su tipo de dato es alfanumérico, su valor por defecto es +0 y no es permitido</t>
   </si>
   <si>
-    <t>Representa el correo electronico del barbero, con el que se va a registrar o iniciar seción. Su tipo de dato es alfanumérico, su valor por defecto es el vacio y no es permitido</t>
-  </si>
-  <si>
     <t>Representa la contraseña del barbebro, con el que se va a registrar o iniciar sesión. Su tipo de dato es alfanumérico, su valor por defecto es el vacio y no esta permitido</t>
+  </si>
+  <si>
+    <t>Tipo de dato</t>
+  </si>
+  <si>
+    <t>Texto</t>
+  </si>
+  <si>
+    <t>Alfanumerico</t>
+  </si>
+  <si>
+    <t>Entero</t>
+  </si>
+  <si>
+    <t>Representa el día de la semana en que aplica este horario, es necesario porque un barbero puede trabajar unos días sí y otros no. Su valor por defecto es el vacío y no es permitido</t>
+  </si>
+  <si>
+    <t>Este dato también lo tengo pensado como una lista. Lo dejé como tipo texto</t>
+  </si>
+  <si>
+    <t>FechaHora</t>
+  </si>
+  <si>
+    <t>Hora</t>
+  </si>
+  <si>
+    <t>Identificador unico</t>
+  </si>
+  <si>
+    <t>Combinacion unica</t>
+  </si>
+  <si>
+    <t>Referencia de otros objetos de dominio</t>
+  </si>
+  <si>
+    <t>Dato calculado</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tipo de dato que solo admite letras de la A a la Z. </t>
+  </si>
+  <si>
+    <t>Tipo de dato que admite cualquier tipo de carácter, combinando letras, números y símbolos.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tipo de dato numérico que solo admite números enteros, sin parte decimal. </t>
+  </si>
+  <si>
+    <t>Tipo de dato que solo representa la hora del día (horas y minutos), sin incluir la fecha.</t>
+  </si>
+  <si>
+    <t>Atributo que identifica de forma única a cada instancia de un objeto de dominio, no se puede repetir entre objetos del mismo tipo.</t>
+  </si>
+  <si>
+    <t>Regla de unicidad construida combinando varios atributos de un mismo objeto de dominio, para garantizar que no existan dos instancias con exactamente los mismos valores en esos campos.</t>
+  </si>
+  <si>
+    <t>Tipo de dato que combina fecha y hora en un mismo valor.</t>
+  </si>
+  <si>
+    <t>Atributo que apunta al identificador o a la combinación única de otro objeto de dominio, materializando la relación de asociación entre ambos.</t>
+  </si>
+  <si>
+    <t>Atributo cuyo valor no lo ingresa el usuario, sino que es un dato calculado sobre otros atributos del mismo objeto o de objetos relacionados. Por ejemplo, la hora de finalización de una cita se calcula sumando la hora de inicio y la duración del servicio agendado.</t>
+  </si>
+  <si>
+    <t>Representa el primer nombre de la persona, que va a estar llendo a la barberia para las citas. Su valor por defecto es el vacío y no es permitido</t>
+  </si>
+  <si>
+    <t>Representa el segundo nombre de la persona, que va a estar llendo a la barberia para las citas. Su valor por defecto es el vacío y es permitido</t>
+  </si>
+  <si>
+    <t>Representa el primer apellido de la persona, que va a estar llendo a la barberia para las citas. Su valor por defecto es el vacío y no es permitido</t>
+  </si>
+  <si>
+    <t>Representa el primer apellido de la persona, que va a estar llendo a la barberia para las citas. Su valor por defecto es el vacío y es permitido</t>
+  </si>
+  <si>
+    <t>Representa de que pais es el numero de celular del cliente. Su valor por defecto es +0 (este prefijo no referencia a ningún país) y no es permitido</t>
+  </si>
+  <si>
+    <t>Representa el numero de celular de la persona que le va a escribir al barbero por WhatsApp para pedirle una cita. Su valor por defecto es el 0 y no es permitido</t>
+  </si>
+  <si>
+    <t>Representa la cantidad de minutos que el cliente puede llegarle tarde un cliente a la cita establecida con el barbero, despues de eso el barbero lo podrá multar. Debe de ser mayor o igual a 0, su valor por defecto es el 0 y es permitido</t>
+  </si>
+  <si>
+    <t>Representa la cantidad de dinero que el cliente debe de pagar en pesos colombianos, por superar la toleranciaTardanza. Debe de ser mayor a cero, su valor por defecto es 0 y no es permitido</t>
+  </si>
+  <si>
+    <t>Representa la maxima de multas que pueda tener un cliente sin pagar, a partir de esta cantidad se le hace un veto al cliente. Debe de ser mayor o igual a cero, su valor por defecto es 0 y es permitido</t>
+  </si>
+  <si>
+    <t>Este dato lo tengo pensado como si fuera una lista, pero no se si esta bien dejarlo tipo texto</t>
+  </si>
+  <si>
+    <t>Representa el día de la semana en que aplica este horario, es necesario para saber que días abrira la barberia. Su valor por defecto es el vacio y no es permitido</t>
+  </si>
+  <si>
+    <t>Representa la hora a la que abre la barbería. Su valor por defecto es 00:00 am y es permitido</t>
+  </si>
+  <si>
+    <t>Representa la hora a la que cierra la barbería. Su valor por defecto es 00:00 am y es permitido</t>
+  </si>
+  <si>
+    <t>Representa el nombre del servicio que va estar en la barberia, que el barbero ofrece y en las citas que esta. Su valor por defecto es el vacio y no es permitido</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Combinacion única </t>
+  </si>
+  <si>
+    <t>Representa lo que va durar en minutos el servicio. Debe de ser mayor a cero, su valor por defecto es 0 y no es permitido</t>
+  </si>
+  <si>
+    <t>Representa cuanto va a valer el servicio en pesos colombianos. Debe de ser mayor a cero, su valor por defecto es 0 y no esta permitido</t>
+  </si>
+  <si>
+    <t>Representa el número de celular del barbero. Su valor por defecto es 0 y no es permitido</t>
+  </si>
+  <si>
+    <t>Representa el correo electronico del barbero, con el que se va a registrar o iniciar seción. Su valor por defecto es el vacio y no es permitido</t>
+  </si>
+  <si>
+    <t>Fecha</t>
+  </si>
+  <si>
+    <t>Tipo de dato que contiene el día, mes y el año.</t>
+  </si>
+  <si>
+    <t>Este es calculado o lo pone el barbero?</t>
+  </si>
+  <si>
+    <t>Tengo pensado que este sea de tipo texto, su valor por defecto sería el vacío y no sería permitido</t>
+  </si>
+  <si>
+    <t>Representa la fecha y la hora en el que se va a realizar la cita al cliente. Su valor por defecto es 01/01/1000 00:00 y no es permitido</t>
+  </si>
+  <si>
+    <t>Representa cuanto valía el servicio en el momento exacto en que se agendó la cita, se guarda aparte del precio del catalogo por si el precio de ese servicio cambia después, las citas ya registradas no se vean afectadas. Debe de ser mayor a cero, su valor por defecto es el 0 y no es permitido</t>
+  </si>
+  <si>
+    <t>Sera que este es calculado o lo pone le barbero</t>
+  </si>
+  <si>
+    <t>Sera que este es calculado o lo pone el barbero</t>
   </si>
 </sst>
 </file>
@@ -713,7 +792,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="10">
+  <fills count="16">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -768,6 +847,42 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="3" tint="0.249977111117893"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF3F3F"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF7030A0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="-0.249977111117893"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -797,7 +912,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="62">
+  <cellXfs count="85">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -848,9 +963,6 @@
     <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
@@ -898,9 +1010,6 @@
     <xf numFmtId="18" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="18" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -915,9 +1024,6 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -957,7 +1063,67 @@
     <xf numFmtId="0" fontId="5" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="15" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="15" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -967,6 +1133,11 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <mruColors>
+      <color rgb="FFFF3F3F"/>
+    </mruColors>
+  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -1359,15 +1530,37 @@
 </a:theme>
 </file>
 
+<file path=xl/webextensions/taskpanes.xml><?xml version="1.0" encoding="utf-8"?>
+<wetp:taskpanes xmlns:wetp="http://schemas.microsoft.com/office/webextensions/taskpanes/2010/11">
+  <wetp:taskpane dockstate="right" visibility="0" width="438" row="0">
+    <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </wetp:taskpane>
+</wetp:taskpanes>
+</file>
+
+<file path=xl/webextensions/webextension1.xml><?xml version="1.0" encoding="utf-8"?>
+<we:webextension xmlns:we="http://schemas.microsoft.com/office/webextensions/webextension/2010/11" id="{E2216492-8388-41E0-BF9F-A7DC14E86A70}">
+  <we:reference id="wa200010725" version="1.0.0.1" store="es-ES" storeType="OMEX"/>
+  <we:alternateReferences>
+    <we:reference id="WA200010725" version="1.0.0.1" store="" storeType="OMEX"/>
+  </we:alternateReferences>
+  <we:properties>
+    <we:property name="claude.fileId" value="&quot;a357427e-8d6b-4b8d-a56c-647f29a36447&quot;"/>
+  </we:properties>
+  <we:bindings/>
+  <we:snapshot xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
+</we:webextension>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D2495362-94CF-4E08-8433-6F4780C6375E}">
   <dimension ref="A1:AD50"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="26.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="26.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A1" s="5" t="s">
         <v>39</v>
       </c>
@@ -1401,7 +1594,7 @@
       <c r="AC1" s="1"/>
       <c r="AD1" s="1"/>
     </row>
-    <row r="2" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
@@ -1433,7 +1626,7 @@
       <c r="AC2" s="1"/>
       <c r="AD2" s="1"/>
     </row>
-    <row r="3" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A3" s="1"/>
       <c r="B3" s="1"/>
       <c r="C3" s="1"/>
@@ -1465,7 +1658,7 @@
       <c r="AC3" s="1"/>
       <c r="AD3" s="1"/>
     </row>
-    <row r="4" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:30" x14ac:dyDescent="0.3">
       <c r="B4" s="1"/>
       <c r="C4" s="1"/>
       <c r="D4" s="1"/>
@@ -1496,7 +1689,7 @@
       <c r="AC4" s="1"/>
       <c r="AD4" s="1"/>
     </row>
-    <row r="5" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A5" s="1"/>
       <c r="B5" s="1"/>
       <c r="C5" s="1"/>
@@ -1528,7 +1721,7 @@
       <c r="AC5" s="1"/>
       <c r="AD5" s="1"/>
     </row>
-    <row r="6" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A6" s="1"/>
       <c r="B6" s="1"/>
       <c r="D6" s="1"/>
@@ -1559,7 +1752,7 @@
       <c r="AC6" s="1"/>
       <c r="AD6" s="1"/>
     </row>
-    <row r="7" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A7" s="1"/>
       <c r="B7" s="1"/>
       <c r="C7" s="1"/>
@@ -1591,7 +1784,7 @@
       <c r="AC7" s="1"/>
       <c r="AD7" s="1"/>
     </row>
-    <row r="8" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A8" s="1"/>
       <c r="B8" s="1"/>
       <c r="C8" s="1"/>
@@ -1623,7 +1816,7 @@
       <c r="AC8" s="1"/>
       <c r="AD8" s="1"/>
     </row>
-    <row r="9" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A9" s="1"/>
       <c r="B9" s="1"/>
       <c r="C9" s="1"/>
@@ -1655,7 +1848,7 @@
       <c r="AC9" s="1"/>
       <c r="AD9" s="1"/>
     </row>
-    <row r="10" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A10" s="1"/>
       <c r="B10" s="1"/>
       <c r="C10" s="1"/>
@@ -1687,7 +1880,7 @@
       <c r="AC10" s="1"/>
       <c r="AD10" s="1"/>
     </row>
-    <row r="11" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A11" s="1"/>
       <c r="B11" s="1"/>
       <c r="C11" s="1"/>
@@ -1719,7 +1912,7 @@
       <c r="AC11" s="1"/>
       <c r="AD11" s="1"/>
     </row>
-    <row r="12" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A12" s="1"/>
       <c r="B12" s="1"/>
       <c r="C12" s="1"/>
@@ -1751,7 +1944,7 @@
       <c r="AC12" s="1"/>
       <c r="AD12" s="1"/>
     </row>
-    <row r="13" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A13" s="1"/>
       <c r="B13" s="1"/>
       <c r="C13" s="1"/>
@@ -1783,7 +1976,7 @@
       <c r="AC13" s="1"/>
       <c r="AD13" s="1"/>
     </row>
-    <row r="14" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A14" s="1"/>
       <c r="B14" s="1"/>
       <c r="C14" s="1"/>
@@ -1815,7 +2008,7 @@
       <c r="AC14" s="1"/>
       <c r="AD14" s="1"/>
     </row>
-    <row r="15" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A15" s="1"/>
       <c r="B15" s="1"/>
       <c r="C15" s="1"/>
@@ -1847,7 +2040,7 @@
       <c r="AC15" s="1"/>
       <c r="AD15" s="1"/>
     </row>
-    <row r="16" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A16" s="1"/>
       <c r="B16" s="1"/>
       <c r="C16" s="1"/>
@@ -1879,7 +2072,7 @@
       <c r="AC16" s="1"/>
       <c r="AD16" s="1"/>
     </row>
-    <row r="17" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A17" s="1"/>
       <c r="B17" s="1"/>
       <c r="C17" s="1"/>
@@ -1911,7 +2104,7 @@
       <c r="AC17" s="1"/>
       <c r="AD17" s="1"/>
     </row>
-    <row r="18" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A18" s="1"/>
       <c r="B18" s="1"/>
       <c r="C18" s="1"/>
@@ -1943,7 +2136,7 @@
       <c r="AC18" s="1"/>
       <c r="AD18" s="1"/>
     </row>
-    <row r="19" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A19" s="1"/>
       <c r="B19" s="1"/>
       <c r="C19" s="1"/>
@@ -1975,7 +2168,7 @@
       <c r="AC19" s="1"/>
       <c r="AD19" s="1"/>
     </row>
-    <row r="20" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A20" s="1"/>
       <c r="B20" s="1"/>
       <c r="C20" s="1"/>
@@ -2007,7 +2200,7 @@
       <c r="AC20" s="1"/>
       <c r="AD20" s="1"/>
     </row>
-    <row r="21" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A21" s="1"/>
       <c r="B21" s="1"/>
       <c r="C21" s="1"/>
@@ -2039,7 +2232,7 @@
       <c r="AC21" s="1"/>
       <c r="AD21" s="1"/>
     </row>
-    <row r="22" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A22" s="1"/>
       <c r="B22" s="1"/>
       <c r="C22" s="1"/>
@@ -2071,7 +2264,7 @@
       <c r="AC22" s="1"/>
       <c r="AD22" s="1"/>
     </row>
-    <row r="23" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A23" s="1"/>
       <c r="B23" s="1"/>
       <c r="C23" s="1"/>
@@ -2103,7 +2296,7 @@
       <c r="AC23" s="1"/>
       <c r="AD23" s="1"/>
     </row>
-    <row r="24" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A24" s="1"/>
       <c r="B24" s="1"/>
       <c r="C24" s="1"/>
@@ -2135,7 +2328,7 @@
       <c r="AC24" s="1"/>
       <c r="AD24" s="1"/>
     </row>
-    <row r="25" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A25" s="1"/>
       <c r="B25" s="1"/>
       <c r="C25" s="1"/>
@@ -2167,7 +2360,7 @@
       <c r="AC25" s="1"/>
       <c r="AD25" s="1"/>
     </row>
-    <row r="26" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A26" s="1"/>
       <c r="B26" s="1"/>
       <c r="C26" s="1"/>
@@ -2199,7 +2392,7 @@
       <c r="AC26" s="1"/>
       <c r="AD26" s="1"/>
     </row>
-    <row r="27" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A27" s="1"/>
       <c r="B27" s="1"/>
       <c r="C27" s="1"/>
@@ -2231,7 +2424,7 @@
       <c r="AC27" s="1"/>
       <c r="AD27" s="1"/>
     </row>
-    <row r="28" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A28" s="1"/>
       <c r="B28" s="1"/>
       <c r="C28" s="1"/>
@@ -2263,7 +2456,7 @@
       <c r="AC28" s="1"/>
       <c r="AD28" s="1"/>
     </row>
-    <row r="29" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A29" s="1"/>
       <c r="B29" s="1"/>
       <c r="C29" s="1"/>
@@ -2295,7 +2488,7 @@
       <c r="AC29" s="1"/>
       <c r="AD29" s="1"/>
     </row>
-    <row r="30" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A30" s="1"/>
       <c r="B30" s="1"/>
       <c r="C30" s="1"/>
@@ -2327,7 +2520,7 @@
       <c r="AC30" s="1"/>
       <c r="AD30" s="1"/>
     </row>
-    <row r="31" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A31" s="1"/>
       <c r="B31" s="1"/>
       <c r="C31" s="1"/>
@@ -2359,7 +2552,7 @@
       <c r="AC31" s="1"/>
       <c r="AD31" s="1"/>
     </row>
-    <row r="32" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A32" s="1"/>
       <c r="B32" s="1"/>
       <c r="C32" s="1"/>
@@ -2391,7 +2584,7 @@
       <c r="AC32" s="1"/>
       <c r="AD32" s="1"/>
     </row>
-    <row r="33" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A33" s="1"/>
       <c r="B33" s="1"/>
       <c r="C33" s="1"/>
@@ -2423,7 +2616,7 @@
       <c r="AC33" s="1"/>
       <c r="AD33" s="1"/>
     </row>
-    <row r="34" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A34" s="1"/>
       <c r="B34" s="1"/>
       <c r="C34" s="1"/>
@@ -2455,7 +2648,7 @@
       <c r="AC34" s="1"/>
       <c r="AD34" s="1"/>
     </row>
-    <row r="35" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A35" s="1"/>
       <c r="B35" s="1"/>
       <c r="C35" s="1"/>
@@ -2487,7 +2680,7 @@
       <c r="AC35" s="1"/>
       <c r="AD35" s="1"/>
     </row>
-    <row r="36" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A36" s="1"/>
       <c r="B36" s="1"/>
       <c r="C36" s="1"/>
@@ -2519,7 +2712,7 @@
       <c r="AC36" s="1"/>
       <c r="AD36" s="1"/>
     </row>
-    <row r="37" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A37" s="1"/>
       <c r="B37" s="1"/>
       <c r="C37" s="1"/>
@@ -2551,7 +2744,7 @@
       <c r="AC37" s="1"/>
       <c r="AD37" s="1"/>
     </row>
-    <row r="38" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A38" s="1"/>
       <c r="B38" s="1"/>
       <c r="C38" s="1"/>
@@ -2583,7 +2776,7 @@
       <c r="AC38" s="1"/>
       <c r="AD38" s="1"/>
     </row>
-    <row r="39" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A39" s="1"/>
       <c r="B39" s="1"/>
       <c r="C39" s="1"/>
@@ -2615,7 +2808,7 @@
       <c r="AC39" s="1"/>
       <c r="AD39" s="1"/>
     </row>
-    <row r="40" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A40" s="1"/>
       <c r="B40" s="1"/>
       <c r="C40" s="1"/>
@@ -2647,7 +2840,7 @@
       <c r="AC40" s="1"/>
       <c r="AD40" s="1"/>
     </row>
-    <row r="41" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A41" s="1"/>
       <c r="B41" s="1"/>
       <c r="C41" s="1"/>
@@ -2679,7 +2872,7 @@
       <c r="AC41" s="1"/>
       <c r="AD41" s="1"/>
     </row>
-    <row r="42" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A42" s="1"/>
       <c r="B42" s="1"/>
       <c r="C42" s="1"/>
@@ -2711,7 +2904,7 @@
       <c r="AC42" s="1"/>
       <c r="AD42" s="1"/>
     </row>
-    <row r="43" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A43" s="1"/>
       <c r="B43" s="1"/>
       <c r="C43" s="1"/>
@@ -2743,7 +2936,7 @@
       <c r="AC43" s="1"/>
       <c r="AD43" s="1"/>
     </row>
-    <row r="44" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A44" s="1"/>
       <c r="B44" s="1"/>
       <c r="C44" s="1"/>
@@ -2775,7 +2968,7 @@
       <c r="AC44" s="1"/>
       <c r="AD44" s="1"/>
     </row>
-    <row r="45" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A45" s="1"/>
       <c r="B45" s="1"/>
       <c r="C45" s="1"/>
@@ -2807,7 +3000,7 @@
       <c r="AC45" s="1"/>
       <c r="AD45" s="1"/>
     </row>
-    <row r="46" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A46" s="1"/>
       <c r="B46" s="1"/>
       <c r="C46" s="1"/>
@@ -2839,7 +3032,7 @@
       <c r="AC46" s="1"/>
       <c r="AD46" s="1"/>
     </row>
-    <row r="47" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A47" s="1"/>
       <c r="B47" s="1"/>
       <c r="C47" s="1"/>
@@ -2871,7 +3064,7 @@
       <c r="AC47" s="1"/>
       <c r="AD47" s="1"/>
     </row>
-    <row r="48" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A48" s="1"/>
       <c r="B48" s="1"/>
       <c r="C48" s="1"/>
@@ -2903,7 +3096,7 @@
       <c r="AC48" s="1"/>
       <c r="AD48" s="1"/>
     </row>
-    <row r="49" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A49" s="1"/>
       <c r="B49" s="1"/>
       <c r="C49" s="1"/>
@@ -2935,7 +3128,7 @@
       <c r="AC49" s="1"/>
       <c r="AD49" s="1"/>
     </row>
-    <row r="50" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A50" s="1"/>
       <c r="B50" s="1"/>
       <c r="C50" s="1"/>
@@ -2978,17 +3171,173 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C828B98D-AAA9-4184-8373-FE2E421AAE23}">
+  <dimension ref="A1:E11"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="27" customWidth="1"/>
+    <col min="2" max="2" width="28.88671875" customWidth="1"/>
+    <col min="3" max="3" width="41" customWidth="1"/>
+    <col min="4" max="4" width="36.109375" customWidth="1"/>
+    <col min="5" max="5" width="26.88671875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A1" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="18" t="s">
+        <v>20</v>
+      </c>
+      <c r="B2" s="18" t="s">
+        <v>58</v>
+      </c>
+      <c r="C2" s="31" t="s">
+        <v>60</v>
+      </c>
+      <c r="D2" s="31" t="s">
+        <v>127</v>
+      </c>
+      <c r="E2" s="31" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A3" s="14" t="s">
+        <v>31</v>
+      </c>
+      <c r="B3" s="32" t="s">
+        <v>61</v>
+      </c>
+      <c r="C3" s="83" t="s">
+        <v>25</v>
+      </c>
+      <c r="D3" s="44" t="s">
+        <v>57</v>
+      </c>
+      <c r="E3" s="29" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A4" s="12">
+        <v>1</v>
+      </c>
+      <c r="B4" s="11">
+        <f>Cliente_D!G4</f>
+        <v>3234528921</v>
+      </c>
+      <c r="C4" s="33">
+        <v>45255</v>
+      </c>
+      <c r="D4" s="12" t="s">
+        <v>50</v>
+      </c>
+      <c r="E4" s="12" t="str">
+        <f>_xlfn.CONCAT(B4,"-",TEXT(C4,"dd/mm/yyyy"))</f>
+        <v>3234528921-25/11/2023</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A5" s="12">
+        <v>2</v>
+      </c>
+      <c r="B5" s="11">
+        <f>Cliente_D!G5</f>
+        <v>3161657782</v>
+      </c>
+      <c r="C5" s="33">
+        <v>45372</v>
+      </c>
+      <c r="D5" s="12" t="s">
+        <v>50</v>
+      </c>
+      <c r="E5" s="12" t="str">
+        <f t="shared" ref="E5:E7" si="0">_xlfn.CONCAT(B5,"-",TEXT(C5,"dd/mm/yyyy"))</f>
+        <v>3161657782-21/03/2024</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A6" s="12">
+        <v>3</v>
+      </c>
+      <c r="B6" s="11">
+        <f>Cliente_D!G6</f>
+        <v>3119884321</v>
+      </c>
+      <c r="C6" s="33">
+        <v>45556</v>
+      </c>
+      <c r="D6" s="12" t="s">
+        <v>49</v>
+      </c>
+      <c r="E6" s="12" t="str">
+        <f t="shared" si="0"/>
+        <v>3119884321-21/09/2024</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A7" s="12">
+        <v>4</v>
+      </c>
+      <c r="B7" s="11">
+        <f>Cliente_D!G7</f>
+        <v>4127359182</v>
+      </c>
+      <c r="C7" s="33">
+        <v>46002</v>
+      </c>
+      <c r="D7" s="12" t="s">
+        <v>49</v>
+      </c>
+      <c r="E7" s="12" t="str">
+        <f t="shared" si="0"/>
+        <v>4127359182-11/12/2025</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="C8" s="30"/>
+      <c r="D8" s="30"/>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="C9" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="C11" s="45"/>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A1" location="'Modelo de Dominio'!A1" display="&lt;&lt;&lt;&lt; Ir al modulo de dominio" xr:uid="{F755F618-0A40-4479-913F-8F6060E94F5B}"/>
+    <hyperlink ref="B1" location="'Objetos de Dominio'!A1" display="&lt;&lt;&lt;&lt; Ir a objetos de dominio" xr:uid="{C5748D80-5E29-4CD8-BA51-198180E61202}"/>
+    <hyperlink ref="B3" location="Cliente_D!A1" display="cliente" xr:uid="{F7C47FD3-2FEB-4E40-8CE8-9FEC66E905E0}"/>
+    <hyperlink ref="B4" location="Cliente_D!A4" display="Cliente_D!A4" xr:uid="{7F6CACFC-57C0-447E-811A-802403EBA0AC}"/>
+    <hyperlink ref="B5" location="Cliente_D!A5" display="Cliente_D!A5" xr:uid="{EE87A799-0DAD-412E-8BF4-24089411596B}"/>
+    <hyperlink ref="B6" location="Cliente_D!A6" display="Cliente_D!A6" xr:uid="{D95F6EBA-51E7-42CB-9EFD-6676C5924513}"/>
+    <hyperlink ref="B7" location="Cliente_D!A7" display="Cliente_D!A7" xr:uid="{9BA1680E-A8A5-4CE9-866D-EC3B5A4F5B91}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A24A074A-5C83-448D-978C-7C1005CE378E}">
   <dimension ref="A1:D7"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="29.140625" customWidth="1"/>
+    <col min="1" max="1" width="29.109375" customWidth="1"/>
     <col min="2" max="2" width="30" customWidth="1"/>
-    <col min="3" max="3" width="41.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="61.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="41.88671875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="61.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="5" t="s">
         <v>32</v>
       </c>
@@ -2996,35 +3345,35 @@
         <v>33</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" ht="36.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="18" t="s">
         <v>20</v>
       </c>
-      <c r="B2" s="35" t="s">
+      <c r="B2" s="34" t="s">
+        <v>63</v>
+      </c>
+      <c r="C2" s="31" t="s">
         <v>64</v>
       </c>
-      <c r="C2" s="32" t="s">
-        <v>65</v>
-      </c>
-      <c r="D2" s="45" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D2" s="43" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" s="14" t="s">
         <v>31</v>
       </c>
-      <c r="B3" s="33" t="s">
+      <c r="B3" s="32" t="s">
         <v>40</v>
       </c>
-      <c r="C3" s="33" t="s">
+      <c r="C3" s="32" t="s">
         <v>41</v>
       </c>
-      <c r="D3" s="37" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D3" s="36" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" s="12">
         <v>1</v>
       </c>
@@ -3041,7 +3390,7 @@
         <v>Juan García-Motilada</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" s="12">
         <v>2</v>
       </c>
@@ -3058,7 +3407,7 @@
         <v>Juan Ortiz-Corte de barba</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" s="12">
         <v>3</v>
       </c>
@@ -3075,7 +3424,7 @@
         <v>Carlos Arbeladez-Perfilada de barba</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" s="12">
         <v>4</v>
       </c>
@@ -3112,17 +3461,17 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2921A3C4-B96A-49A7-8353-9FD37D2F2B74}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
-    <col min="2" max="2" width="42.28515625" customWidth="1"/>
-    <col min="3" max="3" width="37.42578125" customWidth="1"/>
+    <col min="2" max="2" width="42.33203125" customWidth="1"/>
+    <col min="3" max="3" width="37.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="5" t="s">
         <v>32</v>
       </c>
@@ -3130,29 +3479,29 @@
         <v>33</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="28.5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" ht="30" x14ac:dyDescent="0.3">
       <c r="A2" s="18" t="s">
         <v>20</v>
       </c>
       <c r="B2" s="18" t="s">
-        <v>131</v>
+        <v>126</v>
       </c>
       <c r="C2" s="19" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" s="14" t="s">
         <v>31</v>
       </c>
-      <c r="B3" s="33" t="s">
+      <c r="B3" s="32" t="s">
         <v>40</v>
       </c>
-      <c r="C3" s="30" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C3" s="29" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" s="12">
         <v>1</v>
       </c>
@@ -3165,7 +3514,7 @@
         <v>Juan García</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" s="12">
         <v>2</v>
       </c>
@@ -3178,7 +3527,7 @@
         <v>Juan Ortiz</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" s="12">
         <v>3</v>
       </c>
@@ -3191,7 +3540,7 @@
         <v>Carlos Arbeladez</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" s="12">
         <v>4</v>
       </c>
@@ -3219,20 +3568,20 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5CFE76D0-FBB4-4C81-85CC-F644057A8847}">
-  <dimension ref="A1:F7"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:F10"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="27" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="37.140625" customWidth="1"/>
+    <col min="2" max="2" width="37.109375" customWidth="1"/>
     <col min="3" max="3" width="28" customWidth="1"/>
-    <col min="4" max="4" width="18.7109375" customWidth="1"/>
-    <col min="5" max="5" width="31.7109375" customWidth="1"/>
-    <col min="6" max="6" width="37.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="18.6640625" customWidth="1"/>
+    <col min="5" max="5" width="31.6640625" customWidth="1"/>
+    <col min="6" max="6" width="37.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" s="5" t="s">
         <v>32</v>
       </c>
@@ -3240,61 +3589,61 @@
         <v>33</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="40.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" ht="40.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="19" t="s">
         <v>20</v>
       </c>
       <c r="B2" s="19" t="s">
+        <v>88</v>
+      </c>
+      <c r="C2" s="19" t="s">
+        <v>176</v>
+      </c>
+      <c r="D2" s="19" t="s">
+        <v>89</v>
+      </c>
+      <c r="E2" s="19" t="s">
         <v>90</v>
       </c>
-      <c r="C2" s="19" t="s">
+      <c r="F2" s="19" t="s">
         <v>91</v>
       </c>
-      <c r="D2" s="19" t="s">
-        <v>92</v>
-      </c>
-      <c r="E2" s="19" t="s">
-        <v>93</v>
-      </c>
-      <c r="F2" s="19" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" s="14" t="s">
         <v>31</v>
       </c>
-      <c r="B3" s="33" t="s">
-        <v>63</v>
-      </c>
-      <c r="C3" s="40" t="s">
-        <v>79</v>
-      </c>
-      <c r="D3" s="13" t="s">
-        <v>66</v>
-      </c>
-      <c r="E3" s="13" t="s">
-        <v>89</v>
-      </c>
-      <c r="F3" s="30" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B3" s="32" t="s">
+        <v>62</v>
+      </c>
+      <c r="C3" s="59" t="s">
+        <v>77</v>
+      </c>
+      <c r="D3" s="80" t="s">
+        <v>65</v>
+      </c>
+      <c r="E3" s="80" t="s">
+        <v>87</v>
+      </c>
+      <c r="F3" s="29" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" s="12">
         <v>1</v>
       </c>
-      <c r="B4" s="53" t="str">
+      <c r="B4" s="50" t="str">
         <f>Agenda_D!C4</f>
         <v>Juan García</v>
       </c>
-      <c r="C4" s="39" t="s">
-        <v>82</v>
-      </c>
-      <c r="D4" s="39">
+      <c r="C4" s="38" t="s">
+        <v>80</v>
+      </c>
+      <c r="D4" s="38">
         <v>0.41666666666666669</v>
       </c>
-      <c r="E4" s="39">
+      <c r="E4" s="38">
         <v>0.66666666666666663</v>
       </c>
       <c r="F4" s="12" t="str">
@@ -3302,21 +3651,21 @@
         <v>Juan García-Lunes-10-16</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" s="12">
         <v>2</v>
       </c>
-      <c r="B5" s="53" t="str">
+      <c r="B5" s="50" t="str">
         <f>Agenda_D!C5</f>
         <v>Juan Ortiz</v>
       </c>
       <c r="C5" s="12" t="s">
-        <v>83</v>
-      </c>
-      <c r="D5" s="39">
+        <v>81</v>
+      </c>
+      <c r="D5" s="38">
         <v>0.375</v>
       </c>
-      <c r="E5" s="39">
+      <c r="E5" s="38">
         <v>0.625</v>
       </c>
       <c r="F5" s="12" t="str">
@@ -3324,21 +3673,21 @@
         <v>Juan Ortiz-Martes-09-15</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" s="12">
         <v>3</v>
       </c>
-      <c r="B6" s="53" t="str">
+      <c r="B6" s="50" t="str">
         <f>Agenda_D!C6</f>
         <v>Carlos Arbeladez</v>
       </c>
       <c r="C6" s="12" t="s">
-        <v>85</v>
-      </c>
-      <c r="D6" s="39">
+        <v>83</v>
+      </c>
+      <c r="D6" s="38">
         <v>0.54166666666666663</v>
       </c>
-      <c r="E6" s="39">
+      <c r="E6" s="38">
         <v>0.79166666666666663</v>
       </c>
       <c r="F6" s="12" t="str">
@@ -3346,26 +3695,31 @@
         <v>Carlos Arbeladez-Jueves-13-19</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7" s="12">
         <v>4</v>
       </c>
-      <c r="B7" s="53" t="str">
+      <c r="B7" s="50" t="str">
         <f>Agenda_D!C7</f>
         <v>Andres Ramirez</v>
       </c>
       <c r="C7" s="12" t="s">
-        <v>87</v>
-      </c>
-      <c r="D7" s="39">
+        <v>85</v>
+      </c>
+      <c r="D7" s="38">
         <v>0.33333333333333331</v>
       </c>
-      <c r="E7" s="39">
+      <c r="E7" s="38">
         <v>0.58333333333333337</v>
       </c>
       <c r="F7" s="12" t="str">
         <f t="shared" si="0"/>
         <v>Andres Ramirez-Sábado-08-14</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="C10" s="60" t="s">
+        <v>177</v>
       </c>
     </row>
   </sheetData>
@@ -3383,22 +3737,22 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1429879F-6697-4F1F-AF5D-52C4860B7B3E}">
   <dimension ref="A1:H15"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="28" customWidth="1"/>
-    <col min="2" max="2" width="26.5703125" customWidth="1"/>
-    <col min="3" max="3" width="30.42578125" customWidth="1"/>
-    <col min="4" max="4" width="27.5703125" customWidth="1"/>
-    <col min="5" max="5" width="36.5703125" customWidth="1"/>
-    <col min="6" max="6" width="60.28515625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="39.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="26.5546875" customWidth="1"/>
+    <col min="3" max="3" width="30.44140625" customWidth="1"/>
+    <col min="4" max="4" width="27.5546875" customWidth="1"/>
+    <col min="5" max="5" width="36.5546875" customWidth="1"/>
+    <col min="6" max="6" width="60.33203125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="39.33203125" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="22" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A1" s="5" t="s">
         <v>32</v>
       </c>
@@ -3406,53 +3760,53 @@
         <v>33</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" ht="36.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="18" t="s">
         <v>20</v>
       </c>
       <c r="B2" s="18" t="s">
-        <v>67</v>
-      </c>
-      <c r="C2" s="32" t="s">
-        <v>151</v>
-      </c>
-      <c r="D2" s="32" t="s">
-        <v>143</v>
-      </c>
-      <c r="E2" s="32" t="s">
-        <v>148</v>
-      </c>
-      <c r="F2" s="32" t="s">
-        <v>152</v>
-      </c>
-      <c r="G2" s="32" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+        <v>66</v>
+      </c>
+      <c r="C2" s="31" t="s">
+        <v>145</v>
+      </c>
+      <c r="D2" s="31" t="s">
+        <v>216</v>
+      </c>
+      <c r="E2" s="31" t="s">
+        <v>142</v>
+      </c>
+      <c r="F2" s="31" t="s">
+        <v>146</v>
+      </c>
+      <c r="G2" s="31" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" s="14" t="s">
         <v>31</v>
       </c>
-      <c r="B3" s="33" t="s">
+      <c r="B3" s="32" t="s">
         <v>44</v>
       </c>
-      <c r="C3" s="33" t="s">
-        <v>63</v>
-      </c>
-      <c r="D3" s="13" t="s">
-        <v>142</v>
-      </c>
-      <c r="E3" s="47" t="s">
-        <v>89</v>
-      </c>
-      <c r="F3" s="13" t="s">
+      <c r="C3" s="32" t="s">
+        <v>62</v>
+      </c>
+      <c r="D3" s="84" t="s">
+        <v>137</v>
+      </c>
+      <c r="E3" s="44" t="s">
+        <v>87</v>
+      </c>
+      <c r="F3" s="58" t="s">
         <v>26</v>
       </c>
-      <c r="G3" s="30" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G3" s="29" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A4" s="12">
         <v>1</v>
       </c>
@@ -3464,21 +3818,21 @@
         <f>Agenda_D!C4</f>
         <v>Juan García</v>
       </c>
-      <c r="D4" s="55">
+      <c r="D4" s="52">
         <v>46295.416666666664</v>
       </c>
-      <c r="E4" s="39">
+      <c r="E4" s="38">
         <v>0.44791666666666669</v>
       </c>
       <c r="F4" s="12" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="G4" s="12" t="str">
         <f>_xlfn.CONCAT(C4,"-",TEXT(D4,"dd/mm/yyyy/hh:mm"))</f>
         <v>Juan García-30/09/2026/10:00</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A5" s="12">
         <v>2</v>
       </c>
@@ -3490,21 +3844,21 @@
         <f>Agenda_D!C5</f>
         <v>Juan Ortiz</v>
       </c>
-      <c r="D5" s="55">
+      <c r="D5" s="52">
         <v>45983.458333333336</v>
       </c>
-      <c r="E5" s="39">
+      <c r="E5" s="38">
         <v>0.48958333333333331</v>
       </c>
       <c r="F5" s="12" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="G5" s="12" t="str">
         <f t="shared" ref="G5:G8" si="0">_xlfn.CONCAT(C5,"-",TEXT(D5,"dd/mm/yyyy/hh:mm"))</f>
         <v>Juan Ortiz-22/11/2025/11:00</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A6" s="12">
         <v>3</v>
       </c>
@@ -3516,21 +3870,21 @@
         <f>Agenda_D!C6</f>
         <v>Carlos Arbeladez</v>
       </c>
-      <c r="D6" s="55">
+      <c r="D6" s="52">
         <v>45514.583333333336</v>
       </c>
-      <c r="E6" s="39">
+      <c r="E6" s="38">
         <v>0.59375</v>
       </c>
       <c r="F6" s="12" t="s">
-        <v>145</v>
+        <v>139</v>
       </c>
       <c r="G6" s="12" t="str">
         <f t="shared" si="0"/>
         <v>Carlos Arbeladez-10/08/2024/14:00</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A7" s="12">
         <v>4</v>
       </c>
@@ -3542,21 +3896,21 @@
         <f>Agenda_D!C7</f>
         <v>Andres Ramirez</v>
       </c>
-      <c r="D7" s="55">
+      <c r="D7" s="52">
         <v>46289.541666666664</v>
       </c>
-      <c r="E7" s="39">
+      <c r="E7" s="38">
         <v>0.5625</v>
       </c>
       <c r="F7" s="12" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="G7" s="12" t="str">
         <f t="shared" si="0"/>
         <v>Andres Ramirez-24/09/2026/13:00</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A8" s="12">
         <v>5</v>
       </c>
@@ -3568,35 +3922,40 @@
         <f>Agenda_D!C6</f>
         <v>Carlos Arbeladez</v>
       </c>
-      <c r="D8" s="55">
+      <c r="D8" s="52">
         <v>46240.75</v>
       </c>
-      <c r="E8" s="39">
+      <c r="E8" s="38">
         <v>0.75694444444444442</v>
       </c>
       <c r="F8" s="12" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="G8" s="12" t="str">
         <f t="shared" si="0"/>
         <v>Carlos Arbeladez-06/08/2026/18:00</v>
       </c>
-      <c r="H8" s="52"/>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="H10" s="54"/>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="D12" s="56"/>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="D13" s="56"/>
-    </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="D14" s="56"/>
-    </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="D15" s="56"/>
+      <c r="H8" s="49"/>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="H10" s="51"/>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="F11" s="60" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="D12" s="53"/>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="D13" s="53"/>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="D14" s="53"/>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="D15" s="53"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -3621,20 +3980,20 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{766573FB-AAA2-4254-B83C-7C7505540365}">
   <dimension ref="A1:G7"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="26.7109375" customWidth="1"/>
-    <col min="2" max="2" width="38.5703125" customWidth="1"/>
-    <col min="3" max="3" width="39.28515625" bestFit="1" customWidth="1"/>
-    <col min="4" max="5" width="39.7109375" customWidth="1"/>
-    <col min="6" max="6" width="34.28515625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="39.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="26.6640625" customWidth="1"/>
+    <col min="2" max="2" width="38.5546875" customWidth="1"/>
+    <col min="3" max="3" width="39.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="39.6640625" customWidth="1"/>
+    <col min="6" max="6" width="34.33203125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="39.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" s="5" t="s">
         <v>32</v>
       </c>
@@ -3642,53 +4001,53 @@
         <v>33</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" ht="31.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="18" t="s">
         <v>20</v>
       </c>
       <c r="B2" s="18" t="s">
+        <v>96</v>
+      </c>
+      <c r="C2" s="31" t="s">
+        <v>97</v>
+      </c>
+      <c r="D2" s="31" t="s">
+        <v>140</v>
+      </c>
+      <c r="E2" s="31" t="s">
+        <v>148</v>
+      </c>
+      <c r="F2" s="31" t="s">
+        <v>98</v>
+      </c>
+      <c r="G2" s="31" t="s">
         <v>99</v>
       </c>
-      <c r="C2" s="32" t="s">
-        <v>100</v>
-      </c>
-      <c r="D2" s="32" t="s">
-        <v>146</v>
-      </c>
-      <c r="E2" s="32" t="s">
-        <v>154</v>
-      </c>
-      <c r="F2" s="32" t="s">
-        <v>101</v>
-      </c>
-      <c r="G2" s="32" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" s="14" t="s">
         <v>31</v>
       </c>
-      <c r="B3" s="33" t="s">
+      <c r="B3" s="32" t="s">
         <v>44</v>
       </c>
-      <c r="C3" s="33" t="s">
-        <v>98</v>
-      </c>
-      <c r="D3" s="36" t="s">
+      <c r="C3" s="32" t="s">
+        <v>95</v>
+      </c>
+      <c r="D3" s="35" t="s">
         <v>27</v>
       </c>
-      <c r="E3" s="60" t="s">
-        <v>153</v>
-      </c>
-      <c r="F3" s="47" t="s">
+      <c r="E3" s="57" t="s">
+        <v>147</v>
+      </c>
+      <c r="F3" s="44" t="s">
         <v>28</v>
       </c>
-      <c r="G3" s="30" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G3" s="29" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" s="12">
         <v>1</v>
       </c>
@@ -3705,17 +4064,17 @@
         <v>10000</v>
       </c>
       <c r="E4" s="12" t="s">
-        <v>145</v>
+        <v>139</v>
       </c>
       <c r="F4" s="12" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="G4" s="12" t="str">
         <f>C4</f>
         <v>Carlos Arbeladez-10/08/2024/14:00</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" s="12">
         <v>2</v>
       </c>
@@ -3732,17 +4091,17 @@
         <v>35000</v>
       </c>
       <c r="E5" s="12" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="F5" s="12" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="G5" s="12" t="str">
         <f>C5</f>
         <v>Andres Ramirez-24/09/2026/13:00</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" s="10"/>
       <c r="B6" s="10"/>
       <c r="C6" s="10"/>
@@ -3751,7 +4110,7 @@
       <c r="F6" s="10"/>
       <c r="G6" s="10"/>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" s="10"/>
       <c r="B7" s="10"/>
       <c r="C7" s="10"/>
@@ -3775,20 +4134,20 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F470C5A4-8D15-43DA-95FC-91C9614E5EEA}">
-  <dimension ref="A1:F8"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:F10"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="26.42578125" customWidth="1"/>
-    <col min="2" max="2" width="39.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="21.85546875" customWidth="1"/>
-    <col min="4" max="4" width="41.85546875" customWidth="1"/>
-    <col min="5" max="5" width="32.140625" customWidth="1"/>
-    <col min="6" max="6" width="55.85546875" customWidth="1"/>
+    <col min="1" max="1" width="26.44140625" customWidth="1"/>
+    <col min="2" max="2" width="39.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="21.88671875" customWidth="1"/>
+    <col min="4" max="4" width="41.88671875" customWidth="1"/>
+    <col min="5" max="5" width="32.109375" customWidth="1"/>
+    <col min="6" max="6" width="55.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" s="5" t="s">
         <v>32</v>
       </c>
@@ -3796,47 +4155,47 @@
         <v>33</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="33" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" ht="33" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="18" t="s">
         <v>20</v>
       </c>
       <c r="B2" s="18" t="s">
+        <v>100</v>
+      </c>
+      <c r="C2" s="31" t="s">
+        <v>101</v>
+      </c>
+      <c r="D2" s="31" t="s">
+        <v>217</v>
+      </c>
+      <c r="E2" s="31" t="s">
+        <v>102</v>
+      </c>
+      <c r="F2" s="31" t="s">
         <v>103</v>
       </c>
-      <c r="C2" s="32" t="s">
-        <v>104</v>
-      </c>
-      <c r="D2" s="32" t="s">
-        <v>105</v>
-      </c>
-      <c r="E2" s="32" t="s">
-        <v>106</v>
-      </c>
-      <c r="F2" s="32" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" s="43" t="s">
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A3" s="41" t="s">
         <v>31</v>
       </c>
-      <c r="B3" s="33" t="s">
-        <v>98</v>
-      </c>
-      <c r="C3" s="33" t="s">
+      <c r="B3" s="32" t="s">
+        <v>95</v>
+      </c>
+      <c r="C3" s="32" t="s">
         <v>41</v>
       </c>
-      <c r="D3" s="13" t="s">
+      <c r="D3" s="78" t="s">
         <v>29</v>
       </c>
-      <c r="E3" s="13" t="s">
+      <c r="E3" s="78" t="s">
         <v>30</v>
       </c>
-      <c r="F3" s="30" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="F3" s="29" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" s="12">
         <v>1</v>
       </c>
@@ -3859,7 +4218,7 @@
         <v>Juan García-30/09/2026/10:00-Motilada</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" s="12">
         <v>2</v>
       </c>
@@ -3882,7 +4241,7 @@
         <v>Juan Ortiz-22/11/2025/11:00-Motilada</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" s="12">
         <v>3</v>
       </c>
@@ -3905,7 +4264,7 @@
         <v>Carlos Arbeladez-10/08/2024/14:00-Perfilada de barba</v>
       </c>
     </row>
-    <row r="7" spans="1:6" ht="45" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A7" s="12">
         <v>4</v>
       </c>
@@ -3913,7 +4272,7 @@
         <f>Cita_D!G7</f>
         <v>Andres Ramirez-24/09/2026/13:00</v>
       </c>
-      <c r="C7" s="57" t="str">
+      <c r="C7" s="54" t="str">
         <f>Servicio_D!F7</f>
         <v>Arreglo completo de barba con toalla caliente</v>
       </c>
@@ -3923,12 +4282,12 @@
       <c r="E7" s="12">
         <v>30</v>
       </c>
-      <c r="F7" s="26" t="str">
+      <c r="F7" s="25" t="str">
         <f t="shared" si="0"/>
         <v>Andres Ramirez-24/09/2026/13:00-Arreglo completo de barba con toalla caliente</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8" s="12">
         <v>5</v>
       </c>
@@ -3945,9 +4304,17 @@
       <c r="E8" s="12">
         <v>10</v>
       </c>
-      <c r="F8" s="26" t="str">
+      <c r="F8" s="25" t="str">
         <f t="shared" si="0"/>
         <v>Carlos Arbeladez-06/08/2026/18:00-Corte de barba</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="D10" t="s">
+        <v>219</v>
+      </c>
+      <c r="E10" t="s">
+        <v>218</v>
       </c>
     </row>
   </sheetData>
@@ -3975,20 +4342,20 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7A5AA025-A9A3-4E3E-A766-44885AA770B6}">
   <dimension ref="A1:D15"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="27" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="63.7109375" customWidth="1"/>
-    <col min="3" max="3" width="14.42578125" customWidth="1"/>
-    <col min="4" max="4" width="7.7109375" customWidth="1"/>
+    <col min="2" max="2" width="63.6640625" customWidth="1"/>
+    <col min="3" max="3" width="14.44140625" customWidth="1"/>
+    <col min="4" max="4" width="7.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="5" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" s="6" t="s">
         <v>0</v>
       </c>
@@ -4002,7 +4369,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:4" ht="45" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A3" s="7" t="s">
         <v>4</v>
       </c>
@@ -4016,12 +4383,12 @@
         <v>34</v>
       </c>
     </row>
-    <row r="4" spans="1:4" ht="75" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A4" s="7" t="s">
         <v>11</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>161</v>
+        <v>155</v>
       </c>
       <c r="C4" s="7">
         <v>1</v>
@@ -4030,12 +4397,12 @@
         <v>34</v>
       </c>
     </row>
-    <row r="5" spans="1:4" ht="60" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A5" s="7" t="s">
         <v>5</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>162</v>
+        <v>156</v>
       </c>
       <c r="C5" s="7">
         <v>2</v>
@@ -4044,12 +4411,12 @@
         <v>34</v>
       </c>
     </row>
-    <row r="6" spans="1:4" ht="45" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A6" s="7" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>163</v>
+        <v>157</v>
       </c>
       <c r="C6" s="7">
         <v>2</v>
@@ -4058,12 +4425,12 @@
         <v>34</v>
       </c>
     </row>
-    <row r="7" spans="1:4" ht="60" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A7" s="7" t="s">
         <v>6</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>164</v>
+        <v>158</v>
       </c>
       <c r="C7" s="7">
         <v>2</v>
@@ -4072,7 +4439,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="8" spans="1:4" ht="45" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A8" s="7" t="s">
         <v>7</v>
       </c>
@@ -4086,12 +4453,12 @@
         <v>34</v>
       </c>
     </row>
-    <row r="9" spans="1:4" ht="75" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A9" s="7" t="s">
         <v>13</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>165</v>
+        <v>159</v>
       </c>
       <c r="C9" s="7">
         <v>2</v>
@@ -4100,7 +4467,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="10" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A10" s="7" t="s">
         <v>8</v>
       </c>
@@ -4114,12 +4481,12 @@
         <v>34</v>
       </c>
     </row>
-    <row r="11" spans="1:4" ht="45" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A11" s="7" t="s">
         <v>9</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>166</v>
+        <v>160</v>
       </c>
       <c r="C11" s="7">
         <v>3</v>
@@ -4128,12 +4495,12 @@
         <v>34</v>
       </c>
     </row>
-    <row r="12" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A12" s="7" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>167</v>
+        <v>161</v>
       </c>
       <c r="C12" s="7">
         <v>4</v>
@@ -4142,12 +4509,12 @@
         <v>34</v>
       </c>
     </row>
-    <row r="13" spans="1:4" ht="90" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:4" ht="72" x14ac:dyDescent="0.3">
       <c r="A13" s="7" t="s">
         <v>10</v>
       </c>
       <c r="B13" s="8" t="s">
-        <v>168</v>
+        <v>162</v>
       </c>
       <c r="C13" s="7">
         <v>4</v>
@@ -4156,7 +4523,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="14" spans="1:4" ht="45" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A14" s="7" t="s">
         <v>12</v>
       </c>
@@ -4170,7 +4537,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="15" spans="1:4" ht="60" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A15" s="7" t="s">
         <v>14</v>
       </c>
@@ -4206,16 +4573,118 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{387DE6AC-7D92-461D-9DD1-84082B531231}">
+  <dimension ref="A1:B11"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="18.44140625" customWidth="1"/>
+    <col min="2" max="2" width="62.77734375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A1" s="7" t="s">
+        <v>172</v>
+      </c>
+      <c r="B1" s="7" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A2" s="61" t="s">
+        <v>173</v>
+      </c>
+      <c r="B2" s="61" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A3" s="62" t="s">
+        <v>174</v>
+      </c>
+      <c r="B3" s="71" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A4" s="64" t="s">
+        <v>175</v>
+      </c>
+      <c r="B4" s="64" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A5" s="63" t="s">
+        <v>212</v>
+      </c>
+      <c r="B5" s="72" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A6" s="65" t="s">
+        <v>178</v>
+      </c>
+      <c r="B6" s="65" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A7" s="66" t="s">
+        <v>179</v>
+      </c>
+      <c r="B7" s="73" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A8" s="67" t="s">
+        <v>180</v>
+      </c>
+      <c r="B8" s="74" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A9" s="68" t="s">
+        <v>181</v>
+      </c>
+      <c r="B9" s="75" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A10" s="69" t="s">
+        <v>182</v>
+      </c>
+      <c r="B10" s="69" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A11" s="70" t="s">
+        <v>183</v>
+      </c>
+      <c r="B11" s="76" t="s">
+        <v>192</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AAA22F8C-1648-4644-8301-765EB2B8C50B}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="33.85546875" customWidth="1"/>
-    <col min="2" max="2" width="34.7109375" customWidth="1"/>
+    <col min="1" max="1" width="33.88671875" customWidth="1"/>
+    <col min="2" max="2" width="34.6640625" customWidth="1"/>
     <col min="3" max="3" width="21" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="5" t="s">
         <v>32</v>
       </c>
@@ -4223,29 +4692,29 @@
         <v>33</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="19" t="s">
         <v>20</v>
       </c>
       <c r="B2" s="19" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" s="14" t="s">
         <v>31</v>
       </c>
       <c r="B3" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="C3" s="38"/>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C3" s="37"/>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" s="12">
         <v>1</v>
       </c>
-      <c r="B4" s="39" t="s">
-        <v>69</v>
+      <c r="B4" s="38" t="s">
+        <v>68</v>
       </c>
       <c r="C4" s="4"/>
     </row>
@@ -4258,18 +4727,18 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{28259140-2713-4A98-8730-76D57DC1D653}">
   <dimension ref="A1:H11"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="26.85546875" style="10" customWidth="1"/>
-    <col min="2" max="6" width="26.28515625" style="10" customWidth="1"/>
-    <col min="7" max="7" width="23.140625" style="10" customWidth="1"/>
-    <col min="8" max="8" width="38.5703125" style="10" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="26.88671875" style="10" customWidth="1"/>
+    <col min="2" max="6" width="26.33203125" style="10" customWidth="1"/>
+    <col min="7" max="7" width="23.109375" style="10" customWidth="1"/>
+    <col min="8" max="8" width="38.5546875" style="10" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A1" s="11" t="s">
         <v>32</v>
       </c>
@@ -4283,72 +4752,72 @@
       <c r="G1" s="12"/>
       <c r="H1" s="12"/>
     </row>
-    <row r="2" spans="1:8" ht="55.5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" ht="39.6" x14ac:dyDescent="0.3">
       <c r="A2" s="18" t="s">
         <v>20</v>
       </c>
       <c r="B2" s="18" t="s">
-        <v>170</v>
+        <v>193</v>
       </c>
       <c r="C2" s="18" t="s">
-        <v>171</v>
+        <v>194</v>
       </c>
       <c r="D2" s="18" t="s">
-        <v>172</v>
+        <v>195</v>
       </c>
       <c r="E2" s="18" t="s">
-        <v>173</v>
+        <v>196</v>
       </c>
       <c r="F2" s="18" t="s">
-        <v>175</v>
+        <v>197</v>
       </c>
       <c r="G2" s="19" t="s">
-        <v>176</v>
+        <v>198</v>
       </c>
       <c r="H2" s="20" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" s="14" t="s">
         <v>31</v>
       </c>
-      <c r="B3" s="13" t="s">
-        <v>109</v>
-      </c>
-      <c r="C3" s="13" t="s">
-        <v>111</v>
-      </c>
-      <c r="D3" s="13" t="s">
-        <v>110</v>
-      </c>
-      <c r="E3" s="13" t="s">
-        <v>112</v>
-      </c>
-      <c r="F3" s="13" t="s">
-        <v>174</v>
-      </c>
-      <c r="G3" s="13" t="s">
+      <c r="B3" s="58" t="s">
+        <v>105</v>
+      </c>
+      <c r="C3" s="58" t="s">
+        <v>107</v>
+      </c>
+      <c r="D3" s="58" t="s">
+        <v>106</v>
+      </c>
+      <c r="E3" s="58" t="s">
+        <v>108</v>
+      </c>
+      <c r="F3" s="77" t="s">
+        <v>164</v>
+      </c>
+      <c r="G3" s="77" t="s">
         <v>22</v>
       </c>
       <c r="H3" s="15" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A4" s="12">
         <v>1</v>
       </c>
       <c r="B4" s="12" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="C4" s="12"/>
       <c r="D4" s="12" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="E4" s="12"/>
-      <c r="F4" s="51" t="s">
-        <v>138</v>
+      <c r="F4" s="48" t="s">
+        <v>133</v>
       </c>
       <c r="G4" s="12">
         <v>3234528921</v>
@@ -4358,24 +4827,24 @@
         <v>Juan--Gómez--+57-3234528921</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A5" s="12">
         <v>2</v>
       </c>
       <c r="B5" s="12" t="s">
-        <v>124</v>
+        <v>120</v>
       </c>
       <c r="C5" s="12" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="D5" s="12" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="E5" s="12" t="s">
-        <v>120</v>
-      </c>
-      <c r="F5" s="51" t="s">
-        <v>138</v>
+        <v>116</v>
+      </c>
+      <c r="F5" s="48" t="s">
+        <v>133</v>
       </c>
       <c r="G5" s="12">
         <v>3161657782</v>
@@ -4385,22 +4854,22 @@
         <v>Jose-Miguel-Ramirez-Perez-+57-3161657782</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A6" s="12">
         <v>3</v>
       </c>
       <c r="B6" s="12" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="C6" s="12"/>
       <c r="D6" s="12" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="E6" s="12" t="s">
-        <v>121</v>
-      </c>
-      <c r="F6" s="51" t="s">
-        <v>138</v>
+        <v>117</v>
+      </c>
+      <c r="F6" s="48" t="s">
+        <v>133</v>
       </c>
       <c r="G6" s="12">
         <v>3119884321</v>
@@ -4410,20 +4879,20 @@
         <v>Simon--Ochoa-Ramirez-+57-3119884321</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A7" s="12">
         <v>4</v>
       </c>
       <c r="B7" s="12" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="C7" s="12"/>
       <c r="D7" s="12" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="E7" s="12"/>
-      <c r="F7" s="51" t="s">
-        <v>139</v>
+      <c r="F7" s="48" t="s">
+        <v>134</v>
       </c>
       <c r="G7" s="12">
         <v>4127359182</v>
@@ -4433,7 +4902,7 @@
         <v>Alexis--Gallego--+58-4127359182</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
       <c r="C11"/>
     </row>
   </sheetData>
@@ -4446,20 +4915,20 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B0E77388-6266-4A55-B7A3-4FCD2B643D29}">
   <dimension ref="A1:F5"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="26.85546875" customWidth="1"/>
-    <col min="2" max="2" width="32.5703125" customWidth="1"/>
+    <col min="1" max="1" width="26.88671875" customWidth="1"/>
+    <col min="2" max="2" width="32.5546875" customWidth="1"/>
     <col min="3" max="3" width="28" customWidth="1"/>
-    <col min="4" max="4" width="26.7109375" customWidth="1"/>
-    <col min="5" max="5" width="16.28515625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="18.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="26.6640625" customWidth="1"/>
+    <col min="5" max="5" width="16.33203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="18.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" s="5" t="s">
         <v>32</v>
       </c>
@@ -4467,55 +4936,55 @@
         <v>33</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="57" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" ht="49.2" x14ac:dyDescent="0.3">
       <c r="A2" s="18" t="s">
         <v>20</v>
       </c>
       <c r="B2" s="19" t="s">
-        <v>177</v>
+        <v>199</v>
       </c>
       <c r="C2" s="19" t="s">
-        <v>178</v>
+        <v>200</v>
       </c>
       <c r="D2" s="19" t="s">
-        <v>179</v>
+        <v>201</v>
       </c>
       <c r="E2" s="19" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" s="14" t="s">
         <v>31</v>
       </c>
-      <c r="B3" s="13" t="s">
+      <c r="B3" s="78" t="s">
         <v>35</v>
       </c>
-      <c r="C3" s="13" t="s">
+      <c r="C3" s="78" t="s">
         <v>23</v>
       </c>
-      <c r="D3" s="13" t="s">
-        <v>70</v>
-      </c>
-      <c r="E3" s="33" t="s">
+      <c r="D3" s="78" t="s">
+        <v>69</v>
+      </c>
+      <c r="E3" s="32" t="s">
         <v>36</v>
       </c>
       <c r="F3" s="3"/>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" s="12">
         <v>1</v>
       </c>
       <c r="B4" s="12">
         <v>10</v>
       </c>
-      <c r="C4" s="44">
+      <c r="C4" s="42">
         <v>10000</v>
       </c>
       <c r="D4" s="12">
         <v>3</v>
       </c>
-      <c r="E4" s="53" t="str">
+      <c r="E4" s="50" t="str">
         <f>Barberia_D!B4</f>
         <v>Barbería Oriental</v>
       </c>
@@ -4524,7 +4993,7 @@
         <v/>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="D5" s="2"/>
     </row>
   </sheetData>
@@ -4538,20 +5007,20 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2190E1EC-B79B-40C0-AC5B-0E2726DDD399}">
   <dimension ref="A1:F11"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="27" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="26" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="21.28515625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="19.28515625" customWidth="1"/>
-    <col min="5" max="5" width="20.28515625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="34.85546875" customWidth="1"/>
+    <col min="3" max="3" width="22.5546875" customWidth="1"/>
+    <col min="4" max="4" width="23.5546875" customWidth="1"/>
+    <col min="5" max="5" width="23.77734375" customWidth="1"/>
+    <col min="6" max="6" width="34.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" s="5" t="s">
         <v>32</v>
       </c>
@@ -4559,61 +5028,61 @@
         <v>33</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" ht="44.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="19" t="s">
         <v>20</v>
       </c>
       <c r="B2" s="19" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="C2" s="19" t="s">
-        <v>129</v>
+        <v>203</v>
       </c>
       <c r="D2" s="19" t="s">
-        <v>181</v>
+        <v>204</v>
       </c>
       <c r="E2" s="19" t="s">
-        <v>182</v>
+        <v>205</v>
       </c>
       <c r="F2" s="19" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" s="14" t="s">
         <v>31</v>
       </c>
-      <c r="B3" s="33" t="s">
+      <c r="B3" s="32" t="s">
         <v>36</v>
       </c>
-      <c r="C3" s="40" t="s">
+      <c r="C3" s="59" t="s">
+        <v>77</v>
+      </c>
+      <c r="D3" s="79" t="s">
+        <v>78</v>
+      </c>
+      <c r="E3" s="80" t="s">
         <v>79</v>
       </c>
-      <c r="D3" s="46" t="s">
-        <v>80</v>
-      </c>
-      <c r="E3" s="13" t="s">
-        <v>81</v>
-      </c>
-      <c r="F3" s="37" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="F3" s="36" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" s="12">
         <v>1</v>
       </c>
-      <c r="B4" s="53" t="str">
+      <c r="B4" s="50" t="str">
         <f>Barberia_D!B4</f>
         <v>Barbería Oriental</v>
       </c>
-      <c r="C4" s="39" t="s">
-        <v>82</v>
-      </c>
-      <c r="D4" s="39">
+      <c r="C4" s="38" t="s">
+        <v>80</v>
+      </c>
+      <c r="D4" s="38">
         <v>0.375</v>
       </c>
-      <c r="E4" s="39">
+      <c r="E4" s="38">
         <v>0.79166666666666663</v>
       </c>
       <c r="F4" s="12" t="str">
@@ -4621,21 +5090,21 @@
         <v>Barbería Oriental-Lunes-09:00-19:00</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" s="12">
         <v>2</v>
       </c>
-      <c r="B5" s="53" t="str">
+      <c r="B5" s="50" t="str">
         <f>Barberia_D!B4</f>
         <v>Barbería Oriental</v>
       </c>
       <c r="C5" s="12" t="s">
-        <v>83</v>
-      </c>
-      <c r="D5" s="39">
+        <v>81</v>
+      </c>
+      <c r="D5" s="38">
         <v>0.375</v>
       </c>
-      <c r="E5" s="39">
+      <c r="E5" s="38">
         <v>0.79166666666666663</v>
       </c>
       <c r="F5" s="12" t="str">
@@ -4643,21 +5112,21 @@
         <v>Barbería Oriental-Martes-09:00-19:00</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" s="12">
         <v>3</v>
       </c>
-      <c r="B6" s="53" t="str">
+      <c r="B6" s="50" t="str">
         <f>Barberia_D!B4</f>
         <v>Barbería Oriental</v>
       </c>
-      <c r="C6" s="39" t="s">
-        <v>84</v>
-      </c>
-      <c r="D6" s="39">
+      <c r="C6" s="38" t="s">
+        <v>82</v>
+      </c>
+      <c r="D6" s="38">
         <v>0.375</v>
       </c>
-      <c r="E6" s="39">
+      <c r="E6" s="38">
         <v>0.79166666666666696</v>
       </c>
       <c r="F6" s="12" t="str">
@@ -4665,21 +5134,21 @@
         <v>Barbería Oriental-Miércoles-09:00-19:00</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7" s="12">
         <v>4</v>
       </c>
-      <c r="B7" s="53" t="str">
+      <c r="B7" s="50" t="str">
         <f>Barberia_D!B4</f>
         <v>Barbería Oriental</v>
       </c>
       <c r="C7" s="12" t="s">
-        <v>85</v>
-      </c>
-      <c r="D7" s="39">
+        <v>83</v>
+      </c>
+      <c r="D7" s="38">
         <v>0.375</v>
       </c>
-      <c r="E7" s="39">
+      <c r="E7" s="38">
         <v>0.79166666666666696</v>
       </c>
       <c r="F7" s="12" t="str">
@@ -4687,21 +5156,21 @@
         <v>Barbería Oriental-Jueves-09:00-19:00</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8" s="12">
         <v>5</v>
       </c>
-      <c r="B8" s="53" t="str">
+      <c r="B8" s="50" t="str">
         <f>Barberia_D!B4</f>
         <v>Barbería Oriental</v>
       </c>
-      <c r="C8" s="39" t="s">
-        <v>86</v>
-      </c>
-      <c r="D8" s="39">
+      <c r="C8" s="38" t="s">
+        <v>84</v>
+      </c>
+      <c r="D8" s="38">
         <v>0.375</v>
       </c>
-      <c r="E8" s="39">
+      <c r="E8" s="38">
         <v>0.79166666666666696</v>
       </c>
       <c r="F8" s="12" t="str">
@@ -4709,21 +5178,21 @@
         <v>Barbería Oriental-Viernes-09:00-19:00</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A9" s="12">
         <v>6</v>
       </c>
-      <c r="B9" s="53" t="str">
+      <c r="B9" s="50" t="str">
         <f>Barberia_D!B4</f>
         <v>Barbería Oriental</v>
       </c>
       <c r="C9" s="12" t="s">
-        <v>87</v>
-      </c>
-      <c r="D9" s="42">
+        <v>85</v>
+      </c>
+      <c r="D9" s="40">
         <v>0.33333333333333331</v>
       </c>
-      <c r="E9" s="39">
+      <c r="E9" s="38">
         <v>0.875</v>
       </c>
       <c r="F9" s="12" t="str">
@@ -4731,14 +5200,14 @@
         <v>Barbería Oriental-Sábado-08:00-21:00</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A10" s="10"/>
-      <c r="B10" s="41"/>
-      <c r="C10" s="41"/>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="C11" s="61" t="s">
-        <v>180</v>
+      <c r="B10" s="39"/>
+      <c r="C10" s="39"/>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="C11" s="10" t="s">
+        <v>202</v>
       </c>
     </row>
   </sheetData>
@@ -4758,19 +5227,19 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C97B567D-D27E-4BE3-B1E4-8CA267790151}">
   <dimension ref="A1:F12"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="2" width="28.140625" customWidth="1"/>
-    <col min="3" max="3" width="26.5703125" customWidth="1"/>
-    <col min="4" max="4" width="24.42578125" customWidth="1"/>
-    <col min="5" max="5" width="25.28515625" customWidth="1"/>
-    <col min="6" max="6" width="26.5703125" customWidth="1"/>
+    <col min="1" max="2" width="28.109375" customWidth="1"/>
+    <col min="3" max="3" width="26.5546875" customWidth="1"/>
+    <col min="4" max="4" width="24.44140625" customWidth="1"/>
+    <col min="5" max="5" width="25.33203125" customWidth="1"/>
+    <col min="6" max="6" width="26.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" s="16" t="s">
         <v>32</v>
       </c>
@@ -4781,61 +5250,61 @@
       <c r="E1" s="17"/>
       <c r="F1" s="10"/>
     </row>
-    <row r="2" spans="1:6" ht="45.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" ht="45.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="18" t="s">
         <v>20</v>
       </c>
       <c r="B2" s="18" t="s">
-        <v>149</v>
+        <v>143</v>
       </c>
       <c r="C2" s="18" t="s">
-        <v>183</v>
-      </c>
-      <c r="D2" s="32" t="s">
-        <v>184</v>
-      </c>
-      <c r="E2" s="32" t="s">
-        <v>185</v>
+        <v>206</v>
+      </c>
+      <c r="D2" s="31" t="s">
+        <v>208</v>
+      </c>
+      <c r="E2" s="31" t="s">
+        <v>209</v>
       </c>
       <c r="F2" s="19" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" s="21" t="s">
         <v>31</v>
       </c>
-      <c r="B3" s="58" t="s">
+      <c r="B3" s="55" t="s">
         <v>36</v>
       </c>
-      <c r="C3" s="22" t="s">
+      <c r="C3" s="81" t="s">
         <v>21</v>
       </c>
-      <c r="D3" s="22" t="s">
+      <c r="D3" s="82" t="s">
         <v>37</v>
       </c>
-      <c r="E3" s="22" t="s">
+      <c r="E3" s="82" t="s">
         <v>24</v>
       </c>
       <c r="F3" s="15" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4" s="23">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A4" s="22">
         <v>1</v>
       </c>
-      <c r="B4" s="59" t="str">
+      <c r="B4" s="56" t="str">
         <f>Barberia_D!B4</f>
         <v>Barbería Oriental</v>
       </c>
-      <c r="C4" s="23" t="s">
+      <c r="C4" s="22" t="s">
         <v>38</v>
       </c>
-      <c r="D4" s="23">
+      <c r="D4" s="22">
         <v>45</v>
       </c>
-      <c r="E4" s="24">
+      <c r="E4" s="23">
         <v>22000</v>
       </c>
       <c r="F4" s="12" t="str">
@@ -4843,21 +5312,21 @@
         <v>Motilada</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A5" s="23">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A5" s="22">
         <v>2</v>
       </c>
-      <c r="B5" s="59" t="str">
+      <c r="B5" s="56" t="str">
         <f>Barberia_D!B4</f>
         <v>Barbería Oriental</v>
       </c>
-      <c r="C5" s="23" t="s">
+      <c r="C5" s="22" t="s">
         <v>46</v>
       </c>
-      <c r="D5" s="23">
+      <c r="D5" s="22">
         <v>10</v>
       </c>
-      <c r="E5" s="24">
+      <c r="E5" s="23">
         <v>12000</v>
       </c>
       <c r="F5" s="12" t="str">
@@ -4865,21 +5334,21 @@
         <v>Corte de barba</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A6" s="23">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A6" s="22">
         <v>3</v>
       </c>
-      <c r="B6" s="59" t="str">
+      <c r="B6" s="56" t="str">
         <f>Barberia_D!B4</f>
         <v>Barbería Oriental</v>
       </c>
-      <c r="C6" s="23" t="s">
+      <c r="C6" s="22" t="s">
         <v>47</v>
       </c>
-      <c r="D6" s="23">
+      <c r="D6" s="22">
         <v>15</v>
       </c>
-      <c r="E6" s="24">
+      <c r="E6" s="23">
         <v>15000</v>
       </c>
       <c r="F6" s="12" t="str">
@@ -4887,57 +5356,57 @@
         <v>Perfilada de barba</v>
       </c>
     </row>
-    <row r="7" spans="1:6" ht="30" x14ac:dyDescent="0.25">
-      <c r="A7" s="23">
+    <row r="7" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A7" s="22">
         <v>4</v>
       </c>
-      <c r="B7" s="59" t="str">
+      <c r="B7" s="56" t="str">
         <f>Barberia_D!B4</f>
         <v>Barbería Oriental</v>
       </c>
-      <c r="C7" s="25" t="s">
+      <c r="C7" s="24" t="s">
         <v>48</v>
       </c>
-      <c r="D7" s="23">
+      <c r="D7" s="22">
         <v>30</v>
       </c>
-      <c r="E7" s="24">
+      <c r="E7" s="23">
         <v>35000</v>
       </c>
-      <c r="F7" s="26" t="str">
+      <c r="F7" s="25" t="str">
         <f t="shared" si="0"/>
         <v>Arreglo completo de barba con toalla caliente</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8" s="17"/>
       <c r="B8" s="17"/>
       <c r="C8" s="17"/>
       <c r="D8" s="17"/>
       <c r="E8" s="17"/>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A9" s="17"/>
       <c r="B9" s="17"/>
       <c r="C9" s="17"/>
       <c r="D9" s="17"/>
       <c r="E9" s="17"/>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A10" s="17"/>
       <c r="B10" s="17"/>
       <c r="C10" s="17"/>
       <c r="D10" s="17"/>
       <c r="E10" s="17"/>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A11" s="17"/>
       <c r="B11" s="17"/>
       <c r="C11" s="17"/>
       <c r="D11" s="17"/>
       <c r="E11" s="17"/>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A12" s="17"/>
       <c r="B12" s="17"/>
       <c r="C12" s="17"/>
@@ -4958,21 +5427,21 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2DAE59AB-4103-4731-9C3C-4C276F8A29F8}">
   <dimension ref="A1:L14"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="27" bestFit="1" customWidth="1"/>
-    <col min="2" max="6" width="26.7109375" customWidth="1"/>
-    <col min="7" max="7" width="16.28515625" customWidth="1"/>
-    <col min="8" max="9" width="40.7109375" customWidth="1"/>
-    <col min="10" max="10" width="30.28515625" customWidth="1"/>
+    <col min="2" max="6" width="26.6640625" customWidth="1"/>
+    <col min="7" max="7" width="16.33203125" customWidth="1"/>
+    <col min="8" max="9" width="40.6640625" customWidth="1"/>
+    <col min="10" max="10" width="30.33203125" customWidth="1"/>
     <col min="11" max="11" width="21" customWidth="1"/>
-    <col min="12" max="12" width="53.140625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="53.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A1" s="5" t="s">
         <v>32</v>
       </c>
@@ -4984,114 +5453,114 @@
       <c r="E1" s="5"/>
       <c r="F1" s="5"/>
     </row>
-    <row r="2" spans="1:12" ht="45.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="27" t="s">
+    <row r="2" spans="1:12" ht="45.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="26" t="s">
         <v>20</v>
       </c>
-      <c r="B2" s="27" t="s">
-        <v>186</v>
-      </c>
-      <c r="C2" s="27" t="s">
-        <v>187</v>
-      </c>
-      <c r="D2" s="27" t="s">
-        <v>188</v>
-      </c>
-      <c r="E2" s="27" t="s">
-        <v>189</v>
-      </c>
-      <c r="F2" s="27" t="s">
-        <v>191</v>
-      </c>
-      <c r="G2" s="28" t="s">
-        <v>49</v>
-      </c>
-      <c r="H2" s="28" t="s">
-        <v>192</v>
-      </c>
-      <c r="I2" s="28" t="s">
-        <v>193</v>
-      </c>
-      <c r="J2" s="28" t="s">
-        <v>141</v>
-      </c>
-      <c r="K2" s="28" t="s">
-        <v>150</v>
-      </c>
-      <c r="L2" s="29" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="B2" s="26" t="s">
+        <v>165</v>
+      </c>
+      <c r="C2" s="26" t="s">
+        <v>166</v>
+      </c>
+      <c r="D2" s="26" t="s">
+        <v>167</v>
+      </c>
+      <c r="E2" s="26" t="s">
+        <v>168</v>
+      </c>
+      <c r="F2" s="26" t="s">
+        <v>170</v>
+      </c>
+      <c r="G2" s="27" t="s">
+        <v>210</v>
+      </c>
+      <c r="H2" s="27" t="s">
+        <v>211</v>
+      </c>
+      <c r="I2" s="27" t="s">
+        <v>171</v>
+      </c>
+      <c r="J2" s="27" t="s">
+        <v>136</v>
+      </c>
+      <c r="K2" s="27" t="s">
+        <v>144</v>
+      </c>
+      <c r="L2" s="28" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A3" s="14" t="s">
         <v>31</v>
       </c>
-      <c r="B3" s="13" t="s">
-        <v>109</v>
-      </c>
-      <c r="C3" s="13" t="s">
-        <v>111</v>
-      </c>
-      <c r="D3" s="13" t="s">
-        <v>110</v>
-      </c>
-      <c r="E3" s="13" t="s">
-        <v>112</v>
-      </c>
-      <c r="F3" s="13" t="s">
-        <v>137</v>
-      </c>
-      <c r="G3" s="13" t="s">
+      <c r="B3" s="58" t="s">
+        <v>105</v>
+      </c>
+      <c r="C3" s="58" t="s">
+        <v>107</v>
+      </c>
+      <c r="D3" s="58" t="s">
+        <v>106</v>
+      </c>
+      <c r="E3" s="58" t="s">
+        <v>108</v>
+      </c>
+      <c r="F3" s="77" t="s">
+        <v>132</v>
+      </c>
+      <c r="G3" s="77" t="s">
         <v>22</v>
       </c>
-      <c r="H3" s="13" t="s">
+      <c r="H3" s="77" t="s">
         <v>42</v>
       </c>
-      <c r="I3" s="13" t="s">
-        <v>133</v>
-      </c>
-      <c r="J3" s="47" t="s">
+      <c r="I3" s="77" t="s">
+        <v>128</v>
+      </c>
+      <c r="J3" s="44" t="s">
         <v>43</v>
       </c>
-      <c r="K3" s="33" t="s">
+      <c r="K3" s="32" t="s">
         <v>36</v>
       </c>
-      <c r="L3" s="30" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="L3" s="29" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A4" s="12">
         <v>1</v>
       </c>
       <c r="B4" s="12" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="C4" s="12" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="D4" s="12" t="s">
-        <v>156</v>
+        <v>150</v>
       </c>
       <c r="E4" s="12" t="s">
-        <v>115</v>
-      </c>
-      <c r="F4" s="51" t="s">
-        <v>138</v>
+        <v>111</v>
+      </c>
+      <c r="F4" s="48" t="s">
+        <v>133</v>
       </c>
       <c r="G4" s="12">
         <v>3245627890</v>
       </c>
       <c r="H4" s="11" t="s">
-        <v>54</v>
-      </c>
-      <c r="I4" s="49">
+        <v>53</v>
+      </c>
+      <c r="I4" s="46">
         <v>1264267821</v>
       </c>
       <c r="J4" s="12" t="s">
-        <v>50</v>
-      </c>
-      <c r="K4" s="53" t="str">
+        <v>49</v>
+      </c>
+      <c r="K4" s="50" t="str">
         <f>Barberia_D!B4</f>
         <v>Barbería Oriental</v>
       </c>
@@ -5100,38 +5569,38 @@
         <v>Juan-Fernando-García-Lopez-+57-3245627890</v>
       </c>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A5" s="12">
         <v>2</v>
       </c>
       <c r="B5" s="12" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="C5" s="12" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="D5" s="12" t="s">
-        <v>155</v>
+        <v>149</v>
       </c>
       <c r="E5" s="12" t="s">
-        <v>116</v>
-      </c>
-      <c r="F5" s="51" t="s">
-        <v>138</v>
+        <v>112</v>
+      </c>
+      <c r="F5" s="48" t="s">
+        <v>133</v>
       </c>
       <c r="G5" s="12">
         <v>3124518923</v>
       </c>
       <c r="H5" s="11" t="s">
-        <v>55</v>
-      </c>
-      <c r="I5" s="49" t="s">
-        <v>135</v>
+        <v>54</v>
+      </c>
+      <c r="I5" s="46" t="s">
+        <v>130</v>
       </c>
       <c r="J5" s="12" t="s">
-        <v>50</v>
-      </c>
-      <c r="K5" s="53" t="str">
+        <v>49</v>
+      </c>
+      <c r="K5" s="50" t="str">
         <f>Barberia_D!B4</f>
         <v>Barbería Oriental</v>
       </c>
@@ -5140,34 +5609,34 @@
         <v>Juan-David-Ortiz-Sanchez-+57-3124518923</v>
       </c>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A6" s="12">
         <v>3</v>
       </c>
       <c r="B6" s="12" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C6" s="12"/>
       <c r="D6" s="12" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="E6" s="12"/>
-      <c r="F6" s="51" t="s">
-        <v>138</v>
+      <c r="F6" s="48" t="s">
+        <v>133</v>
       </c>
       <c r="G6" s="12">
         <v>3214533321</v>
       </c>
       <c r="H6" s="11" t="s">
-        <v>56</v>
-      </c>
-      <c r="I6" s="50" t="s">
-        <v>134</v>
+        <v>55</v>
+      </c>
+      <c r="I6" s="47" t="s">
+        <v>129</v>
       </c>
       <c r="J6" s="12" t="s">
-        <v>50</v>
-      </c>
-      <c r="K6" s="53" t="str">
+        <v>49</v>
+      </c>
+      <c r="K6" s="50" t="str">
         <f>Barberia_D!B4</f>
         <v>Barbería Oriental</v>
       </c>
@@ -5176,36 +5645,36 @@
         <v>Carlos--Arbeladez--+57-3214533321</v>
       </c>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A7" s="12">
         <v>4</v>
       </c>
       <c r="B7" s="12" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C7" s="12"/>
       <c r="D7" s="12" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="E7" s="12" t="s">
-        <v>117</v>
-      </c>
-      <c r="F7" s="51" t="s">
-        <v>140</v>
+        <v>113</v>
+      </c>
+      <c r="F7" s="48" t="s">
+        <v>135</v>
       </c>
       <c r="G7" s="12">
         <v>9876543210</v>
       </c>
       <c r="H7" s="11" t="s">
-        <v>57</v>
-      </c>
-      <c r="I7" s="49" t="s">
-        <v>136</v>
+        <v>56</v>
+      </c>
+      <c r="I7" s="46" t="s">
+        <v>131</v>
       </c>
       <c r="J7" s="12" t="s">
-        <v>50</v>
-      </c>
-      <c r="K7" s="53" t="str">
+        <v>49</v>
+      </c>
+      <c r="K7" s="50" t="str">
         <f>Barberia_D!B4</f>
         <v>Barbería Oriental</v>
       </c>
@@ -5214,38 +5683,38 @@
         <v>Andres--Ramirez-Patiño-+91-9876543210</v>
       </c>
     </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A8" s="12">
         <v>5</v>
       </c>
       <c r="B8" s="12" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="C8" s="12" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D8" s="12" t="s">
-        <v>157</v>
+        <v>151</v>
       </c>
       <c r="E8" s="12" t="s">
-        <v>120</v>
-      </c>
-      <c r="F8" s="51" t="s">
-        <v>158</v>
+        <v>116</v>
+      </c>
+      <c r="F8" s="48" t="s">
+        <v>152</v>
       </c>
       <c r="G8" s="12">
         <v>998765432</v>
       </c>
       <c r="H8" s="11" t="s">
-        <v>159</v>
+        <v>153</v>
       </c>
       <c r="I8" s="12">
         <v>312334342</v>
       </c>
       <c r="J8" s="12" t="s">
-        <v>51</v>
-      </c>
-      <c r="K8" s="53" t="str">
+        <v>50</v>
+      </c>
+      <c r="K8" s="50" t="str">
         <f>Barberia_D!B4</f>
         <v>Barbería Oriental</v>
       </c>
@@ -5254,13 +5723,13 @@
         <v>Juan-Carlos-Zambrano-Perez-+593-998765432</v>
       </c>
     </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:12" x14ac:dyDescent="0.3">
       <c r="B10" s="10"/>
       <c r="C10" s="10"/>
     </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:12" x14ac:dyDescent="0.3">
       <c r="F14" t="s">
-        <v>190</v>
+        <v>169</v>
       </c>
     </row>
   </sheetData>
@@ -5280,155 +5749,4 @@
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C828B98D-AAA9-4184-8373-FE2E421AAE23}">
-  <dimension ref="A1:E11"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="27" customWidth="1"/>
-    <col min="2" max="2" width="28.85546875" customWidth="1"/>
-    <col min="3" max="3" width="41" customWidth="1"/>
-    <col min="4" max="4" width="36.140625" customWidth="1"/>
-    <col min="5" max="5" width="26.85546875" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1" s="5" t="s">
-        <v>32</v>
-      </c>
-      <c r="B1" s="5" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="18" t="s">
-        <v>20</v>
-      </c>
-      <c r="B2" s="18" t="s">
-        <v>59</v>
-      </c>
-      <c r="C2" s="32" t="s">
-        <v>61</v>
-      </c>
-      <c r="D2" s="32" t="s">
-        <v>132</v>
-      </c>
-      <c r="E2" s="32" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" s="14" t="s">
-        <v>31</v>
-      </c>
-      <c r="B3" s="33" t="s">
-        <v>62</v>
-      </c>
-      <c r="C3" s="13" t="s">
-        <v>25</v>
-      </c>
-      <c r="D3" s="47" t="s">
-        <v>58</v>
-      </c>
-      <c r="E3" s="30" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" s="12">
-        <v>1</v>
-      </c>
-      <c r="B4" s="11">
-        <f>Cliente_D!G4</f>
-        <v>3234528921</v>
-      </c>
-      <c r="C4" s="34">
-        <v>45255</v>
-      </c>
-      <c r="D4" s="12" t="s">
-        <v>51</v>
-      </c>
-      <c r="E4" s="12" t="str">
-        <f>_xlfn.CONCAT(B4,"-",TEXT(C4,"dd/mm/yyyy"))</f>
-        <v>3234528921-25/11/2023</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5" s="12">
-        <v>2</v>
-      </c>
-      <c r="B5" s="11">
-        <f>Cliente_D!G5</f>
-        <v>3161657782</v>
-      </c>
-      <c r="C5" s="34">
-        <v>45372</v>
-      </c>
-      <c r="D5" s="12" t="s">
-        <v>51</v>
-      </c>
-      <c r="E5" s="12" t="str">
-        <f t="shared" ref="E5:E7" si="0">_xlfn.CONCAT(B5,"-",TEXT(C5,"dd/mm/yyyy"))</f>
-        <v>3161657782-21/03/2024</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" s="12">
-        <v>3</v>
-      </c>
-      <c r="B6" s="11">
-        <f>Cliente_D!G6</f>
-        <v>3119884321</v>
-      </c>
-      <c r="C6" s="34">
-        <v>45556</v>
-      </c>
-      <c r="D6" s="12" t="s">
-        <v>50</v>
-      </c>
-      <c r="E6" s="12" t="str">
-        <f t="shared" si="0"/>
-        <v>3119884321-21/09/2024</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A7" s="12">
-        <v>4</v>
-      </c>
-      <c r="B7" s="11">
-        <f>Cliente_D!G7</f>
-        <v>4127359182</v>
-      </c>
-      <c r="C7" s="34">
-        <v>46002</v>
-      </c>
-      <c r="D7" s="12" t="s">
-        <v>50</v>
-      </c>
-      <c r="E7" s="12" t="str">
-        <f t="shared" si="0"/>
-        <v>4127359182-11/12/2025</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="C8" s="31"/>
-      <c r="D8" s="31"/>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="C11" s="48"/>
-    </row>
-  </sheetData>
-  <hyperlinks>
-    <hyperlink ref="A1" location="'Modelo de Dominio'!A1" display="&lt;&lt;&lt;&lt; Ir al modulo de dominio" xr:uid="{F755F618-0A40-4479-913F-8F6060E94F5B}"/>
-    <hyperlink ref="B1" location="'Objetos de Dominio'!A1" display="&lt;&lt;&lt;&lt; Ir a objetos de dominio" xr:uid="{C5748D80-5E29-4CD8-BA51-198180E61202}"/>
-    <hyperlink ref="B3" location="Cliente_D!A1" display="cliente" xr:uid="{F7C47FD3-2FEB-4E40-8CE8-9FEC66E905E0}"/>
-    <hyperlink ref="B4" location="Cliente_D!A4" display="Cliente_D!A4" xr:uid="{7F6CACFC-57C0-447E-811A-802403EBA0AC}"/>
-    <hyperlink ref="B5" location="Cliente_D!A5" display="Cliente_D!A5" xr:uid="{EE87A799-0DAD-412E-8BF4-24089411596B}"/>
-    <hyperlink ref="B6" location="Cliente_D!A6" display="Cliente_D!A6" xr:uid="{D95F6EBA-51E7-42CB-9EFD-6676C5924513}"/>
-    <hyperlink ref="B7" location="Cliente_D!A7" display="Cliente_D!A7" xr:uid="{9BA1680E-A8A5-4CE9-866D-EC3B5A4F5B91}"/>
-  </hyperlinks>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Actualizacion del modelo de dominio (Se le añadieron dos objetos de dominion), falta hacerle el muestreo de datos de esos dos objetos
</commit_message>
<xml_diff>
--- a/Muestreo de datos.xlsx
+++ b/Muestreo de datos.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\leand\Desktop\DOO\DOO\Barberia\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/120f6d501c463b80/Escritorio/leo/Doo/Barberia proyecto/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D2C82A5-CE11-488F-916B-C5EEB7B95CE2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="9" documentId="13_ncr:1_{7D2C82A5-CE11-488F-916B-C5EEB7B95CE2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9F3D621B-2D43-45EE-A08C-EA5144B4F136}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{09A6C7D7-663F-4C06-9D71-8A4E97495CF9}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" firstSheet="1" activeTab="1" xr2:uid="{09A6C7D7-663F-4C06-9D71-8A4E97495CF9}"/>
   </bookViews>
   <sheets>
     <sheet name="Modelo de Dominio" sheetId="1" r:id="rId1"/>
@@ -54,7 +54,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="333" uniqueCount="220">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="336" uniqueCount="223">
   <si>
     <t>Nombre</t>
   </si>
@@ -716,6 +716,15 @@
   </si>
   <si>
     <t>Sera que este es calculado o lo pone el barbero</t>
+  </si>
+  <si>
+    <t>Este objeto de dominio puede no tener ninguna instancia, o es necesario que halla uno</t>
+  </si>
+  <si>
+    <t>Bloqueo</t>
+  </si>
+  <si>
+    <t>Descanso</t>
   </si>
 </sst>
 </file>
@@ -912,7 +921,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="85">
+  <cellXfs count="84">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -1067,9 +1076,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="13" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
@@ -1555,12 +1561,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D2495362-94CF-4E08-8433-6F4780C6375E}">
   <dimension ref="A1:AD50"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="26.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="26.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
         <v>39</v>
       </c>
@@ -1594,7 +1600,7 @@
       <c r="AC1" s="1"/>
       <c r="AD1" s="1"/>
     </row>
-    <row r="2" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A2" s="1"/>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
@@ -1626,7 +1632,7 @@
       <c r="AC2" s="1"/>
       <c r="AD2" s="1"/>
     </row>
-    <row r="3" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
       <c r="B3" s="1"/>
       <c r="C3" s="1"/>
@@ -1658,7 +1664,7 @@
       <c r="AC3" s="1"/>
       <c r="AD3" s="1"/>
     </row>
-    <row r="4" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:30" x14ac:dyDescent="0.25">
       <c r="B4" s="1"/>
       <c r="C4" s="1"/>
       <c r="D4" s="1"/>
@@ -1689,7 +1695,7 @@
       <c r="AC4" s="1"/>
       <c r="AD4" s="1"/>
     </row>
-    <row r="5" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A5" s="1"/>
       <c r="B5" s="1"/>
       <c r="C5" s="1"/>
@@ -1721,7 +1727,7 @@
       <c r="AC5" s="1"/>
       <c r="AD5" s="1"/>
     </row>
-    <row r="6" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A6" s="1"/>
       <c r="B6" s="1"/>
       <c r="D6" s="1"/>
@@ -1752,7 +1758,7 @@
       <c r="AC6" s="1"/>
       <c r="AD6" s="1"/>
     </row>
-    <row r="7" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A7" s="1"/>
       <c r="B7" s="1"/>
       <c r="C7" s="1"/>
@@ -1784,7 +1790,7 @@
       <c r="AC7" s="1"/>
       <c r="AD7" s="1"/>
     </row>
-    <row r="8" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A8" s="1"/>
       <c r="B8" s="1"/>
       <c r="C8" s="1"/>
@@ -1816,7 +1822,7 @@
       <c r="AC8" s="1"/>
       <c r="AD8" s="1"/>
     </row>
-    <row r="9" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A9" s="1"/>
       <c r="B9" s="1"/>
       <c r="C9" s="1"/>
@@ -1848,7 +1854,7 @@
       <c r="AC9" s="1"/>
       <c r="AD9" s="1"/>
     </row>
-    <row r="10" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A10" s="1"/>
       <c r="B10" s="1"/>
       <c r="C10" s="1"/>
@@ -1880,7 +1886,7 @@
       <c r="AC10" s="1"/>
       <c r="AD10" s="1"/>
     </row>
-    <row r="11" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A11" s="1"/>
       <c r="B11" s="1"/>
       <c r="C11" s="1"/>
@@ -1912,7 +1918,7 @@
       <c r="AC11" s="1"/>
       <c r="AD11" s="1"/>
     </row>
-    <row r="12" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A12" s="1"/>
       <c r="B12" s="1"/>
       <c r="C12" s="1"/>
@@ -1944,7 +1950,7 @@
       <c r="AC12" s="1"/>
       <c r="AD12" s="1"/>
     </row>
-    <row r="13" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A13" s="1"/>
       <c r="B13" s="1"/>
       <c r="C13" s="1"/>
@@ -1976,7 +1982,7 @@
       <c r="AC13" s="1"/>
       <c r="AD13" s="1"/>
     </row>
-    <row r="14" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A14" s="1"/>
       <c r="B14" s="1"/>
       <c r="C14" s="1"/>
@@ -2008,7 +2014,7 @@
       <c r="AC14" s="1"/>
       <c r="AD14" s="1"/>
     </row>
-    <row r="15" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A15" s="1"/>
       <c r="B15" s="1"/>
       <c r="C15" s="1"/>
@@ -2040,7 +2046,7 @@
       <c r="AC15" s="1"/>
       <c r="AD15" s="1"/>
     </row>
-    <row r="16" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A16" s="1"/>
       <c r="B16" s="1"/>
       <c r="C16" s="1"/>
@@ -2072,7 +2078,7 @@
       <c r="AC16" s="1"/>
       <c r="AD16" s="1"/>
     </row>
-    <row r="17" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A17" s="1"/>
       <c r="B17" s="1"/>
       <c r="C17" s="1"/>
@@ -2104,7 +2110,7 @@
       <c r="AC17" s="1"/>
       <c r="AD17" s="1"/>
     </row>
-    <row r="18" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A18" s="1"/>
       <c r="B18" s="1"/>
       <c r="C18" s="1"/>
@@ -2136,7 +2142,7 @@
       <c r="AC18" s="1"/>
       <c r="AD18" s="1"/>
     </row>
-    <row r="19" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A19" s="1"/>
       <c r="B19" s="1"/>
       <c r="C19" s="1"/>
@@ -2168,7 +2174,7 @@
       <c r="AC19" s="1"/>
       <c r="AD19" s="1"/>
     </row>
-    <row r="20" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A20" s="1"/>
       <c r="B20" s="1"/>
       <c r="C20" s="1"/>
@@ -2200,7 +2206,7 @@
       <c r="AC20" s="1"/>
       <c r="AD20" s="1"/>
     </row>
-    <row r="21" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A21" s="1"/>
       <c r="B21" s="1"/>
       <c r="C21" s="1"/>
@@ -2232,7 +2238,7 @@
       <c r="AC21" s="1"/>
       <c r="AD21" s="1"/>
     </row>
-    <row r="22" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A22" s="1"/>
       <c r="B22" s="1"/>
       <c r="C22" s="1"/>
@@ -2264,7 +2270,7 @@
       <c r="AC22" s="1"/>
       <c r="AD22" s="1"/>
     </row>
-    <row r="23" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A23" s="1"/>
       <c r="B23" s="1"/>
       <c r="C23" s="1"/>
@@ -2296,7 +2302,7 @@
       <c r="AC23" s="1"/>
       <c r="AD23" s="1"/>
     </row>
-    <row r="24" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A24" s="1"/>
       <c r="B24" s="1"/>
       <c r="C24" s="1"/>
@@ -2328,7 +2334,7 @@
       <c r="AC24" s="1"/>
       <c r="AD24" s="1"/>
     </row>
-    <row r="25" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A25" s="1"/>
       <c r="B25" s="1"/>
       <c r="C25" s="1"/>
@@ -2360,7 +2366,7 @@
       <c r="AC25" s="1"/>
       <c r="AD25" s="1"/>
     </row>
-    <row r="26" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A26" s="1"/>
       <c r="B26" s="1"/>
       <c r="C26" s="1"/>
@@ -2392,7 +2398,7 @@
       <c r="AC26" s="1"/>
       <c r="AD26" s="1"/>
     </row>
-    <row r="27" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A27" s="1"/>
       <c r="B27" s="1"/>
       <c r="C27" s="1"/>
@@ -2424,7 +2430,7 @@
       <c r="AC27" s="1"/>
       <c r="AD27" s="1"/>
     </row>
-    <row r="28" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A28" s="1"/>
       <c r="B28" s="1"/>
       <c r="C28" s="1"/>
@@ -2456,7 +2462,7 @@
       <c r="AC28" s="1"/>
       <c r="AD28" s="1"/>
     </row>
-    <row r="29" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A29" s="1"/>
       <c r="B29" s="1"/>
       <c r="C29" s="1"/>
@@ -2488,7 +2494,7 @@
       <c r="AC29" s="1"/>
       <c r="AD29" s="1"/>
     </row>
-    <row r="30" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A30" s="1"/>
       <c r="B30" s="1"/>
       <c r="C30" s="1"/>
@@ -2520,7 +2526,7 @@
       <c r="AC30" s="1"/>
       <c r="AD30" s="1"/>
     </row>
-    <row r="31" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A31" s="1"/>
       <c r="B31" s="1"/>
       <c r="C31" s="1"/>
@@ -2552,7 +2558,7 @@
       <c r="AC31" s="1"/>
       <c r="AD31" s="1"/>
     </row>
-    <row r="32" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A32" s="1"/>
       <c r="B32" s="1"/>
       <c r="C32" s="1"/>
@@ -2584,7 +2590,7 @@
       <c r="AC32" s="1"/>
       <c r="AD32" s="1"/>
     </row>
-    <row r="33" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A33" s="1"/>
       <c r="B33" s="1"/>
       <c r="C33" s="1"/>
@@ -2616,7 +2622,7 @@
       <c r="AC33" s="1"/>
       <c r="AD33" s="1"/>
     </row>
-    <row r="34" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A34" s="1"/>
       <c r="B34" s="1"/>
       <c r="C34" s="1"/>
@@ -2648,7 +2654,7 @@
       <c r="AC34" s="1"/>
       <c r="AD34" s="1"/>
     </row>
-    <row r="35" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A35" s="1"/>
       <c r="B35" s="1"/>
       <c r="C35" s="1"/>
@@ -2680,7 +2686,7 @@
       <c r="AC35" s="1"/>
       <c r="AD35" s="1"/>
     </row>
-    <row r="36" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A36" s="1"/>
       <c r="B36" s="1"/>
       <c r="C36" s="1"/>
@@ -2712,7 +2718,7 @@
       <c r="AC36" s="1"/>
       <c r="AD36" s="1"/>
     </row>
-    <row r="37" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A37" s="1"/>
       <c r="B37" s="1"/>
       <c r="C37" s="1"/>
@@ -2744,7 +2750,7 @@
       <c r="AC37" s="1"/>
       <c r="AD37" s="1"/>
     </row>
-    <row r="38" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A38" s="1"/>
       <c r="B38" s="1"/>
       <c r="C38" s="1"/>
@@ -2776,7 +2782,7 @@
       <c r="AC38" s="1"/>
       <c r="AD38" s="1"/>
     </row>
-    <row r="39" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A39" s="1"/>
       <c r="B39" s="1"/>
       <c r="C39" s="1"/>
@@ -2808,7 +2814,7 @@
       <c r="AC39" s="1"/>
       <c r="AD39" s="1"/>
     </row>
-    <row r="40" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A40" s="1"/>
       <c r="B40" s="1"/>
       <c r="C40" s="1"/>
@@ -2840,7 +2846,7 @@
       <c r="AC40" s="1"/>
       <c r="AD40" s="1"/>
     </row>
-    <row r="41" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A41" s="1"/>
       <c r="B41" s="1"/>
       <c r="C41" s="1"/>
@@ -2872,7 +2878,7 @@
       <c r="AC41" s="1"/>
       <c r="AD41" s="1"/>
     </row>
-    <row r="42" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A42" s="1"/>
       <c r="B42" s="1"/>
       <c r="C42" s="1"/>
@@ -2904,7 +2910,7 @@
       <c r="AC42" s="1"/>
       <c r="AD42" s="1"/>
     </row>
-    <row r="43" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A43" s="1"/>
       <c r="B43" s="1"/>
       <c r="C43" s="1"/>
@@ -2936,7 +2942,7 @@
       <c r="AC43" s="1"/>
       <c r="AD43" s="1"/>
     </row>
-    <row r="44" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A44" s="1"/>
       <c r="B44" s="1"/>
       <c r="C44" s="1"/>
@@ -2968,7 +2974,7 @@
       <c r="AC44" s="1"/>
       <c r="AD44" s="1"/>
     </row>
-    <row r="45" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A45" s="1"/>
       <c r="B45" s="1"/>
       <c r="C45" s="1"/>
@@ -3000,7 +3006,7 @@
       <c r="AC45" s="1"/>
       <c r="AD45" s="1"/>
     </row>
-    <row r="46" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A46" s="1"/>
       <c r="B46" s="1"/>
       <c r="C46" s="1"/>
@@ -3032,7 +3038,7 @@
       <c r="AC46" s="1"/>
       <c r="AD46" s="1"/>
     </row>
-    <row r="47" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A47" s="1"/>
       <c r="B47" s="1"/>
       <c r="C47" s="1"/>
@@ -3064,7 +3070,7 @@
       <c r="AC47" s="1"/>
       <c r="AD47" s="1"/>
     </row>
-    <row r="48" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A48" s="1"/>
       <c r="B48" s="1"/>
       <c r="C48" s="1"/>
@@ -3096,7 +3102,7 @@
       <c r="AC48" s="1"/>
       <c r="AD48" s="1"/>
     </row>
-    <row r="49" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A49" s="1"/>
       <c r="B49" s="1"/>
       <c r="C49" s="1"/>
@@ -3128,7 +3134,7 @@
       <c r="AC49" s="1"/>
       <c r="AD49" s="1"/>
     </row>
-    <row r="50" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A50" s="1"/>
       <c r="B50" s="1"/>
       <c r="C50" s="1"/>
@@ -3173,16 +3179,16 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C828B98D-AAA9-4184-8373-FE2E421AAE23}">
   <dimension ref="A1:E11"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="27" customWidth="1"/>
-    <col min="2" max="2" width="28.88671875" customWidth="1"/>
+    <col min="2" max="2" width="28.85546875" customWidth="1"/>
     <col min="3" max="3" width="41" customWidth="1"/>
-    <col min="4" max="4" width="36.109375" customWidth="1"/>
-    <col min="5" max="5" width="26.88671875" customWidth="1"/>
+    <col min="4" max="4" width="36.140625" customWidth="1"/>
+    <col min="5" max="5" width="26.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
         <v>32</v>
       </c>
@@ -3190,7 +3196,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:5" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="18" t="s">
         <v>20</v>
       </c>
@@ -3207,14 +3213,14 @@
         <v>59</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="14" t="s">
         <v>31</v>
       </c>
       <c r="B3" s="32" t="s">
         <v>61</v>
       </c>
-      <c r="C3" s="83" t="s">
+      <c r="C3" s="82" t="s">
         <v>25</v>
       </c>
       <c r="D3" s="44" t="s">
@@ -3224,7 +3230,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="12">
         <v>1</v>
       </c>
@@ -3243,7 +3249,7 @@
         <v>3234528921-25/11/2023</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="12">
         <v>2</v>
       </c>
@@ -3262,7 +3268,7 @@
         <v>3161657782-21/03/2024</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="12">
         <v>3</v>
       </c>
@@ -3281,7 +3287,7 @@
         <v>3119884321-21/09/2024</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="12">
         <v>4</v>
       </c>
@@ -3300,16 +3306,16 @@
         <v>4127359182-11/12/2025</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="C8" s="30"/>
       <c r="D8" s="30"/>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="C9" t="s">
         <v>214</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="C11" s="45"/>
     </row>
   </sheetData>
@@ -3329,15 +3335,15 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A24A074A-5C83-448D-978C-7C1005CE378E}">
   <dimension ref="A1:D7"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="29.109375" customWidth="1"/>
+    <col min="1" max="1" width="29.140625" customWidth="1"/>
     <col min="2" max="2" width="30" customWidth="1"/>
-    <col min="3" max="3" width="41.88671875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="61.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="41.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="61.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
         <v>32</v>
       </c>
@@ -3345,7 +3351,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="36.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:4" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="18" t="s">
         <v>20</v>
       </c>
@@ -3359,7 +3365,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="14" t="s">
         <v>31</v>
       </c>
@@ -3373,7 +3379,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="12">
         <v>1</v>
       </c>
@@ -3390,7 +3396,7 @@
         <v>Juan García-Motilada</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="12">
         <v>2</v>
       </c>
@@ -3407,7 +3413,7 @@
         <v>Juan Ortiz-Corte de barba</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="12">
         <v>3</v>
       </c>
@@ -3424,7 +3430,7 @@
         <v>Carlos Arbeladez-Perfilada de barba</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="12">
         <v>4</v>
       </c>
@@ -3464,14 +3470,14 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2921A3C4-B96A-49A7-8353-9FD37D2F2B74}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
-    <col min="2" max="2" width="42.33203125" customWidth="1"/>
-    <col min="3" max="3" width="37.44140625" customWidth="1"/>
+    <col min="2" max="2" width="42.28515625" customWidth="1"/>
+    <col min="3" max="3" width="37.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
         <v>32</v>
       </c>
@@ -3479,7 +3485,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="30" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A2" s="18" t="s">
         <v>20</v>
       </c>
@@ -3490,7 +3496,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="14" t="s">
         <v>31</v>
       </c>
@@ -3501,7 +3507,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="12">
         <v>1</v>
       </c>
@@ -3514,7 +3520,7 @@
         <v>Juan García</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="12">
         <v>2</v>
       </c>
@@ -3527,7 +3533,7 @@
         <v>Juan Ortiz</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="12">
         <v>3</v>
       </c>
@@ -3540,7 +3546,7 @@
         <v>Carlos Arbeladez</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="12">
         <v>4</v>
       </c>
@@ -3571,17 +3577,17 @@
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5CFE76D0-FBB4-4C81-85CC-F644057A8847}">
   <dimension ref="A1:F10"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="27" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="37.109375" customWidth="1"/>
+    <col min="2" max="2" width="37.140625" customWidth="1"/>
     <col min="3" max="3" width="28" customWidth="1"/>
-    <col min="4" max="4" width="18.6640625" customWidth="1"/>
-    <col min="5" max="5" width="31.6640625" customWidth="1"/>
-    <col min="6" max="6" width="37.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="18.7109375" customWidth="1"/>
+    <col min="5" max="5" width="31.7109375" customWidth="1"/>
+    <col min="6" max="6" width="37.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
         <v>32</v>
       </c>
@@ -3589,7 +3595,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="40.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:6" ht="40.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="19" t="s">
         <v>20</v>
       </c>
@@ -3609,7 +3615,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="14" t="s">
         <v>31</v>
       </c>
@@ -3619,17 +3625,17 @@
       <c r="C3" s="59" t="s">
         <v>77</v>
       </c>
-      <c r="D3" s="80" t="s">
+      <c r="D3" s="79" t="s">
         <v>65</v>
       </c>
-      <c r="E3" s="80" t="s">
+      <c r="E3" s="79" t="s">
         <v>87</v>
       </c>
       <c r="F3" s="29" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="12">
         <v>1</v>
       </c>
@@ -3651,7 +3657,7 @@
         <v>Juan García-Lunes-10-16</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="12">
         <v>2</v>
       </c>
@@ -3673,7 +3679,7 @@
         <v>Juan Ortiz-Martes-09-15</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="12">
         <v>3</v>
       </c>
@@ -3695,7 +3701,7 @@
         <v>Carlos Arbeladez-Jueves-13-19</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="12">
         <v>4</v>
       </c>
@@ -3717,8 +3723,8 @@
         <v>Andres Ramirez-Sábado-08-14</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="C10" s="60" t="s">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="C10" s="10" t="s">
         <v>177</v>
       </c>
     </row>
@@ -3740,19 +3746,19 @@
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1429879F-6697-4F1F-AF5D-52C4860B7B3E}">
   <dimension ref="A1:H15"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="28" customWidth="1"/>
-    <col min="2" max="2" width="26.5546875" customWidth="1"/>
-    <col min="3" max="3" width="30.44140625" customWidth="1"/>
-    <col min="4" max="4" width="27.5546875" customWidth="1"/>
-    <col min="5" max="5" width="36.5546875" customWidth="1"/>
-    <col min="6" max="6" width="60.33203125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="39.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="26.5703125" customWidth="1"/>
+    <col min="3" max="3" width="30.42578125" customWidth="1"/>
+    <col min="4" max="4" width="27.5703125" customWidth="1"/>
+    <col min="5" max="5" width="36.5703125" customWidth="1"/>
+    <col min="6" max="6" width="60.28515625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="39.28515625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="22" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
         <v>32</v>
       </c>
@@ -3760,7 +3766,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="36.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="18" t="s">
         <v>20</v>
       </c>
@@ -3783,7 +3789,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" s="14" t="s">
         <v>31</v>
       </c>
@@ -3793,7 +3799,7 @@
       <c r="C3" s="32" t="s">
         <v>62</v>
       </c>
-      <c r="D3" s="84" t="s">
+      <c r="D3" s="83" t="s">
         <v>137</v>
       </c>
       <c r="E3" s="44" t="s">
@@ -3806,7 +3812,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" s="12">
         <v>1</v>
       </c>
@@ -3832,7 +3838,7 @@
         <v>Juan García-30/09/2026/10:00</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" s="12">
         <v>2</v>
       </c>
@@ -3858,7 +3864,7 @@
         <v>Juan Ortiz-22/11/2025/11:00</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" s="12">
         <v>3</v>
       </c>
@@ -3884,7 +3890,7 @@
         <v>Carlos Arbeladez-10/08/2024/14:00</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="12">
         <v>4</v>
       </c>
@@ -3910,7 +3916,7 @@
         <v>Andres Ramirez-24/09/2026/13:00</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" s="12">
         <v>5</v>
       </c>
@@ -3937,24 +3943,24 @@
       </c>
       <c r="H8" s="49"/>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="H10" s="51"/>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="F11" s="60" t="s">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="F11" s="10" t="s">
         <v>215</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="D12" s="53"/>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="D13" s="53"/>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="D14" s="53"/>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="D15" s="53"/>
     </row>
   </sheetData>
@@ -3983,17 +3989,17 @@
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{766573FB-AAA2-4254-B83C-7C7505540365}">
   <dimension ref="A1:G7"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="26.6640625" customWidth="1"/>
-    <col min="2" max="2" width="38.5546875" customWidth="1"/>
-    <col min="3" max="3" width="39.33203125" bestFit="1" customWidth="1"/>
-    <col min="4" max="5" width="39.6640625" customWidth="1"/>
-    <col min="6" max="6" width="34.33203125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="39.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="26.7109375" customWidth="1"/>
+    <col min="2" max="2" width="38.5703125" customWidth="1"/>
+    <col min="3" max="3" width="39.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="39.7109375" customWidth="1"/>
+    <col min="6" max="6" width="34.28515625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="39.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
         <v>32</v>
       </c>
@@ -4001,7 +4007,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="31.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="18" t="s">
         <v>20</v>
       </c>
@@ -4024,7 +4030,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="14" t="s">
         <v>31</v>
       </c>
@@ -4047,7 +4053,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="12">
         <v>1</v>
       </c>
@@ -4074,7 +4080,7 @@
         <v>Carlos Arbeladez-10/08/2024/14:00</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="12">
         <v>2</v>
       </c>
@@ -4101,7 +4107,7 @@
         <v>Andres Ramirez-24/09/2026/13:00</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="10"/>
       <c r="B6" s="10"/>
       <c r="C6" s="10"/>
@@ -4110,7 +4116,7 @@
       <c r="F6" s="10"/>
       <c r="G6" s="10"/>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="10"/>
       <c r="B7" s="10"/>
       <c r="C7" s="10"/>
@@ -4137,17 +4143,17 @@
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F470C5A4-8D15-43DA-95FC-91C9614E5EEA}">
   <dimension ref="A1:F10"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="26.44140625" customWidth="1"/>
-    <col min="2" max="2" width="39.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="21.88671875" customWidth="1"/>
-    <col min="4" max="4" width="41.88671875" customWidth="1"/>
-    <col min="5" max="5" width="32.109375" customWidth="1"/>
-    <col min="6" max="6" width="55.88671875" customWidth="1"/>
+    <col min="1" max="1" width="26.42578125" customWidth="1"/>
+    <col min="2" max="2" width="39.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="21.85546875" customWidth="1"/>
+    <col min="4" max="4" width="41.85546875" customWidth="1"/>
+    <col min="5" max="5" width="32.140625" customWidth="1"/>
+    <col min="6" max="6" width="55.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
         <v>32</v>
       </c>
@@ -4155,7 +4161,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="33" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:6" ht="33" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="18" t="s">
         <v>20</v>
       </c>
@@ -4175,7 +4181,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="41" t="s">
         <v>31</v>
       </c>
@@ -4185,17 +4191,17 @@
       <c r="C3" s="32" t="s">
         <v>41</v>
       </c>
-      <c r="D3" s="78" t="s">
+      <c r="D3" s="77" t="s">
         <v>29</v>
       </c>
-      <c r="E3" s="78" t="s">
+      <c r="E3" s="77" t="s">
         <v>30</v>
       </c>
       <c r="F3" s="29" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="12">
         <v>1</v>
       </c>
@@ -4218,7 +4224,7 @@
         <v>Juan García-30/09/2026/10:00-Motilada</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="12">
         <v>2</v>
       </c>
@@ -4241,7 +4247,7 @@
         <v>Juan Ortiz-22/11/2025/11:00-Motilada</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="12">
         <v>3</v>
       </c>
@@ -4264,7 +4270,7 @@
         <v>Carlos Arbeladez-10/08/2024/14:00-Perfilada de barba</v>
       </c>
     </row>
-    <row r="7" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:6" ht="45" x14ac:dyDescent="0.25">
       <c r="A7" s="12">
         <v>4</v>
       </c>
@@ -4287,7 +4293,7 @@
         <v>Andres Ramirez-24/09/2026/13:00-Arreglo completo de barba con toalla caliente</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="12">
         <v>5</v>
       </c>
@@ -4309,7 +4315,7 @@
         <v>Carlos Arbeladez-06/08/2026/18:00-Corte de barba</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="D10" t="s">
         <v>219</v>
       </c>
@@ -4341,21 +4347,21 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7A5AA025-A9A3-4E3E-A766-44885AA770B6}">
-  <dimension ref="A1:D15"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:D17"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="27" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="63.6640625" customWidth="1"/>
-    <col min="3" max="3" width="14.44140625" customWidth="1"/>
-    <col min="4" max="4" width="7.6640625" customWidth="1"/>
+    <col min="2" max="2" width="63.7109375" customWidth="1"/>
+    <col min="3" max="3" width="14.42578125" customWidth="1"/>
+    <col min="4" max="4" width="7.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
         <v>0</v>
       </c>
@@ -4369,7 +4375,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:4" ht="45" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
         <v>4</v>
       </c>
@@ -4383,7 +4389,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="4" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:4" ht="75" x14ac:dyDescent="0.25">
       <c r="A4" s="7" t="s">
         <v>11</v>
       </c>
@@ -4397,7 +4403,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="5" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:4" ht="60" x14ac:dyDescent="0.25">
       <c r="A5" s="7" t="s">
         <v>5</v>
       </c>
@@ -4411,7 +4417,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="6" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:4" ht="45" x14ac:dyDescent="0.25">
       <c r="A6" s="7" t="s">
         <v>74</v>
       </c>
@@ -4425,7 +4431,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="7" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:4" ht="60" x14ac:dyDescent="0.25">
       <c r="A7" s="7" t="s">
         <v>6</v>
       </c>
@@ -4439,7 +4445,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="8" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:4" ht="45" x14ac:dyDescent="0.25">
       <c r="A8" s="7" t="s">
         <v>7</v>
       </c>
@@ -4453,7 +4459,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="9" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:4" ht="75" x14ac:dyDescent="0.25">
       <c r="A9" s="7" t="s">
         <v>13</v>
       </c>
@@ -4467,7 +4473,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="10" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A10" s="7" t="s">
         <v>8</v>
       </c>
@@ -4481,7 +4487,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="11" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:4" ht="45" x14ac:dyDescent="0.25">
       <c r="A11" s="7" t="s">
         <v>9</v>
       </c>
@@ -4495,26 +4501,22 @@
         <v>34</v>
       </c>
     </row>
-    <row r="12" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="7" t="s">
-        <v>75</v>
-      </c>
-      <c r="B12" s="8" t="s">
-        <v>161</v>
-      </c>
+        <v>221</v>
+      </c>
+      <c r="B12" s="8"/>
       <c r="C12" s="7">
         <v>4</v>
       </c>
-      <c r="D12" s="9" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" ht="72" x14ac:dyDescent="0.3">
+      <c r="D12" s="9"/>
+    </row>
+    <row r="13" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A13" s="7" t="s">
-        <v>10</v>
+        <v>75</v>
       </c>
       <c r="B13" s="8" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="C13" s="7">
         <v>4</v>
@@ -4523,31 +4525,55 @@
         <v>34</v>
       </c>
     </row>
-    <row r="14" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:4" ht="90" x14ac:dyDescent="0.25">
       <c r="A14" s="7" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>18</v>
+        <v>162</v>
       </c>
       <c r="C14" s="7">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D14" s="9" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="15" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" s="7" t="s">
-        <v>14</v>
-      </c>
-      <c r="B15" s="8" t="s">
-        <v>19</v>
-      </c>
+        <v>222</v>
+      </c>
+      <c r="B15" s="8"/>
       <c r="C15" s="7">
         <v>5</v>
       </c>
-      <c r="D15" s="9" t="s">
+      <c r="D15" s="9"/>
+    </row>
+    <row r="16" spans="1:4" ht="45" x14ac:dyDescent="0.25">
+      <c r="A16" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="B16" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="C16" s="7">
+        <v>5</v>
+      </c>
+      <c r="D16" s="9" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" ht="60" x14ac:dyDescent="0.25">
+      <c r="A17" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="B17" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="C17" s="7">
+        <v>5</v>
+      </c>
+      <c r="D17" s="9" t="s">
         <v>34</v>
       </c>
     </row>
@@ -4561,12 +4587,12 @@
     <hyperlink ref="D9" location="Veto_D!A1" display="aquí" xr:uid="{50EEB4A4-A05B-458F-A616-2C079D7BA2A1}"/>
     <hyperlink ref="D10" location="BarberoServicio_D!A1" display="aquí" xr:uid="{AC14820F-CB56-4CB4-B9D5-B9DDBC302113}"/>
     <hyperlink ref="D11" location="Agenda_D!A1" display="aquí" xr:uid="{F2DC45FC-06BF-43EC-8765-3A2CBBBD79CD}"/>
-    <hyperlink ref="D13" location="Cita_D!A1" display="aquí" xr:uid="{3BDFED20-FFB7-4345-9356-B30AC1240BDC}"/>
-    <hyperlink ref="D14" location="Multa_D!A1" display="aquí" xr:uid="{5D100657-ADBE-4AA9-A971-9C9D942C9DAD}"/>
-    <hyperlink ref="D15" location="CitaServicio_D!A1" display="aquí" xr:uid="{F49154C9-A497-4677-B686-F9CF5B536DEC}"/>
+    <hyperlink ref="D14" location="Cita_D!A1" display="aquí" xr:uid="{3BDFED20-FFB7-4345-9356-B30AC1240BDC}"/>
+    <hyperlink ref="D16" location="Multa_D!A1" display="aquí" xr:uid="{5D100657-ADBE-4AA9-A971-9C9D942C9DAD}"/>
+    <hyperlink ref="D17" location="CitaServicio_D!A1" display="aquí" xr:uid="{F49154C9-A497-4677-B686-F9CF5B536DEC}"/>
     <hyperlink ref="A1" location="'Modelo de Dominio'!A1" display="&lt;&lt;&lt;&lt; Ir al modulo de dominio" xr:uid="{A3D1E053-3C90-4C85-85FB-01CE6B92A5EE}"/>
     <hyperlink ref="D6" location="HorarioBarberia_D!A1" display="aquí" xr:uid="{CE45E0DE-1B75-4BE0-8664-81F7834039D9}"/>
-    <hyperlink ref="D12" location="HorarioBarbero_D!A1" display="aquí" xr:uid="{3B048927-BA4F-418A-BCDC-3E65406B8FD1}"/>
+    <hyperlink ref="D13" location="HorarioBarbero_D!A1" display="aquí" xr:uid="{3B048927-BA4F-418A-BCDC-3E65406B8FD1}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -4575,13 +4601,13 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{387DE6AC-7D92-461D-9DD1-84082B531231}">
   <dimension ref="A1:B11"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="18.44140625" customWidth="1"/>
-    <col min="2" max="2" width="62.77734375" customWidth="1"/>
+    <col min="1" max="1" width="18.42578125" customWidth="1"/>
+    <col min="2" max="2" width="62.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
         <v>172</v>
       </c>
@@ -4589,83 +4615,83 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A2" s="61" t="s">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" s="60" t="s">
         <v>173</v>
       </c>
-      <c r="B2" s="61" t="s">
+      <c r="B2" s="60" t="s">
         <v>184</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A3" s="62" t="s">
+    <row r="3" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+      <c r="A3" s="61" t="s">
         <v>174</v>
       </c>
-      <c r="B3" s="71" t="s">
+      <c r="B3" s="70" t="s">
         <v>185</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A4" s="64" t="s">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" s="63" t="s">
         <v>175</v>
       </c>
-      <c r="B4" s="64" t="s">
+      <c r="B4" s="63" t="s">
         <v>186</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A5" s="63" t="s">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" s="62" t="s">
         <v>212</v>
       </c>
-      <c r="B5" s="72" t="s">
+      <c r="B5" s="71" t="s">
         <v>213</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A6" s="65" t="s">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" s="64" t="s">
         <v>178</v>
       </c>
-      <c r="B6" s="65" t="s">
+      <c r="B6" s="64" t="s">
         <v>190</v>
       </c>
     </row>
-    <row r="7" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A7" s="66" t="s">
+    <row r="7" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+      <c r="A7" s="65" t="s">
         <v>179</v>
       </c>
-      <c r="B7" s="73" t="s">
+      <c r="B7" s="72" t="s">
         <v>187</v>
       </c>
     </row>
-    <row r="8" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A8" s="67" t="s">
+    <row r="8" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+      <c r="A8" s="66" t="s">
         <v>180</v>
       </c>
-      <c r="B8" s="74" t="s">
+      <c r="B8" s="73" t="s">
         <v>188</v>
       </c>
     </row>
-    <row r="9" spans="1:2" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A9" s="68" t="s">
+    <row r="9" spans="1:2" ht="45" x14ac:dyDescent="0.25">
+      <c r="A9" s="67" t="s">
         <v>181</v>
       </c>
-      <c r="B9" s="75" t="s">
+      <c r="B9" s="74" t="s">
         <v>189</v>
       </c>
     </row>
-    <row r="10" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A10" s="69" t="s">
+    <row r="10" spans="1:2" ht="45" x14ac:dyDescent="0.25">
+      <c r="A10" s="68" t="s">
         <v>182</v>
       </c>
-      <c r="B10" s="69" t="s">
+      <c r="B10" s="68" t="s">
         <v>191</v>
       </c>
     </row>
-    <row r="11" spans="1:2" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A11" s="70" t="s">
+    <row r="11" spans="1:2" ht="75" x14ac:dyDescent="0.25">
+      <c r="A11" s="69" t="s">
         <v>183</v>
       </c>
-      <c r="B11" s="76" t="s">
+      <c r="B11" s="75" t="s">
         <v>192</v>
       </c>
     </row>
@@ -4677,14 +4703,14 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AAA22F8C-1648-4644-8301-765EB2B8C50B}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="33.88671875" customWidth="1"/>
-    <col min="2" max="2" width="34.6640625" customWidth="1"/>
+    <col min="1" max="1" width="33.85546875" customWidth="1"/>
+    <col min="2" max="2" width="34.7109375" customWidth="1"/>
     <col min="3" max="3" width="21" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
         <v>32</v>
       </c>
@@ -4692,7 +4718,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="19" t="s">
         <v>20</v>
       </c>
@@ -4700,7 +4726,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="14" t="s">
         <v>31</v>
       </c>
@@ -4709,7 +4735,7 @@
       </c>
       <c r="C3" s="37"/>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="12">
         <v>1</v>
       </c>
@@ -4730,15 +4756,15 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{28259140-2713-4A98-8730-76D57DC1D653}">
   <dimension ref="A1:H11"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="26.88671875" style="10" customWidth="1"/>
-    <col min="2" max="6" width="26.33203125" style="10" customWidth="1"/>
-    <col min="7" max="7" width="23.109375" style="10" customWidth="1"/>
-    <col min="8" max="8" width="38.5546875" style="10" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="26.85546875" style="10" customWidth="1"/>
+    <col min="2" max="6" width="26.28515625" style="10" customWidth="1"/>
+    <col min="7" max="7" width="23.140625" style="10" customWidth="1"/>
+    <col min="8" max="8" width="38.5703125" style="10" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="11" t="s">
         <v>32</v>
       </c>
@@ -4752,7 +4778,7 @@
       <c r="G1" s="12"/>
       <c r="H1" s="12"/>
     </row>
-    <row r="2" spans="1:8" ht="39.6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" ht="46.5" x14ac:dyDescent="0.25">
       <c r="A2" s="18" t="s">
         <v>20</v>
       </c>
@@ -4778,7 +4804,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" s="14" t="s">
         <v>31</v>
       </c>
@@ -4794,17 +4820,17 @@
       <c r="E3" s="58" t="s">
         <v>108</v>
       </c>
-      <c r="F3" s="77" t="s">
+      <c r="F3" s="76" t="s">
         <v>164</v>
       </c>
-      <c r="G3" s="77" t="s">
+      <c r="G3" s="76" t="s">
         <v>22</v>
       </c>
       <c r="H3" s="15" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" s="12">
         <v>1</v>
       </c>
@@ -4827,7 +4853,7 @@
         <v>Juan--Gómez--+57-3234528921</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" s="12">
         <v>2</v>
       </c>
@@ -4854,7 +4880,7 @@
         <v>Jose-Miguel-Ramirez-Perez-+57-3161657782</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" s="12">
         <v>3</v>
       </c>
@@ -4879,7 +4905,7 @@
         <v>Simon--Ochoa-Ramirez-+57-3119884321</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="12">
         <v>4</v>
       </c>
@@ -4902,7 +4928,7 @@
         <v>Alexis--Gallego--+58-4127359182</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="C11"/>
     </row>
   </sheetData>
@@ -4918,17 +4944,17 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B0E77388-6266-4A55-B7A3-4FCD2B643D29}">
   <dimension ref="A1:F5"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="26.88671875" customWidth="1"/>
-    <col min="2" max="2" width="32.5546875" customWidth="1"/>
+    <col min="1" max="1" width="26.85546875" customWidth="1"/>
+    <col min="2" max="2" width="32.5703125" customWidth="1"/>
     <col min="3" max="3" width="28" customWidth="1"/>
-    <col min="4" max="4" width="26.6640625" customWidth="1"/>
-    <col min="5" max="5" width="16.33203125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="18.44140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="26.7109375" customWidth="1"/>
+    <col min="5" max="5" width="16.28515625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="18.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
         <v>32</v>
       </c>
@@ -4936,7 +4962,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="49.2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:6" ht="46.5" x14ac:dyDescent="0.25">
       <c r="A2" s="18" t="s">
         <v>20</v>
       </c>
@@ -4953,17 +4979,17 @@
         <v>70</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="14" t="s">
         <v>31</v>
       </c>
-      <c r="B3" s="78" t="s">
+      <c r="B3" s="77" t="s">
         <v>35</v>
       </c>
-      <c r="C3" s="78" t="s">
+      <c r="C3" s="77" t="s">
         <v>23</v>
       </c>
-      <c r="D3" s="78" t="s">
+      <c r="D3" s="77" t="s">
         <v>69</v>
       </c>
       <c r="E3" s="32" t="s">
@@ -4971,7 +4997,7 @@
       </c>
       <c r="F3" s="3"/>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="12">
         <v>1</v>
       </c>
@@ -4993,7 +5019,7 @@
         <v/>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="D5" s="2"/>
     </row>
   </sheetData>
@@ -5009,18 +5035,18 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2190E1EC-B79B-40C0-AC5B-0E2726DDD399}">
-  <dimension ref="A1:F11"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:F14"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="27" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="26" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="22.5546875" customWidth="1"/>
-    <col min="4" max="4" width="23.5546875" customWidth="1"/>
-    <col min="5" max="5" width="23.77734375" customWidth="1"/>
-    <col min="6" max="6" width="34.88671875" customWidth="1"/>
+    <col min="3" max="3" width="22.5703125" customWidth="1"/>
+    <col min="4" max="4" width="23.5703125" customWidth="1"/>
+    <col min="5" max="5" width="23.7109375" customWidth="1"/>
+    <col min="6" max="6" width="34.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
         <v>32</v>
       </c>
@@ -5028,7 +5054,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="44.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:6" ht="44.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="19" t="s">
         <v>20</v>
       </c>
@@ -5048,7 +5074,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="14" t="s">
         <v>31</v>
       </c>
@@ -5058,17 +5084,17 @@
       <c r="C3" s="59" t="s">
         <v>77</v>
       </c>
-      <c r="D3" s="79" t="s">
+      <c r="D3" s="78" t="s">
         <v>78</v>
       </c>
-      <c r="E3" s="80" t="s">
+      <c r="E3" s="79" t="s">
         <v>79</v>
       </c>
       <c r="F3" s="36" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="12">
         <v>1</v>
       </c>
@@ -5090,7 +5116,7 @@
         <v>Barbería Oriental-Lunes-09:00-19:00</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="12">
         <v>2</v>
       </c>
@@ -5112,7 +5138,7 @@
         <v>Barbería Oriental-Martes-09:00-19:00</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="12">
         <v>3</v>
       </c>
@@ -5134,7 +5160,7 @@
         <v>Barbería Oriental-Miércoles-09:00-19:00</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="12">
         <v>4</v>
       </c>
@@ -5156,7 +5182,7 @@
         <v>Barbería Oriental-Jueves-09:00-19:00</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="12">
         <v>5</v>
       </c>
@@ -5178,7 +5204,7 @@
         <v>Barbería Oriental-Viernes-09:00-19:00</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="12">
         <v>6</v>
       </c>
@@ -5200,14 +5226,19 @@
         <v>Barbería Oriental-Sábado-08:00-21:00</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="10"/>
       <c r="B10" s="39"/>
       <c r="C10" s="39"/>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="C11" s="10" t="s">
         <v>202</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B14" t="s">
+        <v>220</v>
       </c>
     </row>
   </sheetData>
@@ -5230,16 +5261,16 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C97B567D-D27E-4BE3-B1E4-8CA267790151}">
   <dimension ref="A1:F12"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="2" width="28.109375" customWidth="1"/>
-    <col min="3" max="3" width="26.5546875" customWidth="1"/>
-    <col min="4" max="4" width="24.44140625" customWidth="1"/>
-    <col min="5" max="5" width="25.33203125" customWidth="1"/>
-    <col min="6" max="6" width="26.5546875" customWidth="1"/>
+    <col min="1" max="2" width="28.140625" customWidth="1"/>
+    <col min="3" max="3" width="26.5703125" customWidth="1"/>
+    <col min="4" max="4" width="24.42578125" customWidth="1"/>
+    <col min="5" max="5" width="25.28515625" customWidth="1"/>
+    <col min="6" max="6" width="26.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="16" t="s">
         <v>32</v>
       </c>
@@ -5250,7 +5281,7 @@
       <c r="E1" s="17"/>
       <c r="F1" s="10"/>
     </row>
-    <row r="2" spans="1:6" ht="45.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:6" ht="45.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="18" t="s">
         <v>20</v>
       </c>
@@ -5270,27 +5301,27 @@
         <v>45</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="21" t="s">
         <v>31</v>
       </c>
       <c r="B3" s="55" t="s">
         <v>36</v>
       </c>
-      <c r="C3" s="81" t="s">
+      <c r="C3" s="80" t="s">
         <v>21</v>
       </c>
-      <c r="D3" s="82" t="s">
+      <c r="D3" s="81" t="s">
         <v>37</v>
       </c>
-      <c r="E3" s="82" t="s">
+      <c r="E3" s="81" t="s">
         <v>24</v>
       </c>
       <c r="F3" s="15" t="s">
         <v>207</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="22">
         <v>1</v>
       </c>
@@ -5312,7 +5343,7 @@
         <v>Motilada</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="22">
         <v>2</v>
       </c>
@@ -5334,7 +5365,7 @@
         <v>Corte de barba</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="22">
         <v>3</v>
       </c>
@@ -5356,7 +5387,7 @@
         <v>Perfilada de barba</v>
       </c>
     </row>
-    <row r="7" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A7" s="22">
         <v>4</v>
       </c>
@@ -5378,35 +5409,35 @@
         <v>Arreglo completo de barba con toalla caliente</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="17"/>
       <c r="B8" s="17"/>
       <c r="C8" s="17"/>
       <c r="D8" s="17"/>
       <c r="E8" s="17"/>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="17"/>
       <c r="B9" s="17"/>
       <c r="C9" s="17"/>
       <c r="D9" s="17"/>
       <c r="E9" s="17"/>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="17"/>
       <c r="B10" s="17"/>
       <c r="C10" s="17"/>
       <c r="D10" s="17"/>
       <c r="E10" s="17"/>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="17"/>
       <c r="B11" s="17"/>
       <c r="C11" s="17"/>
       <c r="D11" s="17"/>
       <c r="E11" s="17"/>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="17"/>
       <c r="B12" s="17"/>
       <c r="C12" s="17"/>
@@ -5430,18 +5461,18 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2DAE59AB-4103-4731-9C3C-4C276F8A29F8}">
   <dimension ref="A1:L14"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="27" bestFit="1" customWidth="1"/>
-    <col min="2" max="6" width="26.6640625" customWidth="1"/>
-    <col min="7" max="7" width="16.33203125" customWidth="1"/>
-    <col min="8" max="9" width="40.6640625" customWidth="1"/>
-    <col min="10" max="10" width="30.33203125" customWidth="1"/>
+    <col min="2" max="6" width="26.7109375" customWidth="1"/>
+    <col min="7" max="7" width="16.28515625" customWidth="1"/>
+    <col min="8" max="9" width="40.7109375" customWidth="1"/>
+    <col min="10" max="10" width="30.28515625" customWidth="1"/>
     <col min="11" max="11" width="21" customWidth="1"/>
-    <col min="12" max="12" width="53.109375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="53.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
         <v>32</v>
       </c>
@@ -5453,7 +5484,7 @@
       <c r="E1" s="5"/>
       <c r="F1" s="5"/>
     </row>
-    <row r="2" spans="1:12" ht="45.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:12" ht="45.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="26" t="s">
         <v>20</v>
       </c>
@@ -5491,7 +5522,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A3" s="14" t="s">
         <v>31</v>
       </c>
@@ -5507,16 +5538,16 @@
       <c r="E3" s="58" t="s">
         <v>108</v>
       </c>
-      <c r="F3" s="77" t="s">
+      <c r="F3" s="76" t="s">
         <v>132</v>
       </c>
-      <c r="G3" s="77" t="s">
+      <c r="G3" s="76" t="s">
         <v>22</v>
       </c>
-      <c r="H3" s="77" t="s">
+      <c r="H3" s="76" t="s">
         <v>42</v>
       </c>
-      <c r="I3" s="77" t="s">
+      <c r="I3" s="76" t="s">
         <v>128</v>
       </c>
       <c r="J3" s="44" t="s">
@@ -5529,7 +5560,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A4" s="12">
         <v>1</v>
       </c>
@@ -5569,7 +5600,7 @@
         <v>Juan-Fernando-García-Lopez-+57-3245627890</v>
       </c>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A5" s="12">
         <v>2</v>
       </c>
@@ -5609,7 +5640,7 @@
         <v>Juan-David-Ortiz-Sanchez-+57-3124518923</v>
       </c>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A6" s="12">
         <v>3</v>
       </c>
@@ -5645,7 +5676,7 @@
         <v>Carlos--Arbeladez--+57-3214533321</v>
       </c>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A7" s="12">
         <v>4</v>
       </c>
@@ -5683,7 +5714,7 @@
         <v>Andres--Ramirez-Patiño-+91-9876543210</v>
       </c>
     </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A8" s="12">
         <v>5</v>
       </c>
@@ -5723,11 +5754,11 @@
         <v>Juan-Carlos-Zambrano-Perez-+593-998765432</v>
       </c>
     </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B10" s="10"/>
       <c r="C10" s="10"/>
     </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F14" t="s">
         <v>169</v>
       </c>

</xml_diff>

<commit_message>
Se definieron los atributos de los dos nuevos objetos de dominio. Tambien se defienieron los tipos de datos de cada uno con su valor por defecto, si es permitido o no
</commit_message>
<xml_diff>
--- a/Muestreo de datos.xlsx
+++ b/Muestreo de datos.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/120f6d501c463b80/Escritorio/leo/Doo/Barberia proyecto/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="9" documentId="13_ncr:1_{7D2C82A5-CE11-488F-916B-C5EEB7B95CE2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9F3D621B-2D43-45EE-A08C-EA5144B4F136}"/>
+  <xr:revisionPtr revIDLastSave="407" documentId="13_ncr:1_{7D2C82A5-CE11-488F-916B-C5EEB7B95CE2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{84D6F366-4DCB-4DED-829F-90BD42E34150}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" firstSheet="1" activeTab="1" xr2:uid="{09A6C7D7-663F-4C06-9D71-8A4E97495CF9}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{09A6C7D7-663F-4C06-9D71-8A4E97495CF9}"/>
   </bookViews>
   <sheets>
     <sheet name="Modelo de Dominio" sheetId="1" r:id="rId1"/>
@@ -25,10 +25,12 @@
     <sheet name="Veto_D" sheetId="10" r:id="rId10"/>
     <sheet name="BarberoServicio_D" sheetId="11" r:id="rId11"/>
     <sheet name="Agenda_D" sheetId="12" r:id="rId12"/>
-    <sheet name="HorarioBarbero_D" sheetId="20" r:id="rId13"/>
-    <sheet name="Cita_D" sheetId="13" r:id="rId14"/>
-    <sheet name="Multa_D" sheetId="16" r:id="rId15"/>
-    <sheet name="CitaServicio_D" sheetId="17" r:id="rId16"/>
+    <sheet name="Bloqueo_D" sheetId="22" r:id="rId13"/>
+    <sheet name="HorarioBarbero_D" sheetId="20" r:id="rId14"/>
+    <sheet name="Descanso_D" sheetId="23" r:id="rId15"/>
+    <sheet name="Cita_D" sheetId="13" r:id="rId16"/>
+    <sheet name="Multa_D" sheetId="16" r:id="rId17"/>
+    <sheet name="CitaServicio_D" sheetId="17" r:id="rId18"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -54,7 +56,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="336" uniqueCount="223">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="376" uniqueCount="244">
   <si>
     <t>Nombre</t>
   </si>
@@ -230,13 +232,7 @@
     <t>activo</t>
   </si>
   <si>
-    <t>Representa el numero de celular del cliente al que se veto, es decir al que no se le podra agendar más citas</t>
-  </si>
-  <si>
     <t>Combinacion única que indica que no puede existir más de un veto con el mismo cliente y la misma fecha</t>
-  </si>
-  <si>
-    <t>Representa la fecha en el que se veto al cliente, por acomular y no pagar las multas, el numero para que se de el veto lo define la regla de la barbería</t>
   </si>
   <si>
     <t>numeroCelularCliente</t>
@@ -324,12 +320,6 @@
 Hace referencia a la agenda (y por lo tanto al barbero) a la que pertenece este horario, permite saber de quién es cada bloque de disponibilidad</t>
   </si>
   <si>
-    <t>Representa la hora en la que el barbero empieza a estar disponible ese dia</t>
-  </si>
-  <si>
-    <t>Representa la hora en la que el barbero deja de estar disponible ese día, junto con horaInicio, es lo que la aplicación usa para saber si hay campo para agendar una cita nueva</t>
-  </si>
-  <si>
     <t>Combinación única que indica que una misma agenda no puede tener dos horarios distintos para el mismo día</t>
   </si>
   <si>
@@ -463,9 +453,6 @@
   </si>
   <si>
     <t>+91</t>
-  </si>
-  <si>
-    <t>Representa si el barbero sigue o no trabajando en la barberia, es un dato calculado cuando el barbero tiene en su agenda un horario de trabajo si es vigente y si no tiene horario de trabajo dice no es vigente</t>
   </si>
   <si>
     <t>fechaHora</t>
@@ -478,9 +465,6 @@
     <t>retraso</t>
   </si>
   <si>
-    <t xml:space="preserve">Representa cuanto dinero en pesos colombianos debe pagar el cliente la multa, si es por retraso se el monto es el que dice en regla y si es por incumplida el monto es del o los servicios que pidio </t>
-  </si>
-  <si>
     <t>Combinacion única que indica que no puede existir más de un cliente con un mismo nombre, apellidos, prefijo de celular y número de celular</t>
   </si>
   <si>
@@ -496,9 +480,6 @@
     <t>Hace referencia a en la agenda de que barbero quedó registrada esta cita, es lo que permite validar que no se cruce con otra cita del mismo barbero</t>
   </si>
   <si>
-    <t>Representa en que momento del proceso está la cita: agendada (se creó y espera a que el cliente llegue), atendida (la cita se cumplió sin ningún inconveniente), retraso (el cliente llegó, pero pasada la tolerancia de tiempo) ,incumplida (el cliente nunca llegó) o cancelada (el cliente avisó con anticipación que ya no la quiere)</t>
-  </si>
-  <si>
     <t>tipo</t>
   </si>
   <si>
@@ -547,9 +528,6 @@
     <t>Representa la reserva de un cliente con un barbero para una fecha y hora puntual. De ella sale tanto el cálculo de cuanto queda ocupado el barbero como la funcionalidad de si hay o no una multa (se genera cuando un barbero pone el estado de la cita en retraso o inclumplida), según cómo haya terminado (atendida, con retraso, incumplida o cancelada)</t>
   </si>
   <si>
-    <t>Representa el nombre de como se llama la barberia en donde trabajan los barberos. El tipo de dato es alfanumérico, su valor por defecto es el vacio y es permitido</t>
-  </si>
-  <si>
     <t>prefijoCelular</t>
   </si>
   <si>
@@ -565,9 +543,6 @@
     <t>Representa el segundo apellido del barbero que trabaja en la barbería. Su tipo de dato es texto, su valor por defecto es el vacio y es permitido</t>
   </si>
   <si>
-    <t>Realmente se necesita saber el numero del barbero</t>
-  </si>
-  <si>
     <t>Representa de que pais es el numero de celular del barbero. Su tipo de dato es alfanumérico, su valor por defecto es +0 y no es permitido</t>
   </si>
   <si>
@@ -586,12 +561,6 @@
     <t>Entero</t>
   </si>
   <si>
-    <t>Representa el día de la semana en que aplica este horario, es necesario porque un barbero puede trabajar unos días sí y otros no. Su valor por defecto es el vacío y no es permitido</t>
-  </si>
-  <si>
-    <t>Este dato también lo tengo pensado como una lista. Lo dejé como tipo texto</t>
-  </si>
-  <si>
     <t>FechaHora</t>
   </si>
   <si>
@@ -601,9 +570,6 @@
     <t>Identificador unico</t>
   </si>
   <si>
-    <t>Combinacion unica</t>
-  </si>
-  <si>
     <t>Referencia de otros objetos de dominio</t>
   </si>
   <si>
@@ -649,33 +615,12 @@
     <t>Representa el primer apellido de la persona, que va a estar llendo a la barberia para las citas. Su valor por defecto es el vacío y es permitido</t>
   </si>
   <si>
-    <t>Representa de que pais es el numero de celular del cliente. Su valor por defecto es +0 (este prefijo no referencia a ningún país) y no es permitido</t>
-  </si>
-  <si>
     <t>Representa el numero de celular de la persona que le va a escribir al barbero por WhatsApp para pedirle una cita. Su valor por defecto es el 0 y no es permitido</t>
   </si>
   <si>
-    <t>Representa la cantidad de minutos que el cliente puede llegarle tarde un cliente a la cita establecida con el barbero, despues de eso el barbero lo podrá multar. Debe de ser mayor o igual a 0, su valor por defecto es el 0 y es permitido</t>
-  </si>
-  <si>
     <t>Representa la cantidad de dinero que el cliente debe de pagar en pesos colombianos, por superar la toleranciaTardanza. Debe de ser mayor a cero, su valor por defecto es 0 y no es permitido</t>
   </si>
   <si>
-    <t>Representa la maxima de multas que pueda tener un cliente sin pagar, a partir de esta cantidad se le hace un veto al cliente. Debe de ser mayor o igual a cero, su valor por defecto es 0 y es permitido</t>
-  </si>
-  <si>
-    <t>Este dato lo tengo pensado como si fuera una lista, pero no se si esta bien dejarlo tipo texto</t>
-  </si>
-  <si>
-    <t>Representa el día de la semana en que aplica este horario, es necesario para saber que días abrira la barberia. Su valor por defecto es el vacio y no es permitido</t>
-  </si>
-  <si>
-    <t>Representa la hora a la que abre la barbería. Su valor por defecto es 00:00 am y es permitido</t>
-  </si>
-  <si>
-    <t>Representa la hora a la que cierra la barbería. Su valor por defecto es 00:00 am y es permitido</t>
-  </si>
-  <si>
     <t>Representa el nombre del servicio que va estar en la barberia, que el barbero ofrece y en las citas que esta. Su valor por defecto es el vacio y no es permitido</t>
   </si>
   <si>
@@ -700,31 +645,152 @@
     <t>Tipo de dato que contiene el día, mes y el año.</t>
   </si>
   <si>
-    <t>Este es calculado o lo pone el barbero?</t>
-  </si>
-  <si>
-    <t>Tengo pensado que este sea de tipo texto, su valor por defecto sería el vacío y no sería permitido</t>
-  </si>
-  <si>
     <t>Representa la fecha y la hora en el que se va a realizar la cita al cliente. Su valor por defecto es 01/01/1000 00:00 y no es permitido</t>
   </si>
   <si>
-    <t>Representa cuanto valía el servicio en el momento exacto en que se agendó la cita, se guarda aparte del precio del catalogo por si el precio de ese servicio cambia después, las citas ya registradas no se vean afectadas. Debe de ser mayor a cero, su valor por defecto es el 0 y no es permitido</t>
-  </si>
-  <si>
-    <t>Sera que este es calculado o lo pone le barbero</t>
-  </si>
-  <si>
-    <t>Sera que este es calculado o lo pone el barbero</t>
-  </si>
-  <si>
-    <t>Este objeto de dominio puede no tener ninguna instancia, o es necesario que halla uno</t>
-  </si>
-  <si>
     <t>Bloqueo</t>
   </si>
   <si>
     <t>Descanso</t>
+  </si>
+  <si>
+    <t>Representa los momentos dentro del horario semanal de un barbero en los que no está disponible para atender, aunque ese día sí trabaje (por ejemplo, la hora del almuerzo). Se repite cada semana junto con el HorarioBarbero al que pertenece</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+Hace referencia a la agenda (y por lo tanto al barbero) a la que pertenece este bloqueo, permite saber en cual agenda se va agregar el bloqueo</t>
+  </si>
+  <si>
+    <t>horaFinal</t>
+  </si>
+  <si>
+    <t>Combinación única que indica que una misma agenda no puede tener dos bloqueos en una misma fecha, horaInicio y horaFinal</t>
+  </si>
+  <si>
+    <t>horarioDelBarbero</t>
+  </si>
+  <si>
+    <t>Hace referencia al dia y las horas que trabaja el barbero</t>
+  </si>
+  <si>
+    <t>Hora de almuerzo</t>
+  </si>
+  <si>
+    <t>Hora en la que almuezo</t>
+  </si>
+  <si>
+    <t>Descansito</t>
+  </si>
+  <si>
+    <t>Hora de descanso</t>
+  </si>
+  <si>
+    <t>Cita medica</t>
+  </si>
+  <si>
+    <t>Vueltas que voy a hacer</t>
+  </si>
+  <si>
+    <t>Incoveniente</t>
+  </si>
+  <si>
+    <t>Compromiso</t>
+  </si>
+  <si>
+    <t>Combinación única que indica que un mismo horario no puede tener dos mismas horas en la que empieze y termine</t>
+  </si>
+  <si>
+    <t>Representa el nombre de como se llama la barberia en donde trabajan los barberos. El tipo de dato es alfanumérico, su valor por defecto es el vacio y es no es permitido</t>
+  </si>
+  <si>
+    <t>Representa el día de la semana en que aplica este horario, es necesario para saber que días abrirá la barberia. Su valor por defecto es el vacio y no es permitido, el barbero solo podra seleccionar los días de la semana</t>
+  </si>
+  <si>
+    <t>Representa la cantidad de minutos que el cliente puede llegarle tarde un cliente a la cita establecida con el barbero, despues de eso el barbero lo podrá multar. Debe de ser mayor o igual a 0, su valor por defecto es el 0 y no es permitido</t>
+  </si>
+  <si>
+    <t>Representa la maxima de multas que pueda tener un cliente sin pagar, a partir de esta cantidad se le hace un veto al cliente. Debe de ser mayor o igual a cero, su valor por defecto es 0 y es no es permitido</t>
+  </si>
+  <si>
+    <t>Representa si el barbero sigue o no trabajando en la barberia. Es un dato calculado, si el barbero tiene en su agenda un horario de trabajo si es vigente y si no tiene horario de trabajo dice no es vigente</t>
+  </si>
+  <si>
+    <t>Representa la fecha en el que se veto al cliente, por acomular y no pagar las multas, el numero para que se de el veto lo define la regla de la barbería. Es un dato calculado, el sistema lo genra cuando detecta que un cliente acaba de tener el numero de multas maximas sin pagar</t>
+  </si>
+  <si>
+    <t>Representa como el barbero va a llamar este bloqueo para su agenda. Su valor por defecto es el vacio y no es permitido</t>
+  </si>
+  <si>
+    <t>Representa cuanto valía el servicio en el momento exacto en que se agendó la cita, se guarda aparte del precio del catalogo por si el precio de ese servicio cambia después, las citas ya registradas no se vean afectadas</t>
+  </si>
+  <si>
+    <t>Representa de que pais es el numero de celular del cliente. Su valor por defecto es +0 (este prefijo no representa a ningún país) y no es permitido</t>
+  </si>
+  <si>
+    <t>nombreCliente</t>
+  </si>
+  <si>
+    <t>Representa el nombre completo del cliente con lo que lo registró el barbero</t>
+  </si>
+  <si>
+    <t>prefijoCelularCliente</t>
+  </si>
+  <si>
+    <t>Representa el nombre del descanso que el barbero considere para su horario de trabajo. Su valor por defecto es vacio y no es permitido</t>
+  </si>
+  <si>
+    <t>Representa la cantidad de minutos dura el descanso de la agenda. Es un dato calculado a partir de la horaInicio y horaFinal, usando horaFinal - horaInicio</t>
+  </si>
+  <si>
+    <t>Representa en que momento del proceso está la cita: agendada (se creó y espera a que el cliente llegue), atendida (la cita se cumplió sin ningún inconveniente), retraso (el cliente llegó, pero pasada la tolerancia de tiempo) ,incumplida (el cliente nunca llegó) o cancelada (el cliente avisó con anticipación que ya no la quiere). Su valor por defecto es agenda y es permitido</t>
+  </si>
+  <si>
+    <t>Representa cuanto dinero en pesos colombianos debe pagar el cliente la multa. Es un dato calculado si es por retraso el monto es el que dice en regla y si es por incumplida el monto es del o los servicios que pidió</t>
+  </si>
+  <si>
+    <t>fechaHoraInicio</t>
+  </si>
+  <si>
+    <t>fechaHoraFinal</t>
+  </si>
+  <si>
+    <t>Representa un momento puntual en una fecha y hora específica, en el que un barbero no puede trabajar por un compromiso personal, aunque ese día normalmente sí trabaje según su horario. A diferencia de Descanso, no se repite semana a semana: aplica solo para esa fecha y hora, y es lo que le permite a la agenda del barbero reflejar cambios temporales sin alterar su horario habitual.</t>
+  </si>
+  <si>
+    <t>Representa la fecha y la hora en el que va a empezar el bloqueo para la agenda del barbero. Su valor por defecto es 01/01/1000 00:00 y no es permitido. No se puden seleccionar fechas antes del momento de hoy, solo fechas futuras</t>
+  </si>
+  <si>
+    <t>Representa la fecha y la hora en el que va a terminar el bloqueo para la agenda del barbero. Su valor por defecto es 01/01/1000 00:00 y no es permitido, la fecha debe de ser mayor a la fecha de inicio</t>
+  </si>
+  <si>
+    <t>Representa la cantidad de minutos dura el bloqueo de la agenda. Es un dato calculado a partir de la fechaHoraInicio y fechaHoraFinal</t>
+  </si>
+  <si>
+    <t>Representa la hora a la que abre la barbería. Su valor por defecto es 00:00 y es permitido</t>
+  </si>
+  <si>
+    <t>Representa el prefijo del celular del cliente, para que los barberos sepan el prefijo del cliente</t>
+  </si>
+  <si>
+    <t>Representa el numero de celular del cliente al que se veto, es decir al que no se le podrá agendar más citas. De modo que sepan los barberos el número del cliente que no van a agendar</t>
+  </si>
+  <si>
+    <t>Representa el día de la semana en que aplica este horario que para la agenda del barbero, es necesario porque un barbero puede trabajar unos días sí y otros no. Su valor por defecto es el vacío y no es permitido, el barbero solo podra seleccionar los días de la semana que la barberia tiene en su horario</t>
+  </si>
+  <si>
+    <t>Representa la hora en la que el barbero empieza a estar disponible ese dia. Su valor por defecto es 00:00 y es permitido. La hora debe de estar dentro del horario barberia</t>
+  </si>
+  <si>
+    <t>Representa la hora a la que cierra la barbería. Su valor por defecto es 00:00 y no es permitido</t>
+  </si>
+  <si>
+    <t>Representa la hora en la que el barbero deja de estar disponible ese día, junto con horaInicio, es lo que la aplicación usa para saber si hay campo para agendar una cita nueva. Su valor por defecto es 00:00 y no es permitido. Esta hora debe de ser mayor a horaInicio y también debe de estar dentro de horario barberia</t>
+  </si>
+  <si>
+    <t>Representa la hora en que el barbero termina su descanso de trabajo. Su valor por defecto es 00:00 no es permitido. La hora debe de ser mayor a la horaInicio y debe estar dentro del horario barbero</t>
+  </si>
+  <si>
+    <t>Representa la hora en que el barbero empieza su descanso de trabajo. Su valor por defecto es 00:00 y es permitido. La hora debe de estar dentro del horario del barbero, es decir que no se puede salir del horario</t>
   </si>
 </sst>
 </file>
@@ -921,7 +987,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="84">
+  <cellXfs count="95">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -945,9 +1011,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1009,9 +1072,6 @@
     <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1022,9 +1082,6 @@
     <xf numFmtId="18" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="18" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1073,9 +1130,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="13" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
@@ -1126,10 +1180,53 @@
     <xf numFmtId="0" fontId="5" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="18" fontId="8" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="18" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="18" fontId="8" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="10" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="14" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="22" fontId="8" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="22" fontId="8" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="20" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="20" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -1160,22 +1257,22 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>202045</xdr:colOff>
-      <xdr:row>2</xdr:row>
-      <xdr:rowOff>192423</xdr:rowOff>
+      <xdr:colOff>259773</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>67347</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>18</xdr:col>
-      <xdr:colOff>329247</xdr:colOff>
-      <xdr:row>31</xdr:row>
-      <xdr:rowOff>163560</xdr:rowOff>
+      <xdr:col>16</xdr:col>
+      <xdr:colOff>752223</xdr:colOff>
+      <xdr:row>33</xdr:row>
+      <xdr:rowOff>48106</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="Imagen 1">
+        <xdr:cNvPr id="3" name="Imagen 2">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{ABE419C4-ED6D-F2DD-03E4-99972CEE0EE1}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{7B8920B4-D75C-E415-61FF-DF31117E7B38}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1198,8 +1295,8 @@
       </xdr:blipFill>
       <xdr:spPr bwMode="auto">
         <a:xfrm>
-          <a:off x="202045" y="577271"/>
-          <a:ext cx="14799550" cy="5551441"/>
+          <a:off x="259773" y="644620"/>
+          <a:ext cx="13644647" cy="5753486"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1219,6 +1316,10 @@
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1760,7 +1861,6 @@
     </row>
     <row r="7" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A7" s="1"/>
-      <c r="B7" s="1"/>
       <c r="C7" s="1"/>
       <c r="D7" s="1"/>
       <c r="E7" s="1"/>
@@ -3178,155 +3278,205 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C828B98D-AAA9-4184-8373-FE2E421AAE23}">
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:G11"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="27" customWidth="1"/>
-    <col min="2" max="2" width="28.85546875" customWidth="1"/>
-    <col min="3" max="3" width="41" customWidth="1"/>
-    <col min="4" max="4" width="36.140625" customWidth="1"/>
-    <col min="5" max="5" width="26.85546875" customWidth="1"/>
+    <col min="1" max="2" width="27" customWidth="1"/>
+    <col min="3" max="4" width="28.85546875" customWidth="1"/>
+    <col min="5" max="5" width="41" customWidth="1"/>
+    <col min="6" max="6" width="36.140625" customWidth="1"/>
+    <col min="7" max="7" width="26.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
         <v>32</v>
       </c>
       <c r="B1" s="5" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="2" spans="1:5" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="18" t="s">
+      <c r="D1" s="5"/>
+    </row>
+    <row r="2" spans="1:7" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="17" t="s">
         <v>20</v>
       </c>
-      <c r="B2" s="18" t="s">
+      <c r="B2" s="17" t="s">
+        <v>236</v>
+      </c>
+      <c r="C2" s="17" t="s">
+        <v>237</v>
+      </c>
+      <c r="D2" s="17" t="s">
+        <v>223</v>
+      </c>
+      <c r="E2" s="30" t="s">
+        <v>218</v>
+      </c>
+      <c r="F2" s="30" t="s">
+        <v>123</v>
+      </c>
+      <c r="G2" s="30" t="s">
         <v>58</v>
       </c>
-      <c r="C2" s="31" t="s">
-        <v>60</v>
-      </c>
-      <c r="D2" s="31" t="s">
-        <v>127</v>
-      </c>
-      <c r="E2" s="31" t="s">
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" s="13" t="s">
+        <v>31</v>
+      </c>
+      <c r="B3" s="31" t="s">
+        <v>224</v>
+      </c>
+      <c r="C3" s="31" t="s">
         <v>59</v>
       </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" s="14" t="s">
-        <v>31</v>
-      </c>
-      <c r="B3" s="32" t="s">
-        <v>61</v>
-      </c>
-      <c r="C3" s="82" t="s">
+      <c r="D3" s="31" t="s">
+        <v>222</v>
+      </c>
+      <c r="E3" s="41" t="s">
         <v>25</v>
       </c>
-      <c r="D3" s="44" t="s">
+      <c r="F3" s="41" t="s">
         <v>57</v>
       </c>
-      <c r="E3" s="29" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="G3" s="28" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="12">
         <v>1</v>
       </c>
-      <c r="B4" s="11">
+      <c r="B4" s="92" t="str">
+        <f>Cliente_D!F4</f>
+        <v>+57</v>
+      </c>
+      <c r="C4" s="11">
         <f>Cliente_D!G4</f>
         <v>3234528921</v>
       </c>
-      <c r="C4" s="33">
+      <c r="D4" s="11" t="str">
+        <f>_xlfn.CONCAT(Cliente_D!B4," ",Cliente_D!C4," ",Cliente_D!D4," ",Cliente_D!E4)</f>
+        <v xml:space="preserve">Juan  Gómez </v>
+      </c>
+      <c r="E4" s="32">
         <v>45255</v>
       </c>
-      <c r="D4" s="12" t="s">
+      <c r="F4" s="12" t="s">
         <v>50</v>
       </c>
-      <c r="E4" s="12" t="str">
-        <f>_xlfn.CONCAT(B4,"-",TEXT(C4,"dd/mm/yyyy"))</f>
+      <c r="G4" s="12" t="str">
+        <f>_xlfn.CONCAT(C4,"-",TEXT(E4,"dd/mm/yyyy"))</f>
         <v>3234528921-25/11/2023</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="12">
         <v>2</v>
       </c>
-      <c r="B5" s="11">
+      <c r="B5" s="92" t="str">
+        <f>Cliente_D!F5</f>
+        <v>+57</v>
+      </c>
+      <c r="C5" s="11">
         <f>Cliente_D!G5</f>
         <v>3161657782</v>
       </c>
-      <c r="C5" s="33">
+      <c r="D5" s="11" t="str">
+        <f>_xlfn.CONCAT(Cliente_D!B5," ",Cliente_D!C5," ",Cliente_D!D5," ",Cliente_D!E5)</f>
+        <v>Jose Miguel Ramirez Perez</v>
+      </c>
+      <c r="E5" s="32">
         <v>45372</v>
       </c>
-      <c r="D5" s="12" t="s">
+      <c r="F5" s="12" t="s">
         <v>50</v>
       </c>
-      <c r="E5" s="12" t="str">
-        <f t="shared" ref="E5:E7" si="0">_xlfn.CONCAT(B5,"-",TEXT(C5,"dd/mm/yyyy"))</f>
+      <c r="G5" s="12" t="str">
+        <f t="shared" ref="G5:G7" si="0">_xlfn.CONCAT(C5,"-",TEXT(E5,"dd/mm/yyyy"))</f>
         <v>3161657782-21/03/2024</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="12">
         <v>3</v>
       </c>
-      <c r="B6" s="11">
+      <c r="B6" s="92" t="str">
+        <f>Cliente_D!F6</f>
+        <v>+57</v>
+      </c>
+      <c r="C6" s="11">
         <f>Cliente_D!G6</f>
         <v>3119884321</v>
       </c>
-      <c r="C6" s="33">
+      <c r="D6" s="11" t="str">
+        <f>_xlfn.CONCAT(Cliente_D!B6," ",Cliente_D!C6," ",Cliente_D!D6," ",Cliente_D!E6)</f>
+        <v>Simon  Ochoa Ramirez</v>
+      </c>
+      <c r="E6" s="32">
         <v>45556</v>
       </c>
-      <c r="D6" s="12" t="s">
+      <c r="F6" s="12" t="s">
         <v>49</v>
       </c>
-      <c r="E6" s="12" t="str">
+      <c r="G6" s="12" t="str">
         <f t="shared" si="0"/>
         <v>3119884321-21/09/2024</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="12">
         <v>4</v>
       </c>
-      <c r="B7" s="11">
+      <c r="B7" s="92" t="str">
+        <f>Cliente_D!F7</f>
+        <v>+58</v>
+      </c>
+      <c r="C7" s="11">
         <f>Cliente_D!G7</f>
         <v>4127359182</v>
       </c>
-      <c r="C7" s="33">
+      <c r="D7" s="11" t="str">
+        <f>_xlfn.CONCAT(Cliente_D!B7," ",Cliente_D!C7," ",Cliente_D!D7," ",Cliente_D!E7)</f>
+        <v xml:space="preserve">Alexis  Gallego </v>
+      </c>
+      <c r="E7" s="32">
         <v>46002</v>
       </c>
-      <c r="D7" s="12" t="s">
+      <c r="F7" s="12" t="s">
         <v>49</v>
       </c>
-      <c r="E7" s="12" t="str">
+      <c r="G7" s="12" t="str">
         <f t="shared" si="0"/>
         <v>4127359182-11/12/2025</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="C8" s="30"/>
-      <c r="D8" s="30"/>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="C9" t="s">
-        <v>214</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="C11" s="45"/>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="E8" s="29"/>
+      <c r="F8" s="29"/>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="E11" s="42"/>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="A1" location="'Modelo de Dominio'!A1" display="&lt;&lt;&lt;&lt; Ir al modulo de dominio" xr:uid="{F755F618-0A40-4479-913F-8F6060E94F5B}"/>
     <hyperlink ref="B1" location="'Objetos de Dominio'!A1" display="&lt;&lt;&lt;&lt; Ir a objetos de dominio" xr:uid="{C5748D80-5E29-4CD8-BA51-198180E61202}"/>
-    <hyperlink ref="B3" location="Cliente_D!A1" display="cliente" xr:uid="{F7C47FD3-2FEB-4E40-8CE8-9FEC66E905E0}"/>
-    <hyperlink ref="B4" location="Cliente_D!A4" display="Cliente_D!A4" xr:uid="{7F6CACFC-57C0-447E-811A-802403EBA0AC}"/>
-    <hyperlink ref="B5" location="Cliente_D!A5" display="Cliente_D!A5" xr:uid="{EE87A799-0DAD-412E-8BF4-24089411596B}"/>
-    <hyperlink ref="B6" location="Cliente_D!A6" display="Cliente_D!A6" xr:uid="{D95F6EBA-51E7-42CB-9EFD-6676C5924513}"/>
-    <hyperlink ref="B7" location="Cliente_D!A7" display="Cliente_D!A7" xr:uid="{9BA1680E-A8A5-4CE9-866D-EC3B5A4F5B91}"/>
+    <hyperlink ref="C3" location="Cliente_D!A1" display="cliente" xr:uid="{F7C47FD3-2FEB-4E40-8CE8-9FEC66E905E0}"/>
+    <hyperlink ref="C4" location="Cliente_D!A4" display="Cliente_D!A4" xr:uid="{7F6CACFC-57C0-447E-811A-802403EBA0AC}"/>
+    <hyperlink ref="C5" location="Cliente_D!A5" display="Cliente_D!A5" xr:uid="{EE87A799-0DAD-412E-8BF4-24089411596B}"/>
+    <hyperlink ref="C6" location="Cliente_D!A6" display="Cliente_D!A6" xr:uid="{D95F6EBA-51E7-42CB-9EFD-6676C5924513}"/>
+    <hyperlink ref="C7" location="Cliente_D!A7" display="Cliente_D!A7" xr:uid="{9BA1680E-A8A5-4CE9-866D-EC3B5A4F5B91}"/>
+    <hyperlink ref="D3" location="Cliente_D!A1" display="nombreCliente" xr:uid="{68430887-3CDA-4C9D-A9B6-DD494CC66E80}"/>
+    <hyperlink ref="D4" location="Cliente_D!A4" display="Cliente_D!A4" xr:uid="{DC10FACA-52DE-4612-881C-57BC4CBD25A5}"/>
+    <hyperlink ref="D5" location="Veto_D!A5" display="Veto_D!A5" xr:uid="{69A54058-DDEF-478F-92C9-1D0A036ECD17}"/>
+    <hyperlink ref="D6" location="Veto_D!A6" display="Veto_D!A6" xr:uid="{3A9B5D93-9BFF-419B-8463-90BD464EE14C}"/>
+    <hyperlink ref="D7" location="Veto_D!A7" display="Veto_D!A7" xr:uid="{DD180C3F-CB53-4CD4-BF38-5DA49CDF6A7A}"/>
+    <hyperlink ref="B3" location="Cliente_D!A1" display="prefijoCelularCliente" xr:uid="{95163A37-51BA-42CF-9077-5A2663E258C4}"/>
+    <hyperlink ref="B4" location="Cliente_D!A4" display="Cliente_D!A4" xr:uid="{F91463B6-23BA-47C1-BDE5-CE760AFC5378}"/>
+    <hyperlink ref="B5" location="Cliente_D!A5" display="Cliente_D!A5" xr:uid="{63234F4D-EF9A-4729-8EBD-7241705C09B7}"/>
+    <hyperlink ref="B6" location="Cliente_D!A6" display="Cliente_D!A6" xr:uid="{8618DC09-780E-4CC7-8513-BFB56E4EC06C}"/>
+    <hyperlink ref="B7" location="Cliente_D!A7" display="Cliente_D!A7" xr:uid="{0B51C16B-0BF1-41D9-8A51-AF1E29A80563}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -3352,31 +3502,31 @@
       </c>
     </row>
     <row r="2" spans="1:4" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="18" t="s">
+      <c r="A2" s="17" t="s">
         <v>20</v>
       </c>
-      <c r="B2" s="34" t="s">
-        <v>63</v>
-      </c>
-      <c r="C2" s="31" t="s">
-        <v>64</v>
-      </c>
-      <c r="D2" s="43" t="s">
-        <v>104</v>
+      <c r="B2" s="33" t="s">
+        <v>61</v>
+      </c>
+      <c r="C2" s="30" t="s">
+        <v>62</v>
+      </c>
+      <c r="D2" s="40" t="s">
+        <v>100</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" s="14" t="s">
+      <c r="A3" s="13" t="s">
         <v>31</v>
       </c>
-      <c r="B3" s="32" t="s">
+      <c r="B3" s="31" t="s">
         <v>40</v>
       </c>
-      <c r="C3" s="32" t="s">
+      <c r="C3" s="31" t="s">
         <v>41</v>
       </c>
-      <c r="D3" s="36" t="s">
-        <v>71</v>
+      <c r="D3" s="34" t="s">
+        <v>69</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
@@ -3486,25 +3636,25 @@
       </c>
     </row>
     <row r="2" spans="1:3" ht="28.5" x14ac:dyDescent="0.25">
-      <c r="A2" s="18" t="s">
+      <c r="A2" s="17" t="s">
         <v>20</v>
       </c>
-      <c r="B2" s="18" t="s">
-        <v>126</v>
-      </c>
-      <c r="C2" s="19" t="s">
-        <v>86</v>
+      <c r="B2" s="17" t="s">
+        <v>122</v>
+      </c>
+      <c r="C2" s="18" t="s">
+        <v>84</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" s="14" t="s">
+      <c r="A3" s="13" t="s">
         <v>31</v>
       </c>
-      <c r="B3" s="32" t="s">
+      <c r="B3" s="31" t="s">
         <v>40</v>
       </c>
-      <c r="C3" s="29" t="s">
-        <v>71</v>
+      <c r="C3" s="28" t="s">
+        <v>69</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
@@ -3575,15 +3725,199 @@
 </file>
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{86AE141B-6E6C-47BF-9B70-297A81AC9A72}">
+  <dimension ref="A1:G7"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="26.85546875" customWidth="1"/>
+    <col min="2" max="2" width="32.5703125" customWidth="1"/>
+    <col min="3" max="3" width="34.5703125" customWidth="1"/>
+    <col min="4" max="4" width="32.5703125" customWidth="1"/>
+    <col min="5" max="5" width="21.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="20.140625" customWidth="1"/>
+    <col min="7" max="7" width="47.140625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A1" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="C1" s="5"/>
+      <c r="D1" s="5"/>
+    </row>
+    <row r="2" spans="1:7" ht="46.5" x14ac:dyDescent="0.25">
+      <c r="A2" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="B2" s="18" t="s">
+        <v>199</v>
+      </c>
+      <c r="C2" s="30" t="s">
+        <v>232</v>
+      </c>
+      <c r="D2" s="30" t="s">
+        <v>233</v>
+      </c>
+      <c r="E2" s="18" t="s">
+        <v>219</v>
+      </c>
+      <c r="F2" s="18" t="s">
+        <v>234</v>
+      </c>
+      <c r="G2" s="18" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" s="13" t="s">
+        <v>31</v>
+      </c>
+      <c r="B3" s="31" t="s">
+        <v>60</v>
+      </c>
+      <c r="C3" s="87" t="s">
+        <v>229</v>
+      </c>
+      <c r="D3" s="87" t="s">
+        <v>230</v>
+      </c>
+      <c r="E3" s="86" t="s">
+        <v>21</v>
+      </c>
+      <c r="F3" s="41" t="s">
+        <v>37</v>
+      </c>
+      <c r="G3" s="28" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" s="12">
+        <v>1</v>
+      </c>
+      <c r="B4" s="11" t="str">
+        <f>Agenda_D!C4</f>
+        <v>Juan García</v>
+      </c>
+      <c r="C4" s="88">
+        <v>46047.458333333336</v>
+      </c>
+      <c r="D4" s="88">
+        <v>46047.541666666664</v>
+      </c>
+      <c r="E4" s="80" t="s">
+        <v>208</v>
+      </c>
+      <c r="F4" s="12">
+        <v>120</v>
+      </c>
+      <c r="G4" s="12" t="str">
+        <f>_xlfn.CONCAT(B4,"-",TEXT(C4,"dd/mm/yyyy hh:mm"),"-",TEXT(D4,"dd/mm/yyyy hh:mm"))</f>
+        <v>Juan García-25/01/2026 11:00-25/01/2026 13:00</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" s="12">
+        <v>2</v>
+      </c>
+      <c r="B5" s="11" t="str">
+        <f>Agenda_D!C5</f>
+        <v>Juan Ortiz</v>
+      </c>
+      <c r="C5" s="88">
+        <v>45362.5</v>
+      </c>
+      <c r="D5" s="88">
+        <v>45362.645833333336</v>
+      </c>
+      <c r="E5" s="82" t="s">
+        <v>209</v>
+      </c>
+      <c r="F5" s="12">
+        <v>210</v>
+      </c>
+      <c r="G5" s="12" t="str">
+        <f t="shared" ref="G5:G7" si="0">_xlfn.CONCAT(B5,"-",TEXT(C5,"dd/mm/yyyy hh:mm"),"-",TEXT(D5,"dd/mm/yyyy hh:mm"))</f>
+        <v>Juan Ortiz-11/03/2024 12:00-11/03/2024 15:30</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" s="12">
+        <v>3</v>
+      </c>
+      <c r="B6" s="11" t="str">
+        <f>Agenda_D!C6</f>
+        <v>Carlos Arbeladez</v>
+      </c>
+      <c r="C6" s="88">
+        <v>46013.541666666664</v>
+      </c>
+      <c r="D6" s="88">
+        <v>46013.583333333336</v>
+      </c>
+      <c r="E6" s="82" t="s">
+        <v>210</v>
+      </c>
+      <c r="F6" s="12">
+        <v>60</v>
+      </c>
+      <c r="G6" s="12" t="str">
+        <f t="shared" si="0"/>
+        <v>Carlos Arbeladez-22/12/2025 13:00-22/12/2025 14:00</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" s="12">
+        <v>4</v>
+      </c>
+      <c r="B7" s="79" t="str">
+        <f>Agenda_D!C7</f>
+        <v>Andres Ramirez</v>
+      </c>
+      <c r="C7" s="89">
+        <v>46241.375</v>
+      </c>
+      <c r="D7" s="89">
+        <v>46241.5</v>
+      </c>
+      <c r="E7" s="82" t="s">
+        <v>211</v>
+      </c>
+      <c r="F7" s="12">
+        <v>180</v>
+      </c>
+      <c r="G7" s="12" t="str">
+        <f t="shared" si="0"/>
+        <v>Andres Ramirez-07/08/2026 09:00-07/08/2026 12:00</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A1" location="'Modelo de Dominio'!A1" display="&lt;&lt;&lt;&lt; Ir al modulo de dominio" xr:uid="{B428C070-F6EA-4693-9030-AA54AF833423}"/>
+    <hyperlink ref="B1" location="'Objetos de Dominio'!A1" display="&lt;&lt;&lt;&lt; Ir a objetos de dominio" xr:uid="{907D0986-51A3-4C83-A3D9-42BF086C4E3E}"/>
+    <hyperlink ref="B3" location="Agenda_D!A1" display="agenda" xr:uid="{ADF6E864-3D66-491F-9B59-46E28FAAD6DA}"/>
+    <hyperlink ref="B4" location="Agenda_D!A4" display="Agenda_D!A4" xr:uid="{780EF3D8-7585-4C31-B2AA-FC1B8C5006F7}"/>
+    <hyperlink ref="B5" location="Agenda_D!A5" display="Agenda_D!A5" xr:uid="{78210E4E-E975-4398-935F-2D4F77890E65}"/>
+    <hyperlink ref="B6" location="Agenda_D!A6" display="Agenda_D!A6" xr:uid="{1994F7F3-CFB6-4C90-85C0-8ADD22510C50}"/>
+    <hyperlink ref="B7" location="Agenda_D!A7" display="Agenda_D!A7" xr:uid="{D0080FB0-93CA-45FC-86C9-19C5C8A97148}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5CFE76D0-FBB4-4C81-85CC-F644057A8847}">
-  <dimension ref="A1:F10"/>
+  <dimension ref="A1:F16"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="27" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="37.140625" customWidth="1"/>
-    <col min="3" max="3" width="28" customWidth="1"/>
-    <col min="4" max="4" width="18.7109375" customWidth="1"/>
-    <col min="5" max="5" width="31.7109375" customWidth="1"/>
+    <col min="3" max="3" width="46.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="26.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="48.5703125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="37.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -3596,60 +3930,60 @@
       </c>
     </row>
     <row r="2" spans="1:6" ht="40.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="19" t="s">
+      <c r="A2" s="18" t="s">
         <v>20</v>
       </c>
-      <c r="B2" s="19" t="s">
-        <v>88</v>
-      </c>
-      <c r="C2" s="19" t="s">
-        <v>176</v>
-      </c>
-      <c r="D2" s="19" t="s">
-        <v>89</v>
-      </c>
-      <c r="E2" s="19" t="s">
-        <v>90</v>
-      </c>
-      <c r="F2" s="19" t="s">
-        <v>91</v>
+      <c r="B2" s="18" t="s">
+        <v>86</v>
+      </c>
+      <c r="C2" s="18" t="s">
+        <v>238</v>
+      </c>
+      <c r="D2" s="18" t="s">
+        <v>239</v>
+      </c>
+      <c r="E2" s="18" t="s">
+        <v>241</v>
+      </c>
+      <c r="F2" s="18" t="s">
+        <v>87</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" s="14" t="s">
+      <c r="A3" s="13" t="s">
         <v>31</v>
       </c>
-      <c r="B3" s="32" t="s">
-        <v>62</v>
-      </c>
-      <c r="C3" s="59" t="s">
-        <v>77</v>
-      </c>
-      <c r="D3" s="79" t="s">
-        <v>65</v>
-      </c>
-      <c r="E3" s="79" t="s">
-        <v>87</v>
-      </c>
-      <c r="F3" s="29" t="s">
-        <v>71</v>
+      <c r="B3" s="31" t="s">
+        <v>60</v>
+      </c>
+      <c r="C3" s="85" t="s">
+        <v>75</v>
+      </c>
+      <c r="D3" s="75" t="s">
+        <v>63</v>
+      </c>
+      <c r="E3" s="75" t="s">
+        <v>85</v>
+      </c>
+      <c r="F3" s="28" t="s">
+        <v>69</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="12">
         <v>1</v>
       </c>
-      <c r="B4" s="50" t="str">
+      <c r="B4" s="47" t="str">
         <f>Agenda_D!C4</f>
         <v>Juan García</v>
       </c>
-      <c r="C4" s="38" t="s">
-        <v>80</v>
-      </c>
-      <c r="D4" s="38">
+      <c r="C4" s="36" t="s">
+        <v>78</v>
+      </c>
+      <c r="D4" s="90">
         <v>0.41666666666666669</v>
       </c>
-      <c r="E4" s="38">
+      <c r="E4" s="90">
         <v>0.66666666666666663</v>
       </c>
       <c r="F4" s="12" t="str">
@@ -3661,17 +3995,17 @@
       <c r="A5" s="12">
         <v>2</v>
       </c>
-      <c r="B5" s="50" t="str">
+      <c r="B5" s="47" t="str">
         <f>Agenda_D!C5</f>
         <v>Juan Ortiz</v>
       </c>
       <c r="C5" s="12" t="s">
-        <v>81</v>
-      </c>
-      <c r="D5" s="38">
+        <v>79</v>
+      </c>
+      <c r="D5" s="90">
         <v>0.375</v>
       </c>
-      <c r="E5" s="38">
+      <c r="E5" s="90">
         <v>0.625</v>
       </c>
       <c r="F5" s="12" t="str">
@@ -3683,17 +4017,17 @@
       <c r="A6" s="12">
         <v>3</v>
       </c>
-      <c r="B6" s="50" t="str">
+      <c r="B6" s="47" t="str">
         <f>Agenda_D!C6</f>
         <v>Carlos Arbeladez</v>
       </c>
       <c r="C6" s="12" t="s">
-        <v>83</v>
-      </c>
-      <c r="D6" s="38">
+        <v>81</v>
+      </c>
+      <c r="D6" s="90">
         <v>0.54166666666666663</v>
       </c>
-      <c r="E6" s="38">
+      <c r="E6" s="90">
         <v>0.79166666666666663</v>
       </c>
       <c r="F6" s="12" t="str">
@@ -3705,17 +4039,17 @@
       <c r="A7" s="12">
         <v>4</v>
       </c>
-      <c r="B7" s="50" t="str">
+      <c r="B7" s="47" t="str">
         <f>Agenda_D!C7</f>
         <v>Andres Ramirez</v>
       </c>
       <c r="C7" s="12" t="s">
-        <v>85</v>
-      </c>
-      <c r="D7" s="38">
+        <v>83</v>
+      </c>
+      <c r="D7" s="90">
         <v>0.33333333333333331</v>
       </c>
-      <c r="E7" s="38">
+      <c r="E7" s="90">
         <v>0.58333333333333337</v>
       </c>
       <c r="F7" s="12" t="str">
@@ -3723,10 +4057,33 @@
         <v>Andres Ramirez-Sábado-08-14</v>
       </c>
     </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="E8" s="93"/>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="E9" s="93"/>
+    </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="C10" s="10" t="s">
-        <v>177</v>
-      </c>
+      <c r="C10" s="10"/>
+      <c r="E10" s="94"/>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="E11" s="94"/>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="E12" s="93"/>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="E13" s="93"/>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="E14" s="93"/>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="E15" s="93"/>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="E16" s="93"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -3743,9 +4100,191 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EB38530B-FD95-4EEF-8F76-78E045637369}">
+  <dimension ref="A1:G7"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="26.85546875" customWidth="1"/>
+    <col min="2" max="2" width="32.5703125" customWidth="1"/>
+    <col min="3" max="3" width="32.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="31.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="26.7109375" customWidth="1"/>
+    <col min="6" max="6" width="29.140625" customWidth="1"/>
+    <col min="7" max="7" width="33.7109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A1" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" ht="40.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="B2" s="18" t="s">
+        <v>203</v>
+      </c>
+      <c r="C2" s="18" t="s">
+        <v>243</v>
+      </c>
+      <c r="D2" s="18" t="s">
+        <v>242</v>
+      </c>
+      <c r="E2" s="18" t="s">
+        <v>225</v>
+      </c>
+      <c r="F2" s="30" t="s">
+        <v>226</v>
+      </c>
+      <c r="G2" s="18" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" s="13" t="s">
+        <v>31</v>
+      </c>
+      <c r="B3" s="31" t="s">
+        <v>202</v>
+      </c>
+      <c r="C3" s="75" t="s">
+        <v>63</v>
+      </c>
+      <c r="D3" s="75" t="s">
+        <v>200</v>
+      </c>
+      <c r="E3" s="72" t="s">
+        <v>21</v>
+      </c>
+      <c r="F3" s="83" t="s">
+        <v>37</v>
+      </c>
+      <c r="G3" s="28" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" s="12">
+        <v>1</v>
+      </c>
+      <c r="B4" s="11" t="str">
+        <f>HorarioBarbero_D!F4</f>
+        <v>Juan García-Lunes-10-16</v>
+      </c>
+      <c r="C4" s="36">
+        <v>0.5</v>
+      </c>
+      <c r="D4" s="36">
+        <v>0.58333333333333337</v>
+      </c>
+      <c r="E4" s="36" t="s">
+        <v>204</v>
+      </c>
+      <c r="F4" s="84">
+        <v>120</v>
+      </c>
+      <c r="G4" s="12" t="str">
+        <f>_xlfn.CONCAT(B4,"-",TEXT(C4,"hh;mm"),"-",TEXT(D4,"hh;mm"))</f>
+        <v>Juan García-Lunes-10-16-12-14</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" s="12">
+        <v>2</v>
+      </c>
+      <c r="B5" s="11" t="str">
+        <f>HorarioBarbero_D!F5</f>
+        <v>Juan Ortiz-Martes-09-15</v>
+      </c>
+      <c r="C5" s="36">
+        <v>0.54166666666666663</v>
+      </c>
+      <c r="D5" s="81">
+        <v>0.625</v>
+      </c>
+      <c r="E5" s="24" t="s">
+        <v>207</v>
+      </c>
+      <c r="F5" s="12">
+        <v>120</v>
+      </c>
+      <c r="G5" s="12" t="str">
+        <f t="shared" ref="G5:G7" si="0">_xlfn.CONCAT(B5,"-",TEXT(C5,"hh;mm"),"-",TEXT(D5,"hh;mm"))</f>
+        <v>Juan Ortiz-Martes-09-15-13-15</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" s="12">
+        <v>3</v>
+      </c>
+      <c r="B6" s="11" t="str">
+        <f>HorarioBarbero_D!F6</f>
+        <v>Carlos Arbeladez-Jueves-13-19</v>
+      </c>
+      <c r="C6" s="36">
+        <v>0.70833333333333337</v>
+      </c>
+      <c r="D6" s="36">
+        <v>0.75</v>
+      </c>
+      <c r="E6" s="12" t="s">
+        <v>206</v>
+      </c>
+      <c r="F6" s="12">
+        <v>60</v>
+      </c>
+      <c r="G6" s="12" t="str">
+        <f t="shared" si="0"/>
+        <v>Carlos Arbeladez-Jueves-13-19-17-18</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" s="12">
+        <v>4</v>
+      </c>
+      <c r="B7" s="11" t="str">
+        <f>HorarioBarbero_D!F7</f>
+        <v>Andres Ramirez-Sábado-08-14</v>
+      </c>
+      <c r="C7" s="36">
+        <v>0.47916666666666669</v>
+      </c>
+      <c r="D7" s="36">
+        <v>0.54166666666666663</v>
+      </c>
+      <c r="E7" s="12" t="s">
+        <v>205</v>
+      </c>
+      <c r="F7" s="12">
+        <v>90</v>
+      </c>
+      <c r="G7" s="12" t="str">
+        <f t="shared" si="0"/>
+        <v>Andres Ramirez-Sábado-08-14-11-13</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A1" location="'Modelo de Dominio'!A1" display="&lt;&lt;&lt;&lt; Ir al modulo de dominio" xr:uid="{28D494EF-6E9C-4926-913D-1C222BAE912F}"/>
+    <hyperlink ref="B1" location="'Objetos de Dominio'!A1" display="&lt;&lt;&lt;&lt; Ir a objetos de dominio" xr:uid="{E603E2D9-858F-4FFA-8815-5567364FE382}"/>
+    <hyperlink ref="B3" location="HorarioBarbero_D!A1" display="horarioDelBarbero" xr:uid="{E895F830-FA04-42C5-BF65-9170EC8A6C40}"/>
+    <hyperlink ref="B4" location="HorarioBarbero_D!A4" display="HorarioBarbero_D!A4" xr:uid="{8EE0E36C-8BF0-4BBA-8EAF-59B76141C41B}"/>
+    <hyperlink ref="B5" location="HorarioBarbero_D!A5" display="HorarioBarbero_D!A5" xr:uid="{B5E52511-94A7-4409-8D8A-54A2A651A3ED}"/>
+    <hyperlink ref="B6" location="HorarioBarbero_D!A6" display="HorarioBarbero_D!A6" xr:uid="{70BE22C1-3690-4C31-BFB5-A4A0D08A8829}"/>
+    <hyperlink ref="B7" location="HorarioBarbero_D!A7" display="HorarioBarbero_D!A7" xr:uid="{8717ACB0-7EC3-4D5F-95F4-D0AF5B38DBFA}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1429879F-6697-4F1F-AF5D-52C4860B7B3E}">
-  <dimension ref="A1:H15"/>
+  <dimension ref="A1:H18"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="28" customWidth="1"/>
@@ -3766,50 +4305,50 @@
         <v>33</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="18" t="s">
+    <row r="2" spans="1:8" ht="44.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="17" t="s">
         <v>20</v>
       </c>
-      <c r="B2" s="18" t="s">
-        <v>66</v>
-      </c>
-      <c r="C2" s="31" t="s">
-        <v>145</v>
-      </c>
-      <c r="D2" s="31" t="s">
-        <v>216</v>
-      </c>
-      <c r="E2" s="31" t="s">
-        <v>142</v>
-      </c>
-      <c r="F2" s="31" t="s">
-        <v>146</v>
-      </c>
-      <c r="G2" s="31" t="s">
-        <v>138</v>
+      <c r="B2" s="17" t="s">
+        <v>64</v>
+      </c>
+      <c r="C2" s="30" t="s">
+        <v>139</v>
+      </c>
+      <c r="D2" s="30" t="s">
+        <v>195</v>
+      </c>
+      <c r="E2" s="30" t="s">
+        <v>136</v>
+      </c>
+      <c r="F2" s="30" t="s">
+        <v>227</v>
+      </c>
+      <c r="G2" s="30" t="s">
+        <v>133</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A3" s="14" t="s">
+      <c r="A3" s="13" t="s">
         <v>31</v>
       </c>
-      <c r="B3" s="32" t="s">
+      <c r="B3" s="31" t="s">
         <v>44</v>
       </c>
-      <c r="C3" s="32" t="s">
-        <v>62</v>
-      </c>
-      <c r="D3" s="83" t="s">
-        <v>137</v>
-      </c>
-      <c r="E3" s="44" t="s">
-        <v>87</v>
-      </c>
-      <c r="F3" s="58" t="s">
+      <c r="C3" s="31" t="s">
+        <v>60</v>
+      </c>
+      <c r="D3" s="78" t="s">
+        <v>132</v>
+      </c>
+      <c r="E3" s="41" t="s">
+        <v>85</v>
+      </c>
+      <c r="F3" s="55" t="s">
         <v>26</v>
       </c>
-      <c r="G3" s="29" t="s">
-        <v>71</v>
+      <c r="G3" s="28" t="s">
+        <v>69</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
@@ -3824,14 +4363,14 @@
         <f>Agenda_D!C4</f>
         <v>Juan García</v>
       </c>
-      <c r="D4" s="52">
+      <c r="D4" s="49">
         <v>46295.416666666664</v>
       </c>
-      <c r="E4" s="38">
+      <c r="E4" s="90">
         <v>0.44791666666666669</v>
       </c>
       <c r="F4" s="12" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="G4" s="12" t="str">
         <f>_xlfn.CONCAT(C4,"-",TEXT(D4,"dd/mm/yyyy/hh:mm"))</f>
@@ -3850,14 +4389,14 @@
         <f>Agenda_D!C5</f>
         <v>Juan Ortiz</v>
       </c>
-      <c r="D5" s="52">
+      <c r="D5" s="49">
         <v>45983.458333333336</v>
       </c>
-      <c r="E5" s="38">
+      <c r="E5" s="90">
         <v>0.48958333333333331</v>
       </c>
       <c r="F5" s="12" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="G5" s="12" t="str">
         <f t="shared" ref="G5:G8" si="0">_xlfn.CONCAT(C5,"-",TEXT(D5,"dd/mm/yyyy/hh:mm"))</f>
@@ -3876,14 +4415,14 @@
         <f>Agenda_D!C6</f>
         <v>Carlos Arbeladez</v>
       </c>
-      <c r="D6" s="52">
+      <c r="D6" s="49">
         <v>45514.583333333336</v>
       </c>
-      <c r="E6" s="38">
+      <c r="E6" s="90">
         <v>0.59375</v>
       </c>
       <c r="F6" s="12" t="s">
-        <v>139</v>
+        <v>134</v>
       </c>
       <c r="G6" s="12" t="str">
         <f t="shared" si="0"/>
@@ -3902,14 +4441,14 @@
         <f>Agenda_D!C7</f>
         <v>Andres Ramirez</v>
       </c>
-      <c r="D7" s="52">
+      <c r="D7" s="49">
         <v>46289.541666666664</v>
       </c>
-      <c r="E7" s="38">
+      <c r="E7" s="90">
         <v>0.5625</v>
       </c>
       <c r="F7" s="12" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="G7" s="12" t="str">
         <f t="shared" si="0"/>
@@ -3928,40 +4467,47 @@
         <f>Agenda_D!C6</f>
         <v>Carlos Arbeladez</v>
       </c>
-      <c r="D8" s="52">
+      <c r="D8" s="49">
         <v>46240.75</v>
       </c>
-      <c r="E8" s="38">
+      <c r="E8" s="90">
         <v>0.75694444444444442</v>
       </c>
       <c r="F8" s="12" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="G8" s="12" t="str">
         <f t="shared" si="0"/>
         <v>Carlos Arbeladez-06/08/2026/18:00</v>
       </c>
-      <c r="H8" s="49"/>
+      <c r="H8" s="46"/>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="H10" s="51"/>
+      <c r="H10" s="48"/>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="F11" s="10" t="s">
-        <v>215</v>
-      </c>
+      <c r="F11" s="10"/>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="D12" s="53"/>
+      <c r="D12" s="50"/>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="D13" s="53"/>
+      <c r="D13" s="50"/>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="D14" s="53"/>
+      <c r="D14" s="50"/>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="D15" s="53"/>
+      <c r="D15" s="50"/>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="E16" s="93"/>
+    </row>
+    <row r="17" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E17" s="93"/>
+    </row>
+    <row r="18" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E18" s="93"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -3986,7 +4532,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{766573FB-AAA2-4254-B83C-7C7505540365}">
   <dimension ref="A1:G7"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -4008,49 +4554,49 @@
       </c>
     </row>
     <row r="2" spans="1:7" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="18" t="s">
+      <c r="A2" s="17" t="s">
         <v>20</v>
       </c>
-      <c r="B2" s="18" t="s">
-        <v>96</v>
-      </c>
-      <c r="C2" s="31" t="s">
-        <v>97</v>
-      </c>
-      <c r="D2" s="31" t="s">
+      <c r="B2" s="17" t="s">
+        <v>92</v>
+      </c>
+      <c r="C2" s="30" t="s">
+        <v>93</v>
+      </c>
+      <c r="D2" s="30" t="s">
+        <v>228</v>
+      </c>
+      <c r="E2" s="30" t="s">
+        <v>141</v>
+      </c>
+      <c r="F2" s="30" t="s">
+        <v>94</v>
+      </c>
+      <c r="G2" s="30" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" s="13" t="s">
+        <v>31</v>
+      </c>
+      <c r="B3" s="31" t="s">
+        <v>44</v>
+      </c>
+      <c r="C3" s="31" t="s">
+        <v>91</v>
+      </c>
+      <c r="D3" s="41" t="s">
+        <v>27</v>
+      </c>
+      <c r="E3" s="54" t="s">
         <v>140</v>
       </c>
-      <c r="E2" s="31" t="s">
-        <v>148</v>
-      </c>
-      <c r="F2" s="31" t="s">
-        <v>98</v>
-      </c>
-      <c r="G2" s="31" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A3" s="14" t="s">
-        <v>31</v>
-      </c>
-      <c r="B3" s="32" t="s">
-        <v>44</v>
-      </c>
-      <c r="C3" s="32" t="s">
-        <v>95</v>
-      </c>
-      <c r="D3" s="35" t="s">
-        <v>27</v>
-      </c>
-      <c r="E3" s="57" t="s">
-        <v>147</v>
-      </c>
-      <c r="F3" s="44" t="s">
+      <c r="F3" s="41" t="s">
         <v>28</v>
       </c>
-      <c r="G3" s="29" t="s">
-        <v>71</v>
+      <c r="G3" s="28" t="s">
+        <v>69</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
@@ -4070,7 +4616,7 @@
         <v>10000</v>
       </c>
       <c r="E4" s="12" t="s">
-        <v>139</v>
+        <v>134</v>
       </c>
       <c r="F4" s="12" t="s">
         <v>49</v>
@@ -4097,7 +4643,7 @@
         <v>35000</v>
       </c>
       <c r="E5" s="12" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="F5" s="12" t="s">
         <v>50</v>
@@ -4140,9 +4686,9 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F470C5A4-8D15-43DA-95FC-91C9614E5EEA}">
-  <dimension ref="A1:F10"/>
+  <dimension ref="A1:F8"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="26.42578125" customWidth="1"/>
@@ -4162,43 +4708,43 @@
       </c>
     </row>
     <row r="2" spans="1:6" ht="33" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="18" t="s">
+      <c r="A2" s="17" t="s">
         <v>20</v>
       </c>
-      <c r="B2" s="18" t="s">
-        <v>100</v>
-      </c>
-      <c r="C2" s="31" t="s">
-        <v>101</v>
-      </c>
-      <c r="D2" s="31" t="s">
-        <v>217</v>
-      </c>
-      <c r="E2" s="31" t="s">
-        <v>102</v>
-      </c>
-      <c r="F2" s="31" t="s">
-        <v>103</v>
+      <c r="B2" s="17" t="s">
+        <v>96</v>
+      </c>
+      <c r="C2" s="30" t="s">
+        <v>97</v>
+      </c>
+      <c r="D2" s="30" t="s">
+        <v>220</v>
+      </c>
+      <c r="E2" s="30" t="s">
+        <v>98</v>
+      </c>
+      <c r="F2" s="30" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" s="41" t="s">
+      <c r="A3" s="38" t="s">
         <v>31</v>
       </c>
-      <c r="B3" s="32" t="s">
-        <v>95</v>
-      </c>
-      <c r="C3" s="32" t="s">
+      <c r="B3" s="31" t="s">
+        <v>91</v>
+      </c>
+      <c r="C3" s="31" t="s">
         <v>41</v>
       </c>
-      <c r="D3" s="77" t="s">
+      <c r="D3" s="73" t="s">
         <v>29</v>
       </c>
-      <c r="E3" s="77" t="s">
+      <c r="E3" s="73" t="s">
         <v>30</v>
       </c>
-      <c r="F3" s="29" t="s">
-        <v>71</v>
+      <c r="F3" s="28" t="s">
+        <v>69</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
@@ -4278,7 +4824,7 @@
         <f>Cita_D!G7</f>
         <v>Andres Ramirez-24/09/2026/13:00</v>
       </c>
-      <c r="C7" s="54" t="str">
+      <c r="C7" s="51" t="str">
         <f>Servicio_D!F7</f>
         <v>Arreglo completo de barba con toalla caliente</v>
       </c>
@@ -4288,7 +4834,7 @@
       <c r="E7" s="12">
         <v>30</v>
       </c>
-      <c r="F7" s="25" t="str">
+      <c r="F7" s="24" t="str">
         <f t="shared" si="0"/>
         <v>Andres Ramirez-24/09/2026/13:00-Arreglo completo de barba con toalla caliente</v>
       </c>
@@ -4310,17 +4856,9 @@
       <c r="E8" s="12">
         <v>10</v>
       </c>
-      <c r="F8" s="25" t="str">
+      <c r="F8" s="24" t="str">
         <f t="shared" si="0"/>
         <v>Carlos Arbeladez-06/08/2026/18:00-Corte de barba</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="D10" t="s">
-        <v>219</v>
-      </c>
-      <c r="E10" t="s">
-        <v>218</v>
       </c>
     </row>
   </sheetData>
@@ -4394,7 +4932,7 @@
         <v>11</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>155</v>
+        <v>148</v>
       </c>
       <c r="C4" s="7">
         <v>1</v>
@@ -4408,7 +4946,7 @@
         <v>5</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>156</v>
+        <v>149</v>
       </c>
       <c r="C5" s="7">
         <v>2</v>
@@ -4419,10 +4957,10 @@
     </row>
     <row r="6" spans="1:4" ht="45" x14ac:dyDescent="0.25">
       <c r="A6" s="7" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>157</v>
+        <v>150</v>
       </c>
       <c r="C6" s="7">
         <v>2</v>
@@ -4436,7 +4974,7 @@
         <v>6</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>158</v>
+        <v>151</v>
       </c>
       <c r="C7" s="7">
         <v>2</v>
@@ -4464,7 +5002,7 @@
         <v>13</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>159</v>
+        <v>152</v>
       </c>
       <c r="C9" s="7">
         <v>2</v>
@@ -4492,7 +5030,7 @@
         <v>9</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>160</v>
+        <v>153</v>
       </c>
       <c r="C11" s="7">
         <v>3</v>
@@ -4501,22 +5039,26 @@
         <v>34</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:4" ht="90" x14ac:dyDescent="0.25">
       <c r="A12" s="7" t="s">
-        <v>221</v>
-      </c>
-      <c r="B12" s="8"/>
+        <v>196</v>
+      </c>
+      <c r="B12" s="8" t="s">
+        <v>231</v>
+      </c>
       <c r="C12" s="7">
         <v>4</v>
       </c>
-      <c r="D12" s="9"/>
+      <c r="D12" s="9" t="s">
+        <v>34</v>
+      </c>
     </row>
     <row r="13" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A13" s="7" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="B13" s="8" t="s">
-        <v>161</v>
+        <v>154</v>
       </c>
       <c r="C13" s="7">
         <v>4</v>
@@ -4530,7 +5072,7 @@
         <v>10</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>162</v>
+        <v>155</v>
       </c>
       <c r="C14" s="7">
         <v>4</v>
@@ -4539,15 +5081,19 @@
         <v>34</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:4" ht="60" x14ac:dyDescent="0.25">
       <c r="A15" s="7" t="s">
-        <v>222</v>
-      </c>
-      <c r="B15" s="8"/>
+        <v>197</v>
+      </c>
+      <c r="B15" s="8" t="s">
+        <v>198</v>
+      </c>
       <c r="C15" s="7">
         <v>5</v>
       </c>
-      <c r="D15" s="9"/>
+      <c r="D15" s="9" t="s">
+        <v>34</v>
+      </c>
     </row>
     <row r="16" spans="1:4" ht="45" x14ac:dyDescent="0.25">
       <c r="A16" s="7" t="s">
@@ -4593,6 +5139,8 @@
     <hyperlink ref="A1" location="'Modelo de Dominio'!A1" display="&lt;&lt;&lt;&lt; Ir al modulo de dominio" xr:uid="{A3D1E053-3C90-4C85-85FB-01CE6B92A5EE}"/>
     <hyperlink ref="D6" location="HorarioBarberia_D!A1" display="aquí" xr:uid="{CE45E0DE-1B75-4BE0-8664-81F7834039D9}"/>
     <hyperlink ref="D13" location="HorarioBarbero_D!A1" display="aquí" xr:uid="{3B048927-BA4F-418A-BCDC-3E65406B8FD1}"/>
+    <hyperlink ref="D12" location="Bloqueo_D!A1" display="aquí" xr:uid="{C19EA470-C149-4E7D-B95C-B02B73C07975}"/>
+    <hyperlink ref="D15" location="Descanso_D!A1" display="aquí" xr:uid="{BA11B464-44BB-488E-84C7-707437A187F8}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -4604,95 +5152,95 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18.42578125" customWidth="1"/>
-    <col min="2" max="2" width="62.7109375" customWidth="1"/>
+    <col min="2" max="2" width="69.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
-        <v>172</v>
+        <v>163</v>
       </c>
       <c r="B1" s="7" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" s="60" t="s">
+      <c r="A2" s="56" t="s">
+        <v>164</v>
+      </c>
+      <c r="B2" s="56" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+      <c r="A3" s="57" t="s">
+        <v>165</v>
+      </c>
+      <c r="B3" s="66" t="s">
         <v>173</v>
       </c>
-      <c r="B2" s="60" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" ht="30" x14ac:dyDescent="0.25">
-      <c r="A3" s="61" t="s">
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" s="59" t="s">
+        <v>166</v>
+      </c>
+      <c r="B4" s="59" t="s">
         <v>174</v>
       </c>
-      <c r="B3" s="70" t="s">
-        <v>185</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" s="63" t="s">
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" s="58" t="s">
+        <v>193</v>
+      </c>
+      <c r="B5" s="67" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" s="60" t="s">
+        <v>167</v>
+      </c>
+      <c r="B6" s="60" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+      <c r="A7" s="61" t="s">
+        <v>168</v>
+      </c>
+      <c r="B7" s="68" t="s">
         <v>175</v>
       </c>
-      <c r="B4" s="63" t="s">
-        <v>186</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5" s="62" t="s">
-        <v>212</v>
-      </c>
-      <c r="B5" s="71" t="s">
-        <v>213</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A6" s="64" t="s">
-        <v>178</v>
-      </c>
-      <c r="B6" s="64" t="s">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" ht="30" x14ac:dyDescent="0.25">
-      <c r="A7" s="65" t="s">
+    </row>
+    <row r="8" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+      <c r="A8" s="62" t="s">
+        <v>169</v>
+      </c>
+      <c r="B8" s="69" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" ht="45" x14ac:dyDescent="0.25">
+      <c r="A9" s="63" t="s">
+        <v>69</v>
+      </c>
+      <c r="B9" s="70" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" ht="45" x14ac:dyDescent="0.25">
+      <c r="A10" s="64" t="s">
+        <v>170</v>
+      </c>
+      <c r="B10" s="64" t="s">
         <v>179</v>
       </c>
-      <c r="B7" s="72" t="s">
-        <v>187</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" ht="30" x14ac:dyDescent="0.25">
-      <c r="A8" s="66" t="s">
+    </row>
+    <row r="11" spans="1:2" ht="75" x14ac:dyDescent="0.25">
+      <c r="A11" s="65" t="s">
+        <v>171</v>
+      </c>
+      <c r="B11" s="71" t="s">
         <v>180</v>
-      </c>
-      <c r="B8" s="73" t="s">
-        <v>188</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" ht="45" x14ac:dyDescent="0.25">
-      <c r="A9" s="67" t="s">
-        <v>181</v>
-      </c>
-      <c r="B9" s="74" t="s">
-        <v>189</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" ht="45" x14ac:dyDescent="0.25">
-      <c r="A10" s="68" t="s">
-        <v>182</v>
-      </c>
-      <c r="B10" s="68" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" ht="75" x14ac:dyDescent="0.25">
-      <c r="A11" s="69" t="s">
-        <v>183</v>
-      </c>
-      <c r="B11" s="75" t="s">
-        <v>192</v>
       </c>
     </row>
   </sheetData>
@@ -4719,28 +5267,28 @@
       </c>
     </row>
     <row r="2" spans="1:3" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="19" t="s">
+      <c r="A2" s="18" t="s">
         <v>20</v>
       </c>
-      <c r="B2" s="19" t="s">
-        <v>163</v>
+      <c r="B2" s="18" t="s">
+        <v>213</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" s="14" t="s">
+      <c r="A3" s="13" t="s">
         <v>31</v>
       </c>
-      <c r="B3" s="13" t="s">
+      <c r="B3" s="72" t="s">
         <v>21</v>
       </c>
-      <c r="C3" s="37"/>
+      <c r="C3" s="35"/>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="12">
         <v>1</v>
       </c>
-      <c r="B4" s="38" t="s">
-        <v>68</v>
+      <c r="B4" s="36" t="s">
+        <v>66</v>
       </c>
       <c r="C4" s="4"/>
     </row>
@@ -4779,55 +5327,55 @@
       <c r="H1" s="12"/>
     </row>
     <row r="2" spans="1:8" ht="46.5" x14ac:dyDescent="0.25">
-      <c r="A2" s="18" t="s">
+      <c r="A2" s="17" t="s">
         <v>20</v>
       </c>
-      <c r="B2" s="18" t="s">
-        <v>193</v>
-      </c>
-      <c r="C2" s="18" t="s">
-        <v>194</v>
-      </c>
-      <c r="D2" s="18" t="s">
-        <v>195</v>
-      </c>
-      <c r="E2" s="18" t="s">
-        <v>196</v>
-      </c>
-      <c r="F2" s="18" t="s">
-        <v>197</v>
-      </c>
-      <c r="G2" s="19" t="s">
-        <v>198</v>
-      </c>
-      <c r="H2" s="20" t="s">
-        <v>141</v>
+      <c r="B2" s="17" t="s">
+        <v>181</v>
+      </c>
+      <c r="C2" s="17" t="s">
+        <v>182</v>
+      </c>
+      <c r="D2" s="17" t="s">
+        <v>183</v>
+      </c>
+      <c r="E2" s="17" t="s">
+        <v>184</v>
+      </c>
+      <c r="F2" s="17" t="s">
+        <v>221</v>
+      </c>
+      <c r="G2" s="18" t="s">
+        <v>185</v>
+      </c>
+      <c r="H2" s="19" t="s">
+        <v>135</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A3" s="14" t="s">
+      <c r="A3" s="13" t="s">
         <v>31</v>
       </c>
-      <c r="B3" s="58" t="s">
-        <v>105</v>
-      </c>
-      <c r="C3" s="58" t="s">
-        <v>107</v>
-      </c>
-      <c r="D3" s="58" t="s">
-        <v>106</v>
-      </c>
-      <c r="E3" s="58" t="s">
-        <v>108</v>
-      </c>
-      <c r="F3" s="76" t="s">
-        <v>164</v>
-      </c>
-      <c r="G3" s="76" t="s">
+      <c r="B3" s="55" t="s">
+        <v>101</v>
+      </c>
+      <c r="C3" s="55" t="s">
+        <v>103</v>
+      </c>
+      <c r="D3" s="55" t="s">
+        <v>102</v>
+      </c>
+      <c r="E3" s="55" t="s">
+        <v>104</v>
+      </c>
+      <c r="F3" s="72" t="s">
+        <v>156</v>
+      </c>
+      <c r="G3" s="72" t="s">
         <v>22</v>
       </c>
-      <c r="H3" s="15" t="s">
-        <v>71</v>
+      <c r="H3" s="14" t="s">
+        <v>69</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
@@ -4835,15 +5383,15 @@
         <v>1</v>
       </c>
       <c r="B4" s="12" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="C4" s="12"/>
       <c r="D4" s="12" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="E4" s="12"/>
-      <c r="F4" s="48" t="s">
-        <v>133</v>
+      <c r="F4" s="45" t="s">
+        <v>129</v>
       </c>
       <c r="G4" s="12">
         <v>3234528921</v>
@@ -4858,19 +5406,19 @@
         <v>2</v>
       </c>
       <c r="B5" s="12" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="C5" s="12" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="D5" s="12" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="E5" s="12" t="s">
-        <v>116</v>
-      </c>
-      <c r="F5" s="48" t="s">
-        <v>133</v>
+        <v>112</v>
+      </c>
+      <c r="F5" s="45" t="s">
+        <v>129</v>
       </c>
       <c r="G5" s="12">
         <v>3161657782</v>
@@ -4885,17 +5433,17 @@
         <v>3</v>
       </c>
       <c r="B6" s="12" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="C6" s="12"/>
       <c r="D6" s="12" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="E6" s="12" t="s">
-        <v>117</v>
-      </c>
-      <c r="F6" s="48" t="s">
-        <v>133</v>
+        <v>113</v>
+      </c>
+      <c r="F6" s="45" t="s">
+        <v>129</v>
       </c>
       <c r="G6" s="12">
         <v>3119884321</v>
@@ -4910,15 +5458,15 @@
         <v>4</v>
       </c>
       <c r="B7" s="12" t="s">
-        <v>124</v>
+        <v>120</v>
       </c>
       <c r="C7" s="12"/>
       <c r="D7" s="12" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="E7" s="12"/>
-      <c r="F7" s="48" t="s">
-        <v>134</v>
+      <c r="F7" s="45" t="s">
+        <v>130</v>
       </c>
       <c r="G7" s="12">
         <v>4127359182</v>
@@ -4963,36 +5511,36 @@
       </c>
     </row>
     <row r="2" spans="1:6" ht="46.5" x14ac:dyDescent="0.25">
-      <c r="A2" s="18" t="s">
+      <c r="A2" s="17" t="s">
         <v>20</v>
       </c>
-      <c r="B2" s="19" t="s">
-        <v>199</v>
-      </c>
-      <c r="C2" s="19" t="s">
-        <v>200</v>
-      </c>
-      <c r="D2" s="19" t="s">
-        <v>201</v>
-      </c>
-      <c r="E2" s="19" t="s">
-        <v>70</v>
+      <c r="B2" s="18" t="s">
+        <v>215</v>
+      </c>
+      <c r="C2" s="18" t="s">
+        <v>186</v>
+      </c>
+      <c r="D2" s="18" t="s">
+        <v>216</v>
+      </c>
+      <c r="E2" s="18" t="s">
+        <v>68</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" s="14" t="s">
+      <c r="A3" s="13" t="s">
         <v>31</v>
       </c>
-      <c r="B3" s="77" t="s">
+      <c r="B3" s="73" t="s">
         <v>35</v>
       </c>
-      <c r="C3" s="77" t="s">
+      <c r="C3" s="73" t="s">
         <v>23</v>
       </c>
-      <c r="D3" s="77" t="s">
-        <v>69</v>
-      </c>
-      <c r="E3" s="32" t="s">
+      <c r="D3" s="73" t="s">
+        <v>67</v>
+      </c>
+      <c r="E3" s="31" t="s">
         <v>36</v>
       </c>
       <c r="F3" s="3"/>
@@ -5004,13 +5552,13 @@
       <c r="B4" s="12">
         <v>10</v>
       </c>
-      <c r="C4" s="42">
+      <c r="C4" s="39">
         <v>10000</v>
       </c>
       <c r="D4" s="12">
         <v>3</v>
       </c>
-      <c r="E4" s="50" t="str">
+      <c r="E4" s="47" t="str">
         <f>Barberia_D!B4</f>
         <v>Barbería Oriental</v>
       </c>
@@ -5035,12 +5583,12 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2190E1EC-B79B-40C0-AC5B-0E2726DDD399}">
-  <dimension ref="A1:F14"/>
+  <dimension ref="A1:F11"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="27" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="26" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="22.5703125" customWidth="1"/>
+    <col min="3" max="3" width="34.42578125" customWidth="1"/>
     <col min="4" max="4" width="23.5703125" customWidth="1"/>
     <col min="5" max="5" width="23.7109375" customWidth="1"/>
     <col min="6" max="6" width="34.85546875" customWidth="1"/>
@@ -5055,60 +5603,60 @@
       </c>
     </row>
     <row r="2" spans="1:6" ht="44.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="19" t="s">
+      <c r="A2" s="18" t="s">
         <v>20</v>
       </c>
-      <c r="B2" s="19" t="s">
+      <c r="B2" s="18" t="s">
+        <v>74</v>
+      </c>
+      <c r="C2" s="18" t="s">
+        <v>214</v>
+      </c>
+      <c r="D2" s="18" t="s">
+        <v>235</v>
+      </c>
+      <c r="E2" s="18" t="s">
+        <v>240</v>
+      </c>
+      <c r="F2" s="18" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" s="13" t="s">
+        <v>31</v>
+      </c>
+      <c r="B3" s="31" t="s">
+        <v>36</v>
+      </c>
+      <c r="C3" s="85" t="s">
+        <v>75</v>
+      </c>
+      <c r="D3" s="74" t="s">
         <v>76</v>
       </c>
-      <c r="C2" s="19" t="s">
-        <v>203</v>
-      </c>
-      <c r="D2" s="19" t="s">
-        <v>204</v>
-      </c>
-      <c r="E2" s="19" t="s">
-        <v>205</v>
-      </c>
-      <c r="F2" s="19" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" s="14" t="s">
-        <v>31</v>
-      </c>
-      <c r="B3" s="32" t="s">
-        <v>36</v>
-      </c>
-      <c r="C3" s="59" t="s">
+      <c r="E3" s="75" t="s">
         <v>77</v>
       </c>
-      <c r="D3" s="78" t="s">
-        <v>78</v>
-      </c>
-      <c r="E3" s="79" t="s">
-        <v>79</v>
-      </c>
-      <c r="F3" s="36" t="s">
-        <v>71</v>
+      <c r="F3" s="34" t="s">
+        <v>69</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="12">
         <v>1</v>
       </c>
-      <c r="B4" s="50" t="str">
+      <c r="B4" s="47" t="str">
         <f>Barberia_D!B4</f>
         <v>Barbería Oriental</v>
       </c>
-      <c r="C4" s="38" t="s">
-        <v>80</v>
-      </c>
-      <c r="D4" s="38">
+      <c r="C4" s="36" t="s">
+        <v>78</v>
+      </c>
+      <c r="D4" s="90">
         <v>0.375</v>
       </c>
-      <c r="E4" s="38">
+      <c r="E4" s="90">
         <v>0.79166666666666663</v>
       </c>
       <c r="F4" s="12" t="str">
@@ -5120,17 +5668,17 @@
       <c r="A5" s="12">
         <v>2</v>
       </c>
-      <c r="B5" s="50" t="str">
+      <c r="B5" s="47" t="str">
         <f>Barberia_D!B4</f>
         <v>Barbería Oriental</v>
       </c>
       <c r="C5" s="12" t="s">
-        <v>81</v>
-      </c>
-      <c r="D5" s="38">
+        <v>79</v>
+      </c>
+      <c r="D5" s="90">
         <v>0.375</v>
       </c>
-      <c r="E5" s="38">
+      <c r="E5" s="90">
         <v>0.79166666666666663</v>
       </c>
       <c r="F5" s="12" t="str">
@@ -5142,17 +5690,17 @@
       <c r="A6" s="12">
         <v>3</v>
       </c>
-      <c r="B6" s="50" t="str">
+      <c r="B6" s="47" t="str">
         <f>Barberia_D!B4</f>
         <v>Barbería Oriental</v>
       </c>
-      <c r="C6" s="38" t="s">
-        <v>82</v>
-      </c>
-      <c r="D6" s="38">
+      <c r="C6" s="36" t="s">
+        <v>80</v>
+      </c>
+      <c r="D6" s="90">
         <v>0.375</v>
       </c>
-      <c r="E6" s="38">
+      <c r="E6" s="90">
         <v>0.79166666666666696</v>
       </c>
       <c r="F6" s="12" t="str">
@@ -5164,17 +5712,17 @@
       <c r="A7" s="12">
         <v>4</v>
       </c>
-      <c r="B7" s="50" t="str">
+      <c r="B7" s="47" t="str">
         <f>Barberia_D!B4</f>
         <v>Barbería Oriental</v>
       </c>
       <c r="C7" s="12" t="s">
-        <v>83</v>
-      </c>
-      <c r="D7" s="38">
+        <v>81</v>
+      </c>
+      <c r="D7" s="90">
         <v>0.375</v>
       </c>
-      <c r="E7" s="38">
+      <c r="E7" s="90">
         <v>0.79166666666666696</v>
       </c>
       <c r="F7" s="12" t="str">
@@ -5186,17 +5734,17 @@
       <c r="A8" s="12">
         <v>5</v>
       </c>
-      <c r="B8" s="50" t="str">
+      <c r="B8" s="47" t="str">
         <f>Barberia_D!B4</f>
         <v>Barbería Oriental</v>
       </c>
-      <c r="C8" s="38" t="s">
-        <v>84</v>
-      </c>
-      <c r="D8" s="38">
+      <c r="C8" s="36" t="s">
+        <v>82</v>
+      </c>
+      <c r="D8" s="90">
         <v>0.375</v>
       </c>
-      <c r="E8" s="38">
+      <c r="E8" s="90">
         <v>0.79166666666666696</v>
       </c>
       <c r="F8" s="12" t="str">
@@ -5208,17 +5756,17 @@
       <c r="A9" s="12">
         <v>6</v>
       </c>
-      <c r="B9" s="50" t="str">
+      <c r="B9" s="47" t="str">
         <f>Barberia_D!B4</f>
         <v>Barbería Oriental</v>
       </c>
       <c r="C9" s="12" t="s">
-        <v>85</v>
-      </c>
-      <c r="D9" s="40">
+        <v>83</v>
+      </c>
+      <c r="D9" s="91">
         <v>0.33333333333333331</v>
       </c>
-      <c r="E9" s="38">
+      <c r="E9" s="90">
         <v>0.875</v>
       </c>
       <c r="F9" s="12" t="str">
@@ -5228,18 +5776,11 @@
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="10"/>
-      <c r="B10" s="39"/>
-      <c r="C10" s="39"/>
+      <c r="B10" s="37"/>
+      <c r="C10" s="37"/>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="C11" s="10" t="s">
-        <v>202</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B14" t="s">
-        <v>220</v>
-      </c>
+      <c r="C11" s="10"/>
     </row>
   </sheetData>
   <phoneticPr fontId="7" type="noConversion"/>
@@ -5271,71 +5812,71 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A1" s="16" t="s">
+      <c r="A1" s="15" t="s">
         <v>32</v>
       </c>
-      <c r="B1" s="16" t="s">
+      <c r="B1" s="15" t="s">
         <v>33</v>
       </c>
-      <c r="D1" s="17"/>
-      <c r="E1" s="17"/>
+      <c r="D1" s="16"/>
+      <c r="E1" s="16"/>
       <c r="F1" s="10"/>
     </row>
     <row r="2" spans="1:6" ht="45.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="18" t="s">
+      <c r="A2" s="17" t="s">
         <v>20</v>
       </c>
-      <c r="B2" s="18" t="s">
-        <v>143</v>
-      </c>
-      <c r="C2" s="18" t="s">
-        <v>206</v>
-      </c>
-      <c r="D2" s="31" t="s">
-        <v>208</v>
-      </c>
-      <c r="E2" s="31" t="s">
-        <v>209</v>
-      </c>
-      <c r="F2" s="19" t="s">
+      <c r="B2" s="17" t="s">
+        <v>137</v>
+      </c>
+      <c r="C2" s="17" t="s">
+        <v>187</v>
+      </c>
+      <c r="D2" s="30" t="s">
+        <v>189</v>
+      </c>
+      <c r="E2" s="30" t="s">
+        <v>190</v>
+      </c>
+      <c r="F2" s="18" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" s="21" t="s">
+      <c r="A3" s="20" t="s">
         <v>31</v>
       </c>
-      <c r="B3" s="55" t="s">
+      <c r="B3" s="52" t="s">
         <v>36</v>
       </c>
-      <c r="C3" s="80" t="s">
+      <c r="C3" s="76" t="s">
         <v>21</v>
       </c>
-      <c r="D3" s="81" t="s">
+      <c r="D3" s="77" t="s">
         <v>37</v>
       </c>
-      <c r="E3" s="81" t="s">
+      <c r="E3" s="77" t="s">
         <v>24</v>
       </c>
-      <c r="F3" s="15" t="s">
-        <v>207</v>
+      <c r="F3" s="14" t="s">
+        <v>188</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4" s="22">
+      <c r="A4" s="21">
         <v>1</v>
       </c>
-      <c r="B4" s="56" t="str">
+      <c r="B4" s="53" t="str">
         <f>Barberia_D!B4</f>
         <v>Barbería Oriental</v>
       </c>
-      <c r="C4" s="22" t="s">
+      <c r="C4" s="21" t="s">
         <v>38</v>
       </c>
-      <c r="D4" s="22">
+      <c r="D4" s="21">
         <v>45</v>
       </c>
-      <c r="E4" s="23">
+      <c r="E4" s="22">
         <v>22000</v>
       </c>
       <c r="F4" s="12" t="str">
@@ -5344,20 +5885,20 @@
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A5" s="22">
+      <c r="A5" s="21">
         <v>2</v>
       </c>
-      <c r="B5" s="56" t="str">
+      <c r="B5" s="53" t="str">
         <f>Barberia_D!B4</f>
         <v>Barbería Oriental</v>
       </c>
-      <c r="C5" s="22" t="s">
+      <c r="C5" s="21" t="s">
         <v>46</v>
       </c>
-      <c r="D5" s="22">
+      <c r="D5" s="21">
         <v>10</v>
       </c>
-      <c r="E5" s="23">
+      <c r="E5" s="22">
         <v>12000</v>
       </c>
       <c r="F5" s="12" t="str">
@@ -5366,20 +5907,20 @@
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A6" s="22">
+      <c r="A6" s="21">
         <v>3</v>
       </c>
-      <c r="B6" s="56" t="str">
+      <c r="B6" s="53" t="str">
         <f>Barberia_D!B4</f>
         <v>Barbería Oriental</v>
       </c>
-      <c r="C6" s="22" t="s">
+      <c r="C6" s="21" t="s">
         <v>47</v>
       </c>
-      <c r="D6" s="22">
+      <c r="D6" s="21">
         <v>15</v>
       </c>
-      <c r="E6" s="23">
+      <c r="E6" s="22">
         <v>15000</v>
       </c>
       <c r="F6" s="12" t="str">
@@ -5388,61 +5929,61 @@
       </c>
     </row>
     <row r="7" spans="1:6" ht="30" x14ac:dyDescent="0.25">
-      <c r="A7" s="22">
+      <c r="A7" s="21">
         <v>4</v>
       </c>
-      <c r="B7" s="56" t="str">
+      <c r="B7" s="53" t="str">
         <f>Barberia_D!B4</f>
         <v>Barbería Oriental</v>
       </c>
-      <c r="C7" s="24" t="s">
+      <c r="C7" s="23" t="s">
         <v>48</v>
       </c>
-      <c r="D7" s="22">
+      <c r="D7" s="21">
         <v>30</v>
       </c>
-      <c r="E7" s="23">
+      <c r="E7" s="22">
         <v>35000</v>
       </c>
-      <c r="F7" s="25" t="str">
+      <c r="F7" s="24" t="str">
         <f t="shared" si="0"/>
         <v>Arreglo completo de barba con toalla caliente</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A8" s="17"/>
-      <c r="B8" s="17"/>
-      <c r="C8" s="17"/>
-      <c r="D8" s="17"/>
-      <c r="E8" s="17"/>
+      <c r="A8" s="16"/>
+      <c r="B8" s="16"/>
+      <c r="C8" s="16"/>
+      <c r="D8" s="16"/>
+      <c r="E8" s="16"/>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A9" s="17"/>
-      <c r="B9" s="17"/>
-      <c r="C9" s="17"/>
-      <c r="D9" s="17"/>
-      <c r="E9" s="17"/>
+      <c r="A9" s="16"/>
+      <c r="B9" s="16"/>
+      <c r="C9" s="16"/>
+      <c r="D9" s="16"/>
+      <c r="E9" s="16"/>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A10" s="17"/>
-      <c r="B10" s="17"/>
-      <c r="C10" s="17"/>
-      <c r="D10" s="17"/>
-      <c r="E10" s="17"/>
+      <c r="A10" s="16"/>
+      <c r="B10" s="16"/>
+      <c r="C10" s="16"/>
+      <c r="D10" s="16"/>
+      <c r="E10" s="16"/>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A11" s="17"/>
-      <c r="B11" s="17"/>
-      <c r="C11" s="17"/>
-      <c r="D11" s="17"/>
-      <c r="E11" s="17"/>
+      <c r="A11" s="16"/>
+      <c r="B11" s="16"/>
+      <c r="C11" s="16"/>
+      <c r="D11" s="16"/>
+      <c r="E11" s="16"/>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A12" s="17"/>
-      <c r="B12" s="17"/>
-      <c r="C12" s="17"/>
-      <c r="D12" s="17"/>
-      <c r="E12" s="17"/>
+      <c r="A12" s="16"/>
+      <c r="B12" s="16"/>
+      <c r="C12" s="16"/>
+      <c r="D12" s="16"/>
+      <c r="E12" s="16"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -5460,7 +6001,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2DAE59AB-4103-4731-9C3C-4C276F8A29F8}">
-  <dimension ref="A1:L14"/>
+  <dimension ref="A1:L10"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="27" bestFit="1" customWidth="1"/>
@@ -5485,79 +6026,79 @@
       <c r="F1" s="5"/>
     </row>
     <row r="2" spans="1:12" ht="45.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="26" t="s">
+      <c r="A2" s="25" t="s">
         <v>20</v>
       </c>
-      <c r="B2" s="26" t="s">
-        <v>165</v>
-      </c>
-      <c r="C2" s="26" t="s">
-        <v>166</v>
-      </c>
-      <c r="D2" s="26" t="s">
-        <v>167</v>
-      </c>
-      <c r="E2" s="26" t="s">
-        <v>168</v>
-      </c>
-      <c r="F2" s="26" t="s">
-        <v>170</v>
-      </c>
-      <c r="G2" s="27" t="s">
-        <v>210</v>
-      </c>
-      <c r="H2" s="27" t="s">
-        <v>211</v>
-      </c>
-      <c r="I2" s="27" t="s">
-        <v>171</v>
-      </c>
-      <c r="J2" s="27" t="s">
-        <v>136</v>
-      </c>
-      <c r="K2" s="27" t="s">
-        <v>144</v>
-      </c>
-      <c r="L2" s="28" t="s">
-        <v>154</v>
+      <c r="B2" s="25" t="s">
+        <v>157</v>
+      </c>
+      <c r="C2" s="25" t="s">
+        <v>158</v>
+      </c>
+      <c r="D2" s="25" t="s">
+        <v>159</v>
+      </c>
+      <c r="E2" s="25" t="s">
+        <v>160</v>
+      </c>
+      <c r="F2" s="25" t="s">
+        <v>161</v>
+      </c>
+      <c r="G2" s="26" t="s">
+        <v>191</v>
+      </c>
+      <c r="H2" s="26" t="s">
+        <v>192</v>
+      </c>
+      <c r="I2" s="26" t="s">
+        <v>162</v>
+      </c>
+      <c r="J2" s="26" t="s">
+        <v>217</v>
+      </c>
+      <c r="K2" s="26" t="s">
+        <v>138</v>
+      </c>
+      <c r="L2" s="27" t="s">
+        <v>147</v>
       </c>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A3" s="14" t="s">
+      <c r="A3" s="13" t="s">
         <v>31</v>
       </c>
-      <c r="B3" s="58" t="s">
-        <v>105</v>
-      </c>
-      <c r="C3" s="58" t="s">
-        <v>107</v>
-      </c>
-      <c r="D3" s="58" t="s">
-        <v>106</v>
-      </c>
-      <c r="E3" s="58" t="s">
-        <v>108</v>
-      </c>
-      <c r="F3" s="76" t="s">
-        <v>132</v>
-      </c>
-      <c r="G3" s="76" t="s">
+      <c r="B3" s="55" t="s">
+        <v>101</v>
+      </c>
+      <c r="C3" s="55" t="s">
+        <v>103</v>
+      </c>
+      <c r="D3" s="55" t="s">
+        <v>102</v>
+      </c>
+      <c r="E3" s="55" t="s">
+        <v>104</v>
+      </c>
+      <c r="F3" s="72" t="s">
+        <v>128</v>
+      </c>
+      <c r="G3" s="72" t="s">
         <v>22</v>
       </c>
-      <c r="H3" s="76" t="s">
+      <c r="H3" s="72" t="s">
         <v>42</v>
       </c>
-      <c r="I3" s="76" t="s">
-        <v>128</v>
-      </c>
-      <c r="J3" s="44" t="s">
+      <c r="I3" s="72" t="s">
+        <v>124</v>
+      </c>
+      <c r="J3" s="41" t="s">
         <v>43</v>
       </c>
-      <c r="K3" s="32" t="s">
+      <c r="K3" s="31" t="s">
         <v>36</v>
       </c>
-      <c r="L3" s="29" t="s">
-        <v>72</v>
+      <c r="L3" s="28" t="s">
+        <v>70</v>
       </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.25">
@@ -5565,19 +6106,19 @@
         <v>1</v>
       </c>
       <c r="B4" s="12" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="C4" s="12" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="D4" s="12" t="s">
-        <v>150</v>
+        <v>143</v>
       </c>
       <c r="E4" s="12" t="s">
-        <v>111</v>
-      </c>
-      <c r="F4" s="48" t="s">
-        <v>133</v>
+        <v>107</v>
+      </c>
+      <c r="F4" s="45" t="s">
+        <v>129</v>
       </c>
       <c r="G4" s="12">
         <v>3245627890</v>
@@ -5585,13 +6126,13 @@
       <c r="H4" s="11" t="s">
         <v>53</v>
       </c>
-      <c r="I4" s="46">
+      <c r="I4" s="43">
         <v>1264267821</v>
       </c>
       <c r="J4" s="12" t="s">
         <v>49</v>
       </c>
-      <c r="K4" s="50" t="str">
+      <c r="K4" s="47" t="str">
         <f>Barberia_D!B4</f>
         <v>Barbería Oriental</v>
       </c>
@@ -5605,19 +6146,19 @@
         <v>2</v>
       </c>
       <c r="B5" s="12" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="C5" s="12" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="D5" s="12" t="s">
-        <v>149</v>
+        <v>142</v>
       </c>
       <c r="E5" s="12" t="s">
-        <v>112</v>
-      </c>
-      <c r="F5" s="48" t="s">
-        <v>133</v>
+        <v>108</v>
+      </c>
+      <c r="F5" s="45" t="s">
+        <v>129</v>
       </c>
       <c r="G5" s="12">
         <v>3124518923</v>
@@ -5625,13 +6166,13 @@
       <c r="H5" s="11" t="s">
         <v>54</v>
       </c>
-      <c r="I5" s="46" t="s">
-        <v>130</v>
+      <c r="I5" s="43" t="s">
+        <v>126</v>
       </c>
       <c r="J5" s="12" t="s">
         <v>49</v>
       </c>
-      <c r="K5" s="50" t="str">
+      <c r="K5" s="47" t="str">
         <f>Barberia_D!B4</f>
         <v>Barbería Oriental</v>
       </c>
@@ -5649,11 +6190,11 @@
       </c>
       <c r="C6" s="12"/>
       <c r="D6" s="12" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="E6" s="12"/>
-      <c r="F6" s="48" t="s">
-        <v>133</v>
+      <c r="F6" s="45" t="s">
+        <v>129</v>
       </c>
       <c r="G6" s="12">
         <v>3214533321</v>
@@ -5661,13 +6202,13 @@
       <c r="H6" s="11" t="s">
         <v>55</v>
       </c>
-      <c r="I6" s="47" t="s">
-        <v>129</v>
+      <c r="I6" s="44" t="s">
+        <v>125</v>
       </c>
       <c r="J6" s="12" t="s">
         <v>49</v>
       </c>
-      <c r="K6" s="50" t="str">
+      <c r="K6" s="47" t="str">
         <f>Barberia_D!B4</f>
         <v>Barbería Oriental</v>
       </c>
@@ -5685,13 +6226,13 @@
       </c>
       <c r="C7" s="12"/>
       <c r="D7" s="12" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="E7" s="12" t="s">
-        <v>113</v>
-      </c>
-      <c r="F7" s="48" t="s">
-        <v>135</v>
+        <v>109</v>
+      </c>
+      <c r="F7" s="45" t="s">
+        <v>131</v>
       </c>
       <c r="G7" s="12">
         <v>9876543210</v>
@@ -5699,13 +6240,13 @@
       <c r="H7" s="11" t="s">
         <v>56</v>
       </c>
-      <c r="I7" s="46" t="s">
-        <v>131</v>
+      <c r="I7" s="43" t="s">
+        <v>127</v>
       </c>
       <c r="J7" s="12" t="s">
         <v>49</v>
       </c>
-      <c r="K7" s="50" t="str">
+      <c r="K7" s="47" t="str">
         <f>Barberia_D!B4</f>
         <v>Barbería Oriental</v>
       </c>
@@ -5719,25 +6260,25 @@
         <v>5</v>
       </c>
       <c r="B8" s="12" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="C8" s="12" t="s">
         <v>51</v>
       </c>
       <c r="D8" s="12" t="s">
-        <v>151</v>
+        <v>144</v>
       </c>
       <c r="E8" s="12" t="s">
-        <v>116</v>
-      </c>
-      <c r="F8" s="48" t="s">
-        <v>152</v>
+        <v>112</v>
+      </c>
+      <c r="F8" s="45" t="s">
+        <v>145</v>
       </c>
       <c r="G8" s="12">
         <v>998765432</v>
       </c>
       <c r="H8" s="11" t="s">
-        <v>153</v>
+        <v>146</v>
       </c>
       <c r="I8" s="12">
         <v>312334342</v>
@@ -5745,7 +6286,7 @@
       <c r="J8" s="12" t="s">
         <v>50</v>
       </c>
-      <c r="K8" s="50" t="str">
+      <c r="K8" s="47" t="str">
         <f>Barberia_D!B4</f>
         <v>Barbería Oriental</v>
       </c>
@@ -5757,11 +6298,6 @@
     <row r="10" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B10" s="10"/>
       <c r="C10" s="10"/>
-    </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="F14" t="s">
-        <v>169</v>
-      </c>
     </row>
   </sheetData>
   <phoneticPr fontId="7" type="noConversion"/>

</xml_diff>

<commit_message>
Se eliminó la relacion entre CLiente y Multa, ya que podría indicar que el cliente siempre tiene una multa. Adicional en el muetreo se añadió un registro en HorarioBarberia y HorarioBarbero,que era si era festivo que pasaba, pues lo pense y no se rompio la logica
</commit_message>
<xml_diff>
--- a/Muestreo de datos.xlsx
+++ b/Muestreo de datos.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/120f6d501c463b80/Escritorio/leo/Doo/Barberia proyecto/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\leand\Desktop\DOO\DOO\Barberia\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="407" documentId="13_ncr:1_{7D2C82A5-CE11-488F-916B-C5EEB7B95CE2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{84D6F366-4DCB-4DED-829F-90BD42E34150}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{686889DE-83BF-4DBB-95FF-005494F7E945}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{09A6C7D7-663F-4C06-9D71-8A4E97495CF9}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{09A6C7D7-663F-4C06-9D71-8A4E97495CF9}"/>
   </bookViews>
   <sheets>
     <sheet name="Modelo de Dominio" sheetId="1" r:id="rId1"/>
@@ -19,9 +19,9 @@
     <sheet name="Barberia_D" sheetId="5" r:id="rId4"/>
     <sheet name="Cliente_D" sheetId="6" r:id="rId5"/>
     <sheet name="Regla_D" sheetId="7" r:id="rId6"/>
-    <sheet name="HorarioBarberia_D" sheetId="18" r:id="rId7"/>
-    <sheet name="Servicio_D" sheetId="8" r:id="rId8"/>
-    <sheet name="Barbero_D" sheetId="9" r:id="rId9"/>
+    <sheet name="Barbero_D" sheetId="9" r:id="rId7"/>
+    <sheet name="HorarioBarberia_D" sheetId="18" r:id="rId8"/>
+    <sheet name="Servicio_D" sheetId="8" r:id="rId9"/>
     <sheet name="Veto_D" sheetId="10" r:id="rId10"/>
     <sheet name="BarberoServicio_D" sheetId="11" r:id="rId11"/>
     <sheet name="Agenda_D" sheetId="12" r:id="rId12"/>
@@ -56,7 +56,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="376" uniqueCount="244">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="378" uniqueCount="247">
   <si>
     <t>Nombre</t>
   </si>
@@ -468,9 +468,6 @@
     <t>Combinacion única que indica que no puede existir más de un cliente con un mismo nombre, apellidos, prefijo de celular y número de celular</t>
   </si>
   <si>
-    <t>Representa la hora prevista a la que finaliza una cita, es un dato calculado a partir de la hora en que empieza la cita y la duración del servicio, sumándole la duración del servicio a la hora de inicio</t>
-  </si>
-  <si>
     <t>Representa el nombre de la barbería que pertenece el servicio</t>
   </si>
   <si>
@@ -637,12 +634,6 @@
   </si>
   <si>
     <t>Representa el correo electronico del barbero, con el que se va a registrar o iniciar seción. Su valor por defecto es el vacio y no es permitido</t>
-  </si>
-  <si>
-    <t>Fecha</t>
-  </si>
-  <si>
-    <t>Tipo de dato que contiene el día, mes y el año.</t>
   </si>
   <si>
     <t>Representa la fecha y la hora en el que se va a realizar la cita al cliente. Su valor por defecto es 01/01/1000 00:00 y no es permitido</t>
@@ -791,6 +782,24 @@
   </si>
   <si>
     <t>Representa la hora en que el barbero empieza su descanso de trabajo. Su valor por defecto es 00:00 y es permitido. La hora debe de estar dentro del horario del barbero, es decir que no se puede salir del horario</t>
+  </si>
+  <si>
+    <t>Logico</t>
+  </si>
+  <si>
+    <t>Tipo de dato que tiene dos posibles valores (Si/No).</t>
+  </si>
+  <si>
+    <t>Necesitare oro objeto de dominio para prefijo</t>
+  </si>
+  <si>
+    <t>Festivo</t>
+  </si>
+  <si>
+    <t>fechaHoraFin</t>
+  </si>
+  <si>
+    <t>Representa la fecha y hora prevista a la que finaliza una cita, es un dato calculado a partir de la fecha y hora en que empieza la cita y la duración del servicio, sumándole la duración del servicio a fechaHora</t>
   </si>
 </sst>
 </file>
@@ -987,7 +996,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="95">
+  <cellXfs count="96">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -1077,9 +1086,6 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="18" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="18" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1225,8 +1231,16 @@
     <xf numFmtId="49" fontId="3" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -1257,22 +1271,22 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>259773</xdr:colOff>
-      <xdr:row>3</xdr:row>
-      <xdr:rowOff>67347</xdr:rowOff>
+      <xdr:colOff>1</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>1</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>16</xdr:col>
-      <xdr:colOff>752223</xdr:colOff>
-      <xdr:row>33</xdr:row>
-      <xdr:rowOff>48106</xdr:rowOff>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>755375</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>90431</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="3" name="Imagen 2">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{7B8920B4-D75C-E415-61FF-DF31117E7B38}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{7CEA3B6A-7E6A-D1B2-1874-4BF2006823E3}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1295,8 +1309,8 @@
       </xdr:blipFill>
       <xdr:spPr bwMode="auto">
         <a:xfrm>
-          <a:off x="259773" y="644620"/>
-          <a:ext cx="13644647" cy="5753486"/>
+          <a:off x="1" y="185531"/>
+          <a:ext cx="10515600" cy="4357630"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1316,10 +1330,6 @@
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1662,12 +1672,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D2495362-94CF-4E08-8433-6F4780C6375E}">
   <dimension ref="A1:AD50"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="26.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="26.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A1" s="5" t="s">
         <v>39</v>
       </c>
@@ -1701,8 +1711,7 @@
       <c r="AC1" s="1"/>
       <c r="AD1" s="1"/>
     </row>
-    <row r="2" spans="1:30" x14ac:dyDescent="0.25">
-      <c r="A2" s="1"/>
+    <row r="2" spans="1:30" x14ac:dyDescent="0.3">
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
@@ -1733,7 +1742,7 @@
       <c r="AC2" s="1"/>
       <c r="AD2" s="1"/>
     </row>
-    <row r="3" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A3" s="1"/>
       <c r="B3" s="1"/>
       <c r="C3" s="1"/>
@@ -1765,7 +1774,7 @@
       <c r="AC3" s="1"/>
       <c r="AD3" s="1"/>
     </row>
-    <row r="4" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:30" x14ac:dyDescent="0.3">
       <c r="B4" s="1"/>
       <c r="C4" s="1"/>
       <c r="D4" s="1"/>
@@ -1796,7 +1805,7 @@
       <c r="AC4" s="1"/>
       <c r="AD4" s="1"/>
     </row>
-    <row r="5" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A5" s="1"/>
       <c r="B5" s="1"/>
       <c r="C5" s="1"/>
@@ -1828,7 +1837,7 @@
       <c r="AC5" s="1"/>
       <c r="AD5" s="1"/>
     </row>
-    <row r="6" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A6" s="1"/>
       <c r="B6" s="1"/>
       <c r="D6" s="1"/>
@@ -1859,7 +1868,7 @@
       <c r="AC6" s="1"/>
       <c r="AD6" s="1"/>
     </row>
-    <row r="7" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A7" s="1"/>
       <c r="C7" s="1"/>
       <c r="D7" s="1"/>
@@ -1890,7 +1899,7 @@
       <c r="AC7" s="1"/>
       <c r="AD7" s="1"/>
     </row>
-    <row r="8" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A8" s="1"/>
       <c r="B8" s="1"/>
       <c r="C8" s="1"/>
@@ -1922,7 +1931,7 @@
       <c r="AC8" s="1"/>
       <c r="AD8" s="1"/>
     </row>
-    <row r="9" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A9" s="1"/>
       <c r="B9" s="1"/>
       <c r="C9" s="1"/>
@@ -1954,7 +1963,7 @@
       <c r="AC9" s="1"/>
       <c r="AD9" s="1"/>
     </row>
-    <row r="10" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A10" s="1"/>
       <c r="B10" s="1"/>
       <c r="C10" s="1"/>
@@ -1986,7 +1995,7 @@
       <c r="AC10" s="1"/>
       <c r="AD10" s="1"/>
     </row>
-    <row r="11" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A11" s="1"/>
       <c r="B11" s="1"/>
       <c r="C11" s="1"/>
@@ -2018,7 +2027,7 @@
       <c r="AC11" s="1"/>
       <c r="AD11" s="1"/>
     </row>
-    <row r="12" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A12" s="1"/>
       <c r="B12" s="1"/>
       <c r="C12" s="1"/>
@@ -2050,7 +2059,7 @@
       <c r="AC12" s="1"/>
       <c r="AD12" s="1"/>
     </row>
-    <row r="13" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A13" s="1"/>
       <c r="B13" s="1"/>
       <c r="C13" s="1"/>
@@ -2082,7 +2091,7 @@
       <c r="AC13" s="1"/>
       <c r="AD13" s="1"/>
     </row>
-    <row r="14" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A14" s="1"/>
       <c r="B14" s="1"/>
       <c r="C14" s="1"/>
@@ -2114,7 +2123,7 @@
       <c r="AC14" s="1"/>
       <c r="AD14" s="1"/>
     </row>
-    <row r="15" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A15" s="1"/>
       <c r="B15" s="1"/>
       <c r="C15" s="1"/>
@@ -2146,7 +2155,7 @@
       <c r="AC15" s="1"/>
       <c r="AD15" s="1"/>
     </row>
-    <row r="16" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A16" s="1"/>
       <c r="B16" s="1"/>
       <c r="C16" s="1"/>
@@ -2178,7 +2187,7 @@
       <c r="AC16" s="1"/>
       <c r="AD16" s="1"/>
     </row>
-    <row r="17" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A17" s="1"/>
       <c r="B17" s="1"/>
       <c r="C17" s="1"/>
@@ -2210,7 +2219,7 @@
       <c r="AC17" s="1"/>
       <c r="AD17" s="1"/>
     </row>
-    <row r="18" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A18" s="1"/>
       <c r="B18" s="1"/>
       <c r="C18" s="1"/>
@@ -2242,7 +2251,7 @@
       <c r="AC18" s="1"/>
       <c r="AD18" s="1"/>
     </row>
-    <row r="19" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A19" s="1"/>
       <c r="B19" s="1"/>
       <c r="C19" s="1"/>
@@ -2274,7 +2283,7 @@
       <c r="AC19" s="1"/>
       <c r="AD19" s="1"/>
     </row>
-    <row r="20" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A20" s="1"/>
       <c r="B20" s="1"/>
       <c r="C20" s="1"/>
@@ -2306,7 +2315,7 @@
       <c r="AC20" s="1"/>
       <c r="AD20" s="1"/>
     </row>
-    <row r="21" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A21" s="1"/>
       <c r="B21" s="1"/>
       <c r="C21" s="1"/>
@@ -2338,7 +2347,7 @@
       <c r="AC21" s="1"/>
       <c r="AD21" s="1"/>
     </row>
-    <row r="22" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A22" s="1"/>
       <c r="B22" s="1"/>
       <c r="C22" s="1"/>
@@ -2370,7 +2379,7 @@
       <c r="AC22" s="1"/>
       <c r="AD22" s="1"/>
     </row>
-    <row r="23" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A23" s="1"/>
       <c r="B23" s="1"/>
       <c r="C23" s="1"/>
@@ -2402,7 +2411,7 @@
       <c r="AC23" s="1"/>
       <c r="AD23" s="1"/>
     </row>
-    <row r="24" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A24" s="1"/>
       <c r="B24" s="1"/>
       <c r="C24" s="1"/>
@@ -2434,7 +2443,7 @@
       <c r="AC24" s="1"/>
       <c r="AD24" s="1"/>
     </row>
-    <row r="25" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A25" s="1"/>
       <c r="B25" s="1"/>
       <c r="C25" s="1"/>
@@ -2466,7 +2475,7 @@
       <c r="AC25" s="1"/>
       <c r="AD25" s="1"/>
     </row>
-    <row r="26" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A26" s="1"/>
       <c r="B26" s="1"/>
       <c r="C26" s="1"/>
@@ -2498,7 +2507,7 @@
       <c r="AC26" s="1"/>
       <c r="AD26" s="1"/>
     </row>
-    <row r="27" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A27" s="1"/>
       <c r="B27" s="1"/>
       <c r="C27" s="1"/>
@@ -2530,7 +2539,7 @@
       <c r="AC27" s="1"/>
       <c r="AD27" s="1"/>
     </row>
-    <row r="28" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A28" s="1"/>
       <c r="B28" s="1"/>
       <c r="C28" s="1"/>
@@ -2562,7 +2571,7 @@
       <c r="AC28" s="1"/>
       <c r="AD28" s="1"/>
     </row>
-    <row r="29" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A29" s="1"/>
       <c r="B29" s="1"/>
       <c r="C29" s="1"/>
@@ -2594,7 +2603,7 @@
       <c r="AC29" s="1"/>
       <c r="AD29" s="1"/>
     </row>
-    <row r="30" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A30" s="1"/>
       <c r="B30" s="1"/>
       <c r="C30" s="1"/>
@@ -2626,7 +2635,7 @@
       <c r="AC30" s="1"/>
       <c r="AD30" s="1"/>
     </row>
-    <row r="31" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A31" s="1"/>
       <c r="B31" s="1"/>
       <c r="C31" s="1"/>
@@ -2658,7 +2667,7 @@
       <c r="AC31" s="1"/>
       <c r="AD31" s="1"/>
     </row>
-    <row r="32" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A32" s="1"/>
       <c r="B32" s="1"/>
       <c r="C32" s="1"/>
@@ -2690,7 +2699,7 @@
       <c r="AC32" s="1"/>
       <c r="AD32" s="1"/>
     </row>
-    <row r="33" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A33" s="1"/>
       <c r="B33" s="1"/>
       <c r="C33" s="1"/>
@@ -2722,7 +2731,7 @@
       <c r="AC33" s="1"/>
       <c r="AD33" s="1"/>
     </row>
-    <row r="34" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A34" s="1"/>
       <c r="B34" s="1"/>
       <c r="C34" s="1"/>
@@ -2754,7 +2763,7 @@
       <c r="AC34" s="1"/>
       <c r="AD34" s="1"/>
     </row>
-    <row r="35" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A35" s="1"/>
       <c r="B35" s="1"/>
       <c r="C35" s="1"/>
@@ -2786,7 +2795,7 @@
       <c r="AC35" s="1"/>
       <c r="AD35" s="1"/>
     </row>
-    <row r="36" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A36" s="1"/>
       <c r="B36" s="1"/>
       <c r="C36" s="1"/>
@@ -2818,7 +2827,7 @@
       <c r="AC36" s="1"/>
       <c r="AD36" s="1"/>
     </row>
-    <row r="37" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A37" s="1"/>
       <c r="B37" s="1"/>
       <c r="C37" s="1"/>
@@ -2850,7 +2859,7 @@
       <c r="AC37" s="1"/>
       <c r="AD37" s="1"/>
     </row>
-    <row r="38" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A38" s="1"/>
       <c r="B38" s="1"/>
       <c r="C38" s="1"/>
@@ -2882,7 +2891,7 @@
       <c r="AC38" s="1"/>
       <c r="AD38" s="1"/>
     </row>
-    <row r="39" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A39" s="1"/>
       <c r="B39" s="1"/>
       <c r="C39" s="1"/>
@@ -2914,7 +2923,7 @@
       <c r="AC39" s="1"/>
       <c r="AD39" s="1"/>
     </row>
-    <row r="40" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A40" s="1"/>
       <c r="B40" s="1"/>
       <c r="C40" s="1"/>
@@ -2946,7 +2955,7 @@
       <c r="AC40" s="1"/>
       <c r="AD40" s="1"/>
     </row>
-    <row r="41" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A41" s="1"/>
       <c r="B41" s="1"/>
       <c r="C41" s="1"/>
@@ -2978,7 +2987,7 @@
       <c r="AC41" s="1"/>
       <c r="AD41" s="1"/>
     </row>
-    <row r="42" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A42" s="1"/>
       <c r="B42" s="1"/>
       <c r="C42" s="1"/>
@@ -3010,7 +3019,7 @@
       <c r="AC42" s="1"/>
       <c r="AD42" s="1"/>
     </row>
-    <row r="43" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A43" s="1"/>
       <c r="B43" s="1"/>
       <c r="C43" s="1"/>
@@ -3042,7 +3051,7 @@
       <c r="AC43" s="1"/>
       <c r="AD43" s="1"/>
     </row>
-    <row r="44" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A44" s="1"/>
       <c r="B44" s="1"/>
       <c r="C44" s="1"/>
@@ -3074,7 +3083,7 @@
       <c r="AC44" s="1"/>
       <c r="AD44" s="1"/>
     </row>
-    <row r="45" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A45" s="1"/>
       <c r="B45" s="1"/>
       <c r="C45" s="1"/>
@@ -3106,7 +3115,7 @@
       <c r="AC45" s="1"/>
       <c r="AD45" s="1"/>
     </row>
-    <row r="46" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A46" s="1"/>
       <c r="B46" s="1"/>
       <c r="C46" s="1"/>
@@ -3138,7 +3147,7 @@
       <c r="AC46" s="1"/>
       <c r="AD46" s="1"/>
     </row>
-    <row r="47" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A47" s="1"/>
       <c r="B47" s="1"/>
       <c r="C47" s="1"/>
@@ -3170,7 +3179,7 @@
       <c r="AC47" s="1"/>
       <c r="AD47" s="1"/>
     </row>
-    <row r="48" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A48" s="1"/>
       <c r="B48" s="1"/>
       <c r="C48" s="1"/>
@@ -3202,7 +3211,7 @@
       <c r="AC48" s="1"/>
       <c r="AD48" s="1"/>
     </row>
-    <row r="49" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A49" s="1"/>
       <c r="B49" s="1"/>
       <c r="C49" s="1"/>
@@ -3234,7 +3243,7 @@
       <c r="AC49" s="1"/>
       <c r="AD49" s="1"/>
     </row>
-    <row r="50" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A50" s="1"/>
       <c r="B50" s="1"/>
       <c r="C50" s="1"/>
@@ -3279,16 +3288,16 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C828B98D-AAA9-4184-8373-FE2E421AAE23}">
   <dimension ref="A1:G11"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="2" width="27" customWidth="1"/>
-    <col min="3" max="4" width="28.85546875" customWidth="1"/>
+    <col min="3" max="4" width="28.88671875" customWidth="1"/>
     <col min="5" max="5" width="41" customWidth="1"/>
-    <col min="6" max="6" width="36.140625" customWidth="1"/>
-    <col min="7" max="7" width="26.85546875" customWidth="1"/>
+    <col min="6" max="6" width="36.109375" customWidth="1"/>
+    <col min="7" max="7" width="26.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" s="5" t="s">
         <v>32</v>
       </c>
@@ -3297,21 +3306,21 @@
       </c>
       <c r="D1" s="5"/>
     </row>
-    <row r="2" spans="1:7" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="17" t="s">
         <v>20</v>
       </c>
       <c r="B2" s="17" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="C2" s="17" t="s">
-        <v>237</v>
+        <v>234</v>
       </c>
       <c r="D2" s="17" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="E2" s="30" t="s">
-        <v>218</v>
+        <v>215</v>
       </c>
       <c r="F2" s="30" t="s">
         <v>123</v>
@@ -3320,34 +3329,34 @@
         <v>58</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" s="13" t="s">
         <v>31</v>
       </c>
       <c r="B3" s="31" t="s">
-        <v>224</v>
+        <v>221</v>
       </c>
       <c r="C3" s="31" t="s">
         <v>59</v>
       </c>
       <c r="D3" s="31" t="s">
-        <v>222</v>
-      </c>
-      <c r="E3" s="41" t="s">
+        <v>219</v>
+      </c>
+      <c r="E3" s="40" t="s">
         <v>25</v>
       </c>
-      <c r="F3" s="41" t="s">
+      <c r="F3" s="40" t="s">
         <v>57</v>
       </c>
       <c r="G3" s="28" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" s="12">
         <v>1</v>
       </c>
-      <c r="B4" s="92" t="str">
+      <c r="B4" s="91" t="str">
         <f>Cliente_D!F4</f>
         <v>+57</v>
       </c>
@@ -3370,11 +3379,11 @@
         <v>3234528921-25/11/2023</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" s="12">
         <v>2</v>
       </c>
-      <c r="B5" s="92" t="str">
+      <c r="B5" s="91" t="str">
         <f>Cliente_D!F5</f>
         <v>+57</v>
       </c>
@@ -3397,11 +3406,11 @@
         <v>3161657782-21/03/2024</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" s="12">
         <v>3</v>
       </c>
-      <c r="B6" s="92" t="str">
+      <c r="B6" s="91" t="str">
         <f>Cliente_D!F6</f>
         <v>+57</v>
       </c>
@@ -3424,11 +3433,11 @@
         <v>3119884321-21/09/2024</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" s="12">
         <v>4</v>
       </c>
-      <c r="B7" s="92" t="str">
+      <c r="B7" s="91" t="str">
         <f>Cliente_D!F7</f>
         <v>+58</v>
       </c>
@@ -3451,12 +3460,12 @@
         <v>4127359182-11/12/2025</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="E8" s="29"/>
       <c r="F8" s="29"/>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="E11" s="42"/>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="E11" s="41"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -3485,15 +3494,15 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A24A074A-5C83-448D-978C-7C1005CE378E}">
   <dimension ref="A1:D7"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="29.140625" customWidth="1"/>
+    <col min="1" max="1" width="29.109375" customWidth="1"/>
     <col min="2" max="2" width="30" customWidth="1"/>
-    <col min="3" max="3" width="41.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="61.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="41.88671875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="61.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="5" t="s">
         <v>32</v>
       </c>
@@ -3501,7 +3510,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" ht="36.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="17" t="s">
         <v>20</v>
       </c>
@@ -3511,11 +3520,11 @@
       <c r="C2" s="30" t="s">
         <v>62</v>
       </c>
-      <c r="D2" s="40" t="s">
+      <c r="D2" s="39" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" s="13" t="s">
         <v>31</v>
       </c>
@@ -3529,7 +3538,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" s="12">
         <v>1</v>
       </c>
@@ -3546,7 +3555,7 @@
         <v>Juan García-Motilada</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" s="12">
         <v>2</v>
       </c>
@@ -3563,7 +3572,7 @@
         <v>Juan Ortiz-Corte de barba</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" s="12">
         <v>3</v>
       </c>
@@ -3580,7 +3589,7 @@
         <v>Carlos Arbeladez-Perfilada de barba</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" s="12">
         <v>4</v>
       </c>
@@ -3620,14 +3629,14 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2921A3C4-B96A-49A7-8353-9FD37D2F2B74}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
-    <col min="2" max="2" width="42.28515625" customWidth="1"/>
-    <col min="3" max="3" width="37.42578125" customWidth="1"/>
+    <col min="2" max="2" width="42.33203125" customWidth="1"/>
+    <col min="3" max="3" width="37.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="5" t="s">
         <v>32</v>
       </c>
@@ -3635,7 +3644,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="28.5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" ht="30" x14ac:dyDescent="0.3">
       <c r="A2" s="17" t="s">
         <v>20</v>
       </c>
@@ -3646,7 +3655,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" s="13" t="s">
         <v>31</v>
       </c>
@@ -3657,7 +3666,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" s="12">
         <v>1</v>
       </c>
@@ -3670,7 +3679,7 @@
         <v>Juan García</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" s="12">
         <v>2</v>
       </c>
@@ -3683,7 +3692,7 @@
         <v>Juan Ortiz</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" s="12">
         <v>3</v>
       </c>
@@ -3696,7 +3705,7 @@
         <v>Carlos Arbeladez</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" s="12">
         <v>4</v>
       </c>
@@ -3727,18 +3736,18 @@
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{86AE141B-6E6C-47BF-9B70-297A81AC9A72}">
   <dimension ref="A1:G7"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="26.85546875" customWidth="1"/>
-    <col min="2" max="2" width="32.5703125" customWidth="1"/>
-    <col min="3" max="3" width="34.5703125" customWidth="1"/>
-    <col min="4" max="4" width="32.5703125" customWidth="1"/>
-    <col min="5" max="5" width="21.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="20.140625" customWidth="1"/>
-    <col min="7" max="7" width="47.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="26.88671875" customWidth="1"/>
+    <col min="2" max="2" width="32.5546875" customWidth="1"/>
+    <col min="3" max="3" width="34.5546875" customWidth="1"/>
+    <col min="4" max="4" width="32.5546875" customWidth="1"/>
+    <col min="5" max="5" width="21.88671875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="20.109375" customWidth="1"/>
+    <col min="7" max="7" width="47.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" s="5" t="s">
         <v>32</v>
       </c>
@@ -3748,53 +3757,53 @@
       <c r="C1" s="5"/>
       <c r="D1" s="5"/>
     </row>
-    <row r="2" spans="1:7" ht="46.5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" ht="39.6" x14ac:dyDescent="0.3">
       <c r="A2" s="17" t="s">
         <v>20</v>
       </c>
       <c r="B2" s="18" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
       <c r="C2" s="30" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
       <c r="D2" s="30" t="s">
-        <v>233</v>
+        <v>230</v>
       </c>
       <c r="E2" s="18" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="F2" s="18" t="s">
-        <v>234</v>
+        <v>231</v>
       </c>
       <c r="G2" s="18" t="s">
-        <v>201</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" s="13" t="s">
         <v>31</v>
       </c>
       <c r="B3" s="31" t="s">
         <v>60</v>
       </c>
-      <c r="C3" s="87" t="s">
-        <v>229</v>
-      </c>
-      <c r="D3" s="87" t="s">
-        <v>230</v>
-      </c>
-      <c r="E3" s="86" t="s">
+      <c r="C3" s="86" t="s">
+        <v>226</v>
+      </c>
+      <c r="D3" s="86" t="s">
+        <v>227</v>
+      </c>
+      <c r="E3" s="85" t="s">
         <v>21</v>
       </c>
-      <c r="F3" s="41" t="s">
+      <c r="F3" s="40" t="s">
         <v>37</v>
       </c>
       <c r="G3" s="28" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" s="12">
         <v>1</v>
       </c>
@@ -3802,14 +3811,14 @@
         <f>Agenda_D!C4</f>
         <v>Juan García</v>
       </c>
-      <c r="C4" s="88">
+      <c r="C4" s="87">
         <v>46047.458333333336</v>
       </c>
-      <c r="D4" s="88">
+      <c r="D4" s="87">
         <v>46047.541666666664</v>
       </c>
-      <c r="E4" s="80" t="s">
-        <v>208</v>
+      <c r="E4" s="79" t="s">
+        <v>205</v>
       </c>
       <c r="F4" s="12">
         <v>120</v>
@@ -3819,7 +3828,7 @@
         <v>Juan García-25/01/2026 11:00-25/01/2026 13:00</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" s="12">
         <v>2</v>
       </c>
@@ -3827,14 +3836,14 @@
         <f>Agenda_D!C5</f>
         <v>Juan Ortiz</v>
       </c>
-      <c r="C5" s="88">
+      <c r="C5" s="87">
         <v>45362.5</v>
       </c>
-      <c r="D5" s="88">
+      <c r="D5" s="87">
         <v>45362.645833333336</v>
       </c>
-      <c r="E5" s="82" t="s">
-        <v>209</v>
+      <c r="E5" s="81" t="s">
+        <v>206</v>
       </c>
       <c r="F5" s="12">
         <v>210</v>
@@ -3844,7 +3853,7 @@
         <v>Juan Ortiz-11/03/2024 12:00-11/03/2024 15:30</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" s="12">
         <v>3</v>
       </c>
@@ -3852,14 +3861,14 @@
         <f>Agenda_D!C6</f>
         <v>Carlos Arbeladez</v>
       </c>
-      <c r="C6" s="88">
+      <c r="C6" s="87">
         <v>46013.541666666664</v>
       </c>
-      <c r="D6" s="88">
+      <c r="D6" s="87">
         <v>46013.583333333336</v>
       </c>
-      <c r="E6" s="82" t="s">
-        <v>210</v>
+      <c r="E6" s="81" t="s">
+        <v>207</v>
       </c>
       <c r="F6" s="12">
         <v>60</v>
@@ -3869,22 +3878,22 @@
         <v>Carlos Arbeladez-22/12/2025 13:00-22/12/2025 14:00</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" s="12">
         <v>4</v>
       </c>
-      <c r="B7" s="79" t="str">
+      <c r="B7" s="78" t="str">
         <f>Agenda_D!C7</f>
         <v>Andres Ramirez</v>
       </c>
-      <c r="C7" s="89">
+      <c r="C7" s="88">
         <v>46241.375</v>
       </c>
-      <c r="D7" s="89">
+      <c r="D7" s="88">
         <v>46241.5</v>
       </c>
-      <c r="E7" s="82" t="s">
-        <v>211</v>
+      <c r="E7" s="81" t="s">
+        <v>208</v>
       </c>
       <c r="F7" s="12">
         <v>180</v>
@@ -3910,18 +3919,18 @@
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5CFE76D0-FBB4-4C81-85CC-F644057A8847}">
-  <dimension ref="A1:F16"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:F11"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="27" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="37.140625" customWidth="1"/>
-    <col min="3" max="3" width="46.5703125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="26.85546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="48.5703125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="37.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="37.109375" customWidth="1"/>
+    <col min="3" max="3" width="46.5546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="26.88671875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="48.5546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="37.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" s="5" t="s">
         <v>32</v>
       </c>
@@ -3929,7 +3938,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="40.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" ht="40.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="18" t="s">
         <v>20</v>
       </c>
@@ -3937,53 +3946,53 @@
         <v>86</v>
       </c>
       <c r="C2" s="18" t="s">
+        <v>235</v>
+      </c>
+      <c r="D2" s="18" t="s">
+        <v>236</v>
+      </c>
+      <c r="E2" s="18" t="s">
         <v>238</v>
-      </c>
-      <c r="D2" s="18" t="s">
-        <v>239</v>
-      </c>
-      <c r="E2" s="18" t="s">
-        <v>241</v>
       </c>
       <c r="F2" s="18" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" s="13" t="s">
         <v>31</v>
       </c>
       <c r="B3" s="31" t="s">
         <v>60</v>
       </c>
-      <c r="C3" s="85" t="s">
+      <c r="C3" s="84" t="s">
         <v>75</v>
       </c>
-      <c r="D3" s="75" t="s">
+      <c r="D3" s="74" t="s">
         <v>63</v>
       </c>
-      <c r="E3" s="75" t="s">
+      <c r="E3" s="74" t="s">
         <v>85</v>
       </c>
       <c r="F3" s="28" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" s="12">
         <v>1</v>
       </c>
-      <c r="B4" s="47" t="str">
+      <c r="B4" s="46" t="str">
         <f>Agenda_D!C4</f>
         <v>Juan García</v>
       </c>
       <c r="C4" s="36" t="s">
         <v>78</v>
       </c>
-      <c r="D4" s="90">
+      <c r="D4" s="89">
         <v>0.41666666666666669</v>
       </c>
-      <c r="E4" s="90">
+      <c r="E4" s="89">
         <v>0.66666666666666663</v>
       </c>
       <c r="F4" s="12" t="str">
@@ -3991,43 +4000,43 @@
         <v>Juan García-Lunes-10-16</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" s="12">
         <v>2</v>
       </c>
-      <c r="B5" s="47" t="str">
+      <c r="B5" s="46" t="str">
         <f>Agenda_D!C5</f>
         <v>Juan Ortiz</v>
       </c>
       <c r="C5" s="12" t="s">
         <v>79</v>
       </c>
-      <c r="D5" s="90">
+      <c r="D5" s="89">
         <v>0.375</v>
       </c>
-      <c r="E5" s="90">
+      <c r="E5" s="89">
         <v>0.625</v>
       </c>
       <c r="F5" s="12" t="str">
-        <f t="shared" ref="F5:F7" si="0">_xlfn.CONCAT(B5,"-",C5,"-",TEXT(D5,"hh;mm"),"-",TEXT(E5,"hh;mm"))</f>
+        <f t="shared" ref="F5:F8" si="0">_xlfn.CONCAT(B5,"-",C5,"-",TEXT(D5,"hh;mm"),"-",TEXT(E5,"hh;mm"))</f>
         <v>Juan Ortiz-Martes-09-15</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" s="12">
         <v>3</v>
       </c>
-      <c r="B6" s="47" t="str">
+      <c r="B6" s="46" t="str">
         <f>Agenda_D!C6</f>
         <v>Carlos Arbeladez</v>
       </c>
       <c r="C6" s="12" t="s">
         <v>81</v>
       </c>
-      <c r="D6" s="90">
+      <c r="D6" s="89">
         <v>0.54166666666666663</v>
       </c>
-      <c r="E6" s="90">
+      <c r="E6" s="89">
         <v>0.79166666666666663</v>
       </c>
       <c r="F6" s="12" t="str">
@@ -4035,21 +4044,21 @@
         <v>Carlos Arbeladez-Jueves-13-19</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7" s="12">
         <v>4</v>
       </c>
-      <c r="B7" s="47" t="str">
+      <c r="B7" s="46" t="str">
         <f>Agenda_D!C7</f>
         <v>Andres Ramirez</v>
       </c>
       <c r="C7" s="12" t="s">
         <v>83</v>
       </c>
-      <c r="D7" s="90">
+      <c r="D7" s="89">
         <v>0.33333333333333331</v>
       </c>
-      <c r="E7" s="90">
+      <c r="E7" s="89">
         <v>0.58333333333333337</v>
       </c>
       <c r="F7" s="12" t="str">
@@ -4057,33 +4066,34 @@
         <v>Andres Ramirez-Sábado-08-14</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="E8" s="93"/>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="E9" s="93"/>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A8" s="94">
+        <v>5</v>
+      </c>
+      <c r="B8" s="11" t="str">
+        <f>Agenda_D!C7</f>
+        <v>Andres Ramirez</v>
+      </c>
+      <c r="C8" s="94" t="s">
+        <v>244</v>
+      </c>
+      <c r="D8" s="89">
+        <v>0.5</v>
+      </c>
+      <c r="E8" s="89">
+        <v>0.625</v>
+      </c>
+      <c r="F8" s="94" t="str">
+        <f t="shared" si="0"/>
+        <v>Andres Ramirez-Festivo-12-15</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
       <c r="C10" s="10"/>
-      <c r="E10" s="94"/>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="E11" s="94"/>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="E12" s="93"/>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="E13" s="93"/>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="E14" s="93"/>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="E15" s="93"/>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="E16" s="93"/>
+      <c r="E10" s="10"/>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E11" s="10"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -4095,6 +4105,7 @@
     <hyperlink ref="B5" location="Agenda_D!A5" display="Agenda_D!A5" xr:uid="{22BB4167-53C0-4D10-9F76-560F79FADE86}"/>
     <hyperlink ref="B6" location="Agenda_D!A6" display="Agenda_D!A6" xr:uid="{36B092FB-CBA5-4E3A-9127-52EA641442EA}"/>
     <hyperlink ref="B7" location="Agenda_D!A7" display="Agenda_D!A7" xr:uid="{59DFEC77-AF33-433C-99D6-F82241ADA5F1}"/>
+    <hyperlink ref="B8" location="Agenda_D!A7" display="Agenda_D!A7" xr:uid="{F90905DD-1298-4E08-99DE-C45A5F8D96D3}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -4103,18 +4114,18 @@
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EB38530B-FD95-4EEF-8F76-78E045637369}">
   <dimension ref="A1:G7"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="26.85546875" customWidth="1"/>
-    <col min="2" max="2" width="32.5703125" customWidth="1"/>
-    <col min="3" max="3" width="32.7109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="31.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="26.7109375" customWidth="1"/>
-    <col min="6" max="6" width="29.140625" customWidth="1"/>
-    <col min="7" max="7" width="33.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="26.88671875" customWidth="1"/>
+    <col min="2" max="2" width="32.5546875" customWidth="1"/>
+    <col min="3" max="3" width="32.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="31.109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="26.6640625" customWidth="1"/>
+    <col min="6" max="6" width="29.109375" customWidth="1"/>
+    <col min="7" max="7" width="33.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" s="5" t="s">
         <v>32</v>
       </c>
@@ -4122,53 +4133,53 @@
         <v>33</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="40.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" ht="40.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="17" t="s">
         <v>20</v>
       </c>
       <c r="B2" s="18" t="s">
-        <v>203</v>
+        <v>200</v>
       </c>
       <c r="C2" s="18" t="s">
-        <v>243</v>
+        <v>240</v>
       </c>
       <c r="D2" s="18" t="s">
-        <v>242</v>
+        <v>239</v>
       </c>
       <c r="E2" s="18" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="F2" s="30" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="G2" s="18" t="s">
-        <v>212</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" s="13" t="s">
         <v>31</v>
       </c>
       <c r="B3" s="31" t="s">
-        <v>202</v>
-      </c>
-      <c r="C3" s="75" t="s">
+        <v>199</v>
+      </c>
+      <c r="C3" s="74" t="s">
         <v>63</v>
       </c>
-      <c r="D3" s="75" t="s">
-        <v>200</v>
-      </c>
-      <c r="E3" s="72" t="s">
+      <c r="D3" s="74" t="s">
+        <v>197</v>
+      </c>
+      <c r="E3" s="71" t="s">
         <v>21</v>
       </c>
-      <c r="F3" s="83" t="s">
+      <c r="F3" s="82" t="s">
         <v>37</v>
       </c>
       <c r="G3" s="28" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" s="12">
         <v>1</v>
       </c>
@@ -4183,9 +4194,9 @@
         <v>0.58333333333333337</v>
       </c>
       <c r="E4" s="36" t="s">
-        <v>204</v>
-      </c>
-      <c r="F4" s="84">
+        <v>201</v>
+      </c>
+      <c r="F4" s="83">
         <v>120</v>
       </c>
       <c r="G4" s="12" t="str">
@@ -4193,7 +4204,7 @@
         <v>Juan García-Lunes-10-16-12-14</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" s="12">
         <v>2</v>
       </c>
@@ -4204,11 +4215,11 @@
       <c r="C5" s="36">
         <v>0.54166666666666663</v>
       </c>
-      <c r="D5" s="81">
+      <c r="D5" s="80">
         <v>0.625</v>
       </c>
       <c r="E5" s="24" t="s">
-        <v>207</v>
+        <v>204</v>
       </c>
       <c r="F5" s="12">
         <v>120</v>
@@ -4218,7 +4229,7 @@
         <v>Juan Ortiz-Martes-09-15-13-15</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" s="12">
         <v>3</v>
       </c>
@@ -4233,7 +4244,7 @@
         <v>0.75</v>
       </c>
       <c r="E6" s="12" t="s">
-        <v>206</v>
+        <v>203</v>
       </c>
       <c r="F6" s="12">
         <v>60</v>
@@ -4243,7 +4254,7 @@
         <v>Carlos Arbeladez-Jueves-13-19-17-18</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" s="12">
         <v>4</v>
       </c>
@@ -4258,7 +4269,7 @@
         <v>0.54166666666666663</v>
       </c>
       <c r="E7" s="12" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
       <c r="F7" s="12">
         <v>90</v>
@@ -4284,20 +4295,20 @@
 
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1429879F-6697-4F1F-AF5D-52C4860B7B3E}">
-  <dimension ref="A1:H18"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:H15"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="28" customWidth="1"/>
-    <col min="2" max="2" width="26.5703125" customWidth="1"/>
-    <col min="3" max="3" width="30.42578125" customWidth="1"/>
-    <col min="4" max="4" width="27.5703125" customWidth="1"/>
-    <col min="5" max="5" width="36.5703125" customWidth="1"/>
-    <col min="6" max="6" width="60.28515625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="39.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="26.5546875" customWidth="1"/>
+    <col min="3" max="3" width="30.44140625" customWidth="1"/>
+    <col min="4" max="4" width="27.5546875" customWidth="1"/>
+    <col min="5" max="5" width="36.5546875" customWidth="1"/>
+    <col min="6" max="6" width="60.33203125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="39.33203125" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="22" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A1" s="5" t="s">
         <v>32</v>
       </c>
@@ -4305,7 +4316,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="44.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" ht="44.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="17" t="s">
         <v>20</v>
       </c>
@@ -4313,22 +4324,22 @@
         <v>64</v>
       </c>
       <c r="C2" s="30" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="D2" s="30" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
       <c r="E2" s="30" t="s">
-        <v>136</v>
+        <v>246</v>
       </c>
       <c r="F2" s="30" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="G2" s="30" t="s">
         <v>133</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" s="13" t="s">
         <v>31</v>
       </c>
@@ -4338,20 +4349,20 @@
       <c r="C3" s="31" t="s">
         <v>60</v>
       </c>
-      <c r="D3" s="78" t="s">
+      <c r="D3" s="77" t="s">
         <v>132</v>
       </c>
-      <c r="E3" s="41" t="s">
-        <v>85</v>
-      </c>
-      <c r="F3" s="55" t="s">
+      <c r="E3" s="40" t="s">
+        <v>245</v>
+      </c>
+      <c r="F3" s="54" t="s">
         <v>26</v>
       </c>
       <c r="G3" s="28" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A4" s="12">
         <v>1</v>
       </c>
@@ -4363,11 +4374,11 @@
         <f>Agenda_D!C4</f>
         <v>Juan García</v>
       </c>
-      <c r="D4" s="49">
+      <c r="D4" s="48">
         <v>46295.416666666664</v>
       </c>
-      <c r="E4" s="90">
-        <v>0.44791666666666669</v>
+      <c r="E4" s="48">
+        <v>46295.447916666664</v>
       </c>
       <c r="F4" s="12" t="s">
         <v>65</v>
@@ -4377,7 +4388,7 @@
         <v>Juan García-30/09/2026/10:00</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A5" s="12">
         <v>2</v>
       </c>
@@ -4389,11 +4400,11 @@
         <f>Agenda_D!C5</f>
         <v>Juan Ortiz</v>
       </c>
-      <c r="D5" s="49">
+      <c r="D5" s="48">
         <v>45983.458333333336</v>
       </c>
-      <c r="E5" s="90">
-        <v>0.48958333333333331</v>
+      <c r="E5" s="48">
+        <v>45983.489583333336</v>
       </c>
       <c r="F5" s="12" t="s">
         <v>88</v>
@@ -4403,7 +4414,7 @@
         <v>Juan Ortiz-22/11/2025/11:00</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A6" s="12">
         <v>3</v>
       </c>
@@ -4415,11 +4426,11 @@
         <f>Agenda_D!C6</f>
         <v>Carlos Arbeladez</v>
       </c>
-      <c r="D6" s="49">
+      <c r="D6" s="48">
         <v>45514.583333333336</v>
       </c>
-      <c r="E6" s="90">
-        <v>0.59375</v>
+      <c r="E6" s="48">
+        <v>45514.59375</v>
       </c>
       <c r="F6" s="12" t="s">
         <v>134</v>
@@ -4429,7 +4440,7 @@
         <v>Carlos Arbeladez-10/08/2024/14:00</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A7" s="12">
         <v>4</v>
       </c>
@@ -4441,11 +4452,11 @@
         <f>Agenda_D!C7</f>
         <v>Andres Ramirez</v>
       </c>
-      <c r="D7" s="49">
+      <c r="D7" s="48">
         <v>46289.541666666664</v>
       </c>
-      <c r="E7" s="90">
-        <v>0.5625</v>
+      <c r="E7" s="48">
+        <v>46289.5625</v>
       </c>
       <c r="F7" s="12" t="s">
         <v>89</v>
@@ -4455,7 +4466,7 @@
         <v>Andres Ramirez-24/09/2026/13:00</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A8" s="12">
         <v>5</v>
       </c>
@@ -4467,11 +4478,11 @@
         <f>Agenda_D!C6</f>
         <v>Carlos Arbeladez</v>
       </c>
-      <c r="D8" s="49">
+      <c r="D8" s="48">
         <v>46240.75</v>
       </c>
-      <c r="E8" s="90">
-        <v>0.75694444444444442</v>
+      <c r="E8" s="48">
+        <v>46240.756944444445</v>
       </c>
       <c r="F8" s="12" t="s">
         <v>90</v>
@@ -4480,34 +4491,30 @@
         <f t="shared" si="0"/>
         <v>Carlos Arbeladez-06/08/2026/18:00</v>
       </c>
-      <c r="H8" s="46"/>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="H10" s="48"/>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="H8" s="45"/>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="E10" s="95"/>
+      <c r="H10" s="47"/>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="E11" s="95"/>
       <c r="F11" s="10"/>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="D12" s="50"/>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="D13" s="50"/>
-    </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="D14" s="50"/>
-    </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="D15" s="50"/>
-    </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="E16" s="93"/>
-    </row>
-    <row r="17" spans="5:5" x14ac:dyDescent="0.25">
-      <c r="E17" s="93"/>
-    </row>
-    <row r="18" spans="5:5" x14ac:dyDescent="0.25">
-      <c r="E18" s="93"/>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="D12" s="49"/>
+      <c r="E12" s="95"/>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="D13" s="49"/>
+      <c r="E13" s="95"/>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="D14" s="49"/>
+      <c r="E14" s="95"/>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="D15" s="49"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -4535,17 +4542,17 @@
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{766573FB-AAA2-4254-B83C-7C7505540365}">
   <dimension ref="A1:G7"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="26.7109375" customWidth="1"/>
-    <col min="2" max="2" width="38.5703125" customWidth="1"/>
-    <col min="3" max="3" width="39.28515625" bestFit="1" customWidth="1"/>
-    <col min="4" max="5" width="39.7109375" customWidth="1"/>
-    <col min="6" max="6" width="34.28515625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="39.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="26.6640625" customWidth="1"/>
+    <col min="2" max="2" width="38.5546875" customWidth="1"/>
+    <col min="3" max="3" width="39.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="39.6640625" customWidth="1"/>
+    <col min="6" max="6" width="34.33203125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="39.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" s="5" t="s">
         <v>32</v>
       </c>
@@ -4553,7 +4560,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" ht="31.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="17" t="s">
         <v>20</v>
       </c>
@@ -4564,10 +4571,10 @@
         <v>93</v>
       </c>
       <c r="D2" s="30" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
       <c r="E2" s="30" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F2" s="30" t="s">
         <v>94</v>
@@ -4576,7 +4583,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" s="13" t="s">
         <v>31</v>
       </c>
@@ -4586,20 +4593,20 @@
       <c r="C3" s="31" t="s">
         <v>91</v>
       </c>
-      <c r="D3" s="41" t="s">
+      <c r="D3" s="40" t="s">
         <v>27</v>
       </c>
-      <c r="E3" s="54" t="s">
-        <v>140</v>
-      </c>
-      <c r="F3" s="41" t="s">
+      <c r="E3" s="53" t="s">
+        <v>139</v>
+      </c>
+      <c r="F3" s="40" t="s">
         <v>28</v>
       </c>
       <c r="G3" s="28" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" s="12">
         <v>1</v>
       </c>
@@ -4626,7 +4633,7 @@
         <v>Carlos Arbeladez-10/08/2024/14:00</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" s="12">
         <v>2</v>
       </c>
@@ -4639,7 +4646,7 @@
         <v>Andres Ramirez-24/09/2026/13:00</v>
       </c>
       <c r="D5" s="12">
-        <f>CitaServicio_D!D7</f>
+        <f>CitaServicio_D!D8</f>
         <v>35000</v>
       </c>
       <c r="E5" s="12" t="s">
@@ -4653,7 +4660,7 @@
         <v>Andres Ramirez-24/09/2026/13:00</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" s="10"/>
       <c r="B6" s="10"/>
       <c r="C6" s="10"/>
@@ -4662,7 +4669,7 @@
       <c r="F6" s="10"/>
       <c r="G6" s="10"/>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" s="10"/>
       <c r="B7" s="10"/>
       <c r="C7" s="10"/>
@@ -4688,18 +4695,18 @@
 
 <file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F470C5A4-8D15-43DA-95FC-91C9614E5EEA}">
-  <dimension ref="A1:F8"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:F9"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="26.42578125" customWidth="1"/>
-    <col min="2" max="2" width="39.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="21.85546875" customWidth="1"/>
-    <col min="4" max="4" width="41.85546875" customWidth="1"/>
-    <col min="5" max="5" width="32.140625" customWidth="1"/>
-    <col min="6" max="6" width="55.85546875" customWidth="1"/>
+    <col min="1" max="1" width="26.44140625" customWidth="1"/>
+    <col min="2" max="2" width="39.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="21.88671875" customWidth="1"/>
+    <col min="4" max="4" width="41.88671875" customWidth="1"/>
+    <col min="5" max="5" width="32.109375" customWidth="1"/>
+    <col min="6" max="6" width="55.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" s="5" t="s">
         <v>32</v>
       </c>
@@ -4707,7 +4714,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="33" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" ht="33" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="17" t="s">
         <v>20</v>
       </c>
@@ -4718,7 +4725,7 @@
         <v>97</v>
       </c>
       <c r="D2" s="30" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="E2" s="30" t="s">
         <v>98</v>
@@ -4727,8 +4734,8 @@
         <v>99</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" s="38" t="s">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A3" s="37" t="s">
         <v>31</v>
       </c>
       <c r="B3" s="31" t="s">
@@ -4737,17 +4744,17 @@
       <c r="C3" s="31" t="s">
         <v>41</v>
       </c>
-      <c r="D3" s="73" t="s">
+      <c r="D3" s="72" t="s">
         <v>29</v>
       </c>
-      <c r="E3" s="73" t="s">
+      <c r="E3" s="72" t="s">
         <v>30</v>
       </c>
       <c r="F3" s="28" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" s="12">
         <v>1</v>
       </c>
@@ -4770,7 +4777,7 @@
         <v>Juan García-30/09/2026/10:00-Motilada</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" s="12">
         <v>2</v>
       </c>
@@ -4779,84 +4786,108 @@
         <v>Juan Ortiz-22/11/2025/11:00</v>
       </c>
       <c r="C5" s="11" t="str">
+        <f>Servicio_D!F5</f>
+        <v>Corte de barba</v>
+      </c>
+      <c r="D5" s="12">
+        <v>12000</v>
+      </c>
+      <c r="E5" s="12">
+        <v>10</v>
+      </c>
+      <c r="F5" s="12" t="str">
+        <f>_xlfn.CONCAT(B5,"-",C5)</f>
+        <v>Juan Ortiz-22/11/2025/11:00-Corte de barba</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A6" s="12">
+        <v>3</v>
+      </c>
+      <c r="B6" s="11" t="str">
+        <f>Cita_D!G5</f>
+        <v>Juan Ortiz-22/11/2025/11:00</v>
+      </c>
+      <c r="C6" s="11" t="str">
         <f>Servicio_D!F4</f>
         <v>Motilada</v>
       </c>
-      <c r="D5" s="12">
+      <c r="D6" s="12">
         <v>22000</v>
       </c>
-      <c r="E5" s="12">
+      <c r="E6" s="12">
         <v>45</v>
       </c>
-      <c r="F5" s="12" t="str">
-        <f t="shared" ref="F5:F8" si="0">_xlfn.CONCAT(B5,"-",C5)</f>
+      <c r="F6" s="12" t="str">
+        <f t="shared" ref="F6:F9" si="0">_xlfn.CONCAT(B6,"-",C6)</f>
         <v>Juan Ortiz-22/11/2025/11:00-Motilada</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A6" s="12">
-        <v>3</v>
-      </c>
-      <c r="B6" s="11" t="str">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A7" s="12">
+        <v>4</v>
+      </c>
+      <c r="B7" s="11" t="str">
         <f>Cita_D!G6</f>
         <v>Carlos Arbeladez-10/08/2024/14:00</v>
       </c>
-      <c r="C6" s="11" t="str">
+      <c r="C7" s="11" t="str">
         <f>Servicio_D!F6</f>
         <v>Perfilada de barba</v>
       </c>
-      <c r="D6" s="12">
+      <c r="D7" s="12">
         <v>15000</v>
       </c>
-      <c r="E6" s="12">
+      <c r="E7" s="12">
         <v>15</v>
       </c>
-      <c r="F6" s="12" t="str">
+      <c r="F7" s="12" t="str">
         <f t="shared" si="0"/>
         <v>Carlos Arbeladez-10/08/2024/14:00-Perfilada de barba</v>
       </c>
     </row>
-    <row r="7" spans="1:6" ht="45" x14ac:dyDescent="0.25">
-      <c r="A7" s="12">
-        <v>4</v>
-      </c>
-      <c r="B7" s="11" t="str">
+    <row r="8" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A8" s="12">
+        <v>5</v>
+      </c>
+      <c r="B8" s="11" t="str">
         <f>Cita_D!G7</f>
         <v>Andres Ramirez-24/09/2026/13:00</v>
       </c>
-      <c r="C7" s="51" t="str">
+      <c r="C8" s="50" t="str">
         <f>Servicio_D!F7</f>
         <v>Arreglo completo de barba con toalla caliente</v>
       </c>
-      <c r="D7" s="12">
+      <c r="D8" s="12">
         <v>35000</v>
       </c>
-      <c r="E7" s="12">
+      <c r="E8" s="12">
         <v>30</v>
       </c>
-      <c r="F7" s="24" t="str">
+      <c r="F8" s="24" t="str">
         <f t="shared" si="0"/>
         <v>Andres Ramirez-24/09/2026/13:00-Arreglo completo de barba con toalla caliente</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A8" s="12">
-        <v>5</v>
-      </c>
-      <c r="B8" s="11" t="str">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A9" s="12">
+        <v>6</v>
+      </c>
+      <c r="B9" s="11" t="str">
         <f>Cita_D!G8</f>
         <v>Carlos Arbeladez-06/08/2026/18:00</v>
       </c>
-      <c r="C8" s="11" t="s">
-        <v>46</v>
-      </c>
-      <c r="D8" s="12">
+      <c r="C9" s="11" t="str">
+        <f>Servicio_D!C5</f>
+        <v>Corte de barba</v>
+      </c>
+      <c r="D9" s="12">
         <v>12000</v>
       </c>
-      <c r="E8" s="12">
+      <c r="E9" s="12">
         <v>10</v>
       </c>
-      <c r="F8" s="24" t="str">
+      <c r="F9" s="24" t="str">
         <f t="shared" si="0"/>
         <v>Carlos Arbeladez-06/08/2026/18:00-Corte de barba</v>
       </c>
@@ -4867,17 +4898,19 @@
     <hyperlink ref="B1" location="'Objetos de Dominio'!A1" display="&lt;&lt;&lt;&lt; Ir a objetos de dominio" xr:uid="{57379F34-219A-4662-8198-09F584C326D5}"/>
     <hyperlink ref="B3" location="Cita_D!A1" display="cita" xr:uid="{E89AB6B9-F364-4BAD-BFEA-CAA2C102229E}"/>
     <hyperlink ref="B4" location="Cita_D!A4" display="Cita_D!A4" xr:uid="{0CF27EF5-B7FA-41F5-B712-E18CF914FB99}"/>
-    <hyperlink ref="B5:B8" location="Cita_D!A4" display="Cita_D!A4" xr:uid="{24E1B3F9-C1C3-4AC0-83CF-93AC9D358E4F}"/>
-    <hyperlink ref="B5" location="Cita_D!A5" display="Cita_D!A5" xr:uid="{54C06FE5-3D1C-4E02-B80F-F52398660735}"/>
-    <hyperlink ref="B6" location="Cita_D!A6" display="Cita_D!A6" xr:uid="{7C3F9E66-FC63-4CC5-A67C-8604702403F0}"/>
-    <hyperlink ref="B7" location="Cita_D!A7" display="Cita_D!A7" xr:uid="{B03F3CEB-2FAE-4C17-B421-BB7244341FF9}"/>
-    <hyperlink ref="B8" location="Cita_D!A8" display="Cita_D!A8" xr:uid="{FA20FBDC-E2C6-44CF-B98E-C85818BE6D1B}"/>
+    <hyperlink ref="B6:B9" location="Cita_D!A4" display="Cita_D!A4" xr:uid="{24E1B3F9-C1C3-4AC0-83CF-93AC9D358E4F}"/>
+    <hyperlink ref="B6" location="Cita_D!A5" display="Cita_D!A5" xr:uid="{54C06FE5-3D1C-4E02-B80F-F52398660735}"/>
+    <hyperlink ref="B7" location="Cita_D!A6" display="Cita_D!A6" xr:uid="{7C3F9E66-FC63-4CC5-A67C-8604702403F0}"/>
+    <hyperlink ref="B8" location="Cita_D!A7" display="Cita_D!A7" xr:uid="{B03F3CEB-2FAE-4C17-B421-BB7244341FF9}"/>
+    <hyperlink ref="B9" location="Cita_D!A8" display="Cita_D!A8" xr:uid="{FA20FBDC-E2C6-44CF-B98E-C85818BE6D1B}"/>
     <hyperlink ref="C3" location="Servicio_D!A1" display="servicio" xr:uid="{46A59B94-B463-41EF-A1B6-2B1BD97218B9}"/>
     <hyperlink ref="C4" location="Servicio_D!A4" display="Servicio_D!A4" xr:uid="{E5D47101-7002-491C-A64F-9E08C0E5E166}"/>
-    <hyperlink ref="C5" location="Servicio_D!A4" display="Servicio_D!A4" xr:uid="{EC363894-A006-45A1-A451-8A105D143020}"/>
-    <hyperlink ref="C6" location="Servicio_D!A6" display="Servicio_D!A6" xr:uid="{2F70A83F-4454-46E6-A1E5-B359824AA24F}"/>
-    <hyperlink ref="C7" location="Servicio_D!A7" display="Servicio_D!A7" xr:uid="{36945D0D-E1EC-4BD2-A67D-287FB73A0E8D}"/>
-    <hyperlink ref="C8" location="Servicio_D!A5" display="Corte de barba" xr:uid="{52D089FF-955D-405E-BFF7-8EABA1516B8E}"/>
+    <hyperlink ref="C6" location="Servicio_D!A4" display="Servicio_D!A4" xr:uid="{EC363894-A006-45A1-A451-8A105D143020}"/>
+    <hyperlink ref="C7" location="Servicio_D!A6" display="Servicio_D!A6" xr:uid="{2F70A83F-4454-46E6-A1E5-B359824AA24F}"/>
+    <hyperlink ref="C8" location="Servicio_D!A7" display="Servicio_D!A7" xr:uid="{36945D0D-E1EC-4BD2-A67D-287FB73A0E8D}"/>
+    <hyperlink ref="C9" location="Servicio_D!A5" display="Corte de barba" xr:uid="{52D089FF-955D-405E-BFF7-8EABA1516B8E}"/>
+    <hyperlink ref="B5" location="Cita_D!A4" display="Cita_D!A4" xr:uid="{39C11A52-01CE-4DAA-BC18-9212C37DBE32}"/>
+    <hyperlink ref="C5" location="Servicio_D!A5" display="Servicio_D!A5" xr:uid="{C52FCEDE-6EC5-4607-AF2D-6AA06D251491}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -4886,20 +4919,20 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7A5AA025-A9A3-4E3E-A766-44885AA770B6}">
   <dimension ref="A1:D17"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="27" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="63.7109375" customWidth="1"/>
-    <col min="3" max="3" width="14.42578125" customWidth="1"/>
-    <col min="4" max="4" width="7.7109375" customWidth="1"/>
+    <col min="2" max="2" width="63.6640625" customWidth="1"/>
+    <col min="3" max="3" width="14.44140625" customWidth="1"/>
+    <col min="4" max="4" width="7.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="5" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" s="6" t="s">
         <v>0</v>
       </c>
@@ -4913,7 +4946,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:4" ht="45" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A3" s="7" t="s">
         <v>4</v>
       </c>
@@ -4927,12 +4960,12 @@
         <v>34</v>
       </c>
     </row>
-    <row r="4" spans="1:4" ht="75" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A4" s="7" t="s">
         <v>11</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="C4" s="7">
         <v>1</v>
@@ -4941,12 +4974,12 @@
         <v>34</v>
       </c>
     </row>
-    <row r="5" spans="1:4" ht="60" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A5" s="7" t="s">
         <v>5</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="C5" s="7">
         <v>2</v>
@@ -4955,12 +4988,12 @@
         <v>34</v>
       </c>
     </row>
-    <row r="6" spans="1:4" ht="45" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A6" s="7" t="s">
         <v>72</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="C6" s="7">
         <v>2</v>
@@ -4969,12 +5002,12 @@
         <v>34</v>
       </c>
     </row>
-    <row r="7" spans="1:4" ht="60" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A7" s="7" t="s">
         <v>6</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C7" s="7">
         <v>2</v>
@@ -4983,7 +5016,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="8" spans="1:4" ht="45" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A8" s="7" t="s">
         <v>7</v>
       </c>
@@ -4997,12 +5030,12 @@
         <v>34</v>
       </c>
     </row>
-    <row r="9" spans="1:4" ht="75" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A9" s="7" t="s">
         <v>13</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="C9" s="7">
         <v>2</v>
@@ -5011,7 +5044,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="10" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A10" s="7" t="s">
         <v>8</v>
       </c>
@@ -5025,12 +5058,12 @@
         <v>34</v>
       </c>
     </row>
-    <row r="11" spans="1:4" ht="45" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A11" s="7" t="s">
         <v>9</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="C11" s="7">
         <v>3</v>
@@ -5039,12 +5072,12 @@
         <v>34</v>
       </c>
     </row>
-    <row r="12" spans="1:4" ht="90" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:4" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A12" s="7" t="s">
-        <v>196</v>
+        <v>193</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
       <c r="C12" s="7">
         <v>4</v>
@@ -5053,12 +5086,12 @@
         <v>34</v>
       </c>
     </row>
-    <row r="13" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A13" s="7" t="s">
         <v>73</v>
       </c>
       <c r="B13" s="8" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="C13" s="7">
         <v>4</v>
@@ -5067,12 +5100,12 @@
         <v>34</v>
       </c>
     </row>
-    <row r="14" spans="1:4" ht="90" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:4" ht="72" x14ac:dyDescent="0.3">
       <c r="A14" s="7" t="s">
         <v>10</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="C14" s="7">
         <v>4</v>
@@ -5081,12 +5114,12 @@
         <v>34</v>
       </c>
     </row>
-    <row r="15" spans="1:4" ht="60" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A15" s="7" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
       <c r="B15" s="8" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
       <c r="C15" s="7">
         <v>5</v>
@@ -5095,7 +5128,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="16" spans="1:4" ht="45" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A16" s="7" t="s">
         <v>12</v>
       </c>
@@ -5109,7 +5142,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="17" spans="1:4" ht="60" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A17" s="7" t="s">
         <v>14</v>
       </c>
@@ -5149,98 +5182,98 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{387DE6AC-7D92-461D-9DD1-84082B531231}">
   <dimension ref="A1:B11"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="18.42578125" customWidth="1"/>
-    <col min="2" max="2" width="69.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="18.44140625" customWidth="1"/>
+    <col min="2" max="2" width="69.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="7" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B1" s="7" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" s="56" t="s">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A2" s="55" t="s">
+        <v>163</v>
+      </c>
+      <c r="B2" s="55" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A3" s="56" t="s">
         <v>164</v>
       </c>
-      <c r="B2" s="56" t="s">
+      <c r="B3" s="65" t="s">
         <v>172</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="30" x14ac:dyDescent="0.25">
-      <c r="A3" s="57" t="s">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A4" s="58" t="s">
         <v>165</v>
       </c>
-      <c r="B3" s="66" t="s">
+      <c r="B4" s="58" t="s">
         <v>173</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" s="59" t="s">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A5" s="57" t="s">
+        <v>241</v>
+      </c>
+      <c r="B5" s="66" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A6" s="59" t="s">
         <v>166</v>
       </c>
-      <c r="B4" s="59" t="s">
+      <c r="B6" s="59" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A7" s="60" t="s">
+        <v>167</v>
+      </c>
+      <c r="B7" s="67" t="s">
         <v>174</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5" s="58" t="s">
-        <v>193</v>
-      </c>
-      <c r="B5" s="67" t="s">
-        <v>194</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A6" s="60" t="s">
-        <v>167</v>
-      </c>
-      <c r="B6" s="60" t="s">
+    <row r="8" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A8" s="61" t="s">
+        <v>168</v>
+      </c>
+      <c r="B8" s="68" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A9" s="62" t="s">
+        <v>69</v>
+      </c>
+      <c r="B9" s="69" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A10" s="63" t="s">
+        <v>169</v>
+      </c>
+      <c r="B10" s="63" t="s">
         <v>178</v>
       </c>
     </row>
-    <row r="7" spans="1:2" ht="30" x14ac:dyDescent="0.25">
-      <c r="A7" s="61" t="s">
-        <v>168</v>
-      </c>
-      <c r="B7" s="68" t="s">
-        <v>175</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" ht="30" x14ac:dyDescent="0.25">
-      <c r="A8" s="62" t="s">
-        <v>169</v>
-      </c>
-      <c r="B8" s="69" t="s">
-        <v>176</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" ht="45" x14ac:dyDescent="0.25">
-      <c r="A9" s="63" t="s">
-        <v>69</v>
-      </c>
-      <c r="B9" s="70" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" ht="45" x14ac:dyDescent="0.25">
-      <c r="A10" s="64" t="s">
+    <row r="11" spans="1:2" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A11" s="64" t="s">
         <v>170</v>
       </c>
-      <c r="B10" s="64" t="s">
+      <c r="B11" s="70" t="s">
         <v>179</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" ht="75" x14ac:dyDescent="0.25">
-      <c r="A11" s="65" t="s">
-        <v>171</v>
-      </c>
-      <c r="B11" s="71" t="s">
-        <v>180</v>
       </c>
     </row>
   </sheetData>
@@ -5251,14 +5284,14 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AAA22F8C-1648-4644-8301-765EB2B8C50B}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="33.85546875" customWidth="1"/>
-    <col min="2" max="2" width="34.7109375" customWidth="1"/>
+    <col min="1" max="1" width="33.88671875" customWidth="1"/>
+    <col min="2" max="2" width="34.6640625" customWidth="1"/>
     <col min="3" max="3" width="21" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="5" t="s">
         <v>32</v>
       </c>
@@ -5266,24 +5299,24 @@
         <v>33</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="18" t="s">
         <v>20</v>
       </c>
       <c r="B2" s="18" t="s">
-        <v>213</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" s="13" t="s">
         <v>31</v>
       </c>
-      <c r="B3" s="72" t="s">
+      <c r="B3" s="71" t="s">
         <v>21</v>
       </c>
       <c r="C3" s="35"/>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" s="12">
         <v>1</v>
       </c>
@@ -5304,15 +5337,15 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{28259140-2713-4A98-8730-76D57DC1D653}">
   <dimension ref="A1:H11"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="26.85546875" style="10" customWidth="1"/>
-    <col min="2" max="6" width="26.28515625" style="10" customWidth="1"/>
-    <col min="7" max="7" width="23.140625" style="10" customWidth="1"/>
-    <col min="8" max="8" width="38.5703125" style="10" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="26.88671875" style="10" customWidth="1"/>
+    <col min="2" max="6" width="26.33203125" style="10" customWidth="1"/>
+    <col min="7" max="7" width="23.109375" style="10" customWidth="1"/>
+    <col min="8" max="8" width="38.5546875" style="10" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A1" s="11" t="s">
         <v>32</v>
       </c>
@@ -5326,59 +5359,59 @@
       <c r="G1" s="12"/>
       <c r="H1" s="12"/>
     </row>
-    <row r="2" spans="1:8" ht="46.5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" ht="39.6" x14ac:dyDescent="0.3">
       <c r="A2" s="17" t="s">
         <v>20</v>
       </c>
       <c r="B2" s="17" t="s">
+        <v>180</v>
+      </c>
+      <c r="C2" s="17" t="s">
         <v>181</v>
       </c>
-      <c r="C2" s="17" t="s">
+      <c r="D2" s="17" t="s">
         <v>182</v>
       </c>
-      <c r="D2" s="17" t="s">
+      <c r="E2" s="17" t="s">
         <v>183</v>
       </c>
-      <c r="E2" s="17" t="s">
+      <c r="F2" s="17" t="s">
+        <v>218</v>
+      </c>
+      <c r="G2" s="18" t="s">
         <v>184</v>
-      </c>
-      <c r="F2" s="17" t="s">
-        <v>221</v>
-      </c>
-      <c r="G2" s="18" t="s">
-        <v>185</v>
       </c>
       <c r="H2" s="19" t="s">
         <v>135</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" s="13" t="s">
         <v>31</v>
       </c>
-      <c r="B3" s="55" t="s">
+      <c r="B3" s="54" t="s">
         <v>101</v>
       </c>
-      <c r="C3" s="55" t="s">
+      <c r="C3" s="54" t="s">
         <v>103</v>
       </c>
-      <c r="D3" s="55" t="s">
+      <c r="D3" s="54" t="s">
         <v>102</v>
       </c>
-      <c r="E3" s="55" t="s">
+      <c r="E3" s="54" t="s">
         <v>104</v>
       </c>
-      <c r="F3" s="72" t="s">
-        <v>156</v>
-      </c>
-      <c r="G3" s="72" t="s">
+      <c r="F3" s="71" t="s">
+        <v>155</v>
+      </c>
+      <c r="G3" s="71" t="s">
         <v>22</v>
       </c>
       <c r="H3" s="14" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A4" s="12">
         <v>1</v>
       </c>
@@ -5390,7 +5423,7 @@
         <v>111</v>
       </c>
       <c r="E4" s="12"/>
-      <c r="F4" s="45" t="s">
+      <c r="F4" s="44" t="s">
         <v>129</v>
       </c>
       <c r="G4" s="12">
@@ -5401,7 +5434,7 @@
         <v>Juan--Gómez--+57-3234528921</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A5" s="12">
         <v>2</v>
       </c>
@@ -5417,7 +5450,7 @@
       <c r="E5" s="12" t="s">
         <v>112</v>
       </c>
-      <c r="F5" s="45" t="s">
+      <c r="F5" s="44" t="s">
         <v>129</v>
       </c>
       <c r="G5" s="12">
@@ -5428,7 +5461,7 @@
         <v>Jose-Miguel-Ramirez-Perez-+57-3161657782</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A6" s="12">
         <v>3</v>
       </c>
@@ -5442,7 +5475,7 @@
       <c r="E6" s="12" t="s">
         <v>113</v>
       </c>
-      <c r="F6" s="45" t="s">
+      <c r="F6" s="44" t="s">
         <v>129</v>
       </c>
       <c r="G6" s="12">
@@ -5453,7 +5486,7 @@
         <v>Simon--Ochoa-Ramirez-+57-3119884321</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A7" s="12">
         <v>4</v>
       </c>
@@ -5465,7 +5498,7 @@
         <v>114</v>
       </c>
       <c r="E7" s="12"/>
-      <c r="F7" s="45" t="s">
+      <c r="F7" s="44" t="s">
         <v>130</v>
       </c>
       <c r="G7" s="12">
@@ -5476,7 +5509,7 @@
         <v>Alexis--Gallego--+58-4127359182</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
       <c r="C11"/>
     </row>
   </sheetData>
@@ -5492,17 +5525,17 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B0E77388-6266-4A55-B7A3-4FCD2B643D29}">
   <dimension ref="A1:F5"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="26.85546875" customWidth="1"/>
-    <col min="2" max="2" width="32.5703125" customWidth="1"/>
+    <col min="1" max="1" width="26.88671875" customWidth="1"/>
+    <col min="2" max="2" width="32.5546875" customWidth="1"/>
     <col min="3" max="3" width="28" customWidth="1"/>
-    <col min="4" max="4" width="26.7109375" customWidth="1"/>
-    <col min="5" max="5" width="16.28515625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="18.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="26.6640625" customWidth="1"/>
+    <col min="5" max="5" width="16.33203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="18.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" s="5" t="s">
         <v>32</v>
       </c>
@@ -5510,34 +5543,34 @@
         <v>33</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="46.5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" ht="49.2" x14ac:dyDescent="0.3">
       <c r="A2" s="17" t="s">
         <v>20</v>
       </c>
       <c r="B2" s="18" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="C2" s="18" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="D2" s="18" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="E2" s="18" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" s="13" t="s">
         <v>31</v>
       </c>
-      <c r="B3" s="73" t="s">
+      <c r="B3" s="72" t="s">
         <v>35</v>
       </c>
-      <c r="C3" s="73" t="s">
+      <c r="C3" s="72" t="s">
         <v>23</v>
       </c>
-      <c r="D3" s="73" t="s">
+      <c r="D3" s="72" t="s">
         <v>67</v>
       </c>
       <c r="E3" s="31" t="s">
@@ -5545,20 +5578,20 @@
       </c>
       <c r="F3" s="3"/>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" s="12">
         <v>1</v>
       </c>
       <c r="B4" s="12">
         <v>10</v>
       </c>
-      <c r="C4" s="39">
+      <c r="C4" s="38">
         <v>10000</v>
       </c>
       <c r="D4" s="12">
         <v>3</v>
       </c>
-      <c r="E4" s="47" t="str">
+      <c r="E4" s="46" t="str">
         <f>Barberia_D!B4</f>
         <v>Barbería Oriental</v>
       </c>
@@ -5567,7 +5600,7 @@
         <v/>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="D5" s="2"/>
     </row>
   </sheetData>
@@ -5582,438 +5615,20 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2190E1EC-B79B-40C0-AC5B-0E2726DDD399}">
-  <dimension ref="A1:F11"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2DAE59AB-4103-4731-9C3C-4C276F8A29F8}">
+  <dimension ref="A1:L11"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="27" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="26" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="34.42578125" customWidth="1"/>
-    <col min="4" max="4" width="23.5703125" customWidth="1"/>
-    <col min="5" max="5" width="23.7109375" customWidth="1"/>
-    <col min="6" max="6" width="34.85546875" customWidth="1"/>
+    <col min="2" max="6" width="26.6640625" customWidth="1"/>
+    <col min="7" max="7" width="16.33203125" customWidth="1"/>
+    <col min="8" max="9" width="40.6640625" customWidth="1"/>
+    <col min="10" max="10" width="30.33203125" customWidth="1"/>
+    <col min="11" max="11" width="21" customWidth="1"/>
+    <col min="12" max="12" width="53.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A1" s="5" t="s">
-        <v>32</v>
-      </c>
-      <c r="B1" s="5" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" ht="44.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="18" t="s">
-        <v>20</v>
-      </c>
-      <c r="B2" s="18" t="s">
-        <v>74</v>
-      </c>
-      <c r="C2" s="18" t="s">
-        <v>214</v>
-      </c>
-      <c r="D2" s="18" t="s">
-        <v>235</v>
-      </c>
-      <c r="E2" s="18" t="s">
-        <v>240</v>
-      </c>
-      <c r="F2" s="18" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" s="13" t="s">
-        <v>31</v>
-      </c>
-      <c r="B3" s="31" t="s">
-        <v>36</v>
-      </c>
-      <c r="C3" s="85" t="s">
-        <v>75</v>
-      </c>
-      <c r="D3" s="74" t="s">
-        <v>76</v>
-      </c>
-      <c r="E3" s="75" t="s">
-        <v>77</v>
-      </c>
-      <c r="F3" s="34" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4" s="12">
-        <v>1</v>
-      </c>
-      <c r="B4" s="47" t="str">
-        <f>Barberia_D!B4</f>
-        <v>Barbería Oriental</v>
-      </c>
-      <c r="C4" s="36" t="s">
-        <v>78</v>
-      </c>
-      <c r="D4" s="90">
-        <v>0.375</v>
-      </c>
-      <c r="E4" s="90">
-        <v>0.79166666666666663</v>
-      </c>
-      <c r="F4" s="12" t="str">
-        <f>_xlfn.CONCAT(B4,"-",C4,"-",TEXT(D4,"hh:mm"),"-",TEXT(E4,"hh:mm"))</f>
-        <v>Barbería Oriental-Lunes-09:00-19:00</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A5" s="12">
-        <v>2</v>
-      </c>
-      <c r="B5" s="47" t="str">
-        <f>Barberia_D!B4</f>
-        <v>Barbería Oriental</v>
-      </c>
-      <c r="C5" s="12" t="s">
-        <v>79</v>
-      </c>
-      <c r="D5" s="90">
-        <v>0.375</v>
-      </c>
-      <c r="E5" s="90">
-        <v>0.79166666666666663</v>
-      </c>
-      <c r="F5" s="12" t="str">
-        <f t="shared" ref="F5:F9" si="0">_xlfn.CONCAT(B5,"-",C5,"-",TEXT(D5,"hh:mm"),"-",TEXT(E5,"hh:mm"))</f>
-        <v>Barbería Oriental-Martes-09:00-19:00</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A6" s="12">
-        <v>3</v>
-      </c>
-      <c r="B6" s="47" t="str">
-        <f>Barberia_D!B4</f>
-        <v>Barbería Oriental</v>
-      </c>
-      <c r="C6" s="36" t="s">
-        <v>80</v>
-      </c>
-      <c r="D6" s="90">
-        <v>0.375</v>
-      </c>
-      <c r="E6" s="90">
-        <v>0.79166666666666696</v>
-      </c>
-      <c r="F6" s="12" t="str">
-        <f t="shared" si="0"/>
-        <v>Barbería Oriental-Miércoles-09:00-19:00</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A7" s="12">
-        <v>4</v>
-      </c>
-      <c r="B7" s="47" t="str">
-        <f>Barberia_D!B4</f>
-        <v>Barbería Oriental</v>
-      </c>
-      <c r="C7" s="12" t="s">
-        <v>81</v>
-      </c>
-      <c r="D7" s="90">
-        <v>0.375</v>
-      </c>
-      <c r="E7" s="90">
-        <v>0.79166666666666696</v>
-      </c>
-      <c r="F7" s="12" t="str">
-        <f t="shared" si="0"/>
-        <v>Barbería Oriental-Jueves-09:00-19:00</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A8" s="12">
-        <v>5</v>
-      </c>
-      <c r="B8" s="47" t="str">
-        <f>Barberia_D!B4</f>
-        <v>Barbería Oriental</v>
-      </c>
-      <c r="C8" s="36" t="s">
-        <v>82</v>
-      </c>
-      <c r="D8" s="90">
-        <v>0.375</v>
-      </c>
-      <c r="E8" s="90">
-        <v>0.79166666666666696</v>
-      </c>
-      <c r="F8" s="12" t="str">
-        <f t="shared" si="0"/>
-        <v>Barbería Oriental-Viernes-09:00-19:00</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A9" s="12">
-        <v>6</v>
-      </c>
-      <c r="B9" s="47" t="str">
-        <f>Barberia_D!B4</f>
-        <v>Barbería Oriental</v>
-      </c>
-      <c r="C9" s="12" t="s">
-        <v>83</v>
-      </c>
-      <c r="D9" s="91">
-        <v>0.33333333333333331</v>
-      </c>
-      <c r="E9" s="90">
-        <v>0.875</v>
-      </c>
-      <c r="F9" s="12" t="str">
-        <f t="shared" si="0"/>
-        <v>Barbería Oriental-Sábado-08:00-21:00</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A10" s="10"/>
-      <c r="B10" s="37"/>
-      <c r="C10" s="37"/>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="C11" s="10"/>
-    </row>
-  </sheetData>
-  <phoneticPr fontId="7" type="noConversion"/>
-  <hyperlinks>
-    <hyperlink ref="A1" location="'Modelo de Dominio'!A1" display="&lt;&lt;&lt;&lt; Ir al modulo de dominio" xr:uid="{8FE767F6-22F1-4F43-85BA-468D80B0CB91}"/>
-    <hyperlink ref="B1" location="'Objetos de Dominio'!A1" display="&lt;&lt;&lt;&lt; Ir a objetos de dominio" xr:uid="{FCE2B5DC-7C40-48F2-89BF-3ECFD15A2C41}"/>
-    <hyperlink ref="B3" location="Barberia_D!A1" display="barberia" xr:uid="{2492FDB7-93E1-4CE3-B41F-90BD0687A121}"/>
-    <hyperlink ref="B4" location="Barberia_D!A4" display="Barberia_D!A4" xr:uid="{CA0BE91C-E243-4E18-9EBC-492DB8F2F841}"/>
-    <hyperlink ref="B5" location="Barberia_D!A4" display="Barberia_D!A4" xr:uid="{8755C4B5-402C-4142-9068-F1A88E40D4BB}"/>
-    <hyperlink ref="B6" location="Barberia_D!A4" display="Barberia_D!A4" xr:uid="{110C1F32-4D8E-40A2-90EC-1FBB2E0B8A29}"/>
-    <hyperlink ref="B7" location="Barberia_D!A4" display="Barberia_D!A4" xr:uid="{EF70DFB1-E188-4E7F-9F0D-1EC2E2330BDA}"/>
-    <hyperlink ref="B8" location="Barberia_D!A4" display="Barberia_D!A4" xr:uid="{FBCD47DD-56CD-4067-A39A-E821892FE723}"/>
-    <hyperlink ref="B9" location="Barberia_D!A4" display="Barberia_D!A4" xr:uid="{11CC4F51-41DB-4B1A-8CAB-35A8FD0DE0E2}"/>
-  </hyperlinks>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C97B567D-D27E-4BE3-B1E4-8CA267790151}">
-  <dimension ref="A1:F12"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="2" width="28.140625" customWidth="1"/>
-    <col min="3" max="3" width="26.5703125" customWidth="1"/>
-    <col min="4" max="4" width="24.42578125" customWidth="1"/>
-    <col min="5" max="5" width="25.28515625" customWidth="1"/>
-    <col min="6" max="6" width="26.5703125" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A1" s="15" t="s">
-        <v>32</v>
-      </c>
-      <c r="B1" s="15" t="s">
-        <v>33</v>
-      </c>
-      <c r="D1" s="16"/>
-      <c r="E1" s="16"/>
-      <c r="F1" s="10"/>
-    </row>
-    <row r="2" spans="1:6" ht="45.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="17" t="s">
-        <v>20</v>
-      </c>
-      <c r="B2" s="17" t="s">
-        <v>137</v>
-      </c>
-      <c r="C2" s="17" t="s">
-        <v>187</v>
-      </c>
-      <c r="D2" s="30" t="s">
-        <v>189</v>
-      </c>
-      <c r="E2" s="30" t="s">
-        <v>190</v>
-      </c>
-      <c r="F2" s="18" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" s="20" t="s">
-        <v>31</v>
-      </c>
-      <c r="B3" s="52" t="s">
-        <v>36</v>
-      </c>
-      <c r="C3" s="76" t="s">
-        <v>21</v>
-      </c>
-      <c r="D3" s="77" t="s">
-        <v>37</v>
-      </c>
-      <c r="E3" s="77" t="s">
-        <v>24</v>
-      </c>
-      <c r="F3" s="14" t="s">
-        <v>188</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4" s="21">
-        <v>1</v>
-      </c>
-      <c r="B4" s="53" t="str">
-        <f>Barberia_D!B4</f>
-        <v>Barbería Oriental</v>
-      </c>
-      <c r="C4" s="21" t="s">
-        <v>38</v>
-      </c>
-      <c r="D4" s="21">
-        <v>45</v>
-      </c>
-      <c r="E4" s="22">
-        <v>22000</v>
-      </c>
-      <c r="F4" s="12" t="str">
-        <f>C4</f>
-        <v>Motilada</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A5" s="21">
-        <v>2</v>
-      </c>
-      <c r="B5" s="53" t="str">
-        <f>Barberia_D!B4</f>
-        <v>Barbería Oriental</v>
-      </c>
-      <c r="C5" s="21" t="s">
-        <v>46</v>
-      </c>
-      <c r="D5" s="21">
-        <v>10</v>
-      </c>
-      <c r="E5" s="22">
-        <v>12000</v>
-      </c>
-      <c r="F5" s="12" t="str">
-        <f t="shared" ref="F5:F7" si="0">C5</f>
-        <v>Corte de barba</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A6" s="21">
-        <v>3</v>
-      </c>
-      <c r="B6" s="53" t="str">
-        <f>Barberia_D!B4</f>
-        <v>Barbería Oriental</v>
-      </c>
-      <c r="C6" s="21" t="s">
-        <v>47</v>
-      </c>
-      <c r="D6" s="21">
-        <v>15</v>
-      </c>
-      <c r="E6" s="22">
-        <v>15000</v>
-      </c>
-      <c r="F6" s="12" t="str">
-        <f t="shared" si="0"/>
-        <v>Perfilada de barba</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" ht="30" x14ac:dyDescent="0.25">
-      <c r="A7" s="21">
-        <v>4</v>
-      </c>
-      <c r="B7" s="53" t="str">
-        <f>Barberia_D!B4</f>
-        <v>Barbería Oriental</v>
-      </c>
-      <c r="C7" s="23" t="s">
-        <v>48</v>
-      </c>
-      <c r="D7" s="21">
-        <v>30</v>
-      </c>
-      <c r="E7" s="22">
-        <v>35000</v>
-      </c>
-      <c r="F7" s="24" t="str">
-        <f t="shared" si="0"/>
-        <v>Arreglo completo de barba con toalla caliente</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A8" s="16"/>
-      <c r="B8" s="16"/>
-      <c r="C8" s="16"/>
-      <c r="D8" s="16"/>
-      <c r="E8" s="16"/>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A9" s="16"/>
-      <c r="B9" s="16"/>
-      <c r="C9" s="16"/>
-      <c r="D9" s="16"/>
-      <c r="E9" s="16"/>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A10" s="16"/>
-      <c r="B10" s="16"/>
-      <c r="C10" s="16"/>
-      <c r="D10" s="16"/>
-      <c r="E10" s="16"/>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A11" s="16"/>
-      <c r="B11" s="16"/>
-      <c r="C11" s="16"/>
-      <c r="D11" s="16"/>
-      <c r="E11" s="16"/>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A12" s="16"/>
-      <c r="B12" s="16"/>
-      <c r="C12" s="16"/>
-      <c r="D12" s="16"/>
-      <c r="E12" s="16"/>
-    </row>
-  </sheetData>
-  <hyperlinks>
-    <hyperlink ref="A1" location="'Modelo de Dominio'!A1" display="&lt;&lt;&lt;&lt; Ir al modulo de dominio" xr:uid="{1232B379-2C8F-4361-B8CE-5CC492F8D207}"/>
-    <hyperlink ref="B1" location="'Objetos de Dominio'!A1" display="&lt;&lt;&lt;&lt; Ir a objetos de dominio" xr:uid="{C4612CEA-B79F-4496-B57E-5F6E72A804C7}"/>
-    <hyperlink ref="B3" location="Barberia_D!A1" display="barberia" xr:uid="{49DC9582-0184-41B1-95D7-525F6EE28820}"/>
-    <hyperlink ref="B4" location="Barberia_D!A4" display="Barberia_D!A4" xr:uid="{9C3C8EC0-3D4B-4A80-9FA2-4578065166BB}"/>
-    <hyperlink ref="B5" location="Barberia_D!A4" display="Barberia_D!A4" xr:uid="{1337E6E0-8BBF-46FA-B386-3E8B848525E7}"/>
-    <hyperlink ref="B6" location="Servicio_D!A4" display="Servicio_D!A4" xr:uid="{F14FFAD6-C31D-4D17-A87C-7C4566115E73}"/>
-    <hyperlink ref="B7" location="Barberia_D!A4" display="Barberia_D!A4" xr:uid="{75AD25E9-0697-4BA2-8F6A-B890AAE2A8F8}"/>
-  </hyperlinks>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2DAE59AB-4103-4731-9C3C-4C276F8A29F8}">
-  <dimension ref="A1:L10"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="27" bestFit="1" customWidth="1"/>
-    <col min="2" max="6" width="26.7109375" customWidth="1"/>
-    <col min="7" max="7" width="16.28515625" customWidth="1"/>
-    <col min="8" max="9" width="40.7109375" customWidth="1"/>
-    <col min="10" max="10" width="30.28515625" customWidth="1"/>
-    <col min="11" max="11" width="21" customWidth="1"/>
-    <col min="12" max="12" width="53.140625" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A1" s="5" t="s">
         <v>32</v>
       </c>
@@ -6025,73 +5640,73 @@
       <c r="E1" s="5"/>
       <c r="F1" s="5"/>
     </row>
-    <row r="2" spans="1:12" ht="45.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:12" ht="45.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="25" t="s">
         <v>20</v>
       </c>
       <c r="B2" s="25" t="s">
+        <v>156</v>
+      </c>
+      <c r="C2" s="25" t="s">
         <v>157</v>
       </c>
-      <c r="C2" s="25" t="s">
+      <c r="D2" s="25" t="s">
         <v>158</v>
       </c>
-      <c r="D2" s="25" t="s">
+      <c r="E2" s="25" t="s">
         <v>159</v>
       </c>
-      <c r="E2" s="25" t="s">
+      <c r="F2" s="25" t="s">
         <v>160</v>
       </c>
-      <c r="F2" s="25" t="s">
+      <c r="G2" s="26" t="s">
+        <v>190</v>
+      </c>
+      <c r="H2" s="26" t="s">
+        <v>191</v>
+      </c>
+      <c r="I2" s="26" t="s">
         <v>161</v>
       </c>
-      <c r="G2" s="26" t="s">
-        <v>191</v>
-      </c>
-      <c r="H2" s="26" t="s">
-        <v>192</v>
-      </c>
-      <c r="I2" s="26" t="s">
-        <v>162</v>
-      </c>
       <c r="J2" s="26" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
       <c r="K2" s="26" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="L2" s="27" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A3" s="13" t="s">
         <v>31</v>
       </c>
-      <c r="B3" s="55" t="s">
+      <c r="B3" s="54" t="s">
         <v>101</v>
       </c>
-      <c r="C3" s="55" t="s">
+      <c r="C3" s="54" t="s">
         <v>103</v>
       </c>
-      <c r="D3" s="55" t="s">
+      <c r="D3" s="54" t="s">
         <v>102</v>
       </c>
-      <c r="E3" s="55" t="s">
+      <c r="E3" s="54" t="s">
         <v>104</v>
       </c>
-      <c r="F3" s="72" t="s">
+      <c r="F3" s="71" t="s">
         <v>128</v>
       </c>
-      <c r="G3" s="72" t="s">
+      <c r="G3" s="71" t="s">
         <v>22</v>
       </c>
-      <c r="H3" s="72" t="s">
+      <c r="H3" s="71" t="s">
         <v>42</v>
       </c>
-      <c r="I3" s="72" t="s">
+      <c r="I3" s="71" t="s">
         <v>124</v>
       </c>
-      <c r="J3" s="41" t="s">
+      <c r="J3" s="40" t="s">
         <v>43</v>
       </c>
       <c r="K3" s="31" t="s">
@@ -6101,7 +5716,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A4" s="12">
         <v>1</v>
       </c>
@@ -6112,12 +5727,12 @@
         <v>105</v>
       </c>
       <c r="D4" s="12" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="E4" s="12" t="s">
         <v>107</v>
       </c>
-      <c r="F4" s="45" t="s">
+      <c r="F4" s="44" t="s">
         <v>129</v>
       </c>
       <c r="G4" s="12">
@@ -6126,13 +5741,13 @@
       <c r="H4" s="11" t="s">
         <v>53</v>
       </c>
-      <c r="I4" s="43">
+      <c r="I4" s="42">
         <v>1264267821</v>
       </c>
       <c r="J4" s="12" t="s">
         <v>49</v>
       </c>
-      <c r="K4" s="47" t="str">
+      <c r="K4" s="46" t="str">
         <f>Barberia_D!B4</f>
         <v>Barbería Oriental</v>
       </c>
@@ -6141,7 +5756,7 @@
         <v>Juan-Fernando-García-Lopez-+57-3245627890</v>
       </c>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A5" s="12">
         <v>2</v>
       </c>
@@ -6152,12 +5767,12 @@
         <v>106</v>
       </c>
       <c r="D5" s="12" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="E5" s="12" t="s">
         <v>108</v>
       </c>
-      <c r="F5" s="45" t="s">
+      <c r="F5" s="44" t="s">
         <v>129</v>
       </c>
       <c r="G5" s="12">
@@ -6166,13 +5781,13 @@
       <c r="H5" s="11" t="s">
         <v>54</v>
       </c>
-      <c r="I5" s="43" t="s">
+      <c r="I5" s="42" t="s">
         <v>126</v>
       </c>
       <c r="J5" s="12" t="s">
         <v>49</v>
       </c>
-      <c r="K5" s="47" t="str">
+      <c r="K5" s="46" t="str">
         <f>Barberia_D!B4</f>
         <v>Barbería Oriental</v>
       </c>
@@ -6181,7 +5796,7 @@
         <v>Juan-David-Ortiz-Sanchez-+57-3124518923</v>
       </c>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A6" s="12">
         <v>3</v>
       </c>
@@ -6193,7 +5808,7 @@
         <v>110</v>
       </c>
       <c r="E6" s="12"/>
-      <c r="F6" s="45" t="s">
+      <c r="F6" s="44" t="s">
         <v>129</v>
       </c>
       <c r="G6" s="12">
@@ -6202,13 +5817,13 @@
       <c r="H6" s="11" t="s">
         <v>55</v>
       </c>
-      <c r="I6" s="44" t="s">
+      <c r="I6" s="43" t="s">
         <v>125</v>
       </c>
       <c r="J6" s="12" t="s">
         <v>49</v>
       </c>
-      <c r="K6" s="47" t="str">
+      <c r="K6" s="46" t="str">
         <f>Barberia_D!B4</f>
         <v>Barbería Oriental</v>
       </c>
@@ -6217,7 +5832,7 @@
         <v>Carlos--Arbeladez--+57-3214533321</v>
       </c>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A7" s="12">
         <v>4</v>
       </c>
@@ -6231,7 +5846,7 @@
       <c r="E7" s="12" t="s">
         <v>109</v>
       </c>
-      <c r="F7" s="45" t="s">
+      <c r="F7" s="44" t="s">
         <v>131</v>
       </c>
       <c r="G7" s="12">
@@ -6240,13 +5855,13 @@
       <c r="H7" s="11" t="s">
         <v>56</v>
       </c>
-      <c r="I7" s="43" t="s">
+      <c r="I7" s="42" t="s">
         <v>127</v>
       </c>
       <c r="J7" s="12" t="s">
         <v>49</v>
       </c>
-      <c r="K7" s="47" t="str">
+      <c r="K7" s="46" t="str">
         <f>Barberia_D!B4</f>
         <v>Barbería Oriental</v>
       </c>
@@ -6255,7 +5870,7 @@
         <v>Andres--Ramirez-Patiño-+91-9876543210</v>
       </c>
     </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A8" s="12">
         <v>5</v>
       </c>
@@ -6266,19 +5881,19 @@
         <v>51</v>
       </c>
       <c r="D8" s="12" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="E8" s="12" t="s">
         <v>112</v>
       </c>
-      <c r="F8" s="45" t="s">
-        <v>145</v>
+      <c r="F8" s="44" t="s">
+        <v>144</v>
       </c>
       <c r="G8" s="12">
         <v>998765432</v>
       </c>
       <c r="H8" s="11" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="I8" s="12">
         <v>312334342</v>
@@ -6286,7 +5901,7 @@
       <c r="J8" s="12" t="s">
         <v>50</v>
       </c>
-      <c r="K8" s="47" t="str">
+      <c r="K8" s="46" t="str">
         <f>Barberia_D!B4</f>
         <v>Barbería Oriental</v>
       </c>
@@ -6295,9 +5910,14 @@
         <v>Juan-Carlos-Zambrano-Perez-+593-998765432</v>
       </c>
     </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:12" x14ac:dyDescent="0.3">
       <c r="B10" s="10"/>
       <c r="C10" s="10"/>
+    </row>
+    <row r="11" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="F11" s="92" t="s">
+        <v>243</v>
+      </c>
     </row>
   </sheetData>
   <phoneticPr fontId="7" type="noConversion"/>
@@ -6316,4 +5936,444 @@
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2190E1EC-B79B-40C0-AC5B-0E2726DDD399}">
+  <dimension ref="A1:F12"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="27" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="26" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="34.44140625" customWidth="1"/>
+    <col min="4" max="4" width="23.5546875" customWidth="1"/>
+    <col min="5" max="5" width="23.6640625" customWidth="1"/>
+    <col min="6" max="6" width="34.88671875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A1" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" ht="44.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="18" t="s">
+        <v>20</v>
+      </c>
+      <c r="B2" s="18" t="s">
+        <v>74</v>
+      </c>
+      <c r="C2" s="18" t="s">
+        <v>211</v>
+      </c>
+      <c r="D2" s="18" t="s">
+        <v>232</v>
+      </c>
+      <c r="E2" s="18" t="s">
+        <v>237</v>
+      </c>
+      <c r="F2" s="18" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A3" s="13" t="s">
+        <v>31</v>
+      </c>
+      <c r="B3" s="31" t="s">
+        <v>36</v>
+      </c>
+      <c r="C3" s="84" t="s">
+        <v>75</v>
+      </c>
+      <c r="D3" s="73" t="s">
+        <v>76</v>
+      </c>
+      <c r="E3" s="74" t="s">
+        <v>77</v>
+      </c>
+      <c r="F3" s="34" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A4" s="12">
+        <v>1</v>
+      </c>
+      <c r="B4" s="46" t="str">
+        <f>Barberia_D!B4</f>
+        <v>Barbería Oriental</v>
+      </c>
+      <c r="C4" s="36" t="s">
+        <v>78</v>
+      </c>
+      <c r="D4" s="89">
+        <v>0.375</v>
+      </c>
+      <c r="E4" s="89">
+        <v>0.79166666666666663</v>
+      </c>
+      <c r="F4" s="12" t="str">
+        <f>_xlfn.CONCAT(B4,"-",C4,"-",TEXT(D4,"hh:mm"),"-",TEXT(E4,"hh:mm"))</f>
+        <v>Barbería Oriental-Lunes-09:00-19:00</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A5" s="12">
+        <v>2</v>
+      </c>
+      <c r="B5" s="46" t="str">
+        <f>Barberia_D!B4</f>
+        <v>Barbería Oriental</v>
+      </c>
+      <c r="C5" s="12" t="s">
+        <v>79</v>
+      </c>
+      <c r="D5" s="89">
+        <v>0.375</v>
+      </c>
+      <c r="E5" s="89">
+        <v>0.79166666666666663</v>
+      </c>
+      <c r="F5" s="12" t="str">
+        <f t="shared" ref="F5:F10" si="0">_xlfn.CONCAT(B5,"-",C5,"-",TEXT(D5,"hh:mm"),"-",TEXT(E5,"hh:mm"))</f>
+        <v>Barbería Oriental-Martes-09:00-19:00</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A6" s="12">
+        <v>3</v>
+      </c>
+      <c r="B6" s="46" t="str">
+        <f>Barberia_D!B4</f>
+        <v>Barbería Oriental</v>
+      </c>
+      <c r="C6" s="36" t="s">
+        <v>80</v>
+      </c>
+      <c r="D6" s="89">
+        <v>0.375</v>
+      </c>
+      <c r="E6" s="89">
+        <v>0.79166666666666696</v>
+      </c>
+      <c r="F6" s="12" t="str">
+        <f t="shared" si="0"/>
+        <v>Barbería Oriental-Miércoles-09:00-19:00</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A7" s="12">
+        <v>4</v>
+      </c>
+      <c r="B7" s="46" t="str">
+        <f>Barberia_D!B4</f>
+        <v>Barbería Oriental</v>
+      </c>
+      <c r="C7" s="12" t="s">
+        <v>81</v>
+      </c>
+      <c r="D7" s="89">
+        <v>0.375</v>
+      </c>
+      <c r="E7" s="89">
+        <v>0.79166666666666696</v>
+      </c>
+      <c r="F7" s="12" t="str">
+        <f t="shared" si="0"/>
+        <v>Barbería Oriental-Jueves-09:00-19:00</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A8" s="12">
+        <v>5</v>
+      </c>
+      <c r="B8" s="46" t="str">
+        <f>Barberia_D!B4</f>
+        <v>Barbería Oriental</v>
+      </c>
+      <c r="C8" s="36" t="s">
+        <v>82</v>
+      </c>
+      <c r="D8" s="89">
+        <v>0.375</v>
+      </c>
+      <c r="E8" s="89">
+        <v>0.79166666666666696</v>
+      </c>
+      <c r="F8" s="12" t="str">
+        <f t="shared" si="0"/>
+        <v>Barbería Oriental-Viernes-09:00-19:00</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A9" s="12">
+        <v>6</v>
+      </c>
+      <c r="B9" s="46" t="str">
+        <f>Barberia_D!B4</f>
+        <v>Barbería Oriental</v>
+      </c>
+      <c r="C9" s="12" t="s">
+        <v>83</v>
+      </c>
+      <c r="D9" s="90">
+        <v>0.33333333333333331</v>
+      </c>
+      <c r="E9" s="89">
+        <v>0.875</v>
+      </c>
+      <c r="F9" s="12" t="str">
+        <f t="shared" si="0"/>
+        <v>Barbería Oriental-Sábado-08:00-21:00</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A10" s="12">
+        <v>7</v>
+      </c>
+      <c r="B10" s="46" t="str">
+        <f>Barberia_D!B4</f>
+        <v>Barbería Oriental</v>
+      </c>
+      <c r="C10" s="36" t="s">
+        <v>244</v>
+      </c>
+      <c r="D10" s="89">
+        <v>0.41666666666666669</v>
+      </c>
+      <c r="E10" s="89">
+        <v>0.625</v>
+      </c>
+      <c r="F10" s="12" t="str">
+        <f t="shared" si="0"/>
+        <v>Barbería Oriental-Festivo-10:00-15:00</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A11" s="93"/>
+      <c r="C11" s="10"/>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A12" s="93"/>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="7" type="noConversion"/>
+  <hyperlinks>
+    <hyperlink ref="A1" location="'Modelo de Dominio'!A1" display="&lt;&lt;&lt;&lt; Ir al modulo de dominio" xr:uid="{8FE767F6-22F1-4F43-85BA-468D80B0CB91}"/>
+    <hyperlink ref="B1" location="'Objetos de Dominio'!A1" display="&lt;&lt;&lt;&lt; Ir a objetos de dominio" xr:uid="{FCE2B5DC-7C40-48F2-89BF-3ECFD15A2C41}"/>
+    <hyperlink ref="B3" location="Barberia_D!A1" display="barberia" xr:uid="{2492FDB7-93E1-4CE3-B41F-90BD0687A121}"/>
+    <hyperlink ref="B4" location="Barberia_D!A4" display="Barberia_D!A4" xr:uid="{CA0BE91C-E243-4E18-9EBC-492DB8F2F841}"/>
+    <hyperlink ref="B5" location="Barberia_D!A4" display="Barberia_D!A4" xr:uid="{8755C4B5-402C-4142-9068-F1A88E40D4BB}"/>
+    <hyperlink ref="B6" location="Barberia_D!A4" display="Barberia_D!A4" xr:uid="{110C1F32-4D8E-40A2-90EC-1FBB2E0B8A29}"/>
+    <hyperlink ref="B7" location="Barberia_D!A4" display="Barberia_D!A4" xr:uid="{EF70DFB1-E188-4E7F-9F0D-1EC2E2330BDA}"/>
+    <hyperlink ref="B8" location="Barberia_D!A4" display="Barberia_D!A4" xr:uid="{FBCD47DD-56CD-4067-A39A-E821892FE723}"/>
+    <hyperlink ref="B9" location="Barberia_D!A4" display="Barberia_D!A4" xr:uid="{11CC4F51-41DB-4B1A-8CAB-35A8FD0DE0E2}"/>
+    <hyperlink ref="B10" location="Barberia_D!A4" display="Barberia_D!A4" xr:uid="{DF73B835-0B1D-44DB-8A25-CFCFDEE0B537}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C97B567D-D27E-4BE3-B1E4-8CA267790151}">
+  <dimension ref="A1:F12"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="2" width="28.109375" customWidth="1"/>
+    <col min="3" max="3" width="26.5546875" customWidth="1"/>
+    <col min="4" max="4" width="24.44140625" customWidth="1"/>
+    <col min="5" max="5" width="25.33203125" customWidth="1"/>
+    <col min="6" max="6" width="26.5546875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A1" s="15" t="s">
+        <v>32</v>
+      </c>
+      <c r="B1" s="15" t="s">
+        <v>33</v>
+      </c>
+      <c r="D1" s="16"/>
+      <c r="E1" s="16"/>
+      <c r="F1" s="10"/>
+    </row>
+    <row r="2" spans="1:6" ht="45.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="B2" s="17" t="s">
+        <v>136</v>
+      </c>
+      <c r="C2" s="17" t="s">
+        <v>186</v>
+      </c>
+      <c r="D2" s="30" t="s">
+        <v>188</v>
+      </c>
+      <c r="E2" s="30" t="s">
+        <v>189</v>
+      </c>
+      <c r="F2" s="18" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A3" s="20" t="s">
+        <v>31</v>
+      </c>
+      <c r="B3" s="51" t="s">
+        <v>36</v>
+      </c>
+      <c r="C3" s="75" t="s">
+        <v>21</v>
+      </c>
+      <c r="D3" s="76" t="s">
+        <v>37</v>
+      </c>
+      <c r="E3" s="76" t="s">
+        <v>24</v>
+      </c>
+      <c r="F3" s="14" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A4" s="21">
+        <v>1</v>
+      </c>
+      <c r="B4" s="52" t="str">
+        <f>Barberia_D!B4</f>
+        <v>Barbería Oriental</v>
+      </c>
+      <c r="C4" s="21" t="s">
+        <v>38</v>
+      </c>
+      <c r="D4" s="21">
+        <v>45</v>
+      </c>
+      <c r="E4" s="22">
+        <v>22000</v>
+      </c>
+      <c r="F4" s="12" t="str">
+        <f>C4</f>
+        <v>Motilada</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A5" s="21">
+        <v>2</v>
+      </c>
+      <c r="B5" s="52" t="str">
+        <f>Barberia_D!B4</f>
+        <v>Barbería Oriental</v>
+      </c>
+      <c r="C5" s="21" t="s">
+        <v>46</v>
+      </c>
+      <c r="D5" s="21">
+        <v>10</v>
+      </c>
+      <c r="E5" s="22">
+        <v>12000</v>
+      </c>
+      <c r="F5" s="12" t="str">
+        <f t="shared" ref="F5:F7" si="0">C5</f>
+        <v>Corte de barba</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A6" s="21">
+        <v>3</v>
+      </c>
+      <c r="B6" s="52" t="str">
+        <f>Barberia_D!B4</f>
+        <v>Barbería Oriental</v>
+      </c>
+      <c r="C6" s="21" t="s">
+        <v>47</v>
+      </c>
+      <c r="D6" s="21">
+        <v>15</v>
+      </c>
+      <c r="E6" s="22">
+        <v>15000</v>
+      </c>
+      <c r="F6" s="12" t="str">
+        <f t="shared" si="0"/>
+        <v>Perfilada de barba</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A7" s="21">
+        <v>4</v>
+      </c>
+      <c r="B7" s="52" t="str">
+        <f>Barberia_D!B4</f>
+        <v>Barbería Oriental</v>
+      </c>
+      <c r="C7" s="23" t="s">
+        <v>48</v>
+      </c>
+      <c r="D7" s="21">
+        <v>30</v>
+      </c>
+      <c r="E7" s="22">
+        <v>35000</v>
+      </c>
+      <c r="F7" s="24" t="str">
+        <f t="shared" si="0"/>
+        <v>Arreglo completo de barba con toalla caliente</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A8" s="16"/>
+      <c r="B8" s="16"/>
+      <c r="C8" s="16"/>
+      <c r="D8" s="16"/>
+      <c r="E8" s="16"/>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A9" s="16"/>
+      <c r="B9" s="16"/>
+      <c r="C9" s="16"/>
+      <c r="D9" s="16"/>
+      <c r="E9" s="16"/>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A10" s="16"/>
+      <c r="B10" s="16"/>
+      <c r="C10" s="16"/>
+      <c r="D10" s="16"/>
+      <c r="E10" s="16"/>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A11" s="16"/>
+      <c r="B11" s="16"/>
+      <c r="C11" s="16"/>
+      <c r="D11" s="16"/>
+      <c r="E11" s="16"/>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A12" s="16"/>
+      <c r="B12" s="16"/>
+      <c r="C12" s="16"/>
+      <c r="D12" s="16"/>
+      <c r="E12" s="16"/>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A1" location="'Modelo de Dominio'!A1" display="&lt;&lt;&lt;&lt; Ir al modulo de dominio" xr:uid="{1232B379-2C8F-4361-B8CE-5CC492F8D207}"/>
+    <hyperlink ref="B1" location="'Objetos de Dominio'!A1" display="&lt;&lt;&lt;&lt; Ir a objetos de dominio" xr:uid="{C4612CEA-B79F-4496-B57E-5F6E72A804C7}"/>
+    <hyperlink ref="B3" location="Barberia_D!A1" display="barberia" xr:uid="{49DC9582-0184-41B1-95D7-525F6EE28820}"/>
+    <hyperlink ref="B4" location="Barberia_D!A4" display="Barberia_D!A4" xr:uid="{9C3C8EC0-3D4B-4A80-9FA2-4578065166BB}"/>
+    <hyperlink ref="B5" location="Barberia_D!A4" display="Barberia_D!A4" xr:uid="{1337E6E0-8BBF-46FA-B386-3E8B848525E7}"/>
+    <hyperlink ref="B6" location="Servicio_D!A4" display="Servicio_D!A4" xr:uid="{F14FFAD6-C31D-4D17-A87C-7C4566115E73}"/>
+    <hyperlink ref="B7" location="Barberia_D!A4" display="Barberia_D!A4" xr:uid="{75AD25E9-0697-4BA2-8F6A-B890AAE2A8F8}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Se añadieron comentarios para pensar la logica de negocio y se cambio la cardinalidad de 1...8 a 1...* de Barberia - Horario Barberia
</commit_message>
<xml_diff>
--- a/Muestreo de datos.xlsx
+++ b/Muestreo de datos.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\leand\Desktop\DOO\DOO\Barberia\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{686889DE-83BF-4DBB-95FF-005494F7E945}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E66909D-5601-4FD5-B019-CA621521DC3F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{09A6C7D7-663F-4C06-9D71-8A4E97495CF9}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="11" activeTab="17" xr2:uid="{09A6C7D7-663F-4C06-9D71-8A4E97495CF9}"/>
   </bookViews>
   <sheets>
     <sheet name="Modelo de Dominio" sheetId="1" r:id="rId1"/>
@@ -56,7 +56,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="378" uniqueCount="247">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="384" uniqueCount="253">
   <si>
     <t>Nombre</t>
   </si>
@@ -790,9 +790,6 @@
     <t>Tipo de dato que tiene dos posibles valores (Si/No).</t>
   </si>
   <si>
-    <t>Necesitare oro objeto de dominio para prefijo</t>
-  </si>
-  <si>
     <t>Festivo</t>
   </si>
   <si>
@@ -800,6 +797,27 @@
   </si>
   <si>
     <t>Representa la fecha y hora prevista a la que finaliza una cita, es un dato calculado a partir de la fecha y hora en que empieza la cita y la duración del servicio, sumándole la duración del servicio a fechaHora</t>
+  </si>
+  <si>
+    <t>**********</t>
+  </si>
+  <si>
+    <t>Analizar combinaciones unicas</t>
+  </si>
+  <si>
+    <t>Sera que necesitamos un objeto de dominio</t>
+  </si>
+  <si>
+    <t>Se necesita el historial</t>
+  </si>
+  <si>
+    <t>Mirar agenda</t>
+  </si>
+  <si>
+    <t>Interesa solo para el futuro</t>
+  </si>
+  <si>
+    <t>Que pasa si el barbero se demora mas de lo previsto</t>
   </si>
 </sst>
 </file>
@@ -1231,16 +1249,16 @@
     <xf numFmtId="49" fontId="3" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="18" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -3464,6 +3482,11 @@
       <c r="E8" s="29"/>
       <c r="F8" s="29"/>
     </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="E10" t="s">
+        <v>249</v>
+      </c>
+    </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="E11" s="41"/>
     </row>
@@ -3628,7 +3651,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2921A3C4-B96A-49A7-8353-9FD37D2F2B74}">
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:C14"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
@@ -3716,6 +3739,11 @@
       <c r="C7" s="12" t="str">
         <f t="shared" si="0"/>
         <v>Andres Ramirez</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="B14" t="s">
+        <v>250</v>
       </c>
     </row>
   </sheetData>
@@ -4067,15 +4095,15 @@
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A8" s="94">
+      <c r="A8" s="12">
         <v>5</v>
       </c>
       <c r="B8" s="11" t="str">
         <f>Agenda_D!C7</f>
         <v>Andres Ramirez</v>
       </c>
-      <c r="C8" s="94" t="s">
-        <v>244</v>
+      <c r="C8" s="12" t="s">
+        <v>243</v>
       </c>
       <c r="D8" s="89">
         <v>0.5</v>
@@ -4083,7 +4111,7 @@
       <c r="E8" s="89">
         <v>0.625</v>
       </c>
-      <c r="F8" s="94" t="str">
+      <c r="F8" s="12" t="str">
         <f t="shared" si="0"/>
         <v>Andres Ramirez-Festivo-12-15</v>
       </c>
@@ -4330,7 +4358,7 @@
         <v>192</v>
       </c>
       <c r="E2" s="30" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="F2" s="30" t="s">
         <v>224</v>
@@ -4353,7 +4381,7 @@
         <v>132</v>
       </c>
       <c r="E3" s="40" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="F3" s="54" t="s">
         <v>26</v>
@@ -4494,24 +4522,24 @@
       <c r="H8" s="45"/>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="E10" s="95"/>
+      <c r="E10" s="93"/>
       <c r="H10" s="47"/>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="E11" s="95"/>
+      <c r="E11" s="93"/>
       <c r="F11" s="10"/>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.3">
       <c r="D12" s="49"/>
-      <c r="E12" s="95"/>
+      <c r="E12" s="93"/>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.3">
       <c r="D13" s="49"/>
-      <c r="E13" s="95"/>
+      <c r="E13" s="93"/>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.3">
       <c r="D14" s="49"/>
-      <c r="E14" s="95"/>
+      <c r="E14" s="93"/>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.3">
       <c r="D15" s="49"/>
@@ -4695,7 +4723,7 @@
 
 <file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F470C5A4-8D15-43DA-95FC-91C9614E5EEA}">
-  <dimension ref="A1:F9"/>
+  <dimension ref="A1:F12"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="26.44140625" customWidth="1"/>
@@ -4890,6 +4918,16 @@
       <c r="F9" s="24" t="str">
         <f t="shared" si="0"/>
         <v>Carlos Arbeladez-06/08/2026/18:00-Corte de barba</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="D11" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E12" t="s">
+        <v>252</v>
       </c>
     </row>
   </sheetData>
@@ -5913,11 +5951,12 @@
     <row r="10" spans="1:12" x14ac:dyDescent="0.3">
       <c r="B10" s="10"/>
       <c r="C10" s="10"/>
+      <c r="I10" s="94" t="s">
+        <v>246</v>
+      </c>
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="F11" s="92" t="s">
-        <v>243</v>
-      </c>
+      <c r="F11" s="92"/>
     </row>
   </sheetData>
   <phoneticPr fontId="7" type="noConversion"/>
@@ -5948,7 +5987,7 @@
     <col min="3" max="3" width="34.44140625" customWidth="1"/>
     <col min="4" max="4" width="23.5546875" customWidth="1"/>
     <col min="5" max="5" width="23.6640625" customWidth="1"/>
-    <col min="6" max="6" width="34.88671875" customWidth="1"/>
+    <col min="6" max="6" width="34.77734375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.3">
@@ -6140,7 +6179,7 @@
         <v>Barbería Oriental</v>
       </c>
       <c r="C10" s="36" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="D10" s="89">
         <v>0.41666666666666669</v>
@@ -6154,11 +6193,14 @@
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A11" s="93"/>
+      <c r="A11" s="10"/>
       <c r="C11" s="10"/>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A12" s="93"/>
+      <c r="A12" s="10"/>
+      <c r="C12" s="95" t="s">
+        <v>247</v>
+      </c>
     </row>
   </sheetData>
   <phoneticPr fontId="7" type="noConversion"/>
@@ -6345,7 +6387,9 @@
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A10" s="16"/>
-      <c r="B10" s="16"/>
+      <c r="B10" s="16" t="s">
+        <v>248</v>
+      </c>
       <c r="C10" s="16"/>
       <c r="D10" s="16"/>
       <c r="E10" s="16"/>

</xml_diff>

<commit_message>
Se elimino el objeto de dominio de HorarioBarbero y se esta pensando algunas logicas de negocio
</commit_message>
<xml_diff>
--- a/Muestreo de datos.xlsx
+++ b/Muestreo de datos.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\leand\Desktop\DOO\DOO\Barberia\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/120f6d501c463b80/Escritorio/leo/Doo/Barberia proyecto/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E66909D-5601-4FD5-B019-CA621521DC3F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="121" documentId="13_ncr:1_{2E66909D-5601-4FD5-B019-CA621521DC3F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F103FF16-41A8-4BCB-BBF4-5C255915BAED}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="11" activeTab="17" xr2:uid="{09A6C7D7-663F-4C06-9D71-8A4E97495CF9}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" firstSheet="8" activeTab="16" xr2:uid="{09A6C7D7-663F-4C06-9D71-8A4E97495CF9}"/>
   </bookViews>
   <sheets>
     <sheet name="Modelo de Dominio" sheetId="1" r:id="rId1"/>
@@ -26,11 +26,10 @@
     <sheet name="BarberoServicio_D" sheetId="11" r:id="rId11"/>
     <sheet name="Agenda_D" sheetId="12" r:id="rId12"/>
     <sheet name="Bloqueo_D" sheetId="22" r:id="rId13"/>
-    <sheet name="HorarioBarbero_D" sheetId="20" r:id="rId14"/>
-    <sheet name="Descanso_D" sheetId="23" r:id="rId15"/>
-    <sheet name="Cita_D" sheetId="13" r:id="rId16"/>
-    <sheet name="Multa_D" sheetId="16" r:id="rId17"/>
-    <sheet name="CitaServicio_D" sheetId="17" r:id="rId18"/>
+    <sheet name="Descanso_D" sheetId="23" r:id="rId14"/>
+    <sheet name="Cita_D" sheetId="13" r:id="rId15"/>
+    <sheet name="Multa_D" sheetId="16" r:id="rId16"/>
+    <sheet name="CitaServicio_D" sheetId="17" r:id="rId17"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -56,7 +55,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="384" uniqueCount="253">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="377" uniqueCount="251">
   <si>
     <t>Nombre</t>
   </si>
@@ -277,9 +276,6 @@
     <t>HorarioBarberia</t>
   </si>
   <si>
-    <t>HorarioBarbero</t>
-  </si>
-  <si>
     <t>Representa el nombre de la barberia que va pertencer los horarios de la barberia</t>
   </si>
   <si>
@@ -313,16 +309,6 @@
     <t>Combinación única que indica que un barbero no puede tener más de una agenda, cada barbero organiza todo su tiempo en un único lugar</t>
   </si>
   <si>
-    <t>horaFin</t>
-  </si>
-  <si>
-    <t xml:space="preserve">
-Hace referencia a la agenda (y por lo tanto al barbero) a la que pertenece este horario, permite saber de quién es cada bloque de disponibilidad</t>
-  </si>
-  <si>
-    <t>Combinación única que indica que una misma agenda no puede tener dos horarios distintos para el mismo día</t>
-  </si>
-  <si>
     <t>atendida</t>
   </si>
   <si>
@@ -432,15 +418,6 @@
   </si>
   <si>
     <t>contraseña</t>
-  </si>
-  <si>
-    <t>Carlos.1995</t>
-  </si>
-  <si>
-    <t>Juan.sanchez2342</t>
-  </si>
-  <si>
-    <t>ramirezpatinio23121</t>
   </si>
   <si>
     <t>prefijo</t>
@@ -519,9 +496,6 @@
     <t>Representa el calendario propio de un barbero. Es donde se organiza su horario de trabajo y las citas que se le van agendando, validando que ninguna se le cruce con otra</t>
   </si>
   <si>
-    <t>Representa cada día de la semana, hora en el que entra, hora a la que sale, para que la agenda del barbero sepa que días trabaja el</t>
-  </si>
-  <si>
     <t>Representa la reserva de un cliente con un barbero para una fecha y hora puntual. De ella sale tanto el cálculo de cuanto queda ocupado el barbero como la funcionalidad de si hay o no una multa (se genera cuando un barbero pone el estado de la cita en retraso o inclumplida), según cómo haya terminado (atendida, con retraso, incumplida o cancelada)</t>
   </si>
   <si>
@@ -541,9 +515,6 @@
   </si>
   <si>
     <t>Representa de que pais es el numero de celular del barbero. Su tipo de dato es alfanumérico, su valor por defecto es +0 y no es permitido</t>
-  </si>
-  <si>
-    <t>Representa la contraseña del barbebro, con el que se va a registrar o iniciar sesión. Su tipo de dato es alfanumérico, su valor por defecto es el vacio y no esta permitido</t>
   </si>
   <si>
     <t>Tipo de dato</t>
@@ -658,9 +629,6 @@
     <t>Combinación única que indica que una misma agenda no puede tener dos bloqueos en una misma fecha, horaInicio y horaFinal</t>
   </si>
   <si>
-    <t>horarioDelBarbero</t>
-  </si>
-  <si>
     <t>Hace referencia al dia y las horas que trabaja el barbero</t>
   </si>
   <si>
@@ -799,25 +767,49 @@
     <t>Representa la fecha y hora prevista a la que finaliza una cita, es un dato calculado a partir de la fecha y hora en que empieza la cita y la duración del servicio, sumándole la duración del servicio a fechaHora</t>
   </si>
   <si>
-    <t>**********</t>
-  </si>
-  <si>
     <t>Analizar combinaciones unicas</t>
   </si>
   <si>
-    <t>Sera que necesitamos un objeto de dominio</t>
-  </si>
-  <si>
     <t>Se necesita el historial</t>
   </si>
   <si>
-    <t>Mirar agenda</t>
-  </si>
-  <si>
     <t>Interesa solo para el futuro</t>
   </si>
   <si>
     <t>Que pasa si el barbero se demora mas de lo previsto</t>
+  </si>
+  <si>
+    <t>Realmente necesitop este objeto de dominio</t>
+  </si>
+  <si>
+    <t>$2b$12$Ce2ZsSJaOpx4iq5W.LNrCuvonh1fxNgpYYqBddeR50IjtYsh9n97C</t>
+  </si>
+  <si>
+    <t>$2b$12$4dn1n10vtv3SpDX5ryR2FOluaaros/pqDXz8liKcEp/7JG7TBvqAK</t>
+  </si>
+  <si>
+    <t>$2b$12$htWWNCh.2QPjVycBmNb5ROHBO21L9p7hlWyFtctUtP4SbV3yBNqei</t>
+  </si>
+  <si>
+    <t>$2b$12$IzNJVnlQl1UX5Py84yi5jOE1yuEdUrA.0Okt.BidVKs8biBdotH7W</t>
+  </si>
+  <si>
+    <t>$2b$12$mlxS0WUooP1stXSQdVR8EeBoYrgBrP5czZRqSvIgvelxUIGcwFgh.</t>
+  </si>
+  <si>
+    <t>Representa la contraseña encriptada del barbero. Su tipo de dato es alfanumérico, su valor por defecto es el vacio y no esta permitido</t>
+  </si>
+  <si>
+    <t>Sera que necesitamos un objeto de dominio barberia</t>
+  </si>
+  <si>
+    <t>horaAperturaBarberia</t>
+  </si>
+  <si>
+    <t>horaCierreBarberia</t>
+  </si>
+  <si>
+    <t xml:space="preserve">El barbero neceta conocer el presente y el futuro o tambien el pasado </t>
   </si>
 </sst>
 </file>
@@ -1014,7 +1006,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="96">
+  <cellXfs count="100">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -1213,9 +1205,6 @@
     <xf numFmtId="18" fontId="8" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="18" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="18" fontId="8" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1258,8 +1247,23 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="18" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="18" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="15" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="20" fontId="3" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="20" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="18" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="18" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1289,22 +1293,22 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>1</xdr:colOff>
+      <xdr:colOff>0</xdr:colOff>
       <xdr:row>1</xdr:row>
-      <xdr:rowOff>1</xdr:rowOff>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>11</xdr:col>
-      <xdr:colOff>755375</xdr:colOff>
-      <xdr:row>24</xdr:row>
-      <xdr:rowOff>90431</xdr:rowOff>
+      <xdr:col>17</xdr:col>
+      <xdr:colOff>132522</xdr:colOff>
+      <xdr:row>31</xdr:row>
+      <xdr:rowOff>68036</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="3" name="Imagen 2">
+        <xdr:cNvPr id="2" name="Imagen 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{7CEA3B6A-7E6A-D1B2-1874-4BF2006823E3}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{966B680E-EB45-290E-275E-F713F60D6F86}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1327,8 +1331,8 @@
       </xdr:blipFill>
       <xdr:spPr bwMode="auto">
         <a:xfrm>
-          <a:off x="1" y="185531"/>
-          <a:ext cx="10515600" cy="4357630"/>
+          <a:off x="0" y="190500"/>
+          <a:ext cx="14080435" cy="5783036"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1348,6 +1352,10 @@
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1690,12 +1698,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D2495362-94CF-4E08-8433-6F4780C6375E}">
   <dimension ref="A1:AD50"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="26.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="26.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
         <v>39</v>
       </c>
@@ -1729,7 +1737,7 @@
       <c r="AC1" s="1"/>
       <c r="AD1" s="1"/>
     </row>
-    <row r="2" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:30" x14ac:dyDescent="0.25">
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
@@ -1760,7 +1768,7 @@
       <c r="AC2" s="1"/>
       <c r="AD2" s="1"/>
     </row>
-    <row r="3" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
       <c r="B3" s="1"/>
       <c r="C3" s="1"/>
@@ -1792,7 +1800,7 @@
       <c r="AC3" s="1"/>
       <c r="AD3" s="1"/>
     </row>
-    <row r="4" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:30" x14ac:dyDescent="0.25">
       <c r="B4" s="1"/>
       <c r="C4" s="1"/>
       <c r="D4" s="1"/>
@@ -1823,7 +1831,7 @@
       <c r="AC4" s="1"/>
       <c r="AD4" s="1"/>
     </row>
-    <row r="5" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A5" s="1"/>
       <c r="B5" s="1"/>
       <c r="C5" s="1"/>
@@ -1855,7 +1863,7 @@
       <c r="AC5" s="1"/>
       <c r="AD5" s="1"/>
     </row>
-    <row r="6" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A6" s="1"/>
       <c r="B6" s="1"/>
       <c r="D6" s="1"/>
@@ -1886,7 +1894,7 @@
       <c r="AC6" s="1"/>
       <c r="AD6" s="1"/>
     </row>
-    <row r="7" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A7" s="1"/>
       <c r="C7" s="1"/>
       <c r="D7" s="1"/>
@@ -1917,7 +1925,7 @@
       <c r="AC7" s="1"/>
       <c r="AD7" s="1"/>
     </row>
-    <row r="8" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A8" s="1"/>
       <c r="B8" s="1"/>
       <c r="C8" s="1"/>
@@ -1949,7 +1957,7 @@
       <c r="AC8" s="1"/>
       <c r="AD8" s="1"/>
     </row>
-    <row r="9" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A9" s="1"/>
       <c r="B9" s="1"/>
       <c r="C9" s="1"/>
@@ -1981,7 +1989,7 @@
       <c r="AC9" s="1"/>
       <c r="AD9" s="1"/>
     </row>
-    <row r="10" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A10" s="1"/>
       <c r="B10" s="1"/>
       <c r="C10" s="1"/>
@@ -2013,7 +2021,7 @@
       <c r="AC10" s="1"/>
       <c r="AD10" s="1"/>
     </row>
-    <row r="11" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A11" s="1"/>
       <c r="B11" s="1"/>
       <c r="C11" s="1"/>
@@ -2045,7 +2053,7 @@
       <c r="AC11" s="1"/>
       <c r="AD11" s="1"/>
     </row>
-    <row r="12" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A12" s="1"/>
       <c r="B12" s="1"/>
       <c r="C12" s="1"/>
@@ -2077,7 +2085,7 @@
       <c r="AC12" s="1"/>
       <c r="AD12" s="1"/>
     </row>
-    <row r="13" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A13" s="1"/>
       <c r="B13" s="1"/>
       <c r="C13" s="1"/>
@@ -2109,7 +2117,7 @@
       <c r="AC13" s="1"/>
       <c r="AD13" s="1"/>
     </row>
-    <row r="14" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A14" s="1"/>
       <c r="B14" s="1"/>
       <c r="C14" s="1"/>
@@ -2141,7 +2149,7 @@
       <c r="AC14" s="1"/>
       <c r="AD14" s="1"/>
     </row>
-    <row r="15" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A15" s="1"/>
       <c r="B15" s="1"/>
       <c r="C15" s="1"/>
@@ -2173,7 +2181,7 @@
       <c r="AC15" s="1"/>
       <c r="AD15" s="1"/>
     </row>
-    <row r="16" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A16" s="1"/>
       <c r="B16" s="1"/>
       <c r="C16" s="1"/>
@@ -2205,7 +2213,7 @@
       <c r="AC16" s="1"/>
       <c r="AD16" s="1"/>
     </row>
-    <row r="17" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A17" s="1"/>
       <c r="B17" s="1"/>
       <c r="C17" s="1"/>
@@ -2237,7 +2245,7 @@
       <c r="AC17" s="1"/>
       <c r="AD17" s="1"/>
     </row>
-    <row r="18" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A18" s="1"/>
       <c r="B18" s="1"/>
       <c r="C18" s="1"/>
@@ -2269,7 +2277,7 @@
       <c r="AC18" s="1"/>
       <c r="AD18" s="1"/>
     </row>
-    <row r="19" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A19" s="1"/>
       <c r="B19" s="1"/>
       <c r="C19" s="1"/>
@@ -2301,7 +2309,7 @@
       <c r="AC19" s="1"/>
       <c r="AD19" s="1"/>
     </row>
-    <row r="20" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A20" s="1"/>
       <c r="B20" s="1"/>
       <c r="C20" s="1"/>
@@ -2333,7 +2341,7 @@
       <c r="AC20" s="1"/>
       <c r="AD20" s="1"/>
     </row>
-    <row r="21" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A21" s="1"/>
       <c r="B21" s="1"/>
       <c r="C21" s="1"/>
@@ -2365,7 +2373,7 @@
       <c r="AC21" s="1"/>
       <c r="AD21" s="1"/>
     </row>
-    <row r="22" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A22" s="1"/>
       <c r="B22" s="1"/>
       <c r="C22" s="1"/>
@@ -2397,7 +2405,7 @@
       <c r="AC22" s="1"/>
       <c r="AD22" s="1"/>
     </row>
-    <row r="23" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A23" s="1"/>
       <c r="B23" s="1"/>
       <c r="C23" s="1"/>
@@ -2429,7 +2437,7 @@
       <c r="AC23" s="1"/>
       <c r="AD23" s="1"/>
     </row>
-    <row r="24" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A24" s="1"/>
       <c r="B24" s="1"/>
       <c r="C24" s="1"/>
@@ -2461,7 +2469,7 @@
       <c r="AC24" s="1"/>
       <c r="AD24" s="1"/>
     </row>
-    <row r="25" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A25" s="1"/>
       <c r="B25" s="1"/>
       <c r="C25" s="1"/>
@@ -2493,7 +2501,7 @@
       <c r="AC25" s="1"/>
       <c r="AD25" s="1"/>
     </row>
-    <row r="26" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A26" s="1"/>
       <c r="B26" s="1"/>
       <c r="C26" s="1"/>
@@ -2525,7 +2533,7 @@
       <c r="AC26" s="1"/>
       <c r="AD26" s="1"/>
     </row>
-    <row r="27" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A27" s="1"/>
       <c r="B27" s="1"/>
       <c r="C27" s="1"/>
@@ -2557,7 +2565,7 @@
       <c r="AC27" s="1"/>
       <c r="AD27" s="1"/>
     </row>
-    <row r="28" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A28" s="1"/>
       <c r="B28" s="1"/>
       <c r="C28" s="1"/>
@@ -2589,7 +2597,7 @@
       <c r="AC28" s="1"/>
       <c r="AD28" s="1"/>
     </row>
-    <row r="29" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A29" s="1"/>
       <c r="B29" s="1"/>
       <c r="C29" s="1"/>
@@ -2621,7 +2629,7 @@
       <c r="AC29" s="1"/>
       <c r="AD29" s="1"/>
     </row>
-    <row r="30" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A30" s="1"/>
       <c r="B30" s="1"/>
       <c r="C30" s="1"/>
@@ -2653,7 +2661,7 @@
       <c r="AC30" s="1"/>
       <c r="AD30" s="1"/>
     </row>
-    <row r="31" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A31" s="1"/>
       <c r="B31" s="1"/>
       <c r="C31" s="1"/>
@@ -2685,7 +2693,7 @@
       <c r="AC31" s="1"/>
       <c r="AD31" s="1"/>
     </row>
-    <row r="32" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A32" s="1"/>
       <c r="B32" s="1"/>
       <c r="C32" s="1"/>
@@ -2717,7 +2725,7 @@
       <c r="AC32" s="1"/>
       <c r="AD32" s="1"/>
     </row>
-    <row r="33" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A33" s="1"/>
       <c r="B33" s="1"/>
       <c r="C33" s="1"/>
@@ -2749,7 +2757,7 @@
       <c r="AC33" s="1"/>
       <c r="AD33" s="1"/>
     </row>
-    <row r="34" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A34" s="1"/>
       <c r="B34" s="1"/>
       <c r="C34" s="1"/>
@@ -2781,7 +2789,7 @@
       <c r="AC34" s="1"/>
       <c r="AD34" s="1"/>
     </row>
-    <row r="35" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A35" s="1"/>
       <c r="B35" s="1"/>
       <c r="C35" s="1"/>
@@ -2813,7 +2821,7 @@
       <c r="AC35" s="1"/>
       <c r="AD35" s="1"/>
     </row>
-    <row r="36" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A36" s="1"/>
       <c r="B36" s="1"/>
       <c r="C36" s="1"/>
@@ -2845,7 +2853,7 @@
       <c r="AC36" s="1"/>
       <c r="AD36" s="1"/>
     </row>
-    <row r="37" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A37" s="1"/>
       <c r="B37" s="1"/>
       <c r="C37" s="1"/>
@@ -2877,7 +2885,7 @@
       <c r="AC37" s="1"/>
       <c r="AD37" s="1"/>
     </row>
-    <row r="38" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A38" s="1"/>
       <c r="B38" s="1"/>
       <c r="C38" s="1"/>
@@ -2909,7 +2917,7 @@
       <c r="AC38" s="1"/>
       <c r="AD38" s="1"/>
     </row>
-    <row r="39" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A39" s="1"/>
       <c r="B39" s="1"/>
       <c r="C39" s="1"/>
@@ -2941,7 +2949,7 @@
       <c r="AC39" s="1"/>
       <c r="AD39" s="1"/>
     </row>
-    <row r="40" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A40" s="1"/>
       <c r="B40" s="1"/>
       <c r="C40" s="1"/>
@@ -2973,7 +2981,7 @@
       <c r="AC40" s="1"/>
       <c r="AD40" s="1"/>
     </row>
-    <row r="41" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A41" s="1"/>
       <c r="B41" s="1"/>
       <c r="C41" s="1"/>
@@ -3005,7 +3013,7 @@
       <c r="AC41" s="1"/>
       <c r="AD41" s="1"/>
     </row>
-    <row r="42" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A42" s="1"/>
       <c r="B42" s="1"/>
       <c r="C42" s="1"/>
@@ -3037,7 +3045,7 @@
       <c r="AC42" s="1"/>
       <c r="AD42" s="1"/>
     </row>
-    <row r="43" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A43" s="1"/>
       <c r="B43" s="1"/>
       <c r="C43" s="1"/>
@@ -3069,7 +3077,7 @@
       <c r="AC43" s="1"/>
       <c r="AD43" s="1"/>
     </row>
-    <row r="44" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A44" s="1"/>
       <c r="B44" s="1"/>
       <c r="C44" s="1"/>
@@ -3101,7 +3109,7 @@
       <c r="AC44" s="1"/>
       <c r="AD44" s="1"/>
     </row>
-    <row r="45" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A45" s="1"/>
       <c r="B45" s="1"/>
       <c r="C45" s="1"/>
@@ -3133,7 +3141,7 @@
       <c r="AC45" s="1"/>
       <c r="AD45" s="1"/>
     </row>
-    <row r="46" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A46" s="1"/>
       <c r="B46" s="1"/>
       <c r="C46" s="1"/>
@@ -3165,7 +3173,7 @@
       <c r="AC46" s="1"/>
       <c r="AD46" s="1"/>
     </row>
-    <row r="47" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A47" s="1"/>
       <c r="B47" s="1"/>
       <c r="C47" s="1"/>
@@ -3197,7 +3205,7 @@
       <c r="AC47" s="1"/>
       <c r="AD47" s="1"/>
     </row>
-    <row r="48" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A48" s="1"/>
       <c r="B48" s="1"/>
       <c r="C48" s="1"/>
@@ -3229,7 +3237,7 @@
       <c r="AC48" s="1"/>
       <c r="AD48" s="1"/>
     </row>
-    <row r="49" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A49" s="1"/>
       <c r="B49" s="1"/>
       <c r="C49" s="1"/>
@@ -3261,7 +3269,7 @@
       <c r="AC49" s="1"/>
       <c r="AD49" s="1"/>
     </row>
-    <row r="50" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A50" s="1"/>
       <c r="B50" s="1"/>
       <c r="C50" s="1"/>
@@ -3306,16 +3314,16 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C828B98D-AAA9-4184-8373-FE2E421AAE23}">
   <dimension ref="A1:G11"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="27" customWidth="1"/>
-    <col min="3" max="4" width="28.88671875" customWidth="1"/>
+    <col min="3" max="4" width="28.85546875" customWidth="1"/>
     <col min="5" max="5" width="41" customWidth="1"/>
-    <col min="6" max="6" width="36.109375" customWidth="1"/>
-    <col min="7" max="7" width="26.88671875" customWidth="1"/>
+    <col min="6" max="6" width="36.140625" customWidth="1"/>
+    <col min="7" max="7" width="26.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
         <v>32</v>
       </c>
@@ -3324,41 +3332,41 @@
       </c>
       <c r="D1" s="5"/>
     </row>
-    <row r="2" spans="1:7" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="17" t="s">
         <v>20</v>
       </c>
       <c r="B2" s="17" t="s">
-        <v>233</v>
+        <v>223</v>
       </c>
       <c r="C2" s="17" t="s">
-        <v>234</v>
+        <v>224</v>
       </c>
       <c r="D2" s="17" t="s">
-        <v>220</v>
+        <v>210</v>
       </c>
       <c r="E2" s="30" t="s">
-        <v>215</v>
+        <v>205</v>
       </c>
       <c r="F2" s="30" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="G2" s="30" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="13" t="s">
         <v>31</v>
       </c>
       <c r="B3" s="31" t="s">
-        <v>221</v>
+        <v>211</v>
       </c>
       <c r="C3" s="31" t="s">
         <v>59</v>
       </c>
       <c r="D3" s="31" t="s">
-        <v>219</v>
+        <v>209</v>
       </c>
       <c r="E3" s="40" t="s">
         <v>25</v>
@@ -3370,11 +3378,11 @@
         <v>71</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="12">
         <v>1</v>
       </c>
-      <c r="B4" s="91" t="str">
+      <c r="B4" s="90" t="str">
         <f>Cliente_D!F4</f>
         <v>+57</v>
       </c>
@@ -3397,11 +3405,11 @@
         <v>3234528921-25/11/2023</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="12">
         <v>2</v>
       </c>
-      <c r="B5" s="91" t="str">
+      <c r="B5" s="90" t="str">
         <f>Cliente_D!F5</f>
         <v>+57</v>
       </c>
@@ -3424,11 +3432,11 @@
         <v>3161657782-21/03/2024</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="12">
         <v>3</v>
       </c>
-      <c r="B6" s="91" t="str">
+      <c r="B6" s="90" t="str">
         <f>Cliente_D!F6</f>
         <v>+57</v>
       </c>
@@ -3451,11 +3459,11 @@
         <v>3119884321-21/09/2024</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="12">
         <v>4</v>
       </c>
-      <c r="B7" s="91" t="str">
+      <c r="B7" s="90" t="str">
         <f>Cliente_D!F7</f>
         <v>+58</v>
       </c>
@@ -3478,16 +3486,16 @@
         <v>4127359182-11/12/2025</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="E8" s="29"/>
       <c r="F8" s="29"/>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="E10" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="E11" s="41"/>
     </row>
   </sheetData>
@@ -3517,15 +3525,15 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A24A074A-5C83-448D-978C-7C1005CE378E}">
   <dimension ref="A1:D7"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="29.109375" customWidth="1"/>
+    <col min="1" max="1" width="29.140625" customWidth="1"/>
     <col min="2" max="2" width="30" customWidth="1"/>
-    <col min="3" max="3" width="41.88671875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="61.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="41.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="61.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
         <v>32</v>
       </c>
@@ -3533,7 +3541,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="36.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:4" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="17" t="s">
         <v>20</v>
       </c>
@@ -3544,10 +3552,10 @@
         <v>62</v>
       </c>
       <c r="D2" s="39" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="13" t="s">
         <v>31</v>
       </c>
@@ -3561,7 +3569,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="12">
         <v>1</v>
       </c>
@@ -3578,7 +3586,7 @@
         <v>Juan García-Motilada</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="12">
         <v>2</v>
       </c>
@@ -3595,7 +3603,7 @@
         <v>Juan Ortiz-Corte de barba</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="12">
         <v>3</v>
       </c>
@@ -3612,7 +3620,7 @@
         <v>Carlos Arbeladez-Perfilada de barba</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="12">
         <v>4</v>
       </c>
@@ -3651,45 +3659,77 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2921A3C4-B96A-49A7-8353-9FD37D2F2B74}">
-  <dimension ref="A1:C14"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:H8"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
-    <col min="2" max="2" width="42.33203125" customWidth="1"/>
-    <col min="3" max="3" width="37.44140625" customWidth="1"/>
+    <col min="2" max="6" width="42.28515625" customWidth="1"/>
+    <col min="7" max="7" width="45.5703125" customWidth="1"/>
+    <col min="8" max="8" width="52.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
         <v>32</v>
       </c>
       <c r="B1" s="5" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="2" spans="1:3" ht="30" x14ac:dyDescent="0.3">
+      <c r="C1" s="5"/>
+      <c r="D1" s="5"/>
+      <c r="E1" s="5"/>
+      <c r="F1" s="5"/>
+      <c r="G1" s="5"/>
+    </row>
+    <row r="2" spans="1:8" ht="46.5" x14ac:dyDescent="0.25">
       <c r="A2" s="17" t="s">
         <v>20</v>
       </c>
       <c r="B2" s="17" t="s">
-        <v>122</v>
-      </c>
-      <c r="C2" s="18" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+        <v>118</v>
+      </c>
+      <c r="C2" s="17" t="s">
+        <v>225</v>
+      </c>
+      <c r="D2" s="17"/>
+      <c r="E2" s="17"/>
+      <c r="F2" s="17" t="s">
+        <v>226</v>
+      </c>
+      <c r="G2" s="17" t="s">
+        <v>228</v>
+      </c>
+      <c r="H2" s="18" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" s="13" t="s">
         <v>31</v>
       </c>
       <c r="B3" s="31" t="s">
         <v>40</v>
       </c>
-      <c r="C3" s="28" t="s">
+      <c r="C3" s="84" t="s">
+        <v>74</v>
+      </c>
+      <c r="D3" s="31" t="s">
+        <v>248</v>
+      </c>
+      <c r="E3" s="31" t="s">
+        <v>249</v>
+      </c>
+      <c r="F3" s="95" t="s">
+        <v>63</v>
+      </c>
+      <c r="G3" s="95" t="s">
+        <v>188</v>
+      </c>
+      <c r="H3" s="28" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" s="12">
         <v>1</v>
       </c>
@@ -3697,12 +3737,29 @@
         <f>_xlfn.CONCAT(Barbero_D!B4," ",Barbero_D!D4)</f>
         <v>Juan García</v>
       </c>
-      <c r="C4" s="12" t="str">
-        <f>B4</f>
-        <v>Juan García</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="C4" s="36" t="s">
+        <v>77</v>
+      </c>
+      <c r="D4" s="96">
+        <f>HorarioBarberia_D!D4</f>
+        <v>0.375</v>
+      </c>
+      <c r="E4" s="96">
+        <f>HorarioBarberia_D!E4</f>
+        <v>0.79166666666666663</v>
+      </c>
+      <c r="F4" s="88">
+        <v>0.41666666666666669</v>
+      </c>
+      <c r="G4" s="88">
+        <v>0.66666666666666663</v>
+      </c>
+      <c r="H4" s="12" t="str">
+        <f>_xlfn.CONCAT(B4,"-",C4,"-",TEXT(F4,"hh:mm"),"-",TEXT(G4,"hh:mm"))</f>
+        <v>Juan García-Lunes-10:00-16:00</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" s="12">
         <v>2</v>
       </c>
@@ -3710,12 +3767,29 @@
         <f>_xlfn.CONCAT(Barbero_D!B5," ",Barbero_D!D5)</f>
         <v>Juan Ortiz</v>
       </c>
-      <c r="C5" s="12" t="str">
-        <f t="shared" ref="C5:C7" si="0">B5</f>
-        <v>Juan Ortiz</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="C5" s="12" t="s">
+        <v>78</v>
+      </c>
+      <c r="D5" s="96">
+        <f>HorarioBarberia_D!D5</f>
+        <v>0.375</v>
+      </c>
+      <c r="E5" s="96">
+        <f>HorarioBarberia_D!E5</f>
+        <v>0.79166666666666663</v>
+      </c>
+      <c r="F5" s="88">
+        <v>0.375</v>
+      </c>
+      <c r="G5" s="88">
+        <v>0.625</v>
+      </c>
+      <c r="H5" s="12" t="str">
+        <f>_xlfn.CONCAT(B5,"-",C5,"-",TEXT(F5,"hh:mm"),"-",TEXT(G5,"hh:mm"))</f>
+        <v>Juan Ortiz-Martes-09:00-15:00</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" s="12">
         <v>3</v>
       </c>
@@ -3723,12 +3797,23 @@
         <f>_xlfn.CONCAT(Barbero_D!B6," ",Barbero_D!D6)</f>
         <v>Carlos Arbeladez</v>
       </c>
-      <c r="C6" s="12" t="str">
-        <f t="shared" si="0"/>
-        <v>Carlos Arbeladez</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="C6" s="12" t="s">
+        <v>80</v>
+      </c>
+      <c r="D6" s="11"/>
+      <c r="E6" s="11"/>
+      <c r="F6" s="88">
+        <v>0.54166666666666663</v>
+      </c>
+      <c r="G6" s="88">
+        <v>0.79166666666666663</v>
+      </c>
+      <c r="H6" s="12" t="str">
+        <f>_xlfn.CONCAT(B6,"-",C6,"-",TEXT(F6,"hh:mm"),"-",TEXT(G6,"hh:mm"))</f>
+        <v>Carlos Arbeladez-Jueves-13:00-19:00</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="12">
         <v>4</v>
       </c>
@@ -3736,14 +3821,44 @@
         <f>_xlfn.CONCAT(Barbero_D!B7," ",Barbero_D!D7)</f>
         <v>Andres Ramirez</v>
       </c>
-      <c r="C7" s="12" t="str">
-        <f t="shared" si="0"/>
+      <c r="C7" s="12" t="s">
+        <v>82</v>
+      </c>
+      <c r="D7" s="11"/>
+      <c r="E7" s="11"/>
+      <c r="F7" s="88">
+        <v>0.33333333333333331</v>
+      </c>
+      <c r="G7" s="88">
+        <v>0.58333333333333337</v>
+      </c>
+      <c r="H7" s="12" t="str">
+        <f>_xlfn.CONCAT(B7,"-",C7,"-",TEXT(F7,"hh:mm"),"-",TEXT(G7,"hh:mm"))</f>
+        <v>Andres Ramirez-Sábado-08:00-14:00</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A8" s="12">
+        <v>5</v>
+      </c>
+      <c r="B8" s="11" t="str">
+        <f>_xlfn.CONCAT(Barbero_D!B7," ",Barbero_D!D7)</f>
         <v>Andres Ramirez</v>
       </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="B14" t="s">
-        <v>250</v>
+      <c r="C8" s="12" t="s">
+        <v>233</v>
+      </c>
+      <c r="D8" s="11"/>
+      <c r="E8" s="11"/>
+      <c r="F8" s="88">
+        <v>0.5</v>
+      </c>
+      <c r="G8" s="88">
+        <v>0.625</v>
+      </c>
+      <c r="H8" s="12" t="str">
+        <f>_xlfn.CONCAT(B8,"-",C8,"-",TEXT(F8,"hh:mm"),"-",TEXT(G8,"hh:mm"))</f>
+        <v>Andres Ramirez-Festivo-12:00-15:00</v>
       </c>
     </row>
   </sheetData>
@@ -3756,6 +3871,8 @@
     <hyperlink ref="B5" location="Barbero_D!A5" display="Barbero_D!A5" xr:uid="{095BCBC5-A9C0-42E2-AF18-87E3049FBEDA}"/>
     <hyperlink ref="B6" location="Barbero_D!A6" display="Barbero_D!A6" xr:uid="{EA02F355-6C5D-4955-BCCD-7B0C9569DCED}"/>
     <hyperlink ref="B7" location="Barbero_D!A7" display="Barbero_D!A7" xr:uid="{979F9DA9-740D-4B06-AD22-BE8F66BD100A}"/>
+    <hyperlink ref="B8" location="Barbero_D!A7" display="Barbero_D!A7" xr:uid="{5A220669-7753-4BEA-B5E1-3132F586A541}"/>
+    <hyperlink ref="D3" location="HorarioBarberia_D!A1" display="horaAperturaBarberia" xr:uid="{2777B03F-8B4F-4798-A955-82C47EDEA18C}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -3764,18 +3881,18 @@
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{86AE141B-6E6C-47BF-9B70-297A81AC9A72}">
   <dimension ref="A1:G7"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="26.88671875" customWidth="1"/>
-    <col min="2" max="2" width="32.5546875" customWidth="1"/>
-    <col min="3" max="3" width="34.5546875" customWidth="1"/>
-    <col min="4" max="4" width="32.5546875" customWidth="1"/>
-    <col min="5" max="5" width="21.88671875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="20.109375" customWidth="1"/>
-    <col min="7" max="7" width="47.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="26.85546875" customWidth="1"/>
+    <col min="2" max="2" width="32.5703125" customWidth="1"/>
+    <col min="3" max="3" width="34.5703125" customWidth="1"/>
+    <col min="4" max="4" width="32.5703125" customWidth="1"/>
+    <col min="5" max="5" width="21.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="20.140625" customWidth="1"/>
+    <col min="7" max="7" width="64.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
         <v>32</v>
       </c>
@@ -3785,43 +3902,43 @@
       <c r="C1" s="5"/>
       <c r="D1" s="5"/>
     </row>
-    <row r="2" spans="1:7" ht="39.6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" ht="46.5" x14ac:dyDescent="0.25">
       <c r="A2" s="17" t="s">
         <v>20</v>
       </c>
       <c r="B2" s="18" t="s">
-        <v>196</v>
+        <v>187</v>
       </c>
       <c r="C2" s="30" t="s">
-        <v>229</v>
+        <v>219</v>
       </c>
       <c r="D2" s="30" t="s">
-        <v>230</v>
+        <v>220</v>
       </c>
       <c r="E2" s="18" t="s">
-        <v>216</v>
+        <v>206</v>
       </c>
       <c r="F2" s="18" t="s">
-        <v>231</v>
+        <v>221</v>
       </c>
       <c r="G2" s="18" t="s">
-        <v>198</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="13" t="s">
         <v>31</v>
       </c>
       <c r="B3" s="31" t="s">
         <v>60</v>
       </c>
-      <c r="C3" s="86" t="s">
-        <v>226</v>
-      </c>
-      <c r="D3" s="86" t="s">
-        <v>227</v>
-      </c>
-      <c r="E3" s="85" t="s">
+      <c r="C3" s="85" t="s">
+        <v>216</v>
+      </c>
+      <c r="D3" s="85" t="s">
+        <v>217</v>
+      </c>
+      <c r="E3" s="84" t="s">
         <v>21</v>
       </c>
       <c r="F3" s="40" t="s">
@@ -3831,104 +3948,104 @@
         <v>69</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="12">
         <v>1</v>
       </c>
       <c r="B4" s="11" t="str">
-        <f>Agenda_D!C4</f>
-        <v>Juan García</v>
-      </c>
-      <c r="C4" s="87">
+        <f>Agenda_D!H4</f>
+        <v>Juan García-Lunes-10:00-16:00</v>
+      </c>
+      <c r="C4" s="86">
         <v>46047.458333333336</v>
       </c>
-      <c r="D4" s="87">
+      <c r="D4" s="86">
         <v>46047.541666666664</v>
       </c>
       <c r="E4" s="79" t="s">
-        <v>205</v>
+        <v>195</v>
       </c>
       <c r="F4" s="12">
         <v>120</v>
       </c>
       <c r="G4" s="12" t="str">
         <f>_xlfn.CONCAT(B4,"-",TEXT(C4,"dd/mm/yyyy hh:mm"),"-",TEXT(D4,"dd/mm/yyyy hh:mm"))</f>
-        <v>Juan García-25/01/2026 11:00-25/01/2026 13:00</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+        <v>Juan García-Lunes-10:00-16:00-25/01/2026 11:00-25/01/2026 13:00</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="12">
         <v>2</v>
       </c>
       <c r="B5" s="11" t="str">
-        <f>Agenda_D!C5</f>
-        <v>Juan Ortiz</v>
-      </c>
-      <c r="C5" s="87">
+        <f>Agenda_D!H5</f>
+        <v>Juan Ortiz-Martes-09:00-15:00</v>
+      </c>
+      <c r="C5" s="86">
         <v>45362.5</v>
       </c>
-      <c r="D5" s="87">
+      <c r="D5" s="86">
         <v>45362.645833333336</v>
       </c>
-      <c r="E5" s="81" t="s">
-        <v>206</v>
+      <c r="E5" s="80" t="s">
+        <v>196</v>
       </c>
       <c r="F5" s="12">
         <v>210</v>
       </c>
       <c r="G5" s="12" t="str">
         <f t="shared" ref="G5:G7" si="0">_xlfn.CONCAT(B5,"-",TEXT(C5,"dd/mm/yyyy hh:mm"),"-",TEXT(D5,"dd/mm/yyyy hh:mm"))</f>
-        <v>Juan Ortiz-11/03/2024 12:00-11/03/2024 15:30</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+        <v>Juan Ortiz-Martes-09:00-15:00-11/03/2024 12:00-11/03/2024 15:30</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="12">
         <v>3</v>
       </c>
       <c r="B6" s="11" t="str">
-        <f>Agenda_D!C6</f>
-        <v>Carlos Arbeladez</v>
-      </c>
-      <c r="C6" s="87">
+        <f>Agenda_D!H6</f>
+        <v>Carlos Arbeladez-Jueves-13:00-19:00</v>
+      </c>
+      <c r="C6" s="86">
         <v>46013.541666666664</v>
       </c>
-      <c r="D6" s="87">
+      <c r="D6" s="86">
         <v>46013.583333333336</v>
       </c>
-      <c r="E6" s="81" t="s">
-        <v>207</v>
+      <c r="E6" s="80" t="s">
+        <v>197</v>
       </c>
       <c r="F6" s="12">
         <v>60</v>
       </c>
       <c r="G6" s="12" t="str">
         <f t="shared" si="0"/>
-        <v>Carlos Arbeladez-22/12/2025 13:00-22/12/2025 14:00</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+        <v>Carlos Arbeladez-Jueves-13:00-19:00-22/12/2025 13:00-22/12/2025 14:00</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="12">
         <v>4</v>
       </c>
       <c r="B7" s="78" t="str">
-        <f>Agenda_D!C7</f>
-        <v>Andres Ramirez</v>
-      </c>
-      <c r="C7" s="88">
+        <f>Agenda_D!H7</f>
+        <v>Andres Ramirez-Sábado-08:00-14:00</v>
+      </c>
+      <c r="C7" s="87">
         <v>46241.375</v>
       </c>
-      <c r="D7" s="88">
+      <c r="D7" s="87">
         <v>46241.5</v>
       </c>
-      <c r="E7" s="81" t="s">
-        <v>208</v>
+      <c r="E7" s="80" t="s">
+        <v>198</v>
       </c>
       <c r="F7" s="12">
         <v>180</v>
       </c>
       <c r="G7" s="12" t="str">
         <f t="shared" si="0"/>
-        <v>Andres Ramirez-07/08/2026 09:00-07/08/2026 12:00</v>
+        <v>Andres Ramirez-Sábado-08:00-14:00-07/08/2026 09:00-07/08/2026 12:00</v>
       </c>
     </row>
   </sheetData>
@@ -3946,19 +4063,20 @@
 </file>
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5CFE76D0-FBB4-4C81-85CC-F644057A8847}">
-  <dimension ref="A1:F11"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EB38530B-FD95-4EEF-8F76-78E045637369}">
+  <dimension ref="A1:G12"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="27" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="37.109375" customWidth="1"/>
-    <col min="3" max="3" width="46.5546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="26.88671875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="48.5546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="37.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="26.85546875" customWidth="1"/>
+    <col min="2" max="2" width="32.5703125" customWidth="1"/>
+    <col min="3" max="3" width="32.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="31.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="26.7109375" customWidth="1"/>
+    <col min="6" max="6" width="29.140625" customWidth="1"/>
+    <col min="7" max="7" width="38.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
         <v>32</v>
       </c>
@@ -3966,352 +4084,173 @@
         <v>33</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="40.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="18" t="s">
+    <row r="2" spans="1:7" ht="40.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="17" t="s">
         <v>20</v>
       </c>
       <c r="B2" s="18" t="s">
-        <v>86</v>
+        <v>190</v>
       </c>
       <c r="C2" s="18" t="s">
-        <v>235</v>
+        <v>230</v>
       </c>
       <c r="D2" s="18" t="s">
-        <v>236</v>
+        <v>229</v>
       </c>
       <c r="E2" s="18" t="s">
-        <v>238</v>
-      </c>
-      <c r="F2" s="18" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+        <v>212</v>
+      </c>
+      <c r="F2" s="30" t="s">
+        <v>213</v>
+      </c>
+      <c r="G2" s="18" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="13" t="s">
         <v>31</v>
       </c>
       <c r="B3" s="31" t="s">
         <v>60</v>
       </c>
-      <c r="C3" s="84" t="s">
-        <v>75</v>
+      <c r="C3" s="74" t="s">
+        <v>63</v>
       </c>
       <c r="D3" s="74" t="s">
-        <v>63</v>
-      </c>
-      <c r="E3" s="74" t="s">
-        <v>85</v>
-      </c>
-      <c r="F3" s="28" t="s">
+        <v>188</v>
+      </c>
+      <c r="E3" s="71" t="s">
+        <v>21</v>
+      </c>
+      <c r="F3" s="81" t="s">
+        <v>37</v>
+      </c>
+      <c r="G3" s="28" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="12">
         <v>1</v>
       </c>
-      <c r="B4" s="46" t="str">
-        <f>Agenda_D!C4</f>
-        <v>Juan García</v>
-      </c>
-      <c r="C4" s="36" t="s">
-        <v>78</v>
-      </c>
-      <c r="D4" s="89">
-        <v>0.41666666666666669</v>
-      </c>
-      <c r="E4" s="89">
-        <v>0.66666666666666663</v>
-      </c>
-      <c r="F4" s="12" t="str">
-        <f>_xlfn.CONCAT(B4,"-",C4,"-",TEXT(D4,"hh;mm"),"-",TEXT(E4,"hh;mm"))</f>
-        <v>Juan García-Lunes-10-16</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="B4" s="11" t="str">
+        <f>Agenda_D!H4</f>
+        <v>Juan García-Lunes-10:00-16:00</v>
+      </c>
+      <c r="C4" s="88">
+        <v>0.5</v>
+      </c>
+      <c r="D4" s="88">
+        <v>0.58333333333333337</v>
+      </c>
+      <c r="E4" s="36" t="s">
+        <v>191</v>
+      </c>
+      <c r="F4" s="82">
+        <v>120</v>
+      </c>
+      <c r="G4" s="12" t="str">
+        <f>_xlfn.CONCAT(B4,"-",TEXT(C4,"hh;mm"),"-",TEXT(D4,"hh;mm"))</f>
+        <v>Juan García-Lunes-10:00-16:00-12-14</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="12">
         <v>2</v>
       </c>
-      <c r="B5" s="46" t="str">
-        <f>Agenda_D!C5</f>
-        <v>Juan Ortiz</v>
-      </c>
-      <c r="C5" s="12" t="s">
-        <v>79</v>
-      </c>
-      <c r="D5" s="89">
-        <v>0.375</v>
-      </c>
-      <c r="E5" s="89">
-        <v>0.625</v>
-      </c>
-      <c r="F5" s="12" t="str">
-        <f t="shared" ref="F5:F8" si="0">_xlfn.CONCAT(B5,"-",C5,"-",TEXT(D5,"hh;mm"),"-",TEXT(E5,"hh;mm"))</f>
-        <v>Juan Ortiz-Martes-09-15</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="B5" s="11" t="str">
+        <f>Agenda_D!H7</f>
+        <v>Andres Ramirez-Sábado-08:00-14:00</v>
+      </c>
+      <c r="C5" s="88">
+        <v>0.52083333333333337</v>
+      </c>
+      <c r="D5" s="97">
+        <v>0.54166666666666663</v>
+      </c>
+      <c r="E5" s="24" t="s">
+        <v>194</v>
+      </c>
+      <c r="F5" s="12">
+        <v>120</v>
+      </c>
+      <c r="G5" s="12" t="str">
+        <f t="shared" ref="G5:G7" si="0">_xlfn.CONCAT(B5,"-",TEXT(C5,"hh;mm"),"-",TEXT(D5,"hh;mm"))</f>
+        <v>Andres Ramirez-Sábado-08:00-14:00-12-13</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="12">
         <v>3</v>
       </c>
-      <c r="B6" s="46" t="str">
-        <f>Agenda_D!C6</f>
-        <v>Carlos Arbeladez</v>
-      </c>
-      <c r="C6" s="12" t="s">
-        <v>81</v>
-      </c>
-      <c r="D6" s="89">
-        <v>0.54166666666666663</v>
-      </c>
-      <c r="E6" s="89">
-        <v>0.79166666666666663</v>
-      </c>
-      <c r="F6" s="12" t="str">
+      <c r="B6" s="11" t="str">
+        <f>Agenda_D!H8</f>
+        <v>Andres Ramirez-Festivo-12:00-15:00</v>
+      </c>
+      <c r="C6" s="88">
+        <v>0.58333333333333337</v>
+      </c>
+      <c r="D6" s="88">
+        <v>0.60416666666666663</v>
+      </c>
+      <c r="E6" s="12" t="s">
+        <v>193</v>
+      </c>
+      <c r="F6" s="12">
+        <v>60</v>
+      </c>
+      <c r="G6" s="12" t="str">
         <f t="shared" si="0"/>
-        <v>Carlos Arbeladez-Jueves-13-19</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+        <v>Andres Ramirez-Festivo-12:00-15:00-14-14</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="12">
         <v>4</v>
       </c>
-      <c r="B7" s="46" t="str">
-        <f>Agenda_D!C7</f>
-        <v>Andres Ramirez</v>
-      </c>
-      <c r="C7" s="12" t="s">
-        <v>83</v>
-      </c>
-      <c r="D7" s="89">
-        <v>0.33333333333333331</v>
-      </c>
-      <c r="E7" s="89">
-        <v>0.58333333333333337</v>
-      </c>
-      <c r="F7" s="12" t="str">
-        <f t="shared" si="0"/>
-        <v>Andres Ramirez-Sábado-08-14</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A8" s="12">
-        <v>5</v>
-      </c>
-      <c r="B8" s="11" t="str">
-        <f>Agenda_D!C7</f>
-        <v>Andres Ramirez</v>
-      </c>
-      <c r="C8" s="12" t="s">
-        <v>243</v>
-      </c>
-      <c r="D8" s="89">
-        <v>0.5</v>
-      </c>
-      <c r="E8" s="89">
-        <v>0.625</v>
-      </c>
-      <c r="F8" s="12" t="str">
-        <f t="shared" si="0"/>
-        <v>Andres Ramirez-Festivo-12-15</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="C10" s="10"/>
-      <c r="E10" s="10"/>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="E11" s="10"/>
-    </row>
-  </sheetData>
-  <hyperlinks>
-    <hyperlink ref="A1" location="'Modelo de Dominio'!A1" display="&lt;&lt;&lt;&lt; Ir al modulo de dominio" xr:uid="{98F427D6-B9F6-42D5-A84C-3F68DE3A5B6E}"/>
-    <hyperlink ref="B1" location="'Objetos de Dominio'!A1" display="&lt;&lt;&lt;&lt; Ir a objetos de dominio" xr:uid="{9EA36EAB-A0B6-4F6C-A61D-44A86E61BF9F}"/>
-    <hyperlink ref="B3" location="Agenda_D!A1" display="agenda" xr:uid="{4824C529-638F-4299-AEE0-9730B3BC73C9}"/>
-    <hyperlink ref="B4" location="Agenda_D!A4" display="Agenda_D!A4" xr:uid="{4DA17190-FFA5-47EF-8FD3-54EA9F7DF58B}"/>
-    <hyperlink ref="B5:B7" location="Agenda_D!A4" display="Agenda_D!A4" xr:uid="{6001330A-45FA-467D-82F2-97DD807F947F}"/>
-    <hyperlink ref="B5" location="Agenda_D!A5" display="Agenda_D!A5" xr:uid="{22BB4167-53C0-4D10-9F76-560F79FADE86}"/>
-    <hyperlink ref="B6" location="Agenda_D!A6" display="Agenda_D!A6" xr:uid="{36B092FB-CBA5-4E3A-9127-52EA641442EA}"/>
-    <hyperlink ref="B7" location="Agenda_D!A7" display="Agenda_D!A7" xr:uid="{59DFEC77-AF33-433C-99D6-F82241ADA5F1}"/>
-    <hyperlink ref="B8" location="Agenda_D!A7" display="Agenda_D!A7" xr:uid="{F90905DD-1298-4E08-99DE-C45A5F8D96D3}"/>
-  </hyperlinks>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EB38530B-FD95-4EEF-8F76-78E045637369}">
-  <dimension ref="A1:G7"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="26.88671875" customWidth="1"/>
-    <col min="2" max="2" width="32.5546875" customWidth="1"/>
-    <col min="3" max="3" width="32.6640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="31.109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="26.6640625" customWidth="1"/>
-    <col min="6" max="6" width="29.109375" customWidth="1"/>
-    <col min="7" max="7" width="33.6640625" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A1" s="5" t="s">
-        <v>32</v>
-      </c>
-      <c r="B1" s="5" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" ht="40.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="17" t="s">
-        <v>20</v>
-      </c>
-      <c r="B2" s="18" t="s">
-        <v>200</v>
-      </c>
-      <c r="C2" s="18" t="s">
-        <v>240</v>
-      </c>
-      <c r="D2" s="18" t="s">
-        <v>239</v>
-      </c>
-      <c r="E2" s="18" t="s">
-        <v>222</v>
-      </c>
-      <c r="F2" s="30" t="s">
-        <v>223</v>
-      </c>
-      <c r="G2" s="18" t="s">
-        <v>209</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A3" s="13" t="s">
-        <v>31</v>
-      </c>
-      <c r="B3" s="31" t="s">
-        <v>199</v>
-      </c>
-      <c r="C3" s="74" t="s">
-        <v>63</v>
-      </c>
-      <c r="D3" s="74" t="s">
-        <v>197</v>
-      </c>
-      <c r="E3" s="71" t="s">
-        <v>21</v>
-      </c>
-      <c r="F3" s="82" t="s">
-        <v>37</v>
-      </c>
-      <c r="G3" s="28" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A4" s="12">
-        <v>1</v>
-      </c>
-      <c r="B4" s="11" t="str">
-        <f>HorarioBarbero_D!F4</f>
-        <v>Juan García-Lunes-10-16</v>
-      </c>
-      <c r="C4" s="36">
-        <v>0.5</v>
-      </c>
-      <c r="D4" s="36">
-        <v>0.58333333333333337</v>
-      </c>
-      <c r="E4" s="36" t="s">
-        <v>201</v>
-      </c>
-      <c r="F4" s="83">
-        <v>120</v>
-      </c>
-      <c r="G4" s="12" t="str">
-        <f>_xlfn.CONCAT(B4,"-",TEXT(C4,"hh;mm"),"-",TEXT(D4,"hh;mm"))</f>
-        <v>Juan García-Lunes-10-16-12-14</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A5" s="12">
-        <v>2</v>
-      </c>
-      <c r="B5" s="11" t="str">
-        <f>HorarioBarbero_D!F5</f>
-        <v>Juan Ortiz-Martes-09-15</v>
-      </c>
-      <c r="C5" s="36">
+      <c r="B7" s="11" t="str">
+        <f>Agenda_D!H5</f>
+        <v>Juan Ortiz-Martes-09:00-15:00</v>
+      </c>
+      <c r="C7" s="88">
+        <v>0.47916666666666669</v>
+      </c>
+      <c r="D7" s="88">
         <v>0.54166666666666663</v>
       </c>
-      <c r="D5" s="80">
-        <v>0.625</v>
-      </c>
-      <c r="E5" s="24" t="s">
-        <v>204</v>
-      </c>
-      <c r="F5" s="12">
-        <v>120</v>
-      </c>
-      <c r="G5" s="12" t="str">
-        <f t="shared" ref="G5:G7" si="0">_xlfn.CONCAT(B5,"-",TEXT(C5,"hh;mm"),"-",TEXT(D5,"hh;mm"))</f>
-        <v>Juan Ortiz-Martes-09-15-13-15</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A6" s="12">
-        <v>3</v>
-      </c>
-      <c r="B6" s="11" t="str">
-        <f>HorarioBarbero_D!F6</f>
-        <v>Carlos Arbeladez-Jueves-13-19</v>
-      </c>
-      <c r="C6" s="36">
-        <v>0.70833333333333337</v>
-      </c>
-      <c r="D6" s="36">
-        <v>0.75</v>
-      </c>
-      <c r="E6" s="12" t="s">
-        <v>203</v>
-      </c>
-      <c r="F6" s="12">
-        <v>60</v>
-      </c>
-      <c r="G6" s="12" t="str">
-        <f t="shared" si="0"/>
-        <v>Carlos Arbeladez-Jueves-13-19-17-18</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A7" s="12">
-        <v>4</v>
-      </c>
-      <c r="B7" s="11" t="str">
-        <f>HorarioBarbero_D!F7</f>
-        <v>Andres Ramirez-Sábado-08-14</v>
-      </c>
-      <c r="C7" s="36">
-        <v>0.47916666666666669</v>
-      </c>
-      <c r="D7" s="36">
-        <v>0.54166666666666663</v>
-      </c>
       <c r="E7" s="12" t="s">
-        <v>202</v>
+        <v>192</v>
       </c>
       <c r="F7" s="12">
         <v>90</v>
       </c>
       <c r="G7" s="12" t="str">
         <f t="shared" si="0"/>
-        <v>Andres Ramirez-Sábado-08-14-11-13</v>
-      </c>
+        <v>Juan Ortiz-Martes-09:00-15:00-11-13</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="C9" s="98"/>
+      <c r="D9" s="98"/>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="C10" s="98"/>
+      <c r="D10" s="99"/>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="C11" s="98"/>
+      <c r="D11" s="98"/>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="C12" s="98"/>
+      <c r="D12" s="98"/>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="A1" location="'Modelo de Dominio'!A1" display="&lt;&lt;&lt;&lt; Ir al modulo de dominio" xr:uid="{28D494EF-6E9C-4926-913D-1C222BAE912F}"/>
     <hyperlink ref="B1" location="'Objetos de Dominio'!A1" display="&lt;&lt;&lt;&lt; Ir a objetos de dominio" xr:uid="{E603E2D9-858F-4FFA-8815-5567364FE382}"/>
-    <hyperlink ref="B3" location="HorarioBarbero_D!A1" display="horarioDelBarbero" xr:uid="{E895F830-FA04-42C5-BF65-9170EC8A6C40}"/>
+    <hyperlink ref="B3" location="Agenda_D!A1" display="agenda" xr:uid="{E895F830-FA04-42C5-BF65-9170EC8A6C40}"/>
     <hyperlink ref="B4" location="HorarioBarbero_D!A4" display="HorarioBarbero_D!A4" xr:uid="{8EE0E36C-8BF0-4BBA-8EAF-59B76141C41B}"/>
     <hyperlink ref="B5" location="HorarioBarbero_D!A5" display="HorarioBarbero_D!A5" xr:uid="{B5E52511-94A7-4409-8D8A-54A2A651A3ED}"/>
     <hyperlink ref="B6" location="HorarioBarbero_D!A6" display="HorarioBarbero_D!A6" xr:uid="{70BE22C1-3690-4C31-BFB5-A4A0D08A8829}"/>
@@ -4321,22 +4260,22 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1429879F-6697-4F1F-AF5D-52C4860B7B3E}">
   <dimension ref="A1:H15"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="28" customWidth="1"/>
-    <col min="2" max="2" width="26.5546875" customWidth="1"/>
-    <col min="3" max="3" width="30.44140625" customWidth="1"/>
-    <col min="4" max="4" width="27.5546875" customWidth="1"/>
-    <col min="5" max="5" width="36.5546875" customWidth="1"/>
-    <col min="6" max="6" width="60.33203125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="39.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="26.5703125" customWidth="1"/>
+    <col min="3" max="3" width="30.42578125" customWidth="1"/>
+    <col min="4" max="4" width="27.5703125" customWidth="1"/>
+    <col min="5" max="5" width="36.5703125" customWidth="1"/>
+    <col min="6" max="6" width="60.28515625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="39.28515625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="22" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
         <v>32</v>
       </c>
@@ -4344,7 +4283,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="44.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" ht="44.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="17" t="s">
         <v>20</v>
       </c>
@@ -4352,22 +4291,22 @@
         <v>64</v>
       </c>
       <c r="C2" s="30" t="s">
-        <v>138</v>
+        <v>131</v>
       </c>
       <c r="D2" s="30" t="s">
-        <v>192</v>
+        <v>183</v>
       </c>
       <c r="E2" s="30" t="s">
-        <v>245</v>
+        <v>235</v>
       </c>
       <c r="F2" s="30" t="s">
-        <v>224</v>
+        <v>214</v>
       </c>
       <c r="G2" s="30" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" s="13" t="s">
         <v>31</v>
       </c>
@@ -4378,10 +4317,10 @@
         <v>60</v>
       </c>
       <c r="D3" s="77" t="s">
-        <v>132</v>
+        <v>125</v>
       </c>
       <c r="E3" s="40" t="s">
-        <v>244</v>
+        <v>234</v>
       </c>
       <c r="F3" s="54" t="s">
         <v>26</v>
@@ -4390,7 +4329,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" s="12">
         <v>1</v>
       </c>
@@ -4399,8 +4338,8 @@
         <v xml:space="preserve">Juan  Gómez </v>
       </c>
       <c r="C4" s="11" t="str">
-        <f>Agenda_D!C4</f>
-        <v>Juan García</v>
+        <f>Agenda_D!H4</f>
+        <v>Juan García-Lunes-10:00-16:00</v>
       </c>
       <c r="D4" s="48">
         <v>46295.416666666664</v>
@@ -4413,10 +4352,10 @@
       </c>
       <c r="G4" s="12" t="str">
         <f>_xlfn.CONCAT(C4,"-",TEXT(D4,"dd/mm/yyyy/hh:mm"))</f>
-        <v>Juan García-30/09/2026/10:00</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+        <v>Juan García-Lunes-10:00-16:00-30/09/2026/10:00</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" s="12">
         <v>2</v>
       </c>
@@ -4425,8 +4364,8 @@
         <v>Jose Miguel Ramirez Perez</v>
       </c>
       <c r="C5" s="11" t="str">
-        <f>Agenda_D!C5</f>
-        <v>Juan Ortiz</v>
+        <f>Agenda_D!H5</f>
+        <v>Juan Ortiz-Martes-09:00-15:00</v>
       </c>
       <c r="D5" s="48">
         <v>45983.458333333336</v>
@@ -4435,14 +4374,14 @@
         <v>45983.489583333336</v>
       </c>
       <c r="F5" s="12" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="G5" s="12" t="str">
         <f t="shared" ref="G5:G8" si="0">_xlfn.CONCAT(C5,"-",TEXT(D5,"dd/mm/yyyy/hh:mm"))</f>
-        <v>Juan Ortiz-22/11/2025/11:00</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+        <v>Juan Ortiz-Martes-09:00-15:00-22/11/2025/11:00</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" s="12">
         <v>3</v>
       </c>
@@ -4451,8 +4390,8 @@
         <v>Simon  Ochoa Ramirez</v>
       </c>
       <c r="C6" s="11" t="str">
-        <f>Agenda_D!C6</f>
-        <v>Carlos Arbeladez</v>
+        <f>Agenda_D!H6</f>
+        <v>Carlos Arbeladez-Jueves-13:00-19:00</v>
       </c>
       <c r="D6" s="48">
         <v>45514.583333333336</v>
@@ -4461,14 +4400,14 @@
         <v>45514.59375</v>
       </c>
       <c r="F6" s="12" t="s">
-        <v>134</v>
+        <v>127</v>
       </c>
       <c r="G6" s="12" t="str">
         <f t="shared" si="0"/>
-        <v>Carlos Arbeladez-10/08/2024/14:00</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+        <v>Carlos Arbeladez-Jueves-13:00-19:00-10/08/2024/14:00</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="12">
         <v>4</v>
       </c>
@@ -4477,8 +4416,8 @@
         <v xml:space="preserve">Alexis  Gallego </v>
       </c>
       <c r="C7" s="11" t="str">
-        <f>Agenda_D!C7</f>
-        <v>Andres Ramirez</v>
+        <f>Agenda_D!H7</f>
+        <v>Andres Ramirez-Sábado-08:00-14:00</v>
       </c>
       <c r="D7" s="48">
         <v>46289.541666666664</v>
@@ -4487,14 +4426,14 @@
         <v>46289.5625</v>
       </c>
       <c r="F7" s="12" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="G7" s="12" t="str">
         <f t="shared" si="0"/>
-        <v>Andres Ramirez-24/09/2026/13:00</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+        <v>Andres Ramirez-Sábado-08:00-14:00-24/09/2026/13:00</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" s="12">
         <v>5</v>
       </c>
@@ -4503,8 +4442,8 @@
         <v xml:space="preserve">Alexis  Gallego </v>
       </c>
       <c r="C8" s="11" t="str">
-        <f>Agenda_D!C6</f>
-        <v>Carlos Arbeladez</v>
+        <f>Agenda_D!H6</f>
+        <v>Carlos Arbeladez-Jueves-13:00-19:00</v>
       </c>
       <c r="D8" s="48">
         <v>46240.75</v>
@@ -4513,35 +4452,35 @@
         <v>46240.756944444445</v>
       </c>
       <c r="F8" s="12" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="G8" s="12" t="str">
         <f t="shared" si="0"/>
-        <v>Carlos Arbeladez-06/08/2026/18:00</v>
+        <v>Carlos Arbeladez-Jueves-13:00-19:00-06/08/2026/18:00</v>
       </c>
       <c r="H8" s="45"/>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="E10" s="93"/>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="E10" s="92"/>
       <c r="H10" s="47"/>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="E11" s="93"/>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="E11" s="92"/>
       <c r="F11" s="10"/>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="D12" s="49"/>
-      <c r="E12" s="93"/>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="E12" s="92"/>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="D13" s="49"/>
-      <c r="E13" s="93"/>
-    </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="E13" s="92"/>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="D14" s="49"/>
-      <c r="E14" s="93"/>
-    </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="E14" s="92"/>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="D15" s="49"/>
     </row>
   </sheetData>
@@ -4567,20 +4506,20 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{766573FB-AAA2-4254-B83C-7C7505540365}">
   <dimension ref="A1:G7"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="26.6640625" customWidth="1"/>
-    <col min="2" max="2" width="38.5546875" customWidth="1"/>
-    <col min="3" max="3" width="39.33203125" bestFit="1" customWidth="1"/>
-    <col min="4" max="5" width="39.6640625" customWidth="1"/>
-    <col min="6" max="6" width="34.33203125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="39.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="26.7109375" customWidth="1"/>
+    <col min="2" max="2" width="38.5703125" customWidth="1"/>
+    <col min="3" max="3" width="39.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="39.7109375" customWidth="1"/>
+    <col min="6" max="6" width="34.28515625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="39.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
         <v>32</v>
       </c>
@@ -4588,30 +4527,30 @@
         <v>33</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="31.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="17" t="s">
         <v>20</v>
       </c>
       <c r="B2" s="17" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="C2" s="30" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="D2" s="30" t="s">
-        <v>225</v>
+        <v>215</v>
       </c>
       <c r="E2" s="30" t="s">
-        <v>140</v>
+        <v>133</v>
       </c>
       <c r="F2" s="30" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="G2" s="30" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="13" t="s">
         <v>31</v>
       </c>
@@ -4619,13 +4558,13 @@
         <v>44</v>
       </c>
       <c r="C3" s="31" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="D3" s="40" t="s">
         <v>27</v>
       </c>
       <c r="E3" s="53" t="s">
-        <v>139</v>
+        <v>132</v>
       </c>
       <c r="F3" s="40" t="s">
         <v>28</v>
@@ -4634,7 +4573,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="12">
         <v>1</v>
       </c>
@@ -4644,24 +4583,24 @@
       </c>
       <c r="C4" s="11" t="str">
         <f>Cita_D!G6</f>
-        <v>Carlos Arbeladez-10/08/2024/14:00</v>
+        <v>Carlos Arbeladez-Jueves-13:00-19:00-10/08/2024/14:00</v>
       </c>
       <c r="D4" s="12">
         <f>Regla_D!C4</f>
         <v>10000</v>
       </c>
       <c r="E4" s="12" t="s">
-        <v>134</v>
+        <v>127</v>
       </c>
       <c r="F4" s="12" t="s">
         <v>49</v>
       </c>
       <c r="G4" s="12" t="str">
         <f>C4</f>
-        <v>Carlos Arbeladez-10/08/2024/14:00</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+        <v>Carlos Arbeladez-Jueves-13:00-19:00-10/08/2024/14:00</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="12">
         <v>2</v>
       </c>
@@ -4671,24 +4610,24 @@
       </c>
       <c r="C5" s="11" t="str">
         <f>Cita_D!G7</f>
-        <v>Andres Ramirez-24/09/2026/13:00</v>
+        <v>Andres Ramirez-Sábado-08:00-14:00-24/09/2026/13:00</v>
       </c>
       <c r="D5" s="12">
         <f>CitaServicio_D!D8</f>
         <v>35000</v>
       </c>
       <c r="E5" s="12" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="F5" s="12" t="s">
         <v>50</v>
       </c>
       <c r="G5" s="12" t="str">
         <f>C5</f>
-        <v>Andres Ramirez-24/09/2026/13:00</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+        <v>Andres Ramirez-Sábado-08:00-14:00-24/09/2026/13:00</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="10"/>
       <c r="B6" s="10"/>
       <c r="C6" s="10"/>
@@ -4697,7 +4636,7 @@
       <c r="F6" s="10"/>
       <c r="G6" s="10"/>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="10"/>
       <c r="B7" s="10"/>
       <c r="C7" s="10"/>
@@ -4721,20 +4660,20 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F470C5A4-8D15-43DA-95FC-91C9614E5EEA}">
   <dimension ref="A1:F12"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="26.44140625" customWidth="1"/>
-    <col min="2" max="2" width="39.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="21.88671875" customWidth="1"/>
-    <col min="4" max="4" width="41.88671875" customWidth="1"/>
-    <col min="5" max="5" width="32.109375" customWidth="1"/>
-    <col min="6" max="6" width="55.88671875" customWidth="1"/>
+    <col min="1" max="1" width="26.42578125" customWidth="1"/>
+    <col min="2" max="2" width="49.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="21.85546875" customWidth="1"/>
+    <col min="4" max="4" width="41.85546875" customWidth="1"/>
+    <col min="5" max="5" width="32.140625" customWidth="1"/>
+    <col min="6" max="6" width="55.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
         <v>32</v>
       </c>
@@ -4742,32 +4681,32 @@
         <v>33</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="33" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:6" ht="33" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="17" t="s">
         <v>20</v>
       </c>
       <c r="B2" s="17" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="C2" s="30" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="D2" s="30" t="s">
-        <v>217</v>
+        <v>207</v>
       </c>
       <c r="E2" s="30" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="F2" s="30" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="37" t="s">
         <v>31</v>
       </c>
       <c r="B3" s="31" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="C3" s="31" t="s">
         <v>41</v>
@@ -4782,13 +4721,13 @@
         <v>69</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="12">
         <v>1</v>
       </c>
       <c r="B4" s="11" t="str">
         <f>Cita_D!G4</f>
-        <v>Juan García-30/09/2026/10:00</v>
+        <v>Juan García-Lunes-10:00-16:00-30/09/2026/10:00</v>
       </c>
       <c r="C4" s="11" t="str">
         <f>Servicio_D!F4</f>
@@ -4802,16 +4741,16 @@
       </c>
       <c r="F4" s="12" t="str">
         <f>_xlfn.CONCAT(B4,"-",C4)</f>
-        <v>Juan García-30/09/2026/10:00-Motilada</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+        <v>Juan García-Lunes-10:00-16:00-30/09/2026/10:00-Motilada</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="12">
         <v>2</v>
       </c>
       <c r="B5" s="11" t="str">
         <f>Cita_D!G5</f>
-        <v>Juan Ortiz-22/11/2025/11:00</v>
+        <v>Juan Ortiz-Martes-09:00-15:00-22/11/2025/11:00</v>
       </c>
       <c r="C5" s="11" t="str">
         <f>Servicio_D!F5</f>
@@ -4825,16 +4764,16 @@
       </c>
       <c r="F5" s="12" t="str">
         <f>_xlfn.CONCAT(B5,"-",C5)</f>
-        <v>Juan Ortiz-22/11/2025/11:00-Corte de barba</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+        <v>Juan Ortiz-Martes-09:00-15:00-22/11/2025/11:00-Corte de barba</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="12">
         <v>3</v>
       </c>
       <c r="B6" s="11" t="str">
         <f>Cita_D!G5</f>
-        <v>Juan Ortiz-22/11/2025/11:00</v>
+        <v>Juan Ortiz-Martes-09:00-15:00-22/11/2025/11:00</v>
       </c>
       <c r="C6" s="11" t="str">
         <f>Servicio_D!F4</f>
@@ -4848,16 +4787,16 @@
       </c>
       <c r="F6" s="12" t="str">
         <f t="shared" ref="F6:F9" si="0">_xlfn.CONCAT(B6,"-",C6)</f>
-        <v>Juan Ortiz-22/11/2025/11:00-Motilada</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+        <v>Juan Ortiz-Martes-09:00-15:00-22/11/2025/11:00-Motilada</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="12">
         <v>4</v>
       </c>
       <c r="B7" s="11" t="str">
         <f>Cita_D!G6</f>
-        <v>Carlos Arbeladez-10/08/2024/14:00</v>
+        <v>Carlos Arbeladez-Jueves-13:00-19:00-10/08/2024/14:00</v>
       </c>
       <c r="C7" s="11" t="str">
         <f>Servicio_D!F6</f>
@@ -4871,16 +4810,16 @@
       </c>
       <c r="F7" s="12" t="str">
         <f t="shared" si="0"/>
-        <v>Carlos Arbeladez-10/08/2024/14:00-Perfilada de barba</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+        <v>Carlos Arbeladez-Jueves-13:00-19:00-10/08/2024/14:00-Perfilada de barba</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" ht="45" x14ac:dyDescent="0.25">
       <c r="A8" s="12">
         <v>5</v>
       </c>
       <c r="B8" s="11" t="str">
         <f>Cita_D!G7</f>
-        <v>Andres Ramirez-24/09/2026/13:00</v>
+        <v>Andres Ramirez-Sábado-08:00-14:00-24/09/2026/13:00</v>
       </c>
       <c r="C8" s="50" t="str">
         <f>Servicio_D!F7</f>
@@ -4894,16 +4833,16 @@
       </c>
       <c r="F8" s="24" t="str">
         <f t="shared" si="0"/>
-        <v>Andres Ramirez-24/09/2026/13:00-Arreglo completo de barba con toalla caliente</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+        <v>Andres Ramirez-Sábado-08:00-14:00-24/09/2026/13:00-Arreglo completo de barba con toalla caliente</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="12">
         <v>6</v>
       </c>
       <c r="B9" s="11" t="str">
         <f>Cita_D!G8</f>
-        <v>Carlos Arbeladez-06/08/2026/18:00</v>
+        <v>Carlos Arbeladez-Jueves-13:00-19:00-06/08/2026/18:00</v>
       </c>
       <c r="C9" s="11" t="str">
         <f>Servicio_D!C5</f>
@@ -4917,17 +4856,17 @@
       </c>
       <c r="F9" s="24" t="str">
         <f t="shared" si="0"/>
-        <v>Carlos Arbeladez-06/08/2026/18:00-Corte de barba</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+        <v>Carlos Arbeladez-Jueves-13:00-19:00-06/08/2026/18:00-Corte de barba</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="D11" t="s">
-        <v>251</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="E12" t="s">
-        <v>252</v>
+        <v>239</v>
       </c>
     </row>
   </sheetData>
@@ -4957,20 +4896,20 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7A5AA025-A9A3-4E3E-A766-44885AA770B6}">
   <dimension ref="A1:D17"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="27" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="63.6640625" customWidth="1"/>
-    <col min="3" max="3" width="14.44140625" customWidth="1"/>
-    <col min="4" max="4" width="7.6640625" customWidth="1"/>
+    <col min="2" max="2" width="63.7109375" customWidth="1"/>
+    <col min="3" max="3" width="14.42578125" customWidth="1"/>
+    <col min="4" max="4" width="7.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
         <v>0</v>
       </c>
@@ -4984,7 +4923,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:4" ht="45" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
         <v>4</v>
       </c>
@@ -4998,12 +4937,12 @@
         <v>34</v>
       </c>
     </row>
-    <row r="4" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:4" ht="75" x14ac:dyDescent="0.25">
       <c r="A4" s="7" t="s">
         <v>11</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>147</v>
+        <v>140</v>
       </c>
       <c r="C4" s="7">
         <v>1</v>
@@ -5012,12 +4951,12 @@
         <v>34</v>
       </c>
     </row>
-    <row r="5" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:4" ht="60" x14ac:dyDescent="0.25">
       <c r="A5" s="7" t="s">
         <v>5</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>148</v>
+        <v>141</v>
       </c>
       <c r="C5" s="7">
         <v>2</v>
@@ -5026,12 +4965,12 @@
         <v>34</v>
       </c>
     </row>
-    <row r="6" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:4" ht="45" x14ac:dyDescent="0.25">
       <c r="A6" s="7" t="s">
         <v>72</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>149</v>
+        <v>142</v>
       </c>
       <c r="C6" s="7">
         <v>2</v>
@@ -5040,12 +4979,12 @@
         <v>34</v>
       </c>
     </row>
-    <row r="7" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:4" ht="60" x14ac:dyDescent="0.25">
       <c r="A7" s="7" t="s">
         <v>6</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>150</v>
+        <v>143</v>
       </c>
       <c r="C7" s="7">
         <v>2</v>
@@ -5054,7 +4993,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="8" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:4" ht="45" x14ac:dyDescent="0.25">
       <c r="A8" s="7" t="s">
         <v>7</v>
       </c>
@@ -5068,12 +5007,12 @@
         <v>34</v>
       </c>
     </row>
-    <row r="9" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:4" ht="75" x14ac:dyDescent="0.25">
       <c r="A9" s="7" t="s">
         <v>13</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>151</v>
+        <v>144</v>
       </c>
       <c r="C9" s="7">
         <v>2</v>
@@ -5082,7 +5021,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="10" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A10" s="7" t="s">
         <v>8</v>
       </c>
@@ -5096,12 +5035,12 @@
         <v>34</v>
       </c>
     </row>
-    <row r="11" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:4" ht="45" x14ac:dyDescent="0.25">
       <c r="A11" s="7" t="s">
         <v>9</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>152</v>
+        <v>145</v>
       </c>
       <c r="C11" s="7">
         <v>3</v>
@@ -5110,12 +5049,12 @@
         <v>34</v>
       </c>
     </row>
-    <row r="12" spans="1:4" ht="86.4" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:4" ht="90" x14ac:dyDescent="0.25">
       <c r="A12" s="7" t="s">
-        <v>193</v>
+        <v>184</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>228</v>
+        <v>218</v>
       </c>
       <c r="C12" s="7">
         <v>4</v>
@@ -5124,26 +5063,18 @@
         <v>34</v>
       </c>
     </row>
-    <row r="13" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A13" s="7" t="s">
-        <v>73</v>
-      </c>
-      <c r="B13" s="8" t="s">
-        <v>153</v>
-      </c>
-      <c r="C13" s="7">
-        <v>4</v>
-      </c>
-      <c r="D13" s="9" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" ht="72" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A13" s="7"/>
+      <c r="B13" s="8"/>
+      <c r="C13" s="7"/>
+      <c r="D13" s="9"/>
+    </row>
+    <row r="14" spans="1:4" ht="90" x14ac:dyDescent="0.25">
       <c r="A14" s="7" t="s">
         <v>10</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>154</v>
+        <v>146</v>
       </c>
       <c r="C14" s="7">
         <v>4</v>
@@ -5152,21 +5083,21 @@
         <v>34</v>
       </c>
     </row>
-    <row r="15" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:4" ht="60" x14ac:dyDescent="0.25">
       <c r="A15" s="7" t="s">
-        <v>194</v>
+        <v>185</v>
       </c>
       <c r="B15" s="8" t="s">
-        <v>195</v>
+        <v>186</v>
       </c>
       <c r="C15" s="7">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D15" s="9" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="16" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:4" ht="45" x14ac:dyDescent="0.25">
       <c r="A16" s="7" t="s">
         <v>12</v>
       </c>
@@ -5180,7 +5111,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="17" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:4" ht="60" x14ac:dyDescent="0.25">
       <c r="A17" s="7" t="s">
         <v>14</v>
       </c>
@@ -5209,7 +5140,6 @@
     <hyperlink ref="D17" location="CitaServicio_D!A1" display="aquí" xr:uid="{F49154C9-A497-4677-B686-F9CF5B536DEC}"/>
     <hyperlink ref="A1" location="'Modelo de Dominio'!A1" display="&lt;&lt;&lt;&lt; Ir al modulo de dominio" xr:uid="{A3D1E053-3C90-4C85-85FB-01CE6B92A5EE}"/>
     <hyperlink ref="D6" location="HorarioBarberia_D!A1" display="aquí" xr:uid="{CE45E0DE-1B75-4BE0-8664-81F7834039D9}"/>
-    <hyperlink ref="D13" location="HorarioBarbero_D!A1" display="aquí" xr:uid="{3B048927-BA4F-418A-BCDC-3E65406B8FD1}"/>
     <hyperlink ref="D12" location="Bloqueo_D!A1" display="aquí" xr:uid="{C19EA470-C149-4E7D-B95C-B02B73C07975}"/>
     <hyperlink ref="D15" location="Descanso_D!A1" display="aquí" xr:uid="{BA11B464-44BB-488E-84C7-707437A187F8}"/>
   </hyperlinks>
@@ -5220,98 +5150,98 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{387DE6AC-7D92-461D-9DD1-84082B531231}">
   <dimension ref="A1:B11"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="18.44140625" customWidth="1"/>
-    <col min="2" max="2" width="69.44140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="18.42578125" customWidth="1"/>
+    <col min="2" max="2" width="69.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
-        <v>162</v>
+        <v>153</v>
       </c>
       <c r="B1" s="7" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="55" t="s">
+        <v>154</v>
+      </c>
+      <c r="B2" s="55" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+      <c r="A3" s="56" t="s">
+        <v>155</v>
+      </c>
+      <c r="B3" s="65" t="s">
         <v>163</v>
       </c>
-      <c r="B2" s="55" t="s">
-        <v>171</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A3" s="56" t="s">
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" s="58" t="s">
+        <v>156</v>
+      </c>
+      <c r="B4" s="58" t="s">
         <v>164</v>
       </c>
-      <c r="B3" s="65" t="s">
-        <v>172</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A4" s="58" t="s">
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" s="57" t="s">
+        <v>231</v>
+      </c>
+      <c r="B5" s="66" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" s="59" t="s">
+        <v>157</v>
+      </c>
+      <c r="B6" s="59" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+      <c r="A7" s="60" t="s">
+        <v>158</v>
+      </c>
+      <c r="B7" s="67" t="s">
         <v>165</v>
       </c>
-      <c r="B4" s="58" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A5" s="57" t="s">
-        <v>241</v>
-      </c>
-      <c r="B5" s="66" t="s">
-        <v>242</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A6" s="59" t="s">
+    </row>
+    <row r="8" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+      <c r="A8" s="61" t="s">
+        <v>159</v>
+      </c>
+      <c r="B8" s="68" t="s">
         <v>166</v>
       </c>
-      <c r="B6" s="59" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A7" s="60" t="s">
-        <v>167</v>
-      </c>
-      <c r="B7" s="67" t="s">
-        <v>174</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A8" s="61" t="s">
-        <v>168</v>
-      </c>
-      <c r="B8" s="68" t="s">
-        <v>175</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" ht="43.2" x14ac:dyDescent="0.3">
+    </row>
+    <row r="9" spans="1:2" ht="45" x14ac:dyDescent="0.25">
       <c r="A9" s="62" t="s">
         <v>69</v>
       </c>
       <c r="B9" s="69" t="s">
-        <v>176</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" ht="30" x14ac:dyDescent="0.25">
       <c r="A10" s="63" t="s">
+        <v>160</v>
+      </c>
+      <c r="B10" s="63" t="s">
         <v>169</v>
       </c>
-      <c r="B10" s="63" t="s">
-        <v>178</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" ht="57.6" x14ac:dyDescent="0.3">
+    </row>
+    <row r="11" spans="1:2" ht="60" x14ac:dyDescent="0.25">
       <c r="A11" s="64" t="s">
+        <v>161</v>
+      </c>
+      <c r="B11" s="70" t="s">
         <v>170</v>
-      </c>
-      <c r="B11" s="70" t="s">
-        <v>179</v>
       </c>
     </row>
   </sheetData>
@@ -5321,15 +5251,15 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AAA22F8C-1648-4644-8301-765EB2B8C50B}">
-  <dimension ref="A1:C4"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:C6"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="33.88671875" customWidth="1"/>
-    <col min="2" max="2" width="34.6640625" customWidth="1"/>
+    <col min="1" max="1" width="33.85546875" customWidth="1"/>
+    <col min="2" max="2" width="34.7109375" customWidth="1"/>
     <col min="3" max="3" width="21" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
         <v>32</v>
       </c>
@@ -5337,15 +5267,15 @@
         <v>33</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="18" t="s">
         <v>20</v>
       </c>
       <c r="B2" s="18" t="s">
-        <v>210</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="13" t="s">
         <v>31</v>
       </c>
@@ -5354,7 +5284,7 @@
       </c>
       <c r="C3" s="35"/>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="12">
         <v>1</v>
       </c>
@@ -5362,6 +5292,11 @@
         <v>66</v>
       </c>
       <c r="C4" s="4"/>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B6" t="s">
+        <v>240</v>
+      </c>
     </row>
   </sheetData>
   <hyperlinks>
@@ -5375,15 +5310,15 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{28259140-2713-4A98-8730-76D57DC1D653}">
   <dimension ref="A1:H11"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="26.88671875" style="10" customWidth="1"/>
-    <col min="2" max="6" width="26.33203125" style="10" customWidth="1"/>
-    <col min="7" max="7" width="23.109375" style="10" customWidth="1"/>
-    <col min="8" max="8" width="38.5546875" style="10" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="26.85546875" style="10" customWidth="1"/>
+    <col min="2" max="6" width="26.28515625" style="10" customWidth="1"/>
+    <col min="7" max="7" width="23.140625" style="10" customWidth="1"/>
+    <col min="8" max="8" width="38.5703125" style="10" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="11" t="s">
         <v>32</v>
       </c>
@@ -5397,50 +5332,50 @@
       <c r="G1" s="12"/>
       <c r="H1" s="12"/>
     </row>
-    <row r="2" spans="1:8" ht="39.6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" ht="46.5" x14ac:dyDescent="0.25">
       <c r="A2" s="17" t="s">
         <v>20</v>
       </c>
       <c r="B2" s="17" t="s">
-        <v>180</v>
+        <v>171</v>
       </c>
       <c r="C2" s="17" t="s">
-        <v>181</v>
+        <v>172</v>
       </c>
       <c r="D2" s="17" t="s">
-        <v>182</v>
+        <v>173</v>
       </c>
       <c r="E2" s="17" t="s">
-        <v>183</v>
+        <v>174</v>
       </c>
       <c r="F2" s="17" t="s">
-        <v>218</v>
+        <v>208</v>
       </c>
       <c r="G2" s="18" t="s">
-        <v>184</v>
+        <v>175</v>
       </c>
       <c r="H2" s="19" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" s="13" t="s">
         <v>31</v>
       </c>
       <c r="B3" s="54" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="C3" s="54" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="D3" s="54" t="s">
-        <v>102</v>
+        <v>98</v>
       </c>
       <c r="E3" s="54" t="s">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="F3" s="71" t="s">
-        <v>155</v>
+        <v>147</v>
       </c>
       <c r="G3" s="71" t="s">
         <v>22</v>
@@ -5449,20 +5384,20 @@
         <v>69</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" s="12">
         <v>1</v>
       </c>
       <c r="B4" s="12" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="C4" s="12"/>
       <c r="D4" s="12" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="E4" s="12"/>
       <c r="F4" s="44" t="s">
-        <v>129</v>
+        <v>122</v>
       </c>
       <c r="G4" s="12">
         <v>3234528921</v>
@@ -5472,24 +5407,24 @@
         <v>Juan--Gómez--+57-3234528921</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" s="12">
         <v>2</v>
       </c>
       <c r="B5" s="12" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="C5" s="12" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="D5" s="12" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="E5" s="12" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="F5" s="44" t="s">
-        <v>129</v>
+        <v>122</v>
       </c>
       <c r="G5" s="12">
         <v>3161657782</v>
@@ -5499,22 +5434,22 @@
         <v>Jose-Miguel-Ramirez-Perez-+57-3161657782</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" s="12">
         <v>3</v>
       </c>
       <c r="B6" s="12" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="C6" s="12"/>
       <c r="D6" s="12" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="E6" s="12" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="F6" s="44" t="s">
-        <v>129</v>
+        <v>122</v>
       </c>
       <c r="G6" s="12">
         <v>3119884321</v>
@@ -5524,20 +5459,20 @@
         <v>Simon--Ochoa-Ramirez-+57-3119884321</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="12">
         <v>4</v>
       </c>
       <c r="B7" s="12" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="C7" s="12"/>
       <c r="D7" s="12" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="E7" s="12"/>
       <c r="F7" s="44" t="s">
-        <v>130</v>
+        <v>123</v>
       </c>
       <c r="G7" s="12">
         <v>4127359182</v>
@@ -5547,7 +5482,7 @@
         <v>Alexis--Gallego--+58-4127359182</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="C11"/>
     </row>
   </sheetData>
@@ -5563,17 +5498,17 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B0E77388-6266-4A55-B7A3-4FCD2B643D29}">
   <dimension ref="A1:F5"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="26.88671875" customWidth="1"/>
-    <col min="2" max="2" width="32.5546875" customWidth="1"/>
+    <col min="1" max="1" width="26.85546875" customWidth="1"/>
+    <col min="2" max="2" width="32.5703125" customWidth="1"/>
     <col min="3" max="3" width="28" customWidth="1"/>
-    <col min="4" max="4" width="26.6640625" customWidth="1"/>
-    <col min="5" max="5" width="16.33203125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="18.44140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="26.7109375" customWidth="1"/>
+    <col min="5" max="5" width="16.28515625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="18.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
         <v>32</v>
       </c>
@@ -5581,24 +5516,24 @@
         <v>33</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="49.2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:6" ht="46.5" x14ac:dyDescent="0.25">
       <c r="A2" s="17" t="s">
         <v>20</v>
       </c>
       <c r="B2" s="18" t="s">
-        <v>212</v>
+        <v>202</v>
       </c>
       <c r="C2" s="18" t="s">
-        <v>185</v>
+        <v>176</v>
       </c>
       <c r="D2" s="18" t="s">
-        <v>213</v>
+        <v>203</v>
       </c>
       <c r="E2" s="18" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="13" t="s">
         <v>31</v>
       </c>
@@ -5616,7 +5551,7 @@
       </c>
       <c r="F3" s="3"/>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="12">
         <v>1</v>
       </c>
@@ -5638,7 +5573,7 @@
         <v/>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="D5" s="2"/>
     </row>
   </sheetData>
@@ -5654,19 +5589,20 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2DAE59AB-4103-4731-9C3C-4C276F8A29F8}">
-  <dimension ref="A1:L11"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:L18"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="27" bestFit="1" customWidth="1"/>
-    <col min="2" max="6" width="26.6640625" customWidth="1"/>
-    <col min="7" max="7" width="16.33203125" customWidth="1"/>
-    <col min="8" max="9" width="40.6640625" customWidth="1"/>
-    <col min="10" max="10" width="30.33203125" customWidth="1"/>
+    <col min="2" max="6" width="26.7109375" customWidth="1"/>
+    <col min="7" max="7" width="16.28515625" customWidth="1"/>
+    <col min="8" max="8" width="40.7109375" customWidth="1"/>
+    <col min="9" max="9" width="67.5703125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="30.28515625" customWidth="1"/>
     <col min="11" max="11" width="21" customWidth="1"/>
-    <col min="12" max="12" width="53.109375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="53.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
         <v>32</v>
       </c>
@@ -5678,62 +5614,62 @@
       <c r="E1" s="5"/>
       <c r="F1" s="5"/>
     </row>
-    <row r="2" spans="1:12" ht="45.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:12" ht="45.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="25" t="s">
         <v>20</v>
       </c>
       <c r="B2" s="25" t="s">
-        <v>156</v>
+        <v>148</v>
       </c>
       <c r="C2" s="25" t="s">
-        <v>157</v>
+        <v>149</v>
       </c>
       <c r="D2" s="25" t="s">
-        <v>158</v>
+        <v>150</v>
       </c>
       <c r="E2" s="25" t="s">
-        <v>159</v>
+        <v>151</v>
       </c>
       <c r="F2" s="25" t="s">
-        <v>160</v>
+        <v>152</v>
       </c>
       <c r="G2" s="26" t="s">
-        <v>190</v>
+        <v>181</v>
       </c>
       <c r="H2" s="26" t="s">
-        <v>191</v>
+        <v>182</v>
       </c>
       <c r="I2" s="26" t="s">
-        <v>161</v>
+        <v>246</v>
       </c>
       <c r="J2" s="26" t="s">
-        <v>214</v>
+        <v>204</v>
       </c>
       <c r="K2" s="26" t="s">
-        <v>137</v>
+        <v>130</v>
       </c>
       <c r="L2" s="27" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A3" s="13" t="s">
         <v>31</v>
       </c>
       <c r="B3" s="54" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="C3" s="54" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="D3" s="54" t="s">
-        <v>102</v>
+        <v>98</v>
       </c>
       <c r="E3" s="54" t="s">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="F3" s="71" t="s">
-        <v>128</v>
+        <v>121</v>
       </c>
       <c r="G3" s="71" t="s">
         <v>22</v>
@@ -5742,7 +5678,7 @@
         <v>42</v>
       </c>
       <c r="I3" s="71" t="s">
-        <v>124</v>
+        <v>120</v>
       </c>
       <c r="J3" s="40" t="s">
         <v>43</v>
@@ -5754,24 +5690,24 @@
         <v>70</v>
       </c>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A4" s="12">
         <v>1</v>
       </c>
       <c r="B4" s="12" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="C4" s="12" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="D4" s="12" t="s">
-        <v>142</v>
+        <v>135</v>
       </c>
       <c r="E4" s="12" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="F4" s="44" t="s">
-        <v>129</v>
+        <v>122</v>
       </c>
       <c r="G4" s="12">
         <v>3245627890</v>
@@ -5779,8 +5715,8 @@
       <c r="H4" s="11" t="s">
         <v>53</v>
       </c>
-      <c r="I4" s="42">
-        <v>1264267821</v>
+      <c r="I4" s="42" t="s">
+        <v>241</v>
       </c>
       <c r="J4" s="12" t="s">
         <v>49</v>
@@ -5794,24 +5730,24 @@
         <v>Juan-Fernando-García-Lopez-+57-3245627890</v>
       </c>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A5" s="12">
         <v>2</v>
       </c>
       <c r="B5" s="12" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="C5" s="12" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="D5" s="12" t="s">
-        <v>141</v>
+        <v>134</v>
       </c>
       <c r="E5" s="12" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="F5" s="44" t="s">
-        <v>129</v>
+        <v>122</v>
       </c>
       <c r="G5" s="12">
         <v>3124518923</v>
@@ -5820,7 +5756,7 @@
         <v>54</v>
       </c>
       <c r="I5" s="42" t="s">
-        <v>126</v>
+        <v>242</v>
       </c>
       <c r="J5" s="12" t="s">
         <v>49</v>
@@ -5834,7 +5770,7 @@
         <v>Juan-David-Ortiz-Sanchez-+57-3124518923</v>
       </c>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A6" s="12">
         <v>3</v>
       </c>
@@ -5843,11 +5779,11 @@
       </c>
       <c r="C6" s="12"/>
       <c r="D6" s="12" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="E6" s="12"/>
       <c r="F6" s="44" t="s">
-        <v>129</v>
+        <v>122</v>
       </c>
       <c r="G6" s="12">
         <v>3214533321</v>
@@ -5856,7 +5792,7 @@
         <v>55</v>
       </c>
       <c r="I6" s="43" t="s">
-        <v>125</v>
+        <v>243</v>
       </c>
       <c r="J6" s="12" t="s">
         <v>49</v>
@@ -5870,7 +5806,7 @@
         <v>Carlos--Arbeladez--+57-3214533321</v>
       </c>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A7" s="12">
         <v>4</v>
       </c>
@@ -5879,13 +5815,13 @@
       </c>
       <c r="C7" s="12"/>
       <c r="D7" s="12" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="E7" s="12" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="F7" s="44" t="s">
-        <v>131</v>
+        <v>124</v>
       </c>
       <c r="G7" s="12">
         <v>9876543210</v>
@@ -5894,7 +5830,7 @@
         <v>56</v>
       </c>
       <c r="I7" s="42" t="s">
-        <v>127</v>
+        <v>244</v>
       </c>
       <c r="J7" s="12" t="s">
         <v>49</v>
@@ -5908,33 +5844,33 @@
         <v>Andres--Ramirez-Patiño-+91-9876543210</v>
       </c>
     </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A8" s="12">
         <v>5</v>
       </c>
       <c r="B8" s="12" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="C8" s="12" t="s">
         <v>51</v>
       </c>
       <c r="D8" s="12" t="s">
-        <v>143</v>
+        <v>136</v>
       </c>
       <c r="E8" s="12" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="F8" s="44" t="s">
-        <v>144</v>
+        <v>137</v>
       </c>
       <c r="G8" s="12">
         <v>998765432</v>
       </c>
       <c r="H8" s="11" t="s">
-        <v>145</v>
-      </c>
-      <c r="I8" s="12">
-        <v>312334342</v>
+        <v>138</v>
+      </c>
+      <c r="I8" s="12" t="s">
+        <v>245</v>
       </c>
       <c r="J8" s="12" t="s">
         <v>50</v>
@@ -5948,15 +5884,18 @@
         <v>Juan-Carlos-Zambrano-Perez-+593-998765432</v>
       </c>
     </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B10" s="10"/>
       <c r="C10" s="10"/>
-      <c r="I10" s="94" t="s">
-        <v>246</v>
-      </c>
-    </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="F11" s="92"/>
+      <c r="I10" s="93"/>
+    </row>
+    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="F11" s="91"/>
+    </row>
+    <row r="18" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C18" t="s">
+        <v>250</v>
+      </c>
     </row>
   </sheetData>
   <phoneticPr fontId="7" type="noConversion"/>
@@ -5980,17 +5919,17 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2190E1EC-B79B-40C0-AC5B-0E2726DDD399}">
   <dimension ref="A1:F12"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="27" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="26" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="34.44140625" customWidth="1"/>
-    <col min="4" max="4" width="23.5546875" customWidth="1"/>
-    <col min="5" max="5" width="23.6640625" customWidth="1"/>
-    <col min="6" max="6" width="34.77734375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="34.42578125" customWidth="1"/>
+    <col min="4" max="4" width="23.5703125" customWidth="1"/>
+    <col min="5" max="5" width="23.7109375" customWidth="1"/>
+    <col min="6" max="6" width="34.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
         <v>32</v>
       </c>
@@ -5998,47 +5937,47 @@
         <v>33</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="44.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:6" ht="44.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="18" t="s">
         <v>20</v>
       </c>
       <c r="B2" s="18" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C2" s="18" t="s">
-        <v>211</v>
+        <v>201</v>
       </c>
       <c r="D2" s="18" t="s">
-        <v>232</v>
+        <v>222</v>
       </c>
       <c r="E2" s="18" t="s">
-        <v>237</v>
+        <v>227</v>
       </c>
       <c r="F2" s="18" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="13" t="s">
         <v>31</v>
       </c>
       <c r="B3" s="31" t="s">
         <v>36</v>
       </c>
-      <c r="C3" s="84" t="s">
+      <c r="C3" s="83" t="s">
+        <v>74</v>
+      </c>
+      <c r="D3" s="73" t="s">
         <v>75</v>
       </c>
-      <c r="D3" s="73" t="s">
+      <c r="E3" s="74" t="s">
         <v>76</v>
-      </c>
-      <c r="E3" s="74" t="s">
-        <v>77</v>
       </c>
       <c r="F3" s="34" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="12">
         <v>1</v>
       </c>
@@ -6047,12 +5986,12 @@
         <v>Barbería Oriental</v>
       </c>
       <c r="C4" s="36" t="s">
-        <v>78</v>
-      </c>
-      <c r="D4" s="89">
+        <v>77</v>
+      </c>
+      <c r="D4" s="88">
         <v>0.375</v>
       </c>
-      <c r="E4" s="89">
+      <c r="E4" s="88">
         <v>0.79166666666666663</v>
       </c>
       <c r="F4" s="12" t="str">
@@ -6060,7 +5999,7 @@
         <v>Barbería Oriental-Lunes-09:00-19:00</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="12">
         <v>2</v>
       </c>
@@ -6069,12 +6008,12 @@
         <v>Barbería Oriental</v>
       </c>
       <c r="C5" s="12" t="s">
-        <v>79</v>
-      </c>
-      <c r="D5" s="89">
+        <v>78</v>
+      </c>
+      <c r="D5" s="88">
         <v>0.375</v>
       </c>
-      <c r="E5" s="89">
+      <c r="E5" s="88">
         <v>0.79166666666666663</v>
       </c>
       <c r="F5" s="12" t="str">
@@ -6082,7 +6021,7 @@
         <v>Barbería Oriental-Martes-09:00-19:00</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="12">
         <v>3</v>
       </c>
@@ -6091,12 +6030,12 @@
         <v>Barbería Oriental</v>
       </c>
       <c r="C6" s="36" t="s">
-        <v>80</v>
-      </c>
-      <c r="D6" s="89">
+        <v>79</v>
+      </c>
+      <c r="D6" s="88">
         <v>0.375</v>
       </c>
-      <c r="E6" s="89">
+      <c r="E6" s="88">
         <v>0.79166666666666696</v>
       </c>
       <c r="F6" s="12" t="str">
@@ -6104,7 +6043,7 @@
         <v>Barbería Oriental-Miércoles-09:00-19:00</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="12">
         <v>4</v>
       </c>
@@ -6113,12 +6052,12 @@
         <v>Barbería Oriental</v>
       </c>
       <c r="C7" s="12" t="s">
-        <v>81</v>
-      </c>
-      <c r="D7" s="89">
+        <v>80</v>
+      </c>
+      <c r="D7" s="88">
         <v>0.375</v>
       </c>
-      <c r="E7" s="89">
+      <c r="E7" s="88">
         <v>0.79166666666666696</v>
       </c>
       <c r="F7" s="12" t="str">
@@ -6126,7 +6065,7 @@
         <v>Barbería Oriental-Jueves-09:00-19:00</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="12">
         <v>5</v>
       </c>
@@ -6135,12 +6074,12 @@
         <v>Barbería Oriental</v>
       </c>
       <c r="C8" s="36" t="s">
-        <v>82</v>
-      </c>
-      <c r="D8" s="89">
+        <v>81</v>
+      </c>
+      <c r="D8" s="88">
         <v>0.375</v>
       </c>
-      <c r="E8" s="89">
+      <c r="E8" s="88">
         <v>0.79166666666666696</v>
       </c>
       <c r="F8" s="12" t="str">
@@ -6148,7 +6087,7 @@
         <v>Barbería Oriental-Viernes-09:00-19:00</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="12">
         <v>6</v>
       </c>
@@ -6157,12 +6096,12 @@
         <v>Barbería Oriental</v>
       </c>
       <c r="C9" s="12" t="s">
-        <v>83</v>
-      </c>
-      <c r="D9" s="90">
+        <v>82</v>
+      </c>
+      <c r="D9" s="89">
         <v>0.33333333333333331</v>
       </c>
-      <c r="E9" s="89">
+      <c r="E9" s="88">
         <v>0.875</v>
       </c>
       <c r="F9" s="12" t="str">
@@ -6170,7 +6109,7 @@
         <v>Barbería Oriental-Sábado-08:00-21:00</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="12">
         <v>7</v>
       </c>
@@ -6179,12 +6118,12 @@
         <v>Barbería Oriental</v>
       </c>
       <c r="C10" s="36" t="s">
-        <v>243</v>
-      </c>
-      <c r="D10" s="89">
+        <v>233</v>
+      </c>
+      <c r="D10" s="88">
         <v>0.41666666666666669</v>
       </c>
-      <c r="E10" s="89">
+      <c r="E10" s="88">
         <v>0.625</v>
       </c>
       <c r="F10" s="12" t="str">
@@ -6192,14 +6131,14 @@
         <v>Barbería Oriental-Festivo-10:00-15:00</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="10"/>
       <c r="C11" s="10"/>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="10"/>
-      <c r="C12" s="95" t="s">
-        <v>247</v>
+      <c r="C12" s="94" t="s">
+        <v>236</v>
       </c>
     </row>
   </sheetData>
@@ -6223,16 +6162,16 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C97B567D-D27E-4BE3-B1E4-8CA267790151}">
   <dimension ref="A1:F12"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="2" width="28.109375" customWidth="1"/>
-    <col min="3" max="3" width="26.5546875" customWidth="1"/>
-    <col min="4" max="4" width="24.44140625" customWidth="1"/>
-    <col min="5" max="5" width="25.33203125" customWidth="1"/>
-    <col min="6" max="6" width="26.5546875" customWidth="1"/>
+    <col min="1" max="2" width="28.140625" customWidth="1"/>
+    <col min="3" max="3" width="26.5703125" customWidth="1"/>
+    <col min="4" max="4" width="24.42578125" customWidth="1"/>
+    <col min="5" max="5" width="25.28515625" customWidth="1"/>
+    <col min="6" max="6" width="26.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="15" t="s">
         <v>32</v>
       </c>
@@ -6243,27 +6182,27 @@
       <c r="E1" s="16"/>
       <c r="F1" s="10"/>
     </row>
-    <row r="2" spans="1:6" ht="45.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:6" ht="45.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="17" t="s">
         <v>20</v>
       </c>
       <c r="B2" s="17" t="s">
-        <v>136</v>
+        <v>129</v>
       </c>
       <c r="C2" s="17" t="s">
-        <v>186</v>
+        <v>177</v>
       </c>
       <c r="D2" s="30" t="s">
-        <v>188</v>
+        <v>179</v>
       </c>
       <c r="E2" s="30" t="s">
-        <v>189</v>
+        <v>180</v>
       </c>
       <c r="F2" s="18" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="20" t="s">
         <v>31</v>
       </c>
@@ -6280,10 +6219,10 @@
         <v>24</v>
       </c>
       <c r="F3" s="14" t="s">
-        <v>187</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="21">
         <v>1</v>
       </c>
@@ -6305,7 +6244,7 @@
         <v>Motilada</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="21">
         <v>2</v>
       </c>
@@ -6327,7 +6266,7 @@
         <v>Corte de barba</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="21">
         <v>3</v>
       </c>
@@ -6349,7 +6288,7 @@
         <v>Perfilada de barba</v>
       </c>
     </row>
-    <row r="7" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A7" s="21">
         <v>4</v>
       </c>
@@ -6371,37 +6310,37 @@
         <v>Arreglo completo de barba con toalla caliente</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="16"/>
       <c r="B8" s="16"/>
       <c r="C8" s="16"/>
       <c r="D8" s="16"/>
       <c r="E8" s="16"/>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="16"/>
       <c r="B9" s="16"/>
       <c r="C9" s="16"/>
       <c r="D9" s="16"/>
       <c r="E9" s="16"/>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="16"/>
       <c r="B10" s="16" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="C10" s="16"/>
       <c r="D10" s="16"/>
       <c r="E10" s="16"/>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="16"/>
       <c r="B11" s="16"/>
       <c r="C11" s="16"/>
       <c r="D11" s="16"/>
       <c r="E11" s="16"/>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="16"/>
       <c r="B12" s="16"/>
       <c r="C12" s="16"/>

</xml_diff>

<commit_message>
Se corrigio la escritura de algunas descripciones
</commit_message>
<xml_diff>
--- a/Muestreo de datos.xlsx
+++ b/Muestreo de datos.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/120f6d501c463b80/Escritorio/leo/Doo/Barberia proyecto/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="121" documentId="13_ncr:1_{2E66909D-5601-4FD5-B019-CA621521DC3F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F103FF16-41A8-4BCB-BBF4-5C255915BAED}"/>
+  <xr:revisionPtr revIDLastSave="126" documentId="13_ncr:1_{2E66909D-5601-4FD5-B019-CA621521DC3F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FE4CB7E7-522D-4B04-A5F9-A71D0E45BE7F}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" firstSheet="8" activeTab="16" xr2:uid="{09A6C7D7-663F-4C06-9D71-8A4E97495CF9}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" firstSheet="8" activeTab="15" xr2:uid="{09A6C7D7-663F-4C06-9D71-8A4E97495CF9}"/>
   </bookViews>
   <sheets>
     <sheet name="Modelo de Dominio" sheetId="1" r:id="rId1"/>
@@ -478,9 +478,6 @@
     <t>Combinacion única que indica que no puede existir más de un barbero con el mismo nombre, apellidos y número de celular</t>
   </si>
   <si>
-    <t>Representa a la persona que solicita citas en la barbería, el se las pide a un barbero por WhatsApp. Su valor esta en darle al sistema un historial por persona: que citas ha pedido, que multas tiene y si esta o no vetado, para que cualquier barbero sepa con quien esta tratando antes de agendarle.</t>
-  </si>
-  <si>
     <t>Representa las políticas de la barbería frente al incumplimiento de los clientes: cuantos minutos de tolerancia se dan antes de considerar tardanza, cuanto vale la multa fija por llegar tarde, y cuantas multas sin pagar activan un veto</t>
   </si>
   <si>
@@ -713,9 +710,6 @@
     <t>fechaHoraFinal</t>
   </si>
   <si>
-    <t>Representa un momento puntual en una fecha y hora específica, en el que un barbero no puede trabajar por un compromiso personal, aunque ese día normalmente sí trabaje según su horario. A diferencia de Descanso, no se repite semana a semana: aplica solo para esa fecha y hora, y es lo que le permite a la agenda del barbero reflejar cambios temporales sin alterar su horario habitual.</t>
-  </si>
-  <si>
     <t>Representa la fecha y la hora en el que va a empezar el bloqueo para la agenda del barbero. Su valor por defecto es 01/01/1000 00:00 y no es permitido. No se puden seleccionar fechas antes del momento de hoy, solo fechas futuras</t>
   </si>
   <si>
@@ -810,6 +804,12 @@
   </si>
   <si>
     <t xml:space="preserve">El barbero neceta conocer el presente y el futuro o tambien el pasado </t>
+  </si>
+  <si>
+    <t>Representa a la persona que solicita citas en la barbería, el se las pide a un barbero por WhatsApp. Su valor esta en darle al sistema un historial por persona: que citas ha pedido, que multas tiene y si esta o no vetado, para que cualquier barbero sepa con quien esta tratando antes de agendarle</t>
+  </si>
+  <si>
+    <t>Representa un momento puntual en una fecha y hora específica, en el que un barbero no puede trabajar por un compromiso personal, aunque ese día normalmente sí trabaje según su horario. A diferencia de Descanso, no se repite semana a semana: aplica solo para esa fecha y hora, y es lo que le permite a la agenda del barbero reflejar cambios temporales sin alterar su horario habitual</t>
   </si>
 </sst>
 </file>
@@ -1006,7 +1006,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="100">
+  <cellXfs count="99">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -1259,10 +1259,7 @@
     <xf numFmtId="20" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="18" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="18" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="18" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -3337,16 +3334,16 @@
         <v>20</v>
       </c>
       <c r="B2" s="17" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="C2" s="17" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="D2" s="17" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="E2" s="30" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="F2" s="30" t="s">
         <v>119</v>
@@ -3360,13 +3357,13 @@
         <v>31</v>
       </c>
       <c r="B3" s="31" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="C3" s="31" t="s">
         <v>59</v>
       </c>
       <c r="D3" s="31" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="E3" s="40" t="s">
         <v>25</v>
@@ -3492,7 +3489,7 @@
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="E10" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
@@ -3689,15 +3686,15 @@
         <v>118</v>
       </c>
       <c r="C2" s="17" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="D2" s="17"/>
       <c r="E2" s="17"/>
       <c r="F2" s="17" t="s">
+        <v>224</v>
+      </c>
+      <c r="G2" s="17" t="s">
         <v>226</v>
-      </c>
-      <c r="G2" s="17" t="s">
-        <v>228</v>
       </c>
       <c r="H2" s="18" t="s">
         <v>83</v>
@@ -3714,16 +3711,16 @@
         <v>74</v>
       </c>
       <c r="D3" s="31" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="E3" s="31" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="F3" s="95" t="s">
         <v>63</v>
       </c>
       <c r="G3" s="95" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="H3" s="28" t="s">
         <v>69</v>
@@ -3846,7 +3843,7 @@
         <v>Andres Ramirez</v>
       </c>
       <c r="C8" s="12" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="D8" s="11"/>
       <c r="E8" s="11"/>
@@ -3907,22 +3904,22 @@
         <v>20</v>
       </c>
       <c r="B2" s="18" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="C2" s="30" t="s">
+        <v>217</v>
+      </c>
+      <c r="D2" s="30" t="s">
+        <v>218</v>
+      </c>
+      <c r="E2" s="18" t="s">
+        <v>205</v>
+      </c>
+      <c r="F2" s="18" t="s">
         <v>219</v>
       </c>
-      <c r="D2" s="30" t="s">
-        <v>220</v>
-      </c>
-      <c r="E2" s="18" t="s">
-        <v>206</v>
-      </c>
-      <c r="F2" s="18" t="s">
-        <v>221</v>
-      </c>
       <c r="G2" s="18" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
@@ -3933,10 +3930,10 @@
         <v>60</v>
       </c>
       <c r="C3" s="85" t="s">
+        <v>215</v>
+      </c>
+      <c r="D3" s="85" t="s">
         <v>216</v>
-      </c>
-      <c r="D3" s="85" t="s">
-        <v>217</v>
       </c>
       <c r="E3" s="84" t="s">
         <v>21</v>
@@ -3963,7 +3960,7 @@
         <v>46047.541666666664</v>
       </c>
       <c r="E4" s="79" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="F4" s="12">
         <v>120</v>
@@ -3988,7 +3985,7 @@
         <v>45362.645833333336</v>
       </c>
       <c r="E5" s="80" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="F5" s="12">
         <v>210</v>
@@ -4013,7 +4010,7 @@
         <v>46013.583333333336</v>
       </c>
       <c r="E6" s="80" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="F6" s="12">
         <v>60</v>
@@ -4038,7 +4035,7 @@
         <v>46241.5</v>
       </c>
       <c r="E7" s="80" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="F7" s="12">
         <v>180</v>
@@ -4089,22 +4086,22 @@
         <v>20</v>
       </c>
       <c r="B2" s="18" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="C2" s="18" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="D2" s="18" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="E2" s="18" t="s">
+        <v>211</v>
+      </c>
+      <c r="F2" s="30" t="s">
         <v>212</v>
       </c>
-      <c r="F2" s="30" t="s">
-        <v>213</v>
-      </c>
       <c r="G2" s="18" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
@@ -4118,7 +4115,7 @@
         <v>63</v>
       </c>
       <c r="D3" s="74" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="E3" s="71" t="s">
         <v>21</v>
@@ -4145,7 +4142,7 @@
         <v>0.58333333333333337</v>
       </c>
       <c r="E4" s="36" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="F4" s="82">
         <v>120</v>
@@ -4170,7 +4167,7 @@
         <v>0.54166666666666663</v>
       </c>
       <c r="E5" s="24" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="F5" s="12">
         <v>120</v>
@@ -4195,7 +4192,7 @@
         <v>0.60416666666666663</v>
       </c>
       <c r="E6" s="12" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="F6" s="12">
         <v>60</v>
@@ -4220,7 +4217,7 @@
         <v>0.54166666666666663</v>
       </c>
       <c r="E7" s="12" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="F7" s="12">
         <v>90</v>
@@ -4231,20 +4228,20 @@
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C9" s="98"/>
-      <c r="D9" s="98"/>
+      <c r="C9" s="94"/>
+      <c r="D9" s="94"/>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C10" s="98"/>
-      <c r="D10" s="99"/>
+      <c r="C10" s="94"/>
+      <c r="D10" s="98"/>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C11" s="98"/>
-      <c r="D11" s="98"/>
+      <c r="C11" s="94"/>
+      <c r="D11" s="94"/>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C12" s="98"/>
-      <c r="D12" s="98"/>
+      <c r="C12" s="94"/>
+      <c r="D12" s="94"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -4271,7 +4268,7 @@
     <col min="4" max="4" width="27.5703125" customWidth="1"/>
     <col min="5" max="5" width="36.5703125" customWidth="1"/>
     <col min="6" max="6" width="60.28515625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="39.28515625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="49.28515625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="22" customWidth="1"/>
   </cols>
   <sheetData>
@@ -4294,13 +4291,13 @@
         <v>131</v>
       </c>
       <c r="D2" s="30" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="E2" s="30" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="F2" s="30" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="G2" s="30" t="s">
         <v>126</v>
@@ -4320,7 +4317,7 @@
         <v>125</v>
       </c>
       <c r="E3" s="40" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="F3" s="54" t="s">
         <v>26</v>
@@ -4513,10 +4510,10 @@
   <cols>
     <col min="1" max="1" width="26.7109375" customWidth="1"/>
     <col min="2" max="2" width="38.5703125" customWidth="1"/>
-    <col min="3" max="3" width="39.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="49.7109375" bestFit="1" customWidth="1"/>
     <col min="4" max="5" width="39.7109375" customWidth="1"/>
     <col min="6" max="6" width="34.28515625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="39.28515625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="49.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
@@ -4538,7 +4535,7 @@
         <v>89</v>
       </c>
       <c r="D2" s="30" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="E2" s="30" t="s">
         <v>133</v>
@@ -4692,7 +4689,7 @@
         <v>93</v>
       </c>
       <c r="D2" s="30" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="E2" s="30" t="s">
         <v>94</v>
@@ -4861,12 +4858,12 @@
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="D11" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="E12" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
     </row>
   </sheetData>
@@ -4942,7 +4939,7 @@
         <v>11</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>140</v>
+        <v>249</v>
       </c>
       <c r="C4" s="7">
         <v>1</v>
@@ -4956,7 +4953,7 @@
         <v>5</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C5" s="7">
         <v>2</v>
@@ -4970,7 +4967,7 @@
         <v>72</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="C6" s="7">
         <v>2</v>
@@ -4984,7 +4981,7 @@
         <v>6</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="C7" s="7">
         <v>2</v>
@@ -5012,7 +5009,7 @@
         <v>13</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C9" s="7">
         <v>2</v>
@@ -5040,7 +5037,7 @@
         <v>9</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="C11" s="7">
         <v>3</v>
@@ -5051,10 +5048,10 @@
     </row>
     <row r="12" spans="1:4" ht="90" x14ac:dyDescent="0.25">
       <c r="A12" s="7" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>218</v>
+        <v>250</v>
       </c>
       <c r="C12" s="7">
         <v>4</v>
@@ -5074,7 +5071,7 @@
         <v>10</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C14" s="7">
         <v>4</v>
@@ -5085,10 +5082,10 @@
     </row>
     <row r="15" spans="1:4" ht="60" x14ac:dyDescent="0.25">
       <c r="A15" s="7" t="s">
+        <v>184</v>
+      </c>
+      <c r="B15" s="8" t="s">
         <v>185</v>
-      </c>
-      <c r="B15" s="8" t="s">
-        <v>186</v>
       </c>
       <c r="C15" s="7">
         <v>4</v>
@@ -5158,7 +5155,7 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="B1" s="7" t="s">
         <v>1</v>
@@ -5166,58 +5163,58 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="55" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="B2" s="55" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="30" x14ac:dyDescent="0.25">
       <c r="A3" s="56" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="B3" s="65" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="58" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="B4" s="58" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="57" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="B5" s="66" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="59" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="B6" s="59" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="30" x14ac:dyDescent="0.25">
       <c r="A7" s="60" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="B7" s="67" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
     </row>
     <row r="8" spans="1:2" ht="30" x14ac:dyDescent="0.25">
       <c r="A8" s="61" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="B8" s="68" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
     </row>
     <row r="9" spans="1:2" ht="45" x14ac:dyDescent="0.25">
@@ -5225,23 +5222,23 @@
         <v>69</v>
       </c>
       <c r="B9" s="69" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
     </row>
     <row r="10" spans="1:2" ht="30" x14ac:dyDescent="0.25">
       <c r="A10" s="63" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="B10" s="63" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
     </row>
     <row r="11" spans="1:2" ht="60" x14ac:dyDescent="0.25">
       <c r="A11" s="64" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="B11" s="70" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
   </sheetData>
@@ -5272,7 +5269,7 @@
         <v>20</v>
       </c>
       <c r="B2" s="18" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -5295,7 +5292,7 @@
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B6" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
     </row>
   </sheetData>
@@ -5337,22 +5334,22 @@
         <v>20</v>
       </c>
       <c r="B2" s="17" t="s">
+        <v>170</v>
+      </c>
+      <c r="C2" s="17" t="s">
         <v>171</v>
       </c>
-      <c r="C2" s="17" t="s">
+      <c r="D2" s="17" t="s">
         <v>172</v>
       </c>
-      <c r="D2" s="17" t="s">
+      <c r="E2" s="17" t="s">
         <v>173</v>
       </c>
-      <c r="E2" s="17" t="s">
+      <c r="F2" s="17" t="s">
+        <v>207</v>
+      </c>
+      <c r="G2" s="18" t="s">
         <v>174</v>
-      </c>
-      <c r="F2" s="17" t="s">
-        <v>208</v>
-      </c>
-      <c r="G2" s="18" t="s">
-        <v>175</v>
       </c>
       <c r="H2" s="19" t="s">
         <v>128</v>
@@ -5375,7 +5372,7 @@
         <v>100</v>
       </c>
       <c r="F3" s="71" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="G3" s="71" t="s">
         <v>22</v>
@@ -5521,13 +5518,13 @@
         <v>20</v>
       </c>
       <c r="B2" s="18" t="s">
+        <v>201</v>
+      </c>
+      <c r="C2" s="18" t="s">
+        <v>175</v>
+      </c>
+      <c r="D2" s="18" t="s">
         <v>202</v>
-      </c>
-      <c r="C2" s="18" t="s">
-        <v>176</v>
-      </c>
-      <c r="D2" s="18" t="s">
-        <v>203</v>
       </c>
       <c r="E2" s="18" t="s">
         <v>68</v>
@@ -5619,31 +5616,31 @@
         <v>20</v>
       </c>
       <c r="B2" s="25" t="s">
+        <v>147</v>
+      </c>
+      <c r="C2" s="25" t="s">
         <v>148</v>
       </c>
-      <c r="C2" s="25" t="s">
+      <c r="D2" s="25" t="s">
         <v>149</v>
       </c>
-      <c r="D2" s="25" t="s">
+      <c r="E2" s="25" t="s">
         <v>150</v>
       </c>
-      <c r="E2" s="25" t="s">
+      <c r="F2" s="25" t="s">
         <v>151</v>
       </c>
-      <c r="F2" s="25" t="s">
-        <v>152</v>
-      </c>
       <c r="G2" s="26" t="s">
+        <v>180</v>
+      </c>
+      <c r="H2" s="26" t="s">
         <v>181</v>
       </c>
-      <c r="H2" s="26" t="s">
-        <v>182</v>
-      </c>
       <c r="I2" s="26" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="J2" s="26" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="K2" s="26" t="s">
         <v>130</v>
@@ -5716,7 +5713,7 @@
         <v>53</v>
       </c>
       <c r="I4" s="42" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="J4" s="12" t="s">
         <v>49</v>
@@ -5756,7 +5753,7 @@
         <v>54</v>
       </c>
       <c r="I5" s="42" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="J5" s="12" t="s">
         <v>49</v>
@@ -5792,7 +5789,7 @@
         <v>55</v>
       </c>
       <c r="I6" s="43" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="J6" s="12" t="s">
         <v>49</v>
@@ -5830,7 +5827,7 @@
         <v>56</v>
       </c>
       <c r="I7" s="42" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="J7" s="12" t="s">
         <v>49</v>
@@ -5870,7 +5867,7 @@
         <v>138</v>
       </c>
       <c r="I8" s="12" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="J8" s="12" t="s">
         <v>50</v>
@@ -5894,7 +5891,7 @@
     </row>
     <row r="18" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C18" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
     </row>
   </sheetData>
@@ -5945,13 +5942,13 @@
         <v>73</v>
       </c>
       <c r="C2" s="18" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="D2" s="18" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="E2" s="18" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="F2" s="18" t="s">
         <v>117</v>
@@ -6118,7 +6115,7 @@
         <v>Barbería Oriental</v>
       </c>
       <c r="C10" s="36" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="D10" s="88">
         <v>0.41666666666666669</v>
@@ -6138,7 +6135,7 @@
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="10"/>
       <c r="C12" s="94" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
     </row>
   </sheetData>
@@ -6190,13 +6187,13 @@
         <v>129</v>
       </c>
       <c r="C2" s="17" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="D2" s="30" t="s">
+        <v>178</v>
+      </c>
+      <c r="E2" s="30" t="s">
         <v>179</v>
-      </c>
-      <c r="E2" s="30" t="s">
-        <v>180</v>
       </c>
       <c r="F2" s="18" t="s">
         <v>45</v>
@@ -6219,7 +6216,7 @@
         <v>24</v>
       </c>
       <c r="F3" s="14" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
@@ -6327,7 +6324,7 @@
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="16"/>
       <c r="B10" s="16" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="C10" s="16"/>
       <c r="D10" s="16"/>

</xml_diff>